<commit_message>
Exclude VAT account from forecast workbook
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/توقع_الفوترة_2026_2027.xlsx
+++ b/توقع_الفوترة_2026_2027.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'التوقعات'!$A$3:$N$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'التوقعات'!$A$3:$N$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1111,17 +1111,17 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>11411</t>
+          <t>144122</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>قيمة الضريبة المضافة</t>
+          <t>إيرادات  متنوعه</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>ضريبة</t>
+          <t>أخرى</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
@@ -1130,16 +1130,16 @@
         </is>
       </c>
       <c r="E13" s="6" t="n">
-        <v>141386313.02</v>
+        <v>9941900.57</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>135239152.29</v>
+        <v>14133817.21</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>123116638.31</v>
+        <v>80747739.2</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>123877773.31</v>
+        <v>316496963.26</v>
       </c>
       <c r="I13" s="6">
         <f>IF(D13="متوقف",0,H13*الافتراضات!$B$4)</f>
@@ -1150,7 +1150,7 @@
         <v/>
       </c>
       <c r="K13" s="7">
-        <f>IF(D13="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.066843)))</f>
+        <f>IF(D13="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,1.849906)))</f>
         <v/>
       </c>
       <c r="L13" s="6">
@@ -1161,22 +1161,26 @@
         <f>IF(G13=0,"",I13/G13-1)</f>
         <v/>
       </c>
-      <c r="N13" s="5" t="inlineStr"/>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>تذبذب عالٍ – راجع التوقع</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>144122</t>
+          <t>1421911</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>إيرادات  متنوعه</t>
+          <t>رسم مبيعات محلات تقديم منتجات التبغ</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>أخرى</t>
+          <t>التبغ والإيواء</t>
         </is>
       </c>
       <c r="D14" s="5" t="inlineStr">
@@ -1185,16 +1189,16 @@
         </is>
       </c>
       <c r="E14" s="6" t="n">
-        <v>9941900.57</v>
+        <v>75066033.04000001</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>14133817.21</v>
+        <v>142202773.54</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>80747739.2</v>
+        <v>105455179.58</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>316496963.26</v>
+        <v>80723092.94</v>
       </c>
       <c r="I14" s="6">
         <f>IF(D14="متوقف",0,H14*الافتراضات!$B$4)</f>
@@ -1205,7 +1209,7 @@
         <v/>
       </c>
       <c r="K14" s="7">
-        <f>IF(D14="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,1.849906)))</f>
+        <f>IF(D14="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.185256)))</f>
         <v/>
       </c>
       <c r="L14" s="6">
@@ -1216,26 +1220,22 @@
         <f>IF(G14=0,"",I14/G14-1)</f>
         <v/>
       </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>تذبذب عالٍ – راجع التوقع</t>
-        </is>
-      </c>
+      <c r="N14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>1421911</t>
+          <t>1421909</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>رسم مبيعات محلات تقديم منتجات التبغ</t>
+          <t>جمع النفايات</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t>التبغ والإيواء</t>
+          <t>الرسوم والتراخيص</t>
         </is>
       </c>
       <c r="D15" s="5" t="inlineStr">
@@ -1244,16 +1244,16 @@
         </is>
       </c>
       <c r="E15" s="6" t="n">
-        <v>75066033.04000001</v>
+        <v>83027851.53</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>142202773.54</v>
+        <v>89269940.62</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>105455179.58</v>
+        <v>80988493.83</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>80723092.94</v>
+        <v>79213506.2</v>
       </c>
       <c r="I15" s="6">
         <f>IF(D15="متوقف",0,H15*الافتراضات!$B$4)</f>
@@ -1264,7 +1264,7 @@
         <v/>
       </c>
       <c r="K15" s="7">
-        <f>IF(D15="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.185256)))</f>
+        <f>IF(D15="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.012358)))</f>
         <v/>
       </c>
       <c r="L15" s="6">
@@ -1280,12 +1280,12 @@
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>1421909</t>
+          <t>11452105</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>جمع النفايات</t>
+          <t>رسوم تراخيص حفر الشوارع</t>
         </is>
       </c>
       <c r="C16" s="5" t="inlineStr">
@@ -1299,16 +1299,16 @@
         </is>
       </c>
       <c r="E16" s="6" t="n">
-        <v>83027851.53</v>
+        <v>66884899.97</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>89269940.62</v>
+        <v>65467285.9</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>80988493.83</v>
+        <v>634736.47</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>79213506.2</v>
+        <v>1350</v>
       </c>
       <c r="I16" s="6">
         <f>IF(D16="متوقف",0,H16*الافتراضات!$B$4)</f>
@@ -1319,7 +1319,7 @@
         <v/>
       </c>
       <c r="K16" s="7">
-        <f>IF(D16="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.012358)))</f>
+        <f>IF(D16="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.902583)))</f>
         <v/>
       </c>
       <c r="L16" s="6">
@@ -1335,12 +1335,12 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>11452105</t>
+          <t>11452108</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>رسوم تراخيص حفر الشوارع</t>
+          <t>ايراد اصدار القرارات المساحية - أمانة منطقة الرياض</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -1354,16 +1354,16 @@
         </is>
       </c>
       <c r="E17" s="6" t="n">
-        <v>66884899.97</v>
+        <v>4422269.64</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>65467285.9</v>
+        <v>19704385.4</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>634736.47</v>
+        <v>26909388.87</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>1350</v>
+        <v>34133807.25</v>
       </c>
       <c r="I17" s="6">
         <f>IF(D17="متوقف",0,H17*الافتراضات!$B$4)</f>
@@ -1374,7 +1374,7 @@
         <v/>
       </c>
       <c r="K17" s="7">
-        <f>IF(D17="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.902583)))</f>
+        <f>IF(D17="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,1.466774)))</f>
         <v/>
       </c>
       <c r="L17" s="6">
@@ -1390,12 +1390,12 @@
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>11452108</t>
+          <t>1422108</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>ايراد اصدار القرارات المساحية - أمانة منطقة الرياض</t>
+          <t>الشهادات الصحية</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
@@ -1409,16 +1409,16 @@
         </is>
       </c>
       <c r="E18" s="6" t="n">
-        <v>4422269.64</v>
+        <v>21268656.03</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>19704385.4</v>
+        <v>13869671.08</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>26909388.87</v>
+        <v>26299399.74</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>34133807.25</v>
+        <v>21634358.52</v>
       </c>
       <c r="I18" s="6">
         <f>IF(D18="متوقف",0,H18*الافتراضات!$B$4)</f>
@@ -1429,7 +1429,7 @@
         <v/>
       </c>
       <c r="K18" s="7">
-        <f>IF(D18="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,1.466774)))</f>
+        <f>IF(D18="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.111995)))</f>
         <v/>
       </c>
       <c r="L18" s="6">
@@ -1445,17 +1445,17 @@
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>1422108</t>
+          <t>1422121</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>الشهادات الصحية</t>
+          <t>رسم ترخيص نشاط تقديم منتجات التبغ</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>الرسوم والتراخيص</t>
+          <t>التبغ والإيواء</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
@@ -1464,16 +1464,16 @@
         </is>
       </c>
       <c r="E19" s="6" t="n">
-        <v>21268656.03</v>
+        <v>16987800</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>13869671.08</v>
+        <v>18210000</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>26299399.74</v>
+        <v>16212478.8</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>21634358.52</v>
+        <v>14308008.01</v>
       </c>
       <c r="I19" s="6">
         <f>IF(D19="متوقف",0,H19*الافتراضات!$B$4)</f>
@@ -1484,7 +1484,7 @@
         <v/>
       </c>
       <c r="K19" s="7">
-        <f>IF(D19="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.111995)))</f>
+        <f>IF(D19="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.023086)))</f>
         <v/>
       </c>
       <c r="L19" s="6">
@@ -1500,17 +1500,17 @@
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>1422121</t>
+          <t>بدون رقم</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>رسم ترخيص نشاط تقديم منتجات التبغ</t>
+          <t>بدون رقم (خدمات علم + جزاءات)</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>التبغ والإيواء</t>
+          <t>علم / جزاءات</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
@@ -1519,16 +1519,16 @@
         </is>
       </c>
       <c r="E20" s="6" t="n">
-        <v>16987800</v>
+        <v>4860068.75</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>18210000</v>
+        <v>14420133.75</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>16212478.8</v>
+        <v>22037760</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>14308008.01</v>
+        <v>21837837.5</v>
       </c>
       <c r="I20" s="6">
         <f>IF(D20="متوقف",0,H20*الافتراضات!$B$4)</f>
@@ -1539,7 +1539,7 @@
         <v/>
       </c>
       <c r="K20" s="7">
-        <f>IF(D20="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.023086)))</f>
+        <f>IF(D20="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,1.129426)))</f>
         <v/>
       </c>
       <c r="L20" s="6">
@@ -1555,17 +1555,17 @@
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>بدون رقم</t>
+          <t>142163</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>بدون رقم (خدمات علم + جزاءات)</t>
+          <t>إيرادات  تأجير مباني تجارية</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>علم / جزاءات</t>
+          <t>إيرادات إستثمارية</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
@@ -1574,16 +1574,16 @@
         </is>
       </c>
       <c r="E21" s="6" t="n">
-        <v>4860068.75</v>
+        <v>9048255.93</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>14420133.75</v>
+        <v>7544256.25</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>22037760</v>
+        <v>4918746.75</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>21837837.5</v>
+        <v>12310614.76</v>
       </c>
       <c r="I21" s="6">
         <f>IF(D21="متوقف",0,H21*الافتراضات!$B$4)</f>
@@ -1594,7 +1594,7 @@
         <v/>
       </c>
       <c r="K21" s="7">
-        <f>IF(D21="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,1.129426)))</f>
+        <f>IF(D21="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.262699)))</f>
         <v/>
       </c>
       <c r="L21" s="6">
@@ -1605,22 +1605,26 @@
         <f>IF(G21=0,"",I21/G21-1)</f>
         <v/>
       </c>
-      <c r="N21" s="5" t="inlineStr"/>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>تذبذب عالٍ – راجع التوقع</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>142163</t>
+          <t>1422109</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>إيرادات  تأجير مباني تجارية</t>
+          <t>ايرادات  الكشفية</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>إيرادات إستثمارية</t>
+          <t>الرسوم والتراخيص</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
@@ -1629,16 +1633,16 @@
         </is>
       </c>
       <c r="E22" s="6" t="n">
-        <v>9048255.93</v>
+        <v>9597160.08</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>7544256.25</v>
+        <v>9593369.65</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>4918746.75</v>
+        <v>7704211.79</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>12310614.76</v>
+        <v>6331998.45</v>
       </c>
       <c r="I22" s="6">
         <f>IF(D22="متوقف",0,H22*الافتراضات!$B$4)</f>
@@ -1649,7 +1653,7 @@
         <v/>
       </c>
       <c r="K22" s="7">
-        <f>IF(D22="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.262699)))</f>
+        <f>IF(D22="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.104032)))</f>
         <v/>
       </c>
       <c r="L22" s="6">
@@ -1660,21 +1664,17 @@
         <f>IF(G22=0,"",I22/G22-1)</f>
         <v/>
       </c>
-      <c r="N22" s="5" t="inlineStr">
-        <is>
-          <t>تذبذب عالٍ – راجع التوقع</t>
-        </is>
-      </c>
+      <c r="N22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>1422109</t>
+          <t>11452111</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>ايرادات  الكشفية</t>
+          <t>المقابل المالي للسماح للأنشطة التجارية بالعمل (24) ساعة</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -1688,16 +1688,16 @@
         </is>
       </c>
       <c r="E23" s="6" t="n">
-        <v>9597160.08</v>
+        <v>6077736.7</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>9593369.65</v>
+        <v>5228065.19</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>7704211.79</v>
+        <v>6051210.16</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>6331998.45</v>
+        <v>12106223.42</v>
       </c>
       <c r="I23" s="6">
         <f>IF(D23="متوقف",0,H23*الافتراضات!$B$4)</f>
@@ -1708,7 +1708,7 @@
         <v/>
       </c>
       <c r="K23" s="7">
-        <f>IF(D23="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.104032)))</f>
+        <f>IF(D23="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.002185)))</f>
         <v/>
       </c>
       <c r="L23" s="6">
@@ -1719,17 +1719,21 @@
         <f>IF(G23=0,"",I23/G23-1)</f>
         <v/>
       </c>
-      <c r="N23" s="5" t="inlineStr"/>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>تذبذب عالٍ – راجع التوقع</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>11452111</t>
+          <t>1421910</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>المقابل المالي للسماح للأنشطة التجارية بالعمل (24) ساعة</t>
+          <t>اصدار تراخيص اشغال الارصفة العامة و الطرق</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
@@ -1743,16 +1747,16 @@
         </is>
       </c>
       <c r="E24" s="6" t="n">
-        <v>6077736.7</v>
+        <v>3853581.36</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>5228065.19</v>
+        <v>2946421.81</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>6051210.16</v>
+        <v>3566627.43</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>12106223.42</v>
+        <v>3660790.62</v>
       </c>
       <c r="I24" s="6">
         <f>IF(D24="متوقف",0,H24*الافتراضات!$B$4)</f>
@@ -1763,7 +1767,7 @@
         <v/>
       </c>
       <c r="K24" s="7">
-        <f>IF(D24="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.002185)))</f>
+        <f>IF(D24="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.037952)))</f>
         <v/>
       </c>
       <c r="L24" s="6">
@@ -1774,26 +1778,22 @@
         <f>IF(G24=0,"",I24/G24-1)</f>
         <v/>
       </c>
-      <c r="N24" s="5" t="inlineStr">
-        <is>
-          <t>تذبذب عالٍ – راجع التوقع</t>
-        </is>
-      </c>
+      <c r="N24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>1421910</t>
+          <t>1439</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>اصدار تراخيص اشغال الارصفة العامة و الطرق</t>
+          <t>ايرادات  مبيعات  ناتجه من النشاط غير مصنفة</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>الرسوم والتراخيص</t>
+          <t>جزاءات وغرامات</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
@@ -1802,16 +1802,16 @@
         </is>
       </c>
       <c r="E25" s="6" t="n">
-        <v>3853581.36</v>
+        <v>3537100</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>2946421.81</v>
+        <v>256186</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>3566627.43</v>
+        <v>8503508</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>3660790.62</v>
+        <v>519000</v>
       </c>
       <c r="I25" s="6">
         <f>IF(D25="متوقف",0,H25*الافتراضات!$B$4)</f>
@@ -1822,7 +1822,7 @@
         <v/>
       </c>
       <c r="K25" s="7">
-        <f>IF(D25="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.037952)))</f>
+        <f>IF(D25="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.550513)))</f>
         <v/>
       </c>
       <c r="L25" s="6">
@@ -1833,22 +1833,26 @@
         <f>IF(G25=0,"",I25/G25-1)</f>
         <v/>
       </c>
-      <c r="N25" s="5" t="inlineStr"/>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>تذبذب عالٍ – راجع التوقع</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>1439</t>
+          <t>1421901</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>ايرادات  مبيعات  ناتجه من النشاط غير مصنفة</t>
+          <t>بيع الوثائق والأنظمة</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t>جزاءات وغرامات</t>
+          <t>أخرى</t>
         </is>
       </c>
       <c r="D26" s="5" t="inlineStr">
@@ -1857,16 +1861,16 @@
         </is>
       </c>
       <c r="E26" s="6" t="n">
-        <v>3537100</v>
+        <v>2945006</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>256186</v>
+        <v>2753795</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>8503508</v>
+        <v>2520477</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>519000</v>
+        <v>1860236</v>
       </c>
       <c r="I26" s="6">
         <f>IF(D26="متوقف",0,H26*الافتراضات!$B$4)</f>
@@ -1877,7 +1881,7 @@
         <v/>
       </c>
       <c r="K26" s="7">
-        <f>IF(D26="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.550513)))</f>
+        <f>IF(D26="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.074880)))</f>
         <v/>
       </c>
       <c r="L26" s="6">
@@ -1888,26 +1892,22 @@
         <f>IF(G26=0,"",I26/G26-1)</f>
         <v/>
       </c>
-      <c r="N26" s="5" t="inlineStr">
-        <is>
-          <t>تذبذب عالٍ – راجع التوقع</t>
-        </is>
-      </c>
+      <c r="N26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>1421901</t>
+          <t>1421903</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>بيع الوثائق والأنظمة</t>
+          <t>مبيعات التيار الكهربائي</t>
         </is>
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t>أخرى</t>
+          <t>إيرادات إستثمارية</t>
         </is>
       </c>
       <c r="D27" s="5" t="inlineStr">
@@ -1916,16 +1916,16 @@
         </is>
       </c>
       <c r="E27" s="6" t="n">
-        <v>2945006</v>
+        <v>0</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>2753795</v>
+        <v>0</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>2520477</v>
+        <v>8083209.81</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>1860236</v>
+        <v>302027.65</v>
       </c>
       <c r="I27" s="6">
         <f>IF(D27="متوقف",0,H27*الافتراضات!$B$4)</f>
@@ -1936,7 +1936,7 @@
         <v/>
       </c>
       <c r="K27" s="7">
-        <f>IF(D27="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.074880)))</f>
+        <f>IF(D27="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.000000)))</f>
         <v/>
       </c>
       <c r="L27" s="6">
@@ -1947,22 +1947,26 @@
         <f>IF(G27=0,"",I27/G27-1)</f>
         <v/>
       </c>
-      <c r="N27" s="5" t="inlineStr"/>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>تذبذب عالٍ – راجع التوقع</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>1421903</t>
+          <t>1438</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>مبيعات التيار الكهربائي</t>
+          <t>جزاءات وغرامات مفروضة بموجب أنظمة الجهة</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>إيرادات إستثمارية</t>
+          <t>جزاءات وغرامات</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
@@ -1971,16 +1975,16 @@
         </is>
       </c>
       <c r="E28" s="6" t="n">
-        <v>0</v>
+        <v>6881203</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>0</v>
+        <v>486100</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>8083209.81</v>
+        <v>352900</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>302027.65</v>
+        <v>59500</v>
       </c>
       <c r="I28" s="6">
         <f>IF(D28="متوقف",0,H28*الافتراضات!$B$4)</f>
@@ -1991,7 +1995,7 @@
         <v/>
       </c>
       <c r="K28" s="7">
-        <f>IF(D28="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.000000)))</f>
+        <f>IF(D28="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.773539)))</f>
         <v/>
       </c>
       <c r="L28" s="6">
@@ -2002,26 +2006,22 @@
         <f>IF(G28=0,"",I28/G28-1)</f>
         <v/>
       </c>
-      <c r="N28" s="5" t="inlineStr">
-        <is>
-          <t>تذبذب عالٍ – راجع التوقع</t>
-        </is>
-      </c>
+      <c r="N28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>1438</t>
+          <t>1421912</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>جزاءات وغرامات مفروضة بموجب أنظمة الجهة</t>
+          <t>تأجير العقارات لأغراض مؤقته</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>جزاءات وغرامات</t>
+          <t>إيرادات إستثمارية</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -2030,16 +2030,16 @@
         </is>
       </c>
       <c r="E29" s="6" t="n">
-        <v>6881203</v>
+        <v>838420.1899999999</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>486100</v>
+        <v>2053263.42</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>352900</v>
+        <v>2460303.51</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>59500</v>
+        <v>1447854.96</v>
       </c>
       <c r="I29" s="6">
         <f>IF(D29="متوقف",0,H29*الافتراضات!$B$4)</f>
@@ -2050,7 +2050,7 @@
         <v/>
       </c>
       <c r="K29" s="7">
-        <f>IF(D29="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.773539)))</f>
+        <f>IF(D29="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.713024)))</f>
         <v/>
       </c>
       <c r="L29" s="6">
@@ -2066,17 +2066,17 @@
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>1421912</t>
+          <t>11452106</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>تأجير العقارات لأغراض مؤقته</t>
+          <t>اصدار التراخيص بتأسيس أو تشغيل ابراج الاتصالات</t>
         </is>
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>إيرادات إستثمارية</t>
+          <t>الرسوم والتراخيص</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -2085,16 +2085,16 @@
         </is>
       </c>
       <c r="E30" s="6" t="n">
-        <v>838420.1899999999</v>
+        <v>1007100</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>2053263.42</v>
+        <v>1570100</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>2460303.51</v>
+        <v>1590000</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>1447854.96</v>
+        <v>476400</v>
       </c>
       <c r="I30" s="6">
         <f>IF(D30="متوقف",0,H30*الافتراضات!$B$4)</f>
@@ -2105,7 +2105,7 @@
         <v/>
       </c>
       <c r="K30" s="7">
-        <f>IF(D30="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.713024)))</f>
+        <f>IF(D30="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.256499)))</f>
         <v/>
       </c>
       <c r="L30" s="6">
@@ -2121,12 +2121,12 @@
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>11452106</t>
+          <t>11452110</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>اصدار التراخيص بتأسيس أو تشغيل ابراج الاتصالات</t>
+          <t>إصدار تراخيص إستخدام أملاك خاصة لإقامة فعاليات</t>
         </is>
       </c>
       <c r="C31" s="5" t="inlineStr">
@@ -2140,16 +2140,16 @@
         </is>
       </c>
       <c r="E31" s="6" t="n">
-        <v>1007100</v>
+        <v>975004.05</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>1570100</v>
+        <v>1038789.25</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>1590000</v>
+        <v>1014443.22</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>476400</v>
+        <v>646845.12</v>
       </c>
       <c r="I31" s="6">
         <f>IF(D31="متوقف",0,H31*الافتراضات!$B$4)</f>
@@ -2160,7 +2160,7 @@
         <v/>
       </c>
       <c r="K31" s="7">
-        <f>IF(D31="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.256499)))</f>
+        <f>IF(D31="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.020025)))</f>
         <v/>
       </c>
       <c r="L31" s="6">
@@ -2176,17 +2176,17 @@
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>11452110</t>
+          <t>141229</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>إصدار تراخيص إستخدام أملاك خاصة لإقامة فعاليات</t>
+          <t>أرباح أخرى</t>
         </is>
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t>الرسوم والتراخيص</t>
+          <t>إيرادات إستثمارية</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
@@ -2195,16 +2195,16 @@
         </is>
       </c>
       <c r="E32" s="6" t="n">
-        <v>975004.05</v>
+        <v>1110572</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>1038789.25</v>
+        <v>2220000</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>1014443.22</v>
+        <v>30000</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>646845.12</v>
+        <v>60000</v>
       </c>
       <c r="I32" s="6">
         <f>IF(D32="متوقف",0,H32*الافتراضات!$B$4)</f>
@@ -2215,7 +2215,7 @@
         <v/>
       </c>
       <c r="K32" s="7">
-        <f>IF(D32="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.020025)))</f>
+        <f>IF(D32="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.835643)))</f>
         <v/>
       </c>
       <c r="L32" s="6">
@@ -2231,17 +2231,17 @@
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>141229</t>
+          <t>11452109</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>أرباح أخرى</t>
+          <t>اعتماد مخططات التطوير العقاري</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t>إيرادات إستثمارية</t>
+          <t>الرسوم والتراخيص</t>
         </is>
       </c>
       <c r="D33" s="5" t="inlineStr">
@@ -2250,16 +2250,16 @@
         </is>
       </c>
       <c r="E33" s="6" t="n">
-        <v>1110572</v>
+        <v>1311574.5</v>
       </c>
       <c r="F33" s="6" t="n">
-        <v>2220000</v>
+        <v>1330639.22</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>30000</v>
+        <v>592396.73</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>60000</v>
+        <v>100</v>
       </c>
       <c r="I33" s="6">
         <f>IF(D33="متوقف",0,H33*الافتراضات!$B$4)</f>
@@ -2270,7 +2270,7 @@
         <v/>
       </c>
       <c r="K33" s="7">
-        <f>IF(D33="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.835643)))</f>
+        <f>IF(D33="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.327937)))</f>
         <v/>
       </c>
       <c r="L33" s="6">
@@ -2286,12 +2286,12 @@
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>11452109</t>
+          <t>11452107</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>اعتماد مخططات التطوير العقاري</t>
+          <t>اصدار التراخيص بتأسيس أو تشغيل الصراف الآلي</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
@@ -2305,16 +2305,16 @@
         </is>
       </c>
       <c r="E34" s="6" t="n">
-        <v>1311574.5</v>
+        <v>54000</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>1330639.22</v>
+        <v>92000</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>592396.73</v>
+        <v>236273.52</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>100</v>
+        <v>200184.61</v>
       </c>
       <c r="I34" s="6">
         <f>IF(D34="متوقف",0,H34*الافتراضات!$B$4)</f>
@@ -2325,7 +2325,7 @@
         <v/>
       </c>
       <c r="K34" s="7">
-        <f>IF(D34="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.327937)))</f>
+        <f>IF(D34="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,1.091754)))</f>
         <v/>
       </c>
       <c r="L34" s="6">
@@ -2341,17 +2341,17 @@
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>11452107</t>
+          <t>3318212</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>اصدار التراخيص بتأسيس أو تشغيل الصراف الآلي</t>
+          <t>مرتجع رواتب - فواتير</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>الرسوم والتراخيص</t>
+          <t>أخرى</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
@@ -2360,16 +2360,16 @@
         </is>
       </c>
       <c r="E35" s="6" t="n">
-        <v>54000</v>
+        <v>0</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>92000</v>
+        <v>0</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>236273.52</v>
+        <v>152767.79</v>
       </c>
       <c r="H35" s="6" t="n">
-        <v>200184.61</v>
+        <v>361665.23</v>
       </c>
       <c r="I35" s="6">
         <f>IF(D35="متوقف",0,H35*الافتراضات!$B$4)</f>
@@ -2380,7 +2380,7 @@
         <v/>
       </c>
       <c r="K35" s="7">
-        <f>IF(D35="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,1.091754)))</f>
+        <f>IF(D35="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.000000)))</f>
         <v/>
       </c>
       <c r="L35" s="6">
@@ -2396,35 +2396,35 @@
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>3318212</t>
+          <t>11422</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>مرتجع رواتب - فواتير</t>
+          <t>رسوم منتجات التبغ</t>
         </is>
       </c>
       <c r="C36" s="5" t="inlineStr">
         <is>
-          <t>أخرى</t>
+          <t>التبغ والإيواء</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>نشط</t>
+          <t>متوقف</t>
         </is>
       </c>
       <c r="E36" s="6" t="n">
-        <v>0</v>
+        <v>27000</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>0</v>
+        <v>5167</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>152767.79</v>
+        <v>72000</v>
       </c>
       <c r="H36" s="6" t="n">
-        <v>361665.23</v>
+        <v>0</v>
       </c>
       <c r="I36" s="6">
         <f>IF(D36="متوقف",0,H36*الافتراضات!$B$4)</f>
@@ -2435,7 +2435,7 @@
         <v/>
       </c>
       <c r="K36" s="7">
-        <f>IF(D36="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.000000)))</f>
+        <f>IF(D36="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.632993)))</f>
         <v/>
       </c>
       <c r="L36" s="6">
@@ -2446,40 +2446,44 @@
         <f>IF(G36=0,"",I36/G36-1)</f>
         <v/>
       </c>
-      <c r="N36" s="5" t="inlineStr"/>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>متوقف في 2026 – توقعه صفر</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>11422</t>
+          <t>1422103</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>رسوم منتجات التبغ</t>
+          <t>تراخيص المحلات</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>التبغ والإيواء</t>
+          <t>إيرادات إستثمارية</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>متوقف</t>
+          <t>نشط</t>
         </is>
       </c>
       <c r="E37" s="6" t="n">
-        <v>27000</v>
+        <v>67711.60000000001</v>
       </c>
       <c r="F37" s="6" t="n">
-        <v>5167</v>
+        <v>16269.6</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>72000</v>
+        <v>1603.2</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>0</v>
+        <v>432</v>
       </c>
       <c r="I37" s="6">
         <f>IF(D37="متوقف",0,H37*الافتراضات!$B$4)</f>
@@ -2490,7 +2494,7 @@
         <v/>
       </c>
       <c r="K37" s="7">
-        <f>IF(D37="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.632993)))</f>
+        <f>IF(D37="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.846127)))</f>
         <v/>
       </c>
       <c r="L37" s="6">
@@ -2501,26 +2505,22 @@
         <f>IF(G37=0,"",I37/G37-1)</f>
         <v/>
       </c>
-      <c r="N37" s="5" t="inlineStr">
-        <is>
-          <t>متوقف في 2026 – توقعه صفر</t>
-        </is>
-      </c>
+      <c r="N37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>1422103</t>
+          <t>11452513</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>تراخيص المحلات</t>
+          <t>لوحات إرشـادية</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>إيرادات إستثمارية</t>
+          <t>الرسوم والتراخيص</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
@@ -2529,16 +2529,16 @@
         </is>
       </c>
       <c r="E38" s="6" t="n">
-        <v>67711.60000000001</v>
+        <v>55525</v>
       </c>
       <c r="F38" s="6" t="n">
-        <v>16269.6</v>
+        <v>12875</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>1603.2</v>
+        <v>9000</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>432</v>
+        <v>600</v>
       </c>
       <c r="I38" s="6">
         <f>IF(D38="متوقف",0,H38*الافتراضات!$B$4)</f>
@@ -2549,7 +2549,7 @@
         <v/>
       </c>
       <c r="K38" s="7">
-        <f>IF(D38="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.846127)))</f>
+        <f>IF(D38="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.597397)))</f>
         <v/>
       </c>
       <c r="L38" s="6">
@@ -2565,12 +2565,12 @@
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>11452513</t>
+          <t>1421907</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>لوحات إرشـادية</t>
+          <t>إيرادات المخططات</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -2584,16 +2584,16 @@
         </is>
       </c>
       <c r="E39" s="6" t="n">
-        <v>55525</v>
+        <v>0</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>12875</v>
+        <v>0</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>9000</v>
+        <v>21950</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>600</v>
+        <v>6350</v>
       </c>
       <c r="I39" s="6">
         <f>IF(D39="متوقف",0,H39*الافتراضات!$B$4)</f>
@@ -2604,7 +2604,7 @@
         <v/>
       </c>
       <c r="K39" s="7">
-        <f>IF(D39="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,-0.597397)))</f>
+        <f>IF(D39="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.000000)))</f>
         <v/>
       </c>
       <c r="L39" s="6">
@@ -2620,35 +2620,35 @@
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>1421907</t>
+          <t>1421908</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>إيرادات المخططات</t>
+          <t>ايرادات  رسوم خدمات  بلدية</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>الرسوم والتراخيص</t>
+          <t>إيرادات إستثمارية</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>نشط</t>
+          <t>متوقف</t>
         </is>
       </c>
       <c r="E40" s="6" t="n">
-        <v>0</v>
+        <v>16385</v>
       </c>
       <c r="F40" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G40" s="6" t="n">
-        <v>21950</v>
+        <v>0</v>
       </c>
       <c r="H40" s="6" t="n">
-        <v>6350</v>
+        <v>0</v>
       </c>
       <c r="I40" s="6">
         <f>IF(D40="متوقف",0,H40*الافتراضات!$B$4)</f>
@@ -2670,17 +2670,21 @@
         <f>IF(G40=0,"",I40/G40-1)</f>
         <v/>
       </c>
-      <c r="N40" s="5" t="inlineStr"/>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>متوقف في 2026 – توقعه صفر</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>1421908</t>
+          <t>142161</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>ايرادات  رسوم خدمات  بلدية</t>
+          <t>تاجير مباني سكنية</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
@@ -2694,13 +2698,13 @@
         </is>
       </c>
       <c r="E41" s="6" t="n">
-        <v>16385</v>
+        <v>0</v>
       </c>
       <c r="F41" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G41" s="6" t="n">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="H41" s="6" t="n">
         <v>0</v>
@@ -2732,113 +2736,54 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>142161</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>تاجير مباني سكنية</t>
-        </is>
-      </c>
-      <c r="C42" s="5" t="inlineStr">
-        <is>
-          <t>إيرادات إستثمارية</t>
-        </is>
-      </c>
-      <c r="D42" s="5" t="inlineStr">
-        <is>
-          <t>متوقف</t>
-        </is>
-      </c>
-      <c r="E42" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="6" t="n">
-        <v>6000</v>
-      </c>
-      <c r="H42" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" s="6">
-        <f>IF(D42="متوقف",0,H42*الافتراضات!$B$4)</f>
-        <v/>
-      </c>
-      <c r="J42" s="6">
-        <f>I42*(1+الافتراضات!$B$5)</f>
-        <v/>
-      </c>
-      <c r="K42" s="7">
-        <f>IF(D42="متوقف",0,MAX(-الافتراضات!$B$6,MIN(الافتراضات!$B$6,0.000000)))</f>
-        <v/>
-      </c>
-      <c r="L42" s="6">
-        <f>I42*(1+K42)</f>
-        <v/>
-      </c>
-      <c r="M42" s="7">
-        <f>IF(G42=0,"",I42/G42-1)</f>
-        <v/>
-      </c>
-      <c r="N42" s="5" t="inlineStr">
-        <is>
-          <t>متوقف في 2026 – توقعه صفر</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n"/>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="C43" s="8" t="n"/>
-      <c r="D43" s="8" t="n"/>
-      <c r="E43" s="9">
-        <f>SUM(E4:E42)</f>
-        <v/>
-      </c>
-      <c r="F43" s="9">
-        <f>SUM(F4:F42)</f>
-        <v/>
-      </c>
-      <c r="G43" s="9">
-        <f>SUM(G4:G42)</f>
-        <v/>
-      </c>
-      <c r="H43" s="9">
-        <f>SUM(H4:H42)</f>
-        <v/>
-      </c>
-      <c r="I43" s="9">
-        <f>SUM(I4:I42)</f>
-        <v/>
-      </c>
-      <c r="J43" s="9">
-        <f>SUM(J4:J42)</f>
-        <v/>
-      </c>
-      <c r="K43" s="10">
-        <f>L43/I43-1</f>
-        <v/>
-      </c>
-      <c r="L43" s="9">
-        <f>SUM(L4:L42)</f>
-        <v/>
-      </c>
-      <c r="M43" s="10">
-        <f>I43/G43-1</f>
-        <v/>
-      </c>
-      <c r="N43" s="8" t="n"/>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="9">
+        <f>SUM(E4:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="9">
+        <f>SUM(F4:F41)</f>
+        <v/>
+      </c>
+      <c r="G42" s="9">
+        <f>SUM(G4:G41)</f>
+        <v/>
+      </c>
+      <c r="H42" s="9">
+        <f>SUM(H4:H41)</f>
+        <v/>
+      </c>
+      <c r="I42" s="9">
+        <f>SUM(I4:I41)</f>
+        <v/>
+      </c>
+      <c r="J42" s="9">
+        <f>SUM(J4:J41)</f>
+        <v/>
+      </c>
+      <c r="K42" s="10">
+        <f>L42/I42-1</f>
+        <v/>
+      </c>
+      <c r="L42" s="9">
+        <f>SUM(L4:L41)</f>
+        <v/>
+      </c>
+      <c r="M42" s="10">
+        <f>I42/G42-1</f>
+        <v/>
+      </c>
+      <c r="N42" s="8" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N42"/>
+  <autoFilter ref="A3:N41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -2849,7 +2794,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H11"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -2918,31 +2863,31 @@
         </is>
       </c>
       <c r="B4" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A4,التوقعات!E$4:E$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A4,التوقعات!E$4:E$41)</f>
         <v/>
       </c>
       <c r="C4" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A4,التوقعات!F$4:F$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A4,التوقعات!F$4:F$41)</f>
         <v/>
       </c>
       <c r="D4" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A4,التوقعات!G$4:G$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A4,التوقعات!G$4:G$41)</f>
         <v/>
       </c>
       <c r="E4" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A4,التوقعات!H$4:H$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A4,التوقعات!H$4:H$41)</f>
         <v/>
       </c>
       <c r="F4" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A4,التوقعات!I$4:I$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A4,التوقعات!I$4:I$41)</f>
         <v/>
       </c>
       <c r="G4" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A4,التوقعات!J$4:J$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A4,التوقعات!J$4:J$41)</f>
         <v/>
       </c>
       <c r="H4" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A4,التوقعات!L$4:L$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A4,التوقعات!L$4:L$41)</f>
         <v/>
       </c>
     </row>
@@ -2953,31 +2898,31 @@
         </is>
       </c>
       <c r="B5" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A5,التوقعات!E$4:E$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A5,التوقعات!E$4:E$41)</f>
         <v/>
       </c>
       <c r="C5" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A5,التوقعات!F$4:F$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A5,التوقعات!F$4:F$41)</f>
         <v/>
       </c>
       <c r="D5" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A5,التوقعات!G$4:G$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A5,التوقعات!G$4:G$41)</f>
         <v/>
       </c>
       <c r="E5" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A5,التوقعات!H$4:H$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A5,التوقعات!H$4:H$41)</f>
         <v/>
       </c>
       <c r="F5" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A5,التوقعات!I$4:I$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A5,التوقعات!I$4:I$41)</f>
         <v/>
       </c>
       <c r="G5" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A5,التوقعات!J$4:J$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A5,التوقعات!J$4:J$41)</f>
         <v/>
       </c>
       <c r="H5" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A5,التوقعات!L$4:L$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A5,التوقعات!L$4:L$41)</f>
         <v/>
       </c>
     </row>
@@ -2988,31 +2933,31 @@
         </is>
       </c>
       <c r="B6" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A6,التوقعات!E$4:E$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A6,التوقعات!E$4:E$41)</f>
         <v/>
       </c>
       <c r="C6" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A6,التوقعات!F$4:F$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A6,التوقعات!F$4:F$41)</f>
         <v/>
       </c>
       <c r="D6" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A6,التوقعات!G$4:G$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A6,التوقعات!G$4:G$41)</f>
         <v/>
       </c>
       <c r="E6" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A6,التوقعات!H$4:H$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A6,التوقعات!H$4:H$41)</f>
         <v/>
       </c>
       <c r="F6" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A6,التوقعات!I$4:I$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A6,التوقعات!I$4:I$41)</f>
         <v/>
       </c>
       <c r="G6" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A6,التوقعات!J$4:J$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A6,التوقعات!J$4:J$41)</f>
         <v/>
       </c>
       <c r="H6" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A6,التوقعات!L$4:L$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A6,التوقعات!L$4:L$41)</f>
         <v/>
       </c>
     </row>
@@ -3023,31 +2968,31 @@
         </is>
       </c>
       <c r="B7" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A7,التوقعات!E$4:E$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A7,التوقعات!E$4:E$41)</f>
         <v/>
       </c>
       <c r="C7" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A7,التوقعات!F$4:F$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A7,التوقعات!F$4:F$41)</f>
         <v/>
       </c>
       <c r="D7" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A7,التوقعات!G$4:G$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A7,التوقعات!G$4:G$41)</f>
         <v/>
       </c>
       <c r="E7" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A7,التوقعات!H$4:H$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A7,التوقعات!H$4:H$41)</f>
         <v/>
       </c>
       <c r="F7" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A7,التوقعات!I$4:I$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A7,التوقعات!I$4:I$41)</f>
         <v/>
       </c>
       <c r="G7" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A7,التوقعات!J$4:J$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A7,التوقعات!J$4:J$41)</f>
         <v/>
       </c>
       <c r="H7" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A7,التوقعات!L$4:L$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A7,التوقعات!L$4:L$41)</f>
         <v/>
       </c>
     </row>
@@ -3058,136 +3003,101 @@
         </is>
       </c>
       <c r="B8" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A8,التوقعات!E$4:E$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A8,التوقعات!E$4:E$41)</f>
         <v/>
       </c>
       <c r="C8" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A8,التوقعات!F$4:F$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A8,التوقعات!F$4:F$41)</f>
         <v/>
       </c>
       <c r="D8" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A8,التوقعات!G$4:G$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A8,التوقعات!G$4:G$41)</f>
         <v/>
       </c>
       <c r="E8" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A8,التوقعات!H$4:H$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A8,التوقعات!H$4:H$41)</f>
         <v/>
       </c>
       <c r="F8" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A8,التوقعات!I$4:I$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A8,التوقعات!I$4:I$41)</f>
         <v/>
       </c>
       <c r="G8" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A8,التوقعات!J$4:J$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A8,التوقعات!J$4:J$41)</f>
         <v/>
       </c>
       <c r="H8" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A8,التوقعات!L$4:L$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A8,التوقعات!L$4:L$41)</f>
         <v/>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>ضريبة</t>
+          <t>علم / جزاءات</t>
         </is>
       </c>
       <c r="B9" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A9,التوقعات!E$4:E$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A9,التوقعات!E$4:E$41)</f>
         <v/>
       </c>
       <c r="C9" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A9,التوقعات!F$4:F$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A9,التوقعات!F$4:F$41)</f>
         <v/>
       </c>
       <c r="D9" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A9,التوقعات!G$4:G$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A9,التوقعات!G$4:G$41)</f>
         <v/>
       </c>
       <c r="E9" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A9,التوقعات!H$4:H$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A9,التوقعات!H$4:H$41)</f>
         <v/>
       </c>
       <c r="F9" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A9,التوقعات!I$4:I$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A9,التوقعات!I$4:I$41)</f>
         <v/>
       </c>
       <c r="G9" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A9,التوقعات!J$4:J$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A9,التوقعات!J$4:J$41)</f>
         <v/>
       </c>
       <c r="H9" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A9,التوقعات!L$4:L$42)</f>
+        <f>SUMIF(التوقعات!$C$4:$C$41,$A9,التوقعات!L$4:L$41)</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
-        <is>
-          <t>علم / جزاءات</t>
-        </is>
-      </c>
-      <c r="B10" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A10,التوقعات!E$4:E$42)</f>
-        <v/>
-      </c>
-      <c r="C10" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A10,التوقعات!F$4:F$42)</f>
-        <v/>
-      </c>
-      <c r="D10" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A10,التوقعات!G$4:G$42)</f>
-        <v/>
-      </c>
-      <c r="E10" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A10,التوقعات!H$4:H$42)</f>
-        <v/>
-      </c>
-      <c r="F10" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A10,التوقعات!I$4:I$42)</f>
-        <v/>
-      </c>
-      <c r="G10" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A10,التوقعات!J$4:J$42)</f>
-        <v/>
-      </c>
-      <c r="H10" s="6">
-        <f>SUMIF(التوقعات!$C$4:$C$42,$A10,التوقعات!L$4:L$42)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="B11" s="9">
-        <f>SUM(B4:B10)</f>
-        <v/>
-      </c>
-      <c r="C11" s="9">
-        <f>SUM(C4:C10)</f>
-        <v/>
-      </c>
-      <c r="D11" s="9">
-        <f>SUM(D4:D10)</f>
-        <v/>
-      </c>
-      <c r="E11" s="9">
-        <f>SUM(E4:E10)</f>
-        <v/>
-      </c>
-      <c r="F11" s="9">
-        <f>SUM(F4:F10)</f>
-        <v/>
-      </c>
-      <c r="G11" s="9">
-        <f>SUM(G4:G10)</f>
-        <v/>
-      </c>
-      <c r="H11" s="9">
-        <f>SUM(H4:H10)</f>
+      <c r="B10" s="9">
+        <f>SUM(B4:B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="9">
+        <f>SUM(C4:C9)</f>
+        <v/>
+      </c>
+      <c r="D10" s="9">
+        <f>SUM(D4:D9)</f>
+        <v/>
+      </c>
+      <c r="E10" s="9">
+        <f>SUM(E4:E9)</f>
+        <v/>
+      </c>
+      <c r="F10" s="9">
+        <f>SUM(F4:F9)</f>
+        <v/>
+      </c>
+      <c r="G10" s="9">
+        <f>SUM(G4:G9)</f>
+        <v/>
+      </c>
+      <c r="H10" s="9">
+        <f>SUM(H4:H9)</f>
         <v/>
       </c>
     </row>
@@ -3202,7 +3112,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3603,862 +3513,862 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>11411</t>
+          <t>144122</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>قيمة الضريبة المضافة</t>
+          <t>إيرادات  متنوعه</t>
         </is>
       </c>
       <c r="C13" s="6" t="n">
-        <v>128903414.3</v>
+        <v>9219073.48</v>
       </c>
       <c r="D13" s="6" t="n">
-        <v>116269653.46</v>
+        <v>13582347.46</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>111903017.85</v>
+        <v>78828800.53</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>100973117.79</v>
+        <v>297191478.48</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>12482898.72</v>
+        <v>722827.09</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>18969498.83</v>
+        <v>551469.75</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>11213620.46</v>
+        <v>1918938.67</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>22904655.52</v>
+        <v>19305484.78</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>144122</t>
+          <t>1421911</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>إيرادات  متنوعه</t>
+          <t>رسم مبيعات محلات تقديم منتجات التبغ</t>
         </is>
       </c>
       <c r="C14" s="6" t="n">
-        <v>9219073.48</v>
+        <v>72701817.54000001</v>
       </c>
       <c r="D14" s="6" t="n">
-        <v>13582347.46</v>
+        <v>140513661.33</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>78828800.53</v>
+        <v>101287573.05</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>297191478.48</v>
+        <v>78309014.93000001</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>722827.09</v>
+        <v>2364215.5</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>551469.75</v>
+        <v>1689112.21</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>1918938.67</v>
+        <v>4167606.53</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>19305484.78</v>
+        <v>2414078.01</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>1421911</t>
+          <t>1421909</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t>رسم مبيعات محلات تقديم منتجات التبغ</t>
+          <t>جمع النفايات</t>
         </is>
       </c>
       <c r="C15" s="6" t="n">
-        <v>72701817.54000001</v>
+        <v>81156665.08</v>
       </c>
       <c r="D15" s="6" t="n">
-        <v>140513661.33</v>
+        <v>87441839.75</v>
       </c>
       <c r="E15" s="6" t="n">
-        <v>101287573.05</v>
+        <v>79209685.56</v>
       </c>
       <c r="F15" s="6" t="n">
-        <v>78309014.93000001</v>
+        <v>76301330.65000001</v>
       </c>
       <c r="G15" s="6" t="n">
-        <v>2364215.5</v>
+        <v>1871186.45</v>
       </c>
       <c r="H15" s="6" t="n">
-        <v>1689112.21</v>
+        <v>1828100.87</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>4167606.53</v>
+        <v>1778808.27</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>2414078.01</v>
+        <v>2912175.55</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
         <is>
-          <t>1421909</t>
+          <t>11452105</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t>جمع النفايات</t>
+          <t>رسوم تراخيص حفر الشوارع</t>
         </is>
       </c>
       <c r="C16" s="6" t="n">
-        <v>81156665.08</v>
+        <v>66565866.19</v>
       </c>
       <c r="D16" s="6" t="n">
-        <v>87441839.75</v>
+        <v>65178247.05</v>
       </c>
       <c r="E16" s="6" t="n">
-        <v>79209685.56</v>
+        <v>560490.41</v>
       </c>
       <c r="F16" s="6" t="n">
-        <v>76301330.65000001</v>
+        <v>0</v>
       </c>
       <c r="G16" s="6" t="n">
-        <v>1871186.45</v>
+        <v>319033.78</v>
       </c>
       <c r="H16" s="6" t="n">
-        <v>1828100.87</v>
+        <v>289038.85</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>1778808.27</v>
+        <v>74246.06</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>2912175.55</v>
+        <v>1350</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>11452105</t>
+          <t>11452108</t>
         </is>
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>رسوم تراخيص حفر الشوارع</t>
+          <t>ايراد اصدار القرارات المساحية - أمانة منطقة الرياض</t>
         </is>
       </c>
       <c r="C17" s="6" t="n">
-        <v>66565866.19</v>
+        <v>4391166.64</v>
       </c>
       <c r="D17" s="6" t="n">
-        <v>65178247.05</v>
+        <v>19598327.65</v>
       </c>
       <c r="E17" s="6" t="n">
-        <v>560490.41</v>
+        <v>26544701.29</v>
       </c>
       <c r="F17" s="6" t="n">
-        <v>0</v>
+        <v>31807755.11</v>
       </c>
       <c r="G17" s="6" t="n">
-        <v>319033.78</v>
+        <v>31103</v>
       </c>
       <c r="H17" s="6" t="n">
-        <v>289038.85</v>
+        <v>106057.75</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>74246.06</v>
+        <v>364687.58</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>1350</v>
+        <v>2326052.14</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
         <is>
-          <t>11452108</t>
+          <t>1422108</t>
         </is>
       </c>
       <c r="B18" s="5" t="inlineStr">
         <is>
-          <t>ايراد اصدار القرارات المساحية - أمانة منطقة الرياض</t>
+          <t>الشهادات الصحية</t>
         </is>
       </c>
       <c r="C18" s="6" t="n">
-        <v>4391166.64</v>
+        <v>19375523.29</v>
       </c>
       <c r="D18" s="6" t="n">
-        <v>19598327.65</v>
+        <v>13396724.24</v>
       </c>
       <c r="E18" s="6" t="n">
-        <v>26544701.29</v>
+        <v>25250138.75</v>
       </c>
       <c r="F18" s="6" t="n">
-        <v>31807755.11</v>
+        <v>21432048.85</v>
       </c>
       <c r="G18" s="6" t="n">
-        <v>31103</v>
+        <v>1893132.74</v>
       </c>
       <c r="H18" s="6" t="n">
-        <v>106057.75</v>
+        <v>472946.84</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>364687.58</v>
+        <v>1049260.99</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>2326052.14</v>
+        <v>202309.67</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
         <is>
-          <t>1422108</t>
+          <t>1422121</t>
         </is>
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>الشهادات الصحية</t>
+          <t>رسم ترخيص نشاط تقديم منتجات التبغ</t>
         </is>
       </c>
       <c r="C19" s="6" t="n">
-        <v>19375523.29</v>
+        <v>16817800</v>
       </c>
       <c r="D19" s="6" t="n">
-        <v>13396724.24</v>
+        <v>16115000</v>
       </c>
       <c r="E19" s="6" t="n">
-        <v>25250138.75</v>
+        <v>15767478.8</v>
       </c>
       <c r="F19" s="6" t="n">
-        <v>21432048.85</v>
+        <v>13744093.5</v>
       </c>
       <c r="G19" s="6" t="n">
-        <v>1893132.74</v>
+        <v>170000</v>
       </c>
       <c r="H19" s="6" t="n">
-        <v>472946.84</v>
+        <v>2095000</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>1049260.99</v>
+        <v>445000</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>202309.67</v>
+        <v>563914.51</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>1422121</t>
+          <t>بدون رقم</t>
         </is>
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>رسم ترخيص نشاط تقديم منتجات التبغ</t>
+          <t>بدون رقم (خدمات علم + جزاءات)</t>
         </is>
       </c>
       <c r="C20" s="6" t="n">
-        <v>16817800</v>
+        <v>4834590</v>
       </c>
       <c r="D20" s="6" t="n">
-        <v>16115000</v>
+        <v>14372921.25</v>
       </c>
       <c r="E20" s="6" t="n">
-        <v>15767478.8</v>
+        <v>21894648.75</v>
       </c>
       <c r="F20" s="6" t="n">
-        <v>13744093.5</v>
+        <v>21614573.75</v>
       </c>
       <c r="G20" s="6" t="n">
-        <v>170000</v>
+        <v>25478.75</v>
       </c>
       <c r="H20" s="6" t="n">
-        <v>2095000</v>
+        <v>47212.5</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>445000</v>
+        <v>143111.25</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>563914.51</v>
+        <v>223263.75</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>بدون رقم</t>
+          <t>142163</t>
         </is>
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>بدون رقم (خدمات علم + جزاءات)</t>
+          <t>إيرادات  تأجير مباني تجارية</t>
         </is>
       </c>
       <c r="C21" s="6" t="n">
-        <v>4834590</v>
+        <v>8085858</v>
       </c>
       <c r="D21" s="6" t="n">
-        <v>14372921.25</v>
+        <v>6095216.75</v>
       </c>
       <c r="E21" s="6" t="n">
-        <v>21894648.75</v>
+        <v>3675127.5</v>
       </c>
       <c r="F21" s="6" t="n">
-        <v>21614573.75</v>
+        <v>9088249.050000001</v>
       </c>
       <c r="G21" s="6" t="n">
-        <v>25478.75</v>
+        <v>962397.9300000001</v>
       </c>
       <c r="H21" s="6" t="n">
-        <v>47212.5</v>
+        <v>1449039.5</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>143111.25</v>
+        <v>1243619.25</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>223263.75</v>
+        <v>3222365.71</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>142163</t>
+          <t>1422109</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
         <is>
-          <t>إيرادات  تأجير مباني تجارية</t>
+          <t>ايرادات  الكشفية</t>
         </is>
       </c>
       <c r="C22" s="6" t="n">
-        <v>8085858</v>
+        <v>9441840.73</v>
       </c>
       <c r="D22" s="6" t="n">
-        <v>6095216.75</v>
+        <v>9503239.65</v>
       </c>
       <c r="E22" s="6" t="n">
-        <v>3675127.5</v>
+        <v>7617004.28</v>
       </c>
       <c r="F22" s="6" t="n">
-        <v>9088249.050000001</v>
+        <v>6172791.57</v>
       </c>
       <c r="G22" s="6" t="n">
-        <v>962397.9300000001</v>
+        <v>155319.35</v>
       </c>
       <c r="H22" s="6" t="n">
-        <v>1449039.5</v>
+        <v>90130</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>1243619.25</v>
+        <v>87207.50999999999</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>3222365.71</v>
+        <v>159206.88</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>1422109</t>
+          <t>11452111</t>
         </is>
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>ايرادات  الكشفية</t>
+          <t>المقابل المالي للسماح للأنشطة التجارية بالعمل (24) ساعة</t>
         </is>
       </c>
       <c r="C23" s="6" t="n">
-        <v>9441840.73</v>
+        <v>6029932.4</v>
       </c>
       <c r="D23" s="6" t="n">
-        <v>9503239.65</v>
+        <v>5182284.58</v>
       </c>
       <c r="E23" s="6" t="n">
-        <v>7617004.28</v>
+        <v>5989835.57</v>
       </c>
       <c r="F23" s="6" t="n">
-        <v>6172791.57</v>
+        <v>11838949.26</v>
       </c>
       <c r="G23" s="6" t="n">
-        <v>155319.35</v>
+        <v>47804.3</v>
       </c>
       <c r="H23" s="6" t="n">
-        <v>90130</v>
+        <v>45780.61</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>87207.50999999999</v>
+        <v>61374.59</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>159206.88</v>
+        <v>267274.16</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>11452111</t>
+          <t>1421910</t>
         </is>
       </c>
       <c r="B24" s="5" t="inlineStr">
         <is>
-          <t>المقابل المالي للسماح للأنشطة التجارية بالعمل (24) ساعة</t>
+          <t>اصدار تراخيص اشغال الارصفة العامة و الطرق</t>
         </is>
       </c>
       <c r="C24" s="6" t="n">
-        <v>6029932.4</v>
+        <v>3769312.51</v>
       </c>
       <c r="D24" s="6" t="n">
-        <v>5182284.58</v>
+        <v>2921517.06</v>
       </c>
       <c r="E24" s="6" t="n">
-        <v>5989835.57</v>
+        <v>3529618.23</v>
       </c>
       <c r="F24" s="6" t="n">
-        <v>11838949.26</v>
+        <v>3571838.39</v>
       </c>
       <c r="G24" s="6" t="n">
-        <v>47804.3</v>
+        <v>84268.85000000001</v>
       </c>
       <c r="H24" s="6" t="n">
-        <v>45780.61</v>
+        <v>24904.75</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>61374.59</v>
+        <v>37009.2</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>267274.16</v>
+        <v>88952.23</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
         <is>
-          <t>1421910</t>
+          <t>1439</t>
         </is>
       </c>
       <c r="B25" s="5" t="inlineStr">
         <is>
-          <t>اصدار تراخيص اشغال الارصفة العامة و الطرق</t>
+          <t>ايرادات  مبيعات  ناتجه من النشاط غير مصنفة</t>
         </is>
       </c>
       <c r="C25" s="6" t="n">
-        <v>3769312.51</v>
+        <v>3533600</v>
       </c>
       <c r="D25" s="6" t="n">
-        <v>2921517.06</v>
+        <v>255186</v>
       </c>
       <c r="E25" s="6" t="n">
-        <v>3529618.23</v>
+        <v>8503508</v>
       </c>
       <c r="F25" s="6" t="n">
-        <v>3571838.39</v>
+        <v>519000</v>
       </c>
       <c r="G25" s="6" t="n">
-        <v>84268.85000000001</v>
+        <v>3500</v>
       </c>
       <c r="H25" s="6" t="n">
-        <v>24904.75</v>
+        <v>1000</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>37009.2</v>
+        <v>0</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>88952.23</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="5" t="inlineStr">
         <is>
-          <t>1439</t>
+          <t>1421901</t>
         </is>
       </c>
       <c r="B26" s="5" t="inlineStr">
         <is>
-          <t>ايرادات  مبيعات  ناتجه من النشاط غير مصنفة</t>
+          <t>بيع الوثائق والأنظمة</t>
         </is>
       </c>
       <c r="C26" s="6" t="n">
-        <v>3533600</v>
+        <v>2937506</v>
       </c>
       <c r="D26" s="6" t="n">
-        <v>255186</v>
+        <v>2737695</v>
       </c>
       <c r="E26" s="6" t="n">
-        <v>8503508</v>
+        <v>2503277</v>
       </c>
       <c r="F26" s="6" t="n">
-        <v>519000</v>
+        <v>1852136</v>
       </c>
       <c r="G26" s="6" t="n">
-        <v>3500</v>
+        <v>7500</v>
       </c>
       <c r="H26" s="6" t="n">
-        <v>1000</v>
+        <v>16100</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>0</v>
+        <v>17200</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0</v>
+        <v>8100</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>1421901</t>
+          <t>1421903</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>بيع الوثائق والأنظمة</t>
+          <t>مبيعات التيار الكهربائي</t>
         </is>
       </c>
       <c r="C27" s="6" t="n">
-        <v>2937506</v>
+        <v>0</v>
       </c>
       <c r="D27" s="6" t="n">
-        <v>2737695</v>
+        <v>0</v>
       </c>
       <c r="E27" s="6" t="n">
-        <v>2503277</v>
+        <v>8083209.81</v>
       </c>
       <c r="F27" s="6" t="n">
-        <v>1852136</v>
+        <v>170710.39</v>
       </c>
       <c r="G27" s="6" t="n">
-        <v>7500</v>
+        <v>0</v>
       </c>
       <c r="H27" s="6" t="n">
-        <v>16100</v>
+        <v>0</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>17200</v>
+        <v>0</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>8100</v>
+        <v>131317.26</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>1421903</t>
+          <t>1438</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr">
         <is>
-          <t>مبيعات التيار الكهربائي</t>
+          <t>جزاءات وغرامات مفروضة بموجب أنظمة الجهة</t>
         </is>
       </c>
       <c r="C28" s="6" t="n">
-        <v>0</v>
+        <v>5975450</v>
       </c>
       <c r="D28" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E28" s="6" t="n">
-        <v>8083209.81</v>
+        <v>0</v>
       </c>
       <c r="F28" s="6" t="n">
-        <v>170710.39</v>
+        <v>0</v>
       </c>
       <c r="G28" s="6" t="n">
-        <v>0</v>
+        <v>905753</v>
       </c>
       <c r="H28" s="6" t="n">
-        <v>0</v>
+        <v>486100</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>0</v>
+        <v>352900</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>131317.26</v>
+        <v>59500</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>1438</t>
+          <t>1421912</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr">
         <is>
-          <t>جزاءات وغرامات مفروضة بموجب أنظمة الجهة</t>
+          <t>تأجير العقارات لأغراض مؤقته</t>
         </is>
       </c>
       <c r="C29" s="6" t="n">
-        <v>5975450</v>
+        <v>836002.1899999999</v>
       </c>
       <c r="D29" s="6" t="n">
-        <v>0</v>
+        <v>2053263.42</v>
       </c>
       <c r="E29" s="6" t="n">
-        <v>0</v>
+        <v>2450880.59</v>
       </c>
       <c r="F29" s="6" t="n">
-        <v>0</v>
+        <v>1444704.96</v>
       </c>
       <c r="G29" s="6" t="n">
-        <v>905753</v>
+        <v>2418</v>
       </c>
       <c r="H29" s="6" t="n">
-        <v>486100</v>
+        <v>0</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>352900</v>
+        <v>9422.92</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>59500</v>
+        <v>3150</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>1421912</t>
+          <t>11452106</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr">
         <is>
-          <t>تأجير العقارات لأغراض مؤقته</t>
+          <t>اصدار التراخيص بتأسيس أو تشغيل ابراج الاتصالات</t>
         </is>
       </c>
       <c r="C30" s="6" t="n">
-        <v>836002.1899999999</v>
+        <v>989500</v>
       </c>
       <c r="D30" s="6" t="n">
-        <v>2053263.42</v>
+        <v>1458100</v>
       </c>
       <c r="E30" s="6" t="n">
-        <v>2450880.59</v>
+        <v>1498900</v>
       </c>
       <c r="F30" s="6" t="n">
-        <v>1444704.96</v>
+        <v>323000</v>
       </c>
       <c r="G30" s="6" t="n">
-        <v>2418</v>
+        <v>17600</v>
       </c>
       <c r="H30" s="6" t="n">
-        <v>0</v>
+        <v>112000</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>9422.92</v>
+        <v>91100</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>3150</v>
+        <v>153400</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>11452106</t>
+          <t>11452110</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr">
         <is>
-          <t>اصدار التراخيص بتأسيس أو تشغيل ابراج الاتصالات</t>
+          <t>إصدار تراخيص إستخدام أملاك خاصة لإقامة فعاليات</t>
         </is>
       </c>
       <c r="C31" s="6" t="n">
-        <v>989500</v>
+        <v>900053.05</v>
       </c>
       <c r="D31" s="6" t="n">
-        <v>1458100</v>
+        <v>804465.15</v>
       </c>
       <c r="E31" s="6" t="n">
-        <v>1498900</v>
+        <v>816539.9300000001</v>
       </c>
       <c r="F31" s="6" t="n">
-        <v>323000</v>
+        <v>631902.8</v>
       </c>
       <c r="G31" s="6" t="n">
-        <v>17600</v>
+        <v>74951</v>
       </c>
       <c r="H31" s="6" t="n">
-        <v>112000</v>
+        <v>234324.1</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>91100</v>
+        <v>197903.29</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>153400</v>
+        <v>14942.32</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
         <is>
-          <t>11452110</t>
+          <t>141229</t>
         </is>
       </c>
       <c r="B32" s="5" t="inlineStr">
         <is>
-          <t>إصدار تراخيص إستخدام أملاك خاصة لإقامة فعاليات</t>
+          <t>أرباح أخرى</t>
         </is>
       </c>
       <c r="C32" s="6" t="n">
-        <v>900053.05</v>
+        <v>1070572</v>
       </c>
       <c r="D32" s="6" t="n">
-        <v>804465.15</v>
+        <v>2100000</v>
       </c>
       <c r="E32" s="6" t="n">
-        <v>816539.9300000001</v>
+        <v>0</v>
       </c>
       <c r="F32" s="6" t="n">
-        <v>631902.8</v>
+        <v>0</v>
       </c>
       <c r="G32" s="6" t="n">
-        <v>74951</v>
+        <v>40000</v>
       </c>
       <c r="H32" s="6" t="n">
-        <v>234324.1</v>
+        <v>120000</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>197903.29</v>
+        <v>30000</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>14942.32</v>
+        <v>60000</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
         <is>
-          <t>141229</t>
+          <t>11452109</t>
         </is>
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>أرباح أخرى</t>
+          <t>اعتماد مخططات التطوير العقاري</t>
         </is>
       </c>
       <c r="C33" s="6" t="n">
-        <v>1070572</v>
+        <v>1309274.5</v>
       </c>
       <c r="D33" s="6" t="n">
-        <v>2100000</v>
+        <v>1328839.22</v>
       </c>
       <c r="E33" s="6" t="n">
-        <v>0</v>
+        <v>590496.73</v>
       </c>
       <c r="F33" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G33" s="6" t="n">
-        <v>40000</v>
+        <v>2300</v>
       </c>
       <c r="H33" s="6" t="n">
-        <v>120000</v>
+        <v>1800</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>30000</v>
+        <v>1900</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>60000</v>
+        <v>100</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
         <is>
-          <t>11452109</t>
+          <t>11452107</t>
         </is>
       </c>
       <c r="B34" s="5" t="inlineStr">
         <is>
-          <t>اعتماد مخططات التطوير العقاري</t>
+          <t>اصدار التراخيص بتأسيس أو تشغيل الصراف الآلي</t>
         </is>
       </c>
       <c r="C34" s="6" t="n">
-        <v>1309274.5</v>
+        <v>49000</v>
       </c>
       <c r="D34" s="6" t="n">
-        <v>1328839.22</v>
+        <v>92000</v>
       </c>
       <c r="E34" s="6" t="n">
-        <v>590496.73</v>
+        <v>234273.52</v>
       </c>
       <c r="F34" s="6" t="n">
-        <v>0</v>
+        <v>193711.09</v>
       </c>
       <c r="G34" s="6" t="n">
-        <v>2300</v>
+        <v>5000</v>
       </c>
       <c r="H34" s="6" t="n">
-        <v>1800</v>
+        <v>0</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>1900</v>
+        <v>2000</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>100</v>
+        <v>6473.52</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
         <is>
-          <t>11452107</t>
+          <t>3318212</t>
         </is>
       </c>
       <c r="B35" s="5" t="inlineStr">
         <is>
-          <t>اصدار التراخيص بتأسيس أو تشغيل الصراف الآلي</t>
+          <t>مرتجع رواتب - فواتير</t>
         </is>
       </c>
       <c r="C35" s="6" t="n">
-        <v>49000</v>
+        <v>0</v>
       </c>
       <c r="D35" s="6" t="n">
-        <v>92000</v>
+        <v>0</v>
       </c>
       <c r="E35" s="6" t="n">
-        <v>234273.52</v>
+        <v>152767.79</v>
       </c>
       <c r="F35" s="6" t="n">
-        <v>193711.09</v>
+        <v>361665.23</v>
       </c>
       <c r="G35" s="6" t="n">
-        <v>5000</v>
+        <v>0</v>
       </c>
       <c r="H35" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>6473.52</v>
+        <v>0</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
         <is>
-          <t>3318212</t>
+          <t>11422</t>
         </is>
       </c>
       <c r="B36" s="5" t="inlineStr">
         <is>
-          <t>مرتجع رواتب - فواتير</t>
+          <t>رسوم منتجات التبغ</t>
         </is>
       </c>
       <c r="C36" s="6" t="n">
-        <v>0</v>
+        <v>3000</v>
       </c>
       <c r="D36" s="6" t="n">
-        <v>0</v>
+        <v>5167</v>
       </c>
       <c r="E36" s="6" t="n">
-        <v>152767.79</v>
+        <v>45000</v>
       </c>
       <c r="F36" s="6" t="n">
-        <v>361665.23</v>
+        <v>0</v>
       </c>
       <c r="G36" s="6" t="n">
-        <v>0</v>
+        <v>24000</v>
       </c>
       <c r="H36" s="6" t="n">
         <v>0</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>0</v>
+        <v>27000</v>
       </c>
       <c r="J36" s="6" t="n">
         <v>0</v>
@@ -4467,48 +4377,48 @@
     <row r="37">
       <c r="A37" s="5" t="inlineStr">
         <is>
-          <t>11422</t>
+          <t>1422103</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>رسوم منتجات التبغ</t>
+          <t>تراخيص المحلات</t>
         </is>
       </c>
       <c r="C37" s="6" t="n">
-        <v>3000</v>
+        <v>0</v>
       </c>
       <c r="D37" s="6" t="n">
-        <v>5167</v>
+        <v>0</v>
       </c>
       <c r="E37" s="6" t="n">
-        <v>45000</v>
+        <v>0</v>
       </c>
       <c r="F37" s="6" t="n">
         <v>0</v>
       </c>
       <c r="G37" s="6" t="n">
-        <v>24000</v>
+        <v>67711.60000000001</v>
       </c>
       <c r="H37" s="6" t="n">
-        <v>0</v>
+        <v>16269.6</v>
       </c>
       <c r="I37" s="6" t="n">
-        <v>27000</v>
+        <v>1603.2</v>
       </c>
       <c r="J37" s="6" t="n">
-        <v>0</v>
+        <v>432</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
         <is>
-          <t>1422103</t>
+          <t>11452513</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>تراخيص المحلات</t>
+          <t>لوحات إرشـادية</t>
         </is>
       </c>
       <c r="C38" s="6" t="n">
@@ -4524,27 +4434,27 @@
         <v>0</v>
       </c>
       <c r="G38" s="6" t="n">
-        <v>67711.60000000001</v>
+        <v>55525</v>
       </c>
       <c r="H38" s="6" t="n">
-        <v>16269.6</v>
+        <v>12875</v>
       </c>
       <c r="I38" s="6" t="n">
-        <v>1603.2</v>
+        <v>9000</v>
       </c>
       <c r="J38" s="6" t="n">
-        <v>432</v>
+        <v>600</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
         <is>
-          <t>11452513</t>
+          <t>1421907</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>لوحات إرشـادية</t>
+          <t>إيرادات المخططات</t>
         </is>
       </c>
       <c r="C39" s="6" t="n">
@@ -4554,46 +4464,46 @@
         <v>0</v>
       </c>
       <c r="E39" s="6" t="n">
-        <v>0</v>
+        <v>21950</v>
       </c>
       <c r="F39" s="6" t="n">
-        <v>0</v>
+        <v>6250</v>
       </c>
       <c r="G39" s="6" t="n">
-        <v>55525</v>
+        <v>0</v>
       </c>
       <c r="H39" s="6" t="n">
-        <v>12875</v>
+        <v>0</v>
       </c>
       <c r="I39" s="6" t="n">
-        <v>9000</v>
+        <v>0</v>
       </c>
       <c r="J39" s="6" t="n">
-        <v>600</v>
+        <v>100</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
         <is>
-          <t>1421907</t>
+          <t>1421908</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>إيرادات المخططات</t>
+          <t>ايرادات  رسوم خدمات  بلدية</t>
         </is>
       </c>
       <c r="C40" s="6" t="n">
-        <v>0</v>
+        <v>16385</v>
       </c>
       <c r="D40" s="6" t="n">
         <v>0</v>
       </c>
       <c r="E40" s="6" t="n">
-        <v>21950</v>
+        <v>0</v>
       </c>
       <c r="F40" s="6" t="n">
-        <v>6250</v>
+        <v>0</v>
       </c>
       <c r="G40" s="6" t="n">
         <v>0</v>
@@ -4605,22 +4515,22 @@
         <v>0</v>
       </c>
       <c r="J40" s="6" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="5" t="inlineStr">
         <is>
-          <t>1421908</t>
+          <t>142161</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>ايرادات  رسوم خدمات  بلدية</t>
+          <t>تاجير مباني سكنية</t>
         </is>
       </c>
       <c r="C41" s="6" t="n">
-        <v>16385</v>
+        <v>0</v>
       </c>
       <c r="D41" s="6" t="n">
         <v>0</v>
@@ -4638,85 +4548,49 @@
         <v>0</v>
       </c>
       <c r="I41" s="6" t="n">
-        <v>0</v>
+        <v>6000</v>
       </c>
       <c r="J41" s="6" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="5" t="inlineStr">
-        <is>
-          <t>142161</t>
-        </is>
-      </c>
-      <c r="B42" s="5" t="inlineStr">
-        <is>
-          <t>تاجير مباني سكنية</t>
-        </is>
-      </c>
-      <c r="C42" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="D42" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="E42" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="F42" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="G42" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="H42" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="I42" s="6" t="n">
-        <v>6000</v>
-      </c>
-      <c r="J42" s="6" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="n"/>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t>الإجمالي</t>
         </is>
       </c>
-      <c r="C43" s="9">
-        <f>SUM(C4:C42)</f>
-        <v/>
-      </c>
-      <c r="D43" s="9">
-        <f>SUM(D4:D42)</f>
-        <v/>
-      </c>
-      <c r="E43" s="9">
-        <f>SUM(E4:E42)</f>
-        <v/>
-      </c>
-      <c r="F43" s="9">
-        <f>SUM(F4:F42)</f>
-        <v/>
-      </c>
-      <c r="G43" s="9">
-        <f>SUM(G4:G42)</f>
-        <v/>
-      </c>
-      <c r="H43" s="9">
-        <f>SUM(H4:H42)</f>
-        <v/>
-      </c>
-      <c r="I43" s="9">
-        <f>SUM(I4:I42)</f>
-        <v/>
-      </c>
-      <c r="J43" s="9">
-        <f>SUM(J4:J42)</f>
+      <c r="C42" s="9">
+        <f>SUM(C4:C41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="9">
+        <f>SUM(D4:D41)</f>
+        <v/>
+      </c>
+      <c r="E42" s="9">
+        <f>SUM(E4:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="9">
+        <f>SUM(F4:F41)</f>
+        <v/>
+      </c>
+      <c r="G42" s="9">
+        <f>SUM(G4:G41)</f>
+        <v/>
+      </c>
+      <c r="H42" s="9">
+        <f>SUM(H4:H41)</f>
+        <v/>
+      </c>
+      <c r="I42" s="9">
+        <f>SUM(I4:I41)</f>
+        <v/>
+      </c>
+      <c r="J42" s="9">
+        <f>SUM(J4:J41)</f>
         <v/>
       </c>
     </row>
@@ -4731,7 +4605,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -4855,12 +4729,19 @@
     <row r="15">
       <c r="A15" s="13" t="inlineStr">
         <is>
-          <t>6) تم دمج صفّي "بدون رقم" (خدمات علم + جزاءات، وجزاءات جزء ضئيل) في صف واحد لكل سنة.</t>
+          <t>6) تم استبعاد حساب قيمة الضريبة المضافة (11411) من كل الحسابات والإجماليات.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="13" t="inlineStr">
+        <is>
+          <t>6b) تم دمج صفّي "بدون رقم" (خدمات علم + جزاءات، وجزاءات جزء ضئيل) في صف واحد لكل سنة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>7) تنبيه: كثير من الحسابات تتذبذب بشدة بين السنوات (لوحات دعائية، تأجير المرافق، إيرادات متنوعة)، ومضاعفة 2026 على 12/9 تضخّم أو تقلّل هذه الأرقام؛ انظر عمود "تنبيه".</t>
         </is>

</xml_diff>

<commit_message>
Add per-year growth rates for each account
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/توقع_الفوترة_2026_2027.xlsx
+++ b/توقع_الفوترة_2026_2027.xlsx
@@ -13,7 +13,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'التوقعات'!$A$3:$N$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'التوقعات'!$A$3:$R$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -494,7 +494,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N42"/>
+  <dimension ref="A1:R42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -510,7 +510,11 @@
     <col width="14" customWidth="1" min="11" max="11"/>
     <col width="18" customWidth="1" min="12" max="12"/>
     <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="30" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -592,10 +596,30 @@
       </c>
       <c r="M3" s="4" t="inlineStr">
         <is>
-          <t>نمو 2026 مقابل 2025</t>
+          <t>نمو 2024 عن 2023</t>
         </is>
       </c>
       <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>نمو 2025 عن 2024</t>
+        </is>
+      </c>
+      <c r="O3" s="4" t="inlineStr">
+        <is>
+          <t>نمو 2026 توقع عن 2025</t>
+        </is>
+      </c>
+      <c r="P3" s="4" t="inlineStr">
+        <is>
+          <t>نمو 2027 (سيناريو النمو الثابت) عن 2026</t>
+        </is>
+      </c>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>نمو 2027 (سيناريو تاريخي) عن 2026</t>
+        </is>
+      </c>
+      <c r="R3" s="4" t="inlineStr">
         <is>
           <t>تنبيه</t>
         </is>
@@ -651,10 +675,26 @@
         <v/>
       </c>
       <c r="M4" s="7">
+        <f>IF(E4=0,"",F4/E4-1)</f>
+        <v/>
+      </c>
+      <c r="N4" s="7">
+        <f>IF(F4=0,"",G4/F4-1)</f>
+        <v/>
+      </c>
+      <c r="O4" s="7">
         <f>IF(G4=0,"",I4/G4-1)</f>
         <v/>
       </c>
-      <c r="N4" s="5" t="inlineStr"/>
+      <c r="P4" s="7">
+        <f>IF(I4=0,"",J4/I4-1)</f>
+        <v/>
+      </c>
+      <c r="Q4" s="7">
+        <f>IF(I4=0,"",L4/I4-1)</f>
+        <v/>
+      </c>
+      <c r="R4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
@@ -706,10 +746,26 @@
         <v/>
       </c>
       <c r="M5" s="7">
+        <f>IF(E5=0,"",F5/E5-1)</f>
+        <v/>
+      </c>
+      <c r="N5" s="7">
+        <f>IF(F5=0,"",G5/F5-1)</f>
+        <v/>
+      </c>
+      <c r="O5" s="7">
         <f>IF(G5=0,"",I5/G5-1)</f>
         <v/>
       </c>
-      <c r="N5" s="5" t="inlineStr"/>
+      <c r="P5" s="7">
+        <f>IF(I5=0,"",J5/I5-1)</f>
+        <v/>
+      </c>
+      <c r="Q5" s="7">
+        <f>IF(I5=0,"",L5/I5-1)</f>
+        <v/>
+      </c>
+      <c r="R5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="5" t="inlineStr">
@@ -761,10 +817,26 @@
         <v/>
       </c>
       <c r="M6" s="7">
+        <f>IF(E6=0,"",F6/E6-1)</f>
+        <v/>
+      </c>
+      <c r="N6" s="7">
+        <f>IF(F6=0,"",G6/F6-1)</f>
+        <v/>
+      </c>
+      <c r="O6" s="7">
         <f>IF(G6=0,"",I6/G6-1)</f>
         <v/>
       </c>
-      <c r="N6" s="5" t="inlineStr">
+      <c r="P6" s="7">
+        <f>IF(I6=0,"",J6/I6-1)</f>
+        <v/>
+      </c>
+      <c r="Q6" s="7">
+        <f>IF(I6=0,"",L6/I6-1)</f>
+        <v/>
+      </c>
+      <c r="R6" s="5" t="inlineStr">
         <is>
           <t>تذبذب عالٍ – راجع التوقع</t>
         </is>
@@ -820,10 +892,26 @@
         <v/>
       </c>
       <c r="M7" s="7">
+        <f>IF(E7=0,"",F7/E7-1)</f>
+        <v/>
+      </c>
+      <c r="N7" s="7">
+        <f>IF(F7=0,"",G7/F7-1)</f>
+        <v/>
+      </c>
+      <c r="O7" s="7">
         <f>IF(G7=0,"",I7/G7-1)</f>
         <v/>
       </c>
-      <c r="N7" s="5" t="inlineStr"/>
+      <c r="P7" s="7">
+        <f>IF(I7=0,"",J7/I7-1)</f>
+        <v/>
+      </c>
+      <c r="Q7" s="7">
+        <f>IF(I7=0,"",L7/I7-1)</f>
+        <v/>
+      </c>
+      <c r="R7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="5" t="inlineStr">
@@ -875,10 +963,26 @@
         <v/>
       </c>
       <c r="M8" s="7">
+        <f>IF(E8=0,"",F8/E8-1)</f>
+        <v/>
+      </c>
+      <c r="N8" s="7">
+        <f>IF(F8=0,"",G8/F8-1)</f>
+        <v/>
+      </c>
+      <c r="O8" s="7">
         <f>IF(G8=0,"",I8/G8-1)</f>
         <v/>
       </c>
-      <c r="N8" s="5" t="inlineStr"/>
+      <c r="P8" s="7">
+        <f>IF(I8=0,"",J8/I8-1)</f>
+        <v/>
+      </c>
+      <c r="Q8" s="7">
+        <f>IF(I8=0,"",L8/I8-1)</f>
+        <v/>
+      </c>
+      <c r="R8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
@@ -930,10 +1034,26 @@
         <v/>
       </c>
       <c r="M9" s="7">
+        <f>IF(E9=0,"",F9/E9-1)</f>
+        <v/>
+      </c>
+      <c r="N9" s="7">
+        <f>IF(F9=0,"",G9/F9-1)</f>
+        <v/>
+      </c>
+      <c r="O9" s="7">
         <f>IF(G9=0,"",I9/G9-1)</f>
         <v/>
       </c>
-      <c r="N9" s="5" t="inlineStr"/>
+      <c r="P9" s="7">
+        <f>IF(I9=0,"",J9/I9-1)</f>
+        <v/>
+      </c>
+      <c r="Q9" s="7">
+        <f>IF(I9=0,"",L9/I9-1)</f>
+        <v/>
+      </c>
+      <c r="R9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="5" t="inlineStr">
@@ -985,10 +1105,26 @@
         <v/>
       </c>
       <c r="M10" s="7">
+        <f>IF(E10=0,"",F10/E10-1)</f>
+        <v/>
+      </c>
+      <c r="N10" s="7">
+        <f>IF(F10=0,"",G10/F10-1)</f>
+        <v/>
+      </c>
+      <c r="O10" s="7">
         <f>IF(G10=0,"",I10/G10-1)</f>
         <v/>
       </c>
-      <c r="N10" s="5" t="inlineStr"/>
+      <c r="P10" s="7">
+        <f>IF(I10=0,"",J10/I10-1)</f>
+        <v/>
+      </c>
+      <c r="Q10" s="7">
+        <f>IF(I10=0,"",L10/I10-1)</f>
+        <v/>
+      </c>
+      <c r="R10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
@@ -1040,10 +1176,26 @@
         <v/>
       </c>
       <c r="M11" s="7">
+        <f>IF(E11=0,"",F11/E11-1)</f>
+        <v/>
+      </c>
+      <c r="N11" s="7">
+        <f>IF(F11=0,"",G11/F11-1)</f>
+        <v/>
+      </c>
+      <c r="O11" s="7">
         <f>IF(G11=0,"",I11/G11-1)</f>
         <v/>
       </c>
-      <c r="N11" s="5" t="inlineStr">
+      <c r="P11" s="7">
+        <f>IF(I11=0,"",J11/I11-1)</f>
+        <v/>
+      </c>
+      <c r="Q11" s="7">
+        <f>IF(I11=0,"",L11/I11-1)</f>
+        <v/>
+      </c>
+      <c r="R11" s="5" t="inlineStr">
         <is>
           <t>تذبذب عالٍ – راجع التوقع</t>
         </is>
@@ -1099,10 +1251,26 @@
         <v/>
       </c>
       <c r="M12" s="7">
+        <f>IF(E12=0,"",F12/E12-1)</f>
+        <v/>
+      </c>
+      <c r="N12" s="7">
+        <f>IF(F12=0,"",G12/F12-1)</f>
+        <v/>
+      </c>
+      <c r="O12" s="7">
         <f>IF(G12=0,"",I12/G12-1)</f>
         <v/>
       </c>
-      <c r="N12" s="5" t="inlineStr">
+      <c r="P12" s="7">
+        <f>IF(I12=0,"",J12/I12-1)</f>
+        <v/>
+      </c>
+      <c r="Q12" s="7">
+        <f>IF(I12=0,"",L12/I12-1)</f>
+        <v/>
+      </c>
+      <c r="R12" s="5" t="inlineStr">
         <is>
           <t>تذبذب عالٍ – راجع التوقع</t>
         </is>
@@ -1158,10 +1326,26 @@
         <v/>
       </c>
       <c r="M13" s="7">
+        <f>IF(E13=0,"",F13/E13-1)</f>
+        <v/>
+      </c>
+      <c r="N13" s="7">
+        <f>IF(F13=0,"",G13/F13-1)</f>
+        <v/>
+      </c>
+      <c r="O13" s="7">
         <f>IF(G13=0,"",I13/G13-1)</f>
         <v/>
       </c>
-      <c r="N13" s="5" t="inlineStr">
+      <c r="P13" s="7">
+        <f>IF(I13=0,"",J13/I13-1)</f>
+        <v/>
+      </c>
+      <c r="Q13" s="7">
+        <f>IF(I13=0,"",L13/I13-1)</f>
+        <v/>
+      </c>
+      <c r="R13" s="5" t="inlineStr">
         <is>
           <t>تذبذب عالٍ – راجع التوقع</t>
         </is>
@@ -1217,10 +1401,26 @@
         <v/>
       </c>
       <c r="M14" s="7">
+        <f>IF(E14=0,"",F14/E14-1)</f>
+        <v/>
+      </c>
+      <c r="N14" s="7">
+        <f>IF(F14=0,"",G14/F14-1)</f>
+        <v/>
+      </c>
+      <c r="O14" s="7">
         <f>IF(G14=0,"",I14/G14-1)</f>
         <v/>
       </c>
-      <c r="N14" s="5" t="inlineStr"/>
+      <c r="P14" s="7">
+        <f>IF(I14=0,"",J14/I14-1)</f>
+        <v/>
+      </c>
+      <c r="Q14" s="7">
+        <f>IF(I14=0,"",L14/I14-1)</f>
+        <v/>
+      </c>
+      <c r="R14" s="5" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
@@ -1272,10 +1472,26 @@
         <v/>
       </c>
       <c r="M15" s="7">
+        <f>IF(E15=0,"",F15/E15-1)</f>
+        <v/>
+      </c>
+      <c r="N15" s="7">
+        <f>IF(F15=0,"",G15/F15-1)</f>
+        <v/>
+      </c>
+      <c r="O15" s="7">
         <f>IF(G15=0,"",I15/G15-1)</f>
         <v/>
       </c>
-      <c r="N15" s="5" t="inlineStr"/>
+      <c r="P15" s="7">
+        <f>IF(I15=0,"",J15/I15-1)</f>
+        <v/>
+      </c>
+      <c r="Q15" s="7">
+        <f>IF(I15=0,"",L15/I15-1)</f>
+        <v/>
+      </c>
+      <c r="R15" s="5" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="5" t="inlineStr">
@@ -1327,10 +1543,26 @@
         <v/>
       </c>
       <c r="M16" s="7">
+        <f>IF(E16=0,"",F16/E16-1)</f>
+        <v/>
+      </c>
+      <c r="N16" s="7">
+        <f>IF(F16=0,"",G16/F16-1)</f>
+        <v/>
+      </c>
+      <c r="O16" s="7">
         <f>IF(G16=0,"",I16/G16-1)</f>
         <v/>
       </c>
-      <c r="N16" s="5" t="inlineStr"/>
+      <c r="P16" s="7">
+        <f>IF(I16=0,"",J16/I16-1)</f>
+        <v/>
+      </c>
+      <c r="Q16" s="7">
+        <f>IF(I16=0,"",L16/I16-1)</f>
+        <v/>
+      </c>
+      <c r="R16" s="5" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
@@ -1382,10 +1614,26 @@
         <v/>
       </c>
       <c r="M17" s="7">
+        <f>IF(E17=0,"",F17/E17-1)</f>
+        <v/>
+      </c>
+      <c r="N17" s="7">
+        <f>IF(F17=0,"",G17/F17-1)</f>
+        <v/>
+      </c>
+      <c r="O17" s="7">
         <f>IF(G17=0,"",I17/G17-1)</f>
         <v/>
       </c>
-      <c r="N17" s="5" t="inlineStr"/>
+      <c r="P17" s="7">
+        <f>IF(I17=0,"",J17/I17-1)</f>
+        <v/>
+      </c>
+      <c r="Q17" s="7">
+        <f>IF(I17=0,"",L17/I17-1)</f>
+        <v/>
+      </c>
+      <c r="R17" s="5" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" s="5" t="inlineStr">
@@ -1437,10 +1685,26 @@
         <v/>
       </c>
       <c r="M18" s="7">
+        <f>IF(E18=0,"",F18/E18-1)</f>
+        <v/>
+      </c>
+      <c r="N18" s="7">
+        <f>IF(F18=0,"",G18/F18-1)</f>
+        <v/>
+      </c>
+      <c r="O18" s="7">
         <f>IF(G18=0,"",I18/G18-1)</f>
         <v/>
       </c>
-      <c r="N18" s="5" t="inlineStr"/>
+      <c r="P18" s="7">
+        <f>IF(I18=0,"",J18/I18-1)</f>
+        <v/>
+      </c>
+      <c r="Q18" s="7">
+        <f>IF(I18=0,"",L18/I18-1)</f>
+        <v/>
+      </c>
+      <c r="R18" s="5" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="5" t="inlineStr">
@@ -1492,10 +1756,26 @@
         <v/>
       </c>
       <c r="M19" s="7">
+        <f>IF(E19=0,"",F19/E19-1)</f>
+        <v/>
+      </c>
+      <c r="N19" s="7">
+        <f>IF(F19=0,"",G19/F19-1)</f>
+        <v/>
+      </c>
+      <c r="O19" s="7">
         <f>IF(G19=0,"",I19/G19-1)</f>
         <v/>
       </c>
-      <c r="N19" s="5" t="inlineStr"/>
+      <c r="P19" s="7">
+        <f>IF(I19=0,"",J19/I19-1)</f>
+        <v/>
+      </c>
+      <c r="Q19" s="7">
+        <f>IF(I19=0,"",L19/I19-1)</f>
+        <v/>
+      </c>
+      <c r="R19" s="5" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
@@ -1547,10 +1827,26 @@
         <v/>
       </c>
       <c r="M20" s="7">
+        <f>IF(E20=0,"",F20/E20-1)</f>
+        <v/>
+      </c>
+      <c r="N20" s="7">
+        <f>IF(F20=0,"",G20/F20-1)</f>
+        <v/>
+      </c>
+      <c r="O20" s="7">
         <f>IF(G20=0,"",I20/G20-1)</f>
         <v/>
       </c>
-      <c r="N20" s="5" t="inlineStr"/>
+      <c r="P20" s="7">
+        <f>IF(I20=0,"",J20/I20-1)</f>
+        <v/>
+      </c>
+      <c r="Q20" s="7">
+        <f>IF(I20=0,"",L20/I20-1)</f>
+        <v/>
+      </c>
+      <c r="R20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
@@ -1602,10 +1898,26 @@
         <v/>
       </c>
       <c r="M21" s="7">
+        <f>IF(E21=0,"",F21/E21-1)</f>
+        <v/>
+      </c>
+      <c r="N21" s="7">
+        <f>IF(F21=0,"",G21/F21-1)</f>
+        <v/>
+      </c>
+      <c r="O21" s="7">
         <f>IF(G21=0,"",I21/G21-1)</f>
         <v/>
       </c>
-      <c r="N21" s="5" t="inlineStr">
+      <c r="P21" s="7">
+        <f>IF(I21=0,"",J21/I21-1)</f>
+        <v/>
+      </c>
+      <c r="Q21" s="7">
+        <f>IF(I21=0,"",L21/I21-1)</f>
+        <v/>
+      </c>
+      <c r="R21" s="5" t="inlineStr">
         <is>
           <t>تذبذب عالٍ – راجع التوقع</t>
         </is>
@@ -1661,10 +1973,26 @@
         <v/>
       </c>
       <c r="M22" s="7">
+        <f>IF(E22=0,"",F22/E22-1)</f>
+        <v/>
+      </c>
+      <c r="N22" s="7">
+        <f>IF(F22=0,"",G22/F22-1)</f>
+        <v/>
+      </c>
+      <c r="O22" s="7">
         <f>IF(G22=0,"",I22/G22-1)</f>
         <v/>
       </c>
-      <c r="N22" s="5" t="inlineStr"/>
+      <c r="P22" s="7">
+        <f>IF(I22=0,"",J22/I22-1)</f>
+        <v/>
+      </c>
+      <c r="Q22" s="7">
+        <f>IF(I22=0,"",L22/I22-1)</f>
+        <v/>
+      </c>
+      <c r="R22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
@@ -1716,10 +2044,26 @@
         <v/>
       </c>
       <c r="M23" s="7">
+        <f>IF(E23=0,"",F23/E23-1)</f>
+        <v/>
+      </c>
+      <c r="N23" s="7">
+        <f>IF(F23=0,"",G23/F23-1)</f>
+        <v/>
+      </c>
+      <c r="O23" s="7">
         <f>IF(G23=0,"",I23/G23-1)</f>
         <v/>
       </c>
-      <c r="N23" s="5" t="inlineStr">
+      <c r="P23" s="7">
+        <f>IF(I23=0,"",J23/I23-1)</f>
+        <v/>
+      </c>
+      <c r="Q23" s="7">
+        <f>IF(I23=0,"",L23/I23-1)</f>
+        <v/>
+      </c>
+      <c r="R23" s="5" t="inlineStr">
         <is>
           <t>تذبذب عالٍ – راجع التوقع</t>
         </is>
@@ -1775,10 +2119,26 @@
         <v/>
       </c>
       <c r="M24" s="7">
+        <f>IF(E24=0,"",F24/E24-1)</f>
+        <v/>
+      </c>
+      <c r="N24" s="7">
+        <f>IF(F24=0,"",G24/F24-1)</f>
+        <v/>
+      </c>
+      <c r="O24" s="7">
         <f>IF(G24=0,"",I24/G24-1)</f>
         <v/>
       </c>
-      <c r="N24" s="5" t="inlineStr"/>
+      <c r="P24" s="7">
+        <f>IF(I24=0,"",J24/I24-1)</f>
+        <v/>
+      </c>
+      <c r="Q24" s="7">
+        <f>IF(I24=0,"",L24/I24-1)</f>
+        <v/>
+      </c>
+      <c r="R24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="5" t="inlineStr">
@@ -1830,10 +2190,26 @@
         <v/>
       </c>
       <c r="M25" s="7">
+        <f>IF(E25=0,"",F25/E25-1)</f>
+        <v/>
+      </c>
+      <c r="N25" s="7">
+        <f>IF(F25=0,"",G25/F25-1)</f>
+        <v/>
+      </c>
+      <c r="O25" s="7">
         <f>IF(G25=0,"",I25/G25-1)</f>
         <v/>
       </c>
-      <c r="N25" s="5" t="inlineStr">
+      <c r="P25" s="7">
+        <f>IF(I25=0,"",J25/I25-1)</f>
+        <v/>
+      </c>
+      <c r="Q25" s="7">
+        <f>IF(I25=0,"",L25/I25-1)</f>
+        <v/>
+      </c>
+      <c r="R25" s="5" t="inlineStr">
         <is>
           <t>تذبذب عالٍ – راجع التوقع</t>
         </is>
@@ -1889,10 +2265,26 @@
         <v/>
       </c>
       <c r="M26" s="7">
+        <f>IF(E26=0,"",F26/E26-1)</f>
+        <v/>
+      </c>
+      <c r="N26" s="7">
+        <f>IF(F26=0,"",G26/F26-1)</f>
+        <v/>
+      </c>
+      <c r="O26" s="7">
         <f>IF(G26=0,"",I26/G26-1)</f>
         <v/>
       </c>
-      <c r="N26" s="5" t="inlineStr"/>
+      <c r="P26" s="7">
+        <f>IF(I26=0,"",J26/I26-1)</f>
+        <v/>
+      </c>
+      <c r="Q26" s="7">
+        <f>IF(I26=0,"",L26/I26-1)</f>
+        <v/>
+      </c>
+      <c r="R26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
@@ -1944,10 +2336,26 @@
         <v/>
       </c>
       <c r="M27" s="7">
+        <f>IF(E27=0,"",F27/E27-1)</f>
+        <v/>
+      </c>
+      <c r="N27" s="7">
+        <f>IF(F27=0,"",G27/F27-1)</f>
+        <v/>
+      </c>
+      <c r="O27" s="7">
         <f>IF(G27=0,"",I27/G27-1)</f>
         <v/>
       </c>
-      <c r="N27" s="5" t="inlineStr">
+      <c r="P27" s="7">
+        <f>IF(I27=0,"",J27/I27-1)</f>
+        <v/>
+      </c>
+      <c r="Q27" s="7">
+        <f>IF(I27=0,"",L27/I27-1)</f>
+        <v/>
+      </c>
+      <c r="R27" s="5" t="inlineStr">
         <is>
           <t>تذبذب عالٍ – راجع التوقع</t>
         </is>
@@ -2003,10 +2411,26 @@
         <v/>
       </c>
       <c r="M28" s="7">
+        <f>IF(E28=0,"",F28/E28-1)</f>
+        <v/>
+      </c>
+      <c r="N28" s="7">
+        <f>IF(F28=0,"",G28/F28-1)</f>
+        <v/>
+      </c>
+      <c r="O28" s="7">
         <f>IF(G28=0,"",I28/G28-1)</f>
         <v/>
       </c>
-      <c r="N28" s="5" t="inlineStr"/>
+      <c r="P28" s="7">
+        <f>IF(I28=0,"",J28/I28-1)</f>
+        <v/>
+      </c>
+      <c r="Q28" s="7">
+        <f>IF(I28=0,"",L28/I28-1)</f>
+        <v/>
+      </c>
+      <c r="R28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
@@ -2058,10 +2482,26 @@
         <v/>
       </c>
       <c r="M29" s="7">
+        <f>IF(E29=0,"",F29/E29-1)</f>
+        <v/>
+      </c>
+      <c r="N29" s="7">
+        <f>IF(F29=0,"",G29/F29-1)</f>
+        <v/>
+      </c>
+      <c r="O29" s="7">
         <f>IF(G29=0,"",I29/G29-1)</f>
         <v/>
       </c>
-      <c r="N29" s="5" t="inlineStr"/>
+      <c r="P29" s="7">
+        <f>IF(I29=0,"",J29/I29-1)</f>
+        <v/>
+      </c>
+      <c r="Q29" s="7">
+        <f>IF(I29=0,"",L29/I29-1)</f>
+        <v/>
+      </c>
+      <c r="R29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
@@ -2113,10 +2553,26 @@
         <v/>
       </c>
       <c r="M30" s="7">
+        <f>IF(E30=0,"",F30/E30-1)</f>
+        <v/>
+      </c>
+      <c r="N30" s="7">
+        <f>IF(F30=0,"",G30/F30-1)</f>
+        <v/>
+      </c>
+      <c r="O30" s="7">
         <f>IF(G30=0,"",I30/G30-1)</f>
         <v/>
       </c>
-      <c r="N30" s="5" t="inlineStr"/>
+      <c r="P30" s="7">
+        <f>IF(I30=0,"",J30/I30-1)</f>
+        <v/>
+      </c>
+      <c r="Q30" s="7">
+        <f>IF(I30=0,"",L30/I30-1)</f>
+        <v/>
+      </c>
+      <c r="R30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
@@ -2168,10 +2624,26 @@
         <v/>
       </c>
       <c r="M31" s="7">
+        <f>IF(E31=0,"",F31/E31-1)</f>
+        <v/>
+      </c>
+      <c r="N31" s="7">
+        <f>IF(F31=0,"",G31/F31-1)</f>
+        <v/>
+      </c>
+      <c r="O31" s="7">
         <f>IF(G31=0,"",I31/G31-1)</f>
         <v/>
       </c>
-      <c r="N31" s="5" t="inlineStr"/>
+      <c r="P31" s="7">
+        <f>IF(I31=0,"",J31/I31-1)</f>
+        <v/>
+      </c>
+      <c r="Q31" s="7">
+        <f>IF(I31=0,"",L31/I31-1)</f>
+        <v/>
+      </c>
+      <c r="R31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="5" t="inlineStr">
@@ -2223,10 +2695,26 @@
         <v/>
       </c>
       <c r="M32" s="7">
+        <f>IF(E32=0,"",F32/E32-1)</f>
+        <v/>
+      </c>
+      <c r="N32" s="7">
+        <f>IF(F32=0,"",G32/F32-1)</f>
+        <v/>
+      </c>
+      <c r="O32" s="7">
         <f>IF(G32=0,"",I32/G32-1)</f>
         <v/>
       </c>
-      <c r="N32" s="5" t="inlineStr"/>
+      <c r="P32" s="7">
+        <f>IF(I32=0,"",J32/I32-1)</f>
+        <v/>
+      </c>
+      <c r="Q32" s="7">
+        <f>IF(I32=0,"",L32/I32-1)</f>
+        <v/>
+      </c>
+      <c r="R32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="5" t="inlineStr">
@@ -2278,10 +2766,26 @@
         <v/>
       </c>
       <c r="M33" s="7">
+        <f>IF(E33=0,"",F33/E33-1)</f>
+        <v/>
+      </c>
+      <c r="N33" s="7">
+        <f>IF(F33=0,"",G33/F33-1)</f>
+        <v/>
+      </c>
+      <c r="O33" s="7">
         <f>IF(G33=0,"",I33/G33-1)</f>
         <v/>
       </c>
-      <c r="N33" s="5" t="inlineStr"/>
+      <c r="P33" s="7">
+        <f>IF(I33=0,"",J33/I33-1)</f>
+        <v/>
+      </c>
+      <c r="Q33" s="7">
+        <f>IF(I33=0,"",L33/I33-1)</f>
+        <v/>
+      </c>
+      <c r="R33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="5" t="inlineStr">
@@ -2333,10 +2837,26 @@
         <v/>
       </c>
       <c r="M34" s="7">
+        <f>IF(E34=0,"",F34/E34-1)</f>
+        <v/>
+      </c>
+      <c r="N34" s="7">
+        <f>IF(F34=0,"",G34/F34-1)</f>
+        <v/>
+      </c>
+      <c r="O34" s="7">
         <f>IF(G34=0,"",I34/G34-1)</f>
         <v/>
       </c>
-      <c r="N34" s="5" t="inlineStr"/>
+      <c r="P34" s="7">
+        <f>IF(I34=0,"",J34/I34-1)</f>
+        <v/>
+      </c>
+      <c r="Q34" s="7">
+        <f>IF(I34=0,"",L34/I34-1)</f>
+        <v/>
+      </c>
+      <c r="R34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="5" t="inlineStr">
@@ -2388,10 +2908,26 @@
         <v/>
       </c>
       <c r="M35" s="7">
+        <f>IF(E35=0,"",F35/E35-1)</f>
+        <v/>
+      </c>
+      <c r="N35" s="7">
+        <f>IF(F35=0,"",G35/F35-1)</f>
+        <v/>
+      </c>
+      <c r="O35" s="7">
         <f>IF(G35=0,"",I35/G35-1)</f>
         <v/>
       </c>
-      <c r="N35" s="5" t="inlineStr"/>
+      <c r="P35" s="7">
+        <f>IF(I35=0,"",J35/I35-1)</f>
+        <v/>
+      </c>
+      <c r="Q35" s="7">
+        <f>IF(I35=0,"",L35/I35-1)</f>
+        <v/>
+      </c>
+      <c r="R35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="5" t="inlineStr">
@@ -2443,10 +2979,26 @@
         <v/>
       </c>
       <c r="M36" s="7">
+        <f>IF(E36=0,"",F36/E36-1)</f>
+        <v/>
+      </c>
+      <c r="N36" s="7">
+        <f>IF(F36=0,"",G36/F36-1)</f>
+        <v/>
+      </c>
+      <c r="O36" s="7">
         <f>IF(G36=0,"",I36/G36-1)</f>
         <v/>
       </c>
-      <c r="N36" s="5" t="inlineStr">
+      <c r="P36" s="7">
+        <f>IF(I36=0,"",J36/I36-1)</f>
+        <v/>
+      </c>
+      <c r="Q36" s="7">
+        <f>IF(I36=0,"",L36/I36-1)</f>
+        <v/>
+      </c>
+      <c r="R36" s="5" t="inlineStr">
         <is>
           <t>متوقف في 2026 – توقعه صفر</t>
         </is>
@@ -2502,10 +3054,26 @@
         <v/>
       </c>
       <c r="M37" s="7">
+        <f>IF(E37=0,"",F37/E37-1)</f>
+        <v/>
+      </c>
+      <c r="N37" s="7">
+        <f>IF(F37=0,"",G37/F37-1)</f>
+        <v/>
+      </c>
+      <c r="O37" s="7">
         <f>IF(G37=0,"",I37/G37-1)</f>
         <v/>
       </c>
-      <c r="N37" s="5" t="inlineStr"/>
+      <c r="P37" s="7">
+        <f>IF(I37=0,"",J37/I37-1)</f>
+        <v/>
+      </c>
+      <c r="Q37" s="7">
+        <f>IF(I37=0,"",L37/I37-1)</f>
+        <v/>
+      </c>
+      <c r="R37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="5" t="inlineStr">
@@ -2557,10 +3125,26 @@
         <v/>
       </c>
       <c r="M38" s="7">
+        <f>IF(E38=0,"",F38/E38-1)</f>
+        <v/>
+      </c>
+      <c r="N38" s="7">
+        <f>IF(F38=0,"",G38/F38-1)</f>
+        <v/>
+      </c>
+      <c r="O38" s="7">
         <f>IF(G38=0,"",I38/G38-1)</f>
         <v/>
       </c>
-      <c r="N38" s="5" t="inlineStr"/>
+      <c r="P38" s="7">
+        <f>IF(I38=0,"",J38/I38-1)</f>
+        <v/>
+      </c>
+      <c r="Q38" s="7">
+        <f>IF(I38=0,"",L38/I38-1)</f>
+        <v/>
+      </c>
+      <c r="R38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="5" t="inlineStr">
@@ -2612,10 +3196,26 @@
         <v/>
       </c>
       <c r="M39" s="7">
+        <f>IF(E39=0,"",F39/E39-1)</f>
+        <v/>
+      </c>
+      <c r="N39" s="7">
+        <f>IF(F39=0,"",G39/F39-1)</f>
+        <v/>
+      </c>
+      <c r="O39" s="7">
         <f>IF(G39=0,"",I39/G39-1)</f>
         <v/>
       </c>
-      <c r="N39" s="5" t="inlineStr"/>
+      <c r="P39" s="7">
+        <f>IF(I39=0,"",J39/I39-1)</f>
+        <v/>
+      </c>
+      <c r="Q39" s="7">
+        <f>IF(I39=0,"",L39/I39-1)</f>
+        <v/>
+      </c>
+      <c r="R39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="5" t="inlineStr">
@@ -2667,10 +3267,26 @@
         <v/>
       </c>
       <c r="M40" s="7">
+        <f>IF(E40=0,"",F40/E40-1)</f>
+        <v/>
+      </c>
+      <c r="N40" s="7">
+        <f>IF(F40=0,"",G40/F40-1)</f>
+        <v/>
+      </c>
+      <c r="O40" s="7">
         <f>IF(G40=0,"",I40/G40-1)</f>
         <v/>
       </c>
-      <c r="N40" s="5" t="inlineStr">
+      <c r="P40" s="7">
+        <f>IF(I40=0,"",J40/I40-1)</f>
+        <v/>
+      </c>
+      <c r="Q40" s="7">
+        <f>IF(I40=0,"",L40/I40-1)</f>
+        <v/>
+      </c>
+      <c r="R40" s="5" t="inlineStr">
         <is>
           <t>متوقف في 2026 – توقعه صفر</t>
         </is>
@@ -2726,10 +3342,26 @@
         <v/>
       </c>
       <c r="M41" s="7">
+        <f>IF(E41=0,"",F41/E41-1)</f>
+        <v/>
+      </c>
+      <c r="N41" s="7">
+        <f>IF(F41=0,"",G41/F41-1)</f>
+        <v/>
+      </c>
+      <c r="O41" s="7">
         <f>IF(G41=0,"",I41/G41-1)</f>
         <v/>
       </c>
-      <c r="N41" s="5" t="inlineStr">
+      <c r="P41" s="7">
+        <f>IF(I41=0,"",J41/I41-1)</f>
+        <v/>
+      </c>
+      <c r="Q41" s="7">
+        <f>IF(I41=0,"",L41/I41-1)</f>
+        <v/>
+      </c>
+      <c r="R41" s="5" t="inlineStr">
         <is>
           <t>متوقف في 2026 – توقعه صفر</t>
         </is>
@@ -2777,13 +3409,29 @@
         <v/>
       </c>
       <c r="M42" s="10">
-        <f>I42/G42-1</f>
-        <v/>
-      </c>
-      <c r="N42" s="8" t="n"/>
+        <f>IF(E42=0,"",F42/E42-1)</f>
+        <v/>
+      </c>
+      <c r="N42" s="10">
+        <f>IF(F42=0,"",G42/F42-1)</f>
+        <v/>
+      </c>
+      <c r="O42" s="10">
+        <f>IF(G42=0,"",I42/G42-1)</f>
+        <v/>
+      </c>
+      <c r="P42" s="10">
+        <f>IF(I42=0,"",J42/I42-1)</f>
+        <v/>
+      </c>
+      <c r="Q42" s="10">
+        <f>IF(I42=0,"",L42/I42-1)</f>
+        <v/>
+      </c>
+      <c r="R42" s="8" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A3:N41"/>
+  <autoFilter ref="A3:R41"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -4605,7 +5253,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C17"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -4743,6 +5391,13 @@
     <row r="17">
       <c r="A17" s="13" t="inlineStr">
         <is>
+          <t>6c) أعمدة النمو لكل حساب: نمو كل سنة عن السنة السابقة (2024 عن 2023، 2025 عن 2024، 2026 توقع عن 2025، و2027 عن 2026 للسيناريوهين). تظهر فارغة عندما تكون السنة السابقة صفراً.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="13" t="inlineStr">
+        <is>
           <t>7) تنبيه: كثير من الحسابات تتذبذب بشدة بين السنوات (لوحات دعائية، تأجير المرافق، إيرادات متنوعة)، ومضاعفة 2026 على 12/9 تضخّم أو تقلّل هذه الأرقام؛ انظر عمود "تنبيه".</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add collected (actual) 2026 closing forecast sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/توقع_الفوترة_2026_2027.xlsx
+++ b/توقع_الفوترة_2026_2027.xlsx
@@ -10,10 +10,12 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="التوقعات" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حسب التبويب" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تفصيل المكونات" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="توقع المحصل 2026" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'التوقعات'!$A$3:$R$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'توقع المحصل 2026'!$A$3:$N$41</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -26,7 +28,7 @@
     <numFmt numFmtId="165" formatCode="0.0%"/>
     <numFmt numFmtId="166" formatCode="#,##0;(#,##0);&quot;-&quot;"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,6 +61,10 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="9"/>
     </font>
   </fonts>
   <fills count="5">
@@ -110,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -126,6 +132,7 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -5253,7 +5260,2264 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C18"/>
+  <dimension ref="A1:N42"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>توقع إقفال 2026 كمحصّل فعلي (مسدد عن السنة + محصل سنوات سابقة)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>توقع 2026 = المحصل الفعلي حتى سبتمبر × معامل الافتراضات (12÷9). الحسابات المتوقفة في 2026 (لا فوترة ولا تحصيل) توقعها صفر. الضريبة مستبعدة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>رقم الحساب</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>اسم الحساب</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>التبويب</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>الحالة</t>
+        </is>
+      </c>
+      <c r="E3" s="4" t="inlineStr">
+        <is>
+          <t>2023 محصّل</t>
+        </is>
+      </c>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>2024 محصّل</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>2025 محصّل</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>2026 محصّل حتى سبتمبر</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>منه: مسدد عن 2026</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>منه: محصل سنوات سابقة</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>2026 توقع إقفال (محصّل)</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>نمو التوقع عن 2025</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="inlineStr">
+        <is>
+          <t>توقع الفوترة 2026</t>
+        </is>
+      </c>
+      <c r="N3" s="4" t="inlineStr">
+        <is>
+          <t>نسبة المحصّل إلى المفوتر (توقع)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>1438001</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات و غرامات مفروضة بموجب أنظمة الجهة</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D4" s="5">
+        <f>IF(AND(1065200061.32=0,370612328.79=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E4" s="6" t="n">
+        <v>459891610.83</v>
+      </c>
+      <c r="F4" s="6" t="n">
+        <v>303585685.79</v>
+      </c>
+      <c r="G4" s="6" t="n">
+        <v>308012204.69</v>
+      </c>
+      <c r="H4" s="6" t="n">
+        <v>370612328.79</v>
+      </c>
+      <c r="I4" s="6" t="n">
+        <v>204559511.42</v>
+      </c>
+      <c r="J4" s="6" t="n">
+        <v>166052817.37</v>
+      </c>
+      <c r="K4" s="6">
+        <f>IF(D4="متوقف",0,H4*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L4" s="7">
+        <f>IF(G4=0,"",K4/G4-1)</f>
+        <v/>
+      </c>
+      <c r="M4" s="6">
+        <f>IFERROR(VLOOKUP(A4,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N4" s="7">
+        <f>IF(M4=0,"",K4/M4)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>14155</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>ريع الأراضي (تأجير الأراض )</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D5" s="5">
+        <f>IF(AND(803599432.03=0,612889120.88=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>779186906.26</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>803323461.12</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>649331791.52</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>612889120.88</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>453484669.92</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>159404450.96</v>
+      </c>
+      <c r="K5" s="6">
+        <f>IF(D5="متوقف",0,H5*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L5" s="7">
+        <f>IF(G5=0,"",K5/G5-1)</f>
+        <v/>
+      </c>
+      <c r="M5" s="6">
+        <f>IFERROR(VLOOKUP(A5,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N5" s="7">
+        <f>IF(M5=0,"",K5/M5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>142113</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  اللوحات الدعائية</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D6" s="5">
+        <f>IF(AND(126475270.21=0,122031767.73=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>157946538.8</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>609523702.9299999</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>1016877058.52</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>122031767.73</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>84830327.73</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>37201440</v>
+      </c>
+      <c r="K6" s="6">
+        <f>IF(D6="متوقف",0,H6*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L6" s="7">
+        <f>IF(G6=0,"",K6/G6-1)</f>
+        <v/>
+      </c>
+      <c r="M6" s="6">
+        <f>IFERROR(VLOOKUP(A6,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N6" s="7">
+        <f>IF(M6=0,"",K6/M6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>11452104</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>إصدار رخص الأنشطة التجارية</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D7" s="5">
+        <f>IF(AND(266305026.42=0,250375647.47=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>260667489.98</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>276275913.44</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>267496278.85</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>250375647.47</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>242883840.52</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>7491806.95</v>
+      </c>
+      <c r="K7" s="6">
+        <f>IF(D7="متوقف",0,H7*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L7" s="7">
+        <f>IF(G7=0,"",K7/G7-1)</f>
+        <v/>
+      </c>
+      <c r="M7" s="6">
+        <f>IFERROR(VLOOKUP(A7,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N7" s="7">
+        <f>IF(M7=0,"",K7/M7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>11452103</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>ايراد اصدار تراخيص المباني والاسوار - أمانة منطقة الرياض</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D8" s="5">
+        <f>IF(AND(206131241.55=0,204002823.21=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>224939645.24</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>244582493.3</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>319675274.54</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>204002823.21</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>201825904.56</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>2176918.65</v>
+      </c>
+      <c r="K8" s="6">
+        <f>IF(D8="متوقف",0,H8*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L8" s="7">
+        <f>IF(G8=0,"",K8/G8-1)</f>
+        <v/>
+      </c>
+      <c r="M8" s="6">
+        <f>IFERROR(VLOOKUP(A8,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N8" s="7">
+        <f>IF(M8=0,"",K8/M8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>11452512</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات لوحات المحلات</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D9" s="5">
+        <f>IF(AND(187729029.22=0,174294501.5=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>218503365</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>219218740</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>193830778.44</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>174294501.5</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>168452157.32</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>5842344.18</v>
+      </c>
+      <c r="K9" s="6">
+        <f>IF(D9="متوقف",0,H9*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L9" s="7">
+        <f>IF(G9=0,"",K9/G9-1)</f>
+        <v/>
+      </c>
+      <c r="M9" s="6">
+        <f>IFERROR(VLOOKUP(A9,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N9" s="7">
+        <f>IF(M9=0,"",K9/M9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>11442</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>اشغال مرافق الايواء</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D10" s="5">
+        <f>IF(AND(156682947.06=0,136639761.84=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>219905861.19</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>256726800.98</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>199149669.75</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>136639761.84</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>130009859.83</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>6629902.01</v>
+      </c>
+      <c r="K10" s="6">
+        <f>IF(D10="متوقف",0,H10*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L10" s="7">
+        <f>IF(G10=0,"",K10/G10-1)</f>
+        <v/>
+      </c>
+      <c r="M10" s="6">
+        <f>IFERROR(VLOOKUP(A10,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N10" s="7">
+        <f>IF(M10=0,"",K10/M10)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>142162</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  تأجير المرافق</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D11" s="5">
+        <f>IF(AND(430765503.41=0,428460046.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>29573714.25</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>45452213.03</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>25602601.22</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>428460046</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>419189059.67</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>9270986.33</v>
+      </c>
+      <c r="K11" s="6">
+        <f>IF(D11="متوقف",0,H11*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L11" s="7">
+        <f>IF(G11=0,"",K11/G11-1)</f>
+        <v/>
+      </c>
+      <c r="M11" s="6">
+        <f>IFERROR(VLOOKUP(A11,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N11" s="7">
+        <f>IF(M11=0,"",K11/M11)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>1421999</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>مبيعات أخرى</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D12" s="5">
+        <f>IF(AND(147700656.12=0,134076434.91=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>110542302.74</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>106593084.61</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>60096373.96</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>134076434.91</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>131555252.54</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>2521182.37</v>
+      </c>
+      <c r="K12" s="6">
+        <f>IF(D12="متوقف",0,H12*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L12" s="7">
+        <f>IF(G12=0,"",K12/G12-1)</f>
+        <v/>
+      </c>
+      <c r="M12" s="6">
+        <f>IFERROR(VLOOKUP(A12,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N12" s="7">
+        <f>IF(M12=0,"",K12/M12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>144122</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  متنوعه</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D13" s="5">
+        <f>IF(AND(316496963.26=0,20815752.14=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>8992323.98</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>8297789.75</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>2477531.42</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>20815752.14</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>1510267.36</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>19305484.78</v>
+      </c>
+      <c r="K13" s="6">
+        <f>IF(D13="متوقف",0,H13*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L13" s="7">
+        <f>IF(G13=0,"",K13/G13-1)</f>
+        <v/>
+      </c>
+      <c r="M13" s="6">
+        <f>IFERROR(VLOOKUP(A13,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N13" s="7">
+        <f>IF(M13=0,"",K13/M13)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>1421911</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>رسم مبيعات محلات تقديم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D14" s="5">
+        <f>IF(AND(80723092.94=0,56671709.72=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>65864668.18</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>79278364.97</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>67630101.28</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>56671709.72</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>54257631.71</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>2414078.01</v>
+      </c>
+      <c r="K14" s="6">
+        <f>IF(D14="متوقف",0,H14*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L14" s="7">
+        <f>IF(G14=0,"",K14/G14-1)</f>
+        <v/>
+      </c>
+      <c r="M14" s="6">
+        <f>IFERROR(VLOOKUP(A14,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N14" s="7">
+        <f>IF(M14=0,"",K14/M14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>1421909</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>جمع النفايات</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D15" s="5">
+        <f>IF(AND(79213506.2=0,72223518.14=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>72026385.34999999</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>76106716.86</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>72842923.63</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>72223518.14</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>69311342.59</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>2912175.55</v>
+      </c>
+      <c r="K15" s="6">
+        <f>IF(D15="متوقف",0,H15*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L15" s="7">
+        <f>IF(G15=0,"",K15/G15-1)</f>
+        <v/>
+      </c>
+      <c r="M15" s="6">
+        <f>IFERROR(VLOOKUP(A15,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N15" s="7">
+        <f>IF(M15=0,"",K15/M15)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>11452105</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>رسوم تراخيص حفر الشوارع</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D16" s="5">
+        <f>IF(AND(1350.0=0,1350.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>66558861.24</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>65200590.52</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>590915.4300000001</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>1350</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>1350</v>
+      </c>
+      <c r="K16" s="6">
+        <f>IF(D16="متوقف",0,H16*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L16" s="7">
+        <f>IF(G16=0,"",K16/G16-1)</f>
+        <v/>
+      </c>
+      <c r="M16" s="6">
+        <f>IFERROR(VLOOKUP(A16,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N16" s="7">
+        <f>IF(M16=0,"",K16/M16)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>11452108</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>ايراد اصدار القرارات المساحية - أمانة منطقة الرياض</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D17" s="5">
+        <f>IF(AND(34133807.25=0,31178848.2=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>4316211.89</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>19339697.82</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>24531493.81</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>31178848.2</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>28852796.06</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>2326052.14</v>
+      </c>
+      <c r="K17" s="6">
+        <f>IF(D17="متوقف",0,H17*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L17" s="7">
+        <f>IF(G17=0,"",K17/G17-1)</f>
+        <v/>
+      </c>
+      <c r="M17" s="6">
+        <f>IFERROR(VLOOKUP(A17,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N17" s="7">
+        <f>IF(M17=0,"",K17/M17)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>1422108</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>الشهادات الصحية</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D18" s="5">
+        <f>IF(AND(21634358.52=0,17601110.76=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>20767064.19</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>12367178.86</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>26098550.07</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>17601110.76</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>17398801.09</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>202309.67</v>
+      </c>
+      <c r="K18" s="6">
+        <f>IF(D18="متوقف",0,H18*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L18" s="7">
+        <f>IF(G18=0,"",K18/G18-1)</f>
+        <v/>
+      </c>
+      <c r="M18" s="6">
+        <f>IFERROR(VLOOKUP(A18,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N18" s="7">
+        <f>IF(M18=0,"",K18/M18)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>1422121</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>رسم ترخيص نشاط تقديم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D19" s="5">
+        <f>IF(AND(14308008.01=0,13896650.67=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>13322800</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>17925000</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>15681460.95</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>13896650.67</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>13332736.16</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>563914.51</v>
+      </c>
+      <c r="K19" s="6">
+        <f>IF(D19="متوقف",0,H19*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L19" s="7">
+        <f>IF(G19=0,"",K19/G19-1)</f>
+        <v/>
+      </c>
+      <c r="M19" s="6">
+        <f>IFERROR(VLOOKUP(A19,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N19" s="7">
+        <f>IF(M19=0,"",K19/M19)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>بدون رقم</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>بدون رقم (خدمات علم + جزاءات)</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>علم / جزاءات</t>
+        </is>
+      </c>
+      <c r="D20" s="5">
+        <f>IF(AND(21837837.5=0,2122923.75=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>4815218.75</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>14256546.25</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>21814890</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>2122923.75</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>1899660</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>223263.75</v>
+      </c>
+      <c r="K20" s="6">
+        <f>IF(D20="متوقف",0,H20*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L20" s="7">
+        <f>IF(G20=0,"",K20/G20-1)</f>
+        <v/>
+      </c>
+      <c r="M20" s="6">
+        <f>IFERROR(VLOOKUP(A20,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N20" s="7">
+        <f>IF(M20=0,"",K20/M20)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>142163</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  تأجير مباني تجارية</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D21" s="5">
+        <f>IF(AND(12310614.76=0,10169478.26=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>6866663.43</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>6179302.5</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>3001651.75</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>10169478.26</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>6947112.55</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>3222365.71</v>
+      </c>
+      <c r="K21" s="6">
+        <f>IF(D21="متوقف",0,H21*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L21" s="7">
+        <f>IF(G21=0,"",K21/G21-1)</f>
+        <v/>
+      </c>
+      <c r="M21" s="6">
+        <f>IFERROR(VLOOKUP(A21,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N21" s="7">
+        <f>IF(M21=0,"",K21/M21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>1422109</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  الكشفية</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D22" s="5">
+        <f>IF(AND(6331998.45=0,5723153.45=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>9211384.77</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>8995823.25</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>7132142.91</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>5723153.45</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>5563946.57</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>159206.88</v>
+      </c>
+      <c r="K22" s="6">
+        <f>IF(D22="متوقف",0,H22*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L22" s="7">
+        <f>IF(G22=0,"",K22/G22-1)</f>
+        <v/>
+      </c>
+      <c r="M22" s="6">
+        <f>IFERROR(VLOOKUP(A22,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N22" s="7">
+        <f>IF(M22=0,"",K22/M22)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>11452111</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>المقابل المالي للسماح للأنشطة التجارية بالعمل (24) ساعة</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D23" s="5">
+        <f>IF(AND(12106223.42=0,11409758.77=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>6031956.09</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>5166690.6</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>5751371.82</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>11409758.77</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>11142484.61</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>267274.16</v>
+      </c>
+      <c r="K23" s="6">
+        <f>IF(D23="متوقف",0,H23*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L23" s="7">
+        <f>IF(G23=0,"",K23/G23-1)</f>
+        <v/>
+      </c>
+      <c r="M23" s="6">
+        <f>IFERROR(VLOOKUP(A23,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N23" s="7">
+        <f>IF(M23=0,"",K23/M23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>1421910</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>اصدار تراخيص اشغال الارصفة العامة و الطرق</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D24" s="5">
+        <f>IF(AND(3660790.62=0,3564931.07=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>3828676.61</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>2909412.61</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>3477675.2</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>3564931.07</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>3475978.84</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>88952.23</v>
+      </c>
+      <c r="K24" s="6">
+        <f>IF(D24="متوقف",0,H24*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L24" s="7">
+        <f>IF(G24=0,"",K24/G24-1)</f>
+        <v/>
+      </c>
+      <c r="M24" s="6">
+        <f>IFERROR(VLOOKUP(A24,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N24" s="7">
+        <f>IF(M24=0,"",K24/M24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>1439</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  مبيعات  ناتجه من النشاط غير مصنفة</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D25" s="5">
+        <f>IF(AND(519000.0=0,183000.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>3537100</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>227000</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>8503508</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>183000</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>183000</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K25" s="6">
+        <f>IF(D25="متوقف",0,H25*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L25" s="7">
+        <f>IF(G25=0,"",K25/G25-1)</f>
+        <v/>
+      </c>
+      <c r="M25" s="6">
+        <f>IFERROR(VLOOKUP(A25,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N25" s="7">
+        <f>IF(M25=0,"",K25/M25)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>1421901</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>بيع الوثائق والأنظمة</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D26" s="5">
+        <f>IF(AND(1860236.0=0,1624137.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>2928906</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>2736595</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>2512377</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>1624137</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>1616037</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>8100</v>
+      </c>
+      <c r="K26" s="6">
+        <f>IF(D26="متوقف",0,H26*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L26" s="7">
+        <f>IF(G26=0,"",K26/G26-1)</f>
+        <v/>
+      </c>
+      <c r="M26" s="6">
+        <f>IFERROR(VLOOKUP(A26,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N26" s="7">
+        <f>IF(M26=0,"",K26/M26)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>1421903</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>مبيعات التيار الكهربائي</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D27" s="5">
+        <f>IF(AND(302027.65=0,274868.65=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>1464687.1</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>274868.65</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>143551.39</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>131317.26</v>
+      </c>
+      <c r="K27" s="6">
+        <f>IF(D27="متوقف",0,H27*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L27" s="7">
+        <f>IF(G27=0,"",K27/G27-1)</f>
+        <v/>
+      </c>
+      <c r="M27" s="6">
+        <f>IFERROR(VLOOKUP(A27,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N27" s="7">
+        <f>IF(M27=0,"",K27/M27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>1438</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات مفروضة بموجب أنظمة الجهة</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D28" s="5">
+        <f>IF(AND(59500.0=0,59500.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>4544553</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>486100</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>352900</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>59500</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>59500</v>
+      </c>
+      <c r="K28" s="6">
+        <f>IF(D28="متوقف",0,H28*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L28" s="7">
+        <f>IF(G28=0,"",K28/G28-1)</f>
+        <v/>
+      </c>
+      <c r="M28" s="6">
+        <f>IFERROR(VLOOKUP(A28,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N28" s="7">
+        <f>IF(M28=0,"",K28/M28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>1421912</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>تأجير العقارات لأغراض مؤقته</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D29" s="5">
+        <f>IF(AND(1447854.96=0,1357611.55=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>838420.1899999999</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>2043840.5</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>2454143.51</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>1357611.55</v>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>1354461.55</v>
+      </c>
+      <c r="J29" s="6" t="n">
+        <v>3150</v>
+      </c>
+      <c r="K29" s="6">
+        <f>IF(D29="متوقف",0,H29*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L29" s="7">
+        <f>IF(G29=0,"",K29/G29-1)</f>
+        <v/>
+      </c>
+      <c r="M29" s="6">
+        <f>IFERROR(VLOOKUP(A29,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N29" s="7">
+        <f>IF(M29=0,"",K29/M29)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>11452106</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>اصدار التراخيص بتأسيس أو تشغيل ابراج الاتصالات</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D30" s="5">
+        <f>IF(AND(476400.0=0,342700.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>845300</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>1408700</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>1275300</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>342700</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>189300</v>
+      </c>
+      <c r="J30" s="6" t="n">
+        <v>153400</v>
+      </c>
+      <c r="K30" s="6">
+        <f>IF(D30="متوقف",0,H30*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L30" s="7">
+        <f>IF(G30=0,"",K30/G30-1)</f>
+        <v/>
+      </c>
+      <c r="M30" s="6">
+        <f>IFERROR(VLOOKUP(A30,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N30" s="7">
+        <f>IF(M30=0,"",K30/M30)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>11452110</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>إصدار تراخيص إستخدام أملاك خاصة لإقامة فعاليات</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D31" s="5">
+        <f>IF(AND(646845.12=0,594187.77=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>609446.45</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>1038687.25</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>809215.9</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>594187.77</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>579245.45</v>
+      </c>
+      <c r="J31" s="6" t="n">
+        <v>14942.32</v>
+      </c>
+      <c r="K31" s="6">
+        <f>IF(D31="متوقف",0,H31*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L31" s="7">
+        <f>IF(G31=0,"",K31/G31-1)</f>
+        <v/>
+      </c>
+      <c r="M31" s="6">
+        <f>IFERROR(VLOOKUP(A31,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N31" s="7">
+        <f>IF(M31=0,"",K31/M31)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>141229</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>أرباح أخرى</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D32" s="5">
+        <f>IF(AND(60000.0=0,60000.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>910572</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>2120000</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>60000</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>60000</v>
+      </c>
+      <c r="K32" s="6">
+        <f>IF(D32="متوقف",0,H32*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L32" s="7">
+        <f>IF(G32=0,"",K32/G32-1)</f>
+        <v/>
+      </c>
+      <c r="M32" s="6">
+        <f>IFERROR(VLOOKUP(A32,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N32" s="7">
+        <f>IF(M32=0,"",K32/M32)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>11452109</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>اعتماد مخططات التطوير العقاري</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D33" s="5">
+        <f>IF(AND(100.0=0,100.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>536299.9399999999</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>1217856.22</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>591946.73</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="I33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="K33" s="6">
+        <f>IF(D33="متوقف",0,H33*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L33" s="7">
+        <f>IF(G33=0,"",K33/G33-1)</f>
+        <v/>
+      </c>
+      <c r="M33" s="6">
+        <f>IFERROR(VLOOKUP(A33,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N33" s="7">
+        <f>IF(M33=0,"",K33/M33)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>11452107</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>اصدار التراخيص بتأسيس أو تشغيل الصراف الآلي</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D34" s="5">
+        <f>IF(AND(200184.61=0,158934.61=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>54000</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>90000</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>229800</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>158934.61</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>152461.09</v>
+      </c>
+      <c r="J34" s="6" t="n">
+        <v>6473.52</v>
+      </c>
+      <c r="K34" s="6">
+        <f>IF(D34="متوقف",0,H34*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L34" s="7">
+        <f>IF(G34=0,"",K34/G34-1)</f>
+        <v/>
+      </c>
+      <c r="M34" s="6">
+        <f>IFERROR(VLOOKUP(A34,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N34" s="7">
+        <f>IF(M34=0,"",K34/M34)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>3318212</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>مرتجع رواتب - فواتير</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D35" s="5">
+        <f>IF(AND(361665.23=0,216725.66=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>152767.79</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>216725.66</v>
+      </c>
+      <c r="I35" s="6" t="n">
+        <v>216725.66</v>
+      </c>
+      <c r="J35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K35" s="6">
+        <f>IF(D35="متوقف",0,H35*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L35" s="7">
+        <f>IF(G35=0,"",K35/G35-1)</f>
+        <v/>
+      </c>
+      <c r="M35" s="6">
+        <f>IFERROR(VLOOKUP(A35,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N35" s="7">
+        <f>IF(M35=0,"",K35/M35)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>11422</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>رسوم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D36" s="5">
+        <f>IF(AND(0.0=0,0.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>27000</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>5167</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>27000</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K36" s="6">
+        <f>IF(D36="متوقف",0,H36*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L36" s="7">
+        <f>IF(G36=0,"",K36/G36-1)</f>
+        <v/>
+      </c>
+      <c r="M36" s="6">
+        <f>IFERROR(VLOOKUP(A36,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N36" s="7">
+        <f>IF(M36=0,"",K36/M36)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>1422103</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>تراخيص المحلات</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D37" s="5">
+        <f>IF(AND(432.0=0,432.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>67711.60000000001</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>16269.6</v>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>1603.2</v>
+      </c>
+      <c r="H37" s="6" t="n">
+        <v>432</v>
+      </c>
+      <c r="I37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="6" t="n">
+        <v>432</v>
+      </c>
+      <c r="K37" s="6">
+        <f>IF(D37="متوقف",0,H37*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L37" s="7">
+        <f>IF(G37=0,"",K37/G37-1)</f>
+        <v/>
+      </c>
+      <c r="M37" s="6">
+        <f>IFERROR(VLOOKUP(A37,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N37" s="7">
+        <f>IF(M37=0,"",K37/M37)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>11452513</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>لوحات إرشـادية</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D38" s="5">
+        <f>IF(AND(600.0=0,600.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>55525</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>12875</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>9000</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>600</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="6" t="n">
+        <v>600</v>
+      </c>
+      <c r="K38" s="6">
+        <f>IF(D38="متوقف",0,H38*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L38" s="7">
+        <f>IF(G38=0,"",K38/G38-1)</f>
+        <v/>
+      </c>
+      <c r="M38" s="6">
+        <f>IFERROR(VLOOKUP(A38,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N38" s="7">
+        <f>IF(M38=0,"",K38/M38)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>1421907</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات المخططات</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D39" s="5">
+        <f>IF(AND(6350.0=0,5550.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>20650</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>5550</v>
+      </c>
+      <c r="I39" s="6" t="n">
+        <v>5450</v>
+      </c>
+      <c r="J39" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="K39" s="6">
+        <f>IF(D39="متوقف",0,H39*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L39" s="7">
+        <f>IF(G39=0,"",K39/G39-1)</f>
+        <v/>
+      </c>
+      <c r="M39" s="6">
+        <f>IFERROR(VLOOKUP(A39,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N39" s="7">
+        <f>IF(M39=0,"",K39/M39)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>1421908</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  رسوم خدمات  بلدية</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D40" s="5">
+        <f>IF(AND(0.0=0,0.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>16385</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" s="6">
+        <f>IF(D40="متوقف",0,H40*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L40" s="7">
+        <f>IF(G40=0,"",K40/G40-1)</f>
+        <v/>
+      </c>
+      <c r="M40" s="6">
+        <f>IFERROR(VLOOKUP(A40,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N40" s="7">
+        <f>IF(M40=0,"",K40/M40)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>142161</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>تاجير مباني سكنية</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D41" s="5">
+        <f>IF(AND(0.0=0,0.0=0),"متوقف","نشط")</f>
+        <v/>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" s="6">
+        <f>IF(D41="متوقف",0,H41*الافتراضات!$B$4)</f>
+        <v/>
+      </c>
+      <c r="L41" s="7">
+        <f>IF(G41=0,"",K41/G41-1)</f>
+        <v/>
+      </c>
+      <c r="M41" s="6">
+        <f>IFERROR(VLOOKUP(A41,التوقعات!$A$4:$I$41,9,FALSE),0)</f>
+        <v/>
+      </c>
+      <c r="N41" s="7">
+        <f>IF(M41=0,"",K41/M41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="8" t="n"/>
+      <c r="B42" s="8" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="C42" s="8" t="n"/>
+      <c r="D42" s="8" t="n"/>
+      <c r="E42" s="9">
+        <f>SUM(E4:E41)</f>
+        <v/>
+      </c>
+      <c r="F42" s="9">
+        <f>SUM(F4:F41)</f>
+        <v/>
+      </c>
+      <c r="G42" s="9">
+        <f>SUM(G4:G41)</f>
+        <v/>
+      </c>
+      <c r="H42" s="9">
+        <f>SUM(H4:H41)</f>
+        <v/>
+      </c>
+      <c r="I42" s="9">
+        <f>SUM(I4:I41)</f>
+        <v/>
+      </c>
+      <c r="J42" s="9">
+        <f>SUM(J4:J41)</f>
+        <v/>
+      </c>
+      <c r="K42" s="9">
+        <f>SUM(K4:K41)</f>
+        <v/>
+      </c>
+      <c r="L42" s="10">
+        <f>K42/G42-1</f>
+        <v/>
+      </c>
+      <c r="M42" s="9">
+        <f>SUM(M4:M41)</f>
+        <v/>
+      </c>
+      <c r="N42" s="10">
+        <f>K42/M42</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A3:N41"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -5291,7 +7555,7 @@
           <t>معامل تحويل 2026 إلى سنة كاملة (12÷9)</t>
         </is>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="12">
         <f>12/9</f>
         <v/>
       </c>
@@ -5307,7 +7571,7 @@
           <t>نسبة النمو – السيناريو الأول (ثابتة)</t>
         </is>
       </c>
-      <c r="B5" s="12">
+      <c r="B5" s="13">
         <f>التوقعات!C2</f>
         <v/>
       </c>
@@ -5323,7 +7587,7 @@
           <t>سقف معدل النمو التاريخي (±)</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="13" t="n">
         <v>0.25</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -5340,63 +7604,70 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="13" t="inlineStr">
+      <c r="A10" s="14" t="inlineStr">
         <is>
           <t>1) الإجمالي المفوتر للحساب = المفوتر + المحصل عن سنوات سابقة (حسب طلبك).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="13" t="inlineStr">
+      <c r="A11" s="14" t="inlineStr">
         <is>
           <t>2) توقع 2026 = الفعلي حتى سبتمبر × 12/9 (لا توجد بيانات شهرية، فلا موسمية في التوقع).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="13" t="inlineStr">
+      <c r="A12" s="14" t="inlineStr">
         <is>
           <t>3) الحسابات التي فوترتها وتحصيلها صفر في 2026 تُعتبر متوقفة وتوقعها صفر في 2026 و2027.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="inlineStr">
+      <c r="A13" s="14" t="inlineStr">
         <is>
           <t>4) 2027 – السيناريو الأول: توقع 2026 × (1 + نسبة النمو في خلية C2 بورقة التوقعات؛ الافتراضي 7%).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="13" t="inlineStr">
+      <c r="A14" s="14" t="inlineStr">
         <is>
           <t>5) 2027 – السيناريو الثاني: توقع 2026 × (1 + معدل النمو السنوي المركب التاريخي للحساب بين أول سنة فيها فوترة و2025، بسقف ±25%). إن توفرت سنة واحدة فقط من البيانات = نمو 0%.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>6) تم استبعاد حساب قيمة الضريبة المضافة (11411) من كل الحسابات والإجماليات.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>6b) تم دمج صفّي "بدون رقم" (خدمات علم + جزاءات، وجزاءات جزء ضئيل) في صف واحد لكل سنة.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>6c) أعمدة النمو لكل حساب: نمو كل سنة عن السنة السابقة (2024 عن 2023، 2025 عن 2024، 2026 توقع عن 2025، و2027 عن 2026 للسيناريوهين). تظهر فارغة عندما تكون السنة السابقة صفراً.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>6d) ورقة "توقع المحصل 2026": توقع إقفال 2026 كمحصّل فعلي = المحصل حتى سبتمبر × 12÷9 (مسدد عن السنة + محصل سنوات سابقة).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>7) تنبيه: كثير من الحسابات تتذبذب بشدة بين السنوات (لوحات دعائية، تأجير المرافق، إيرادات متنوعة)، ومضاعفة 2026 على 12/9 تضخّم أو تقلّل هذه الأرقام؛ انظر عمود "تنبيه".</t>
         </is>

</xml_diff>

<commit_message>
Add forecast rationale and worst-case scenario sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/توقع_الفوترة_2026_2027.xlsx
+++ b/توقع_الفوترة_2026_2027.xlsx
@@ -11,11 +11,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="حسب التبويب" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تفصيل المكونات" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="توقع المحصل 2026" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تحليل التوقع والأسوأ" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'التوقعات'!$A$3:$R$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'توقع المحصل 2026'!$A$3:$N$41</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'تحليل التوقع والأسوأ'!$A$4:$O$42</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -116,7 +118,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -133,6 +135,19 @@
     <xf numFmtId="166" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -7517,6 +7532,2772 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
+    <col width="90" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>لماذا هذا التوقع؟ تحليل كل حساب والسيناريو الأسوأ لإقفال 2026 (محصّل)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="44" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>التوقع الأساسي = المحصل حتى سبتمبر × 12÷9. السيناريو الأسوأ لكل حساب = الأكبر بين (المحصل حتى سبتمبر) و(الأصغر بين التوقع الأساسي ومحصل 2025)، أي: لا نمو عن 2025، والقفزات لا تتكرر، ولا ينزل الحساب عما حُصّل فعلاً. الحد الأدنى المطلق = المحصل حتى سبتمبر بدون أي تحصيل في الربع الأخير. نص السبب ثابت بحسب الافتراضات الحالية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>الملخص:</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>التوقع الأساسي</t>
+        </is>
+      </c>
+      <c r="D3" s="14">
+        <f>J43</f>
+        <v/>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>السيناريو الأسوأ</t>
+        </is>
+      </c>
+      <c r="F3" s="14">
+        <f>K43</f>
+        <v/>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>الحد الأدنى المطلق</t>
+        </is>
+      </c>
+      <c r="H3" s="14">
+        <f>G43</f>
+        <v/>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>محصل 2025</t>
+        </is>
+      </c>
+      <c r="J3" s="14">
+        <f>F43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>رقم الحساب</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>اسم الحساب</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>التبويب</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>2023 محصّل</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>2024 محصّل</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>2025 محصّل</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>2026 حتى سبتمبر</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>حتى سبتمبر ÷ 2025</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>تحصيل الربع الأخير المتوقع</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>التوقع الأساسي</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>السيناريو الأسوأ</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>الفرق (أسوأ − أساسي)</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>حصة الحساب من الأساسي</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>مستوى الخطر</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>سبب التوقع</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>1438001</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات و غرامات مفروضة بموجب أنظمة الجهة</t>
+        </is>
+      </c>
+      <c r="C5" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D5" s="6">
+        <f>'توقع المحصل 2026'!E4</f>
+        <v/>
+      </c>
+      <c r="E5" s="6">
+        <f>'توقع المحصل 2026'!F4</f>
+        <v/>
+      </c>
+      <c r="F5" s="6">
+        <f>'توقع المحصل 2026'!G4</f>
+        <v/>
+      </c>
+      <c r="G5" s="6">
+        <f>'توقع المحصل 2026'!H4</f>
+        <v/>
+      </c>
+      <c r="H5" s="15">
+        <f>IF(F5=0,"",G5/F5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="6">
+        <f>J5-G5</f>
+        <v/>
+      </c>
+      <c r="J5" s="6">
+        <f>'توقع المحصل 2026'!K4</f>
+        <v/>
+      </c>
+      <c r="K5" s="6">
+        <f>IF(J5=0,0,MAX(G5,MIN(J5,F5)))</f>
+        <v/>
+      </c>
+      <c r="L5" s="6">
+        <f>K5-J5</f>
+        <v/>
+      </c>
+      <c r="M5" s="7">
+        <f>J5/J$43</f>
+        <v/>
+      </c>
+      <c r="N5" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O5" s="16" t="inlineStr">
+        <is>
+          <t>قفزة: المحصل حتى سبتمبر (370.6م) يعادل 120% من كل 2025 (308.0م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>14155</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>ريع الأراضي (تأجير الأراض )</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D6" s="6">
+        <f>'توقع المحصل 2026'!E5</f>
+        <v/>
+      </c>
+      <c r="E6" s="6">
+        <f>'توقع المحصل 2026'!F5</f>
+        <v/>
+      </c>
+      <c r="F6" s="6">
+        <f>'توقع المحصل 2026'!G5</f>
+        <v/>
+      </c>
+      <c r="G6" s="6">
+        <f>'توقع المحصل 2026'!H5</f>
+        <v/>
+      </c>
+      <c r="H6" s="15">
+        <f>IF(F6=0,"",G6/F6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="6">
+        <f>J6-G6</f>
+        <v/>
+      </c>
+      <c r="J6" s="6">
+        <f>'توقع المحصل 2026'!K5</f>
+        <v/>
+      </c>
+      <c r="K6" s="6">
+        <f>IF(J6=0,0,MAX(G6,MIN(J6,F6)))</f>
+        <v/>
+      </c>
+      <c r="L6" s="6">
+        <f>K6-J6</f>
+        <v/>
+      </c>
+      <c r="M6" s="7">
+        <f>J6/J$43</f>
+        <v/>
+      </c>
+      <c r="N6" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O6" s="16" t="inlineStr">
+        <is>
+          <t>المحصل حتى سبتمبر (612.9م) بلغ 94% من كل 2025 (649.3م). إضافة الربع الأخير بنفس الوتيرة ترفع التوقع 26% فوق 2025، وإن كان التحصيل يتركز في بداية السنة فالتوقع مبالغ فيه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>142113</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  اللوحات الدعائية</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D7" s="6">
+        <f>'توقع المحصل 2026'!E6</f>
+        <v/>
+      </c>
+      <c r="E7" s="6">
+        <f>'توقع المحصل 2026'!F6</f>
+        <v/>
+      </c>
+      <c r="F7" s="6">
+        <f>'توقع المحصل 2026'!G6</f>
+        <v/>
+      </c>
+      <c r="G7" s="6">
+        <f>'توقع المحصل 2026'!H6</f>
+        <v/>
+      </c>
+      <c r="H7" s="15">
+        <f>IF(F7=0,"",G7/F7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="6">
+        <f>J7-G7</f>
+        <v/>
+      </c>
+      <c r="J7" s="6">
+        <f>'توقع المحصل 2026'!K6</f>
+        <v/>
+      </c>
+      <c r="K7" s="6">
+        <f>IF(J7=0,0,MAX(G7,MIN(J7,F7)))</f>
+        <v/>
+      </c>
+      <c r="L7" s="6">
+        <f>K7-J7</f>
+        <v/>
+      </c>
+      <c r="M7" s="7">
+        <f>J7/J$43</f>
+        <v/>
+      </c>
+      <c r="N7" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O7" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (122.0م) يعادل 12% فقط من 2025 (1,016.9م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>11452104</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>إصدار رخص الأنشطة التجارية</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D8" s="6">
+        <f>'توقع المحصل 2026'!E7</f>
+        <v/>
+      </c>
+      <c r="E8" s="6">
+        <f>'توقع المحصل 2026'!F7</f>
+        <v/>
+      </c>
+      <c r="F8" s="6">
+        <f>'توقع المحصل 2026'!G7</f>
+        <v/>
+      </c>
+      <c r="G8" s="6">
+        <f>'توقع المحصل 2026'!H7</f>
+        <v/>
+      </c>
+      <c r="H8" s="15">
+        <f>IF(F8=0,"",G8/F8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="6">
+        <f>J8-G8</f>
+        <v/>
+      </c>
+      <c r="J8" s="6">
+        <f>'توقع المحصل 2026'!K7</f>
+        <v/>
+      </c>
+      <c r="K8" s="6">
+        <f>IF(J8=0,0,MAX(G8,MIN(J8,F8)))</f>
+        <v/>
+      </c>
+      <c r="L8" s="6">
+        <f>K8-J8</f>
+        <v/>
+      </c>
+      <c r="M8" s="7">
+        <f>J8/J$43</f>
+        <v/>
+      </c>
+      <c r="N8" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O8" s="16" t="inlineStr">
+        <is>
+          <t>المحصل حتى سبتمبر (250.4م) بلغ 94% من كل 2025 (267.5م). إضافة الربع الأخير بنفس الوتيرة ترفع التوقع 25% فوق 2025، وإن كان التحصيل يتركز في بداية السنة فالتوقع مبالغ فيه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>11452103</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>ايراد اصدار تراخيص المباني والاسوار - أمانة منطقة الرياض</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D9" s="6">
+        <f>'توقع المحصل 2026'!E8</f>
+        <v/>
+      </c>
+      <c r="E9" s="6">
+        <f>'توقع المحصل 2026'!F8</f>
+        <v/>
+      </c>
+      <c r="F9" s="6">
+        <f>'توقع المحصل 2026'!G8</f>
+        <v/>
+      </c>
+      <c r="G9" s="6">
+        <f>'توقع المحصل 2026'!H8</f>
+        <v/>
+      </c>
+      <c r="H9" s="15">
+        <f>IF(F9=0,"",G9/F9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="6">
+        <f>J9-G9</f>
+        <v/>
+      </c>
+      <c r="J9" s="6">
+        <f>'توقع المحصل 2026'!K8</f>
+        <v/>
+      </c>
+      <c r="K9" s="6">
+        <f>IF(J9=0,0,MAX(G9,MIN(J9,F9)))</f>
+        <v/>
+      </c>
+      <c r="L9" s="6">
+        <f>K9-J9</f>
+        <v/>
+      </c>
+      <c r="M9" s="7">
+        <f>J9/J$43</f>
+        <v/>
+      </c>
+      <c r="N9" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O9" s="16" t="inlineStr">
+        <is>
+          <t>مستقر: التوقع (272.0م) قريب من محصل 2025 (319.7م).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>11452512</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات لوحات المحلات</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D10" s="6">
+        <f>'توقع المحصل 2026'!E9</f>
+        <v/>
+      </c>
+      <c r="E10" s="6">
+        <f>'توقع المحصل 2026'!F9</f>
+        <v/>
+      </c>
+      <c r="F10" s="6">
+        <f>'توقع المحصل 2026'!G9</f>
+        <v/>
+      </c>
+      <c r="G10" s="6">
+        <f>'توقع المحصل 2026'!H9</f>
+        <v/>
+      </c>
+      <c r="H10" s="15">
+        <f>IF(F10=0,"",G10/F10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="6">
+        <f>J10-G10</f>
+        <v/>
+      </c>
+      <c r="J10" s="6">
+        <f>'توقع المحصل 2026'!K9</f>
+        <v/>
+      </c>
+      <c r="K10" s="6">
+        <f>IF(J10=0,0,MAX(G10,MIN(J10,F10)))</f>
+        <v/>
+      </c>
+      <c r="L10" s="6">
+        <f>K10-J10</f>
+        <v/>
+      </c>
+      <c r="M10" s="7">
+        <f>J10/J$43</f>
+        <v/>
+      </c>
+      <c r="N10" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
+        </is>
+      </c>
+      <c r="O10" s="16" t="inlineStr">
+        <is>
+          <t>التوقع أعلى من 2025 بنسبة 20% لأن وتيرة التحصيل حتى سبتمبر أعلى.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>11442</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>اشغال مرافق الايواء</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D11" s="6">
+        <f>'توقع المحصل 2026'!E10</f>
+        <v/>
+      </c>
+      <c r="E11" s="6">
+        <f>'توقع المحصل 2026'!F10</f>
+        <v/>
+      </c>
+      <c r="F11" s="6">
+        <f>'توقع المحصل 2026'!G10</f>
+        <v/>
+      </c>
+      <c r="G11" s="6">
+        <f>'توقع المحصل 2026'!H10</f>
+        <v/>
+      </c>
+      <c r="H11" s="15">
+        <f>IF(F11=0,"",G11/F11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="6">
+        <f>J11-G11</f>
+        <v/>
+      </c>
+      <c r="J11" s="6">
+        <f>'توقع المحصل 2026'!K10</f>
+        <v/>
+      </c>
+      <c r="K11" s="6">
+        <f>IF(J11=0,0,MAX(G11,MIN(J11,F11)))</f>
+        <v/>
+      </c>
+      <c r="L11" s="6">
+        <f>K11-J11</f>
+        <v/>
+      </c>
+      <c r="M11" s="7">
+        <f>J11/J$43</f>
+        <v/>
+      </c>
+      <c r="N11" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O11" s="16" t="inlineStr">
+        <is>
+          <t>مستقر: التوقع (182.2م) قريب من محصل 2025 (199.1م).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>142162</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  تأجير المرافق</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D12" s="6">
+        <f>'توقع المحصل 2026'!E11</f>
+        <v/>
+      </c>
+      <c r="E12" s="6">
+        <f>'توقع المحصل 2026'!F11</f>
+        <v/>
+      </c>
+      <c r="F12" s="6">
+        <f>'توقع المحصل 2026'!G11</f>
+        <v/>
+      </c>
+      <c r="G12" s="6">
+        <f>'توقع المحصل 2026'!H11</f>
+        <v/>
+      </c>
+      <c r="H12" s="15">
+        <f>IF(F12=0,"",G12/F12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="6">
+        <f>J12-G12</f>
+        <v/>
+      </c>
+      <c r="J12" s="6">
+        <f>'توقع المحصل 2026'!K11</f>
+        <v/>
+      </c>
+      <c r="K12" s="6">
+        <f>IF(J12=0,0,MAX(G12,MIN(J12,F12)))</f>
+        <v/>
+      </c>
+      <c r="L12" s="6">
+        <f>K12-J12</f>
+        <v/>
+      </c>
+      <c r="M12" s="7">
+        <f>J12/J$43</f>
+        <v/>
+      </c>
+      <c r="N12" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O12" s="16" t="inlineStr">
+        <is>
+          <t>قفزة: المحصل حتى سبتمبر (428.5م) يعادل 1,674% من كل 2025 (25.6م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>1421999</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>مبيعات أخرى</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D13" s="6">
+        <f>'توقع المحصل 2026'!E12</f>
+        <v/>
+      </c>
+      <c r="E13" s="6">
+        <f>'توقع المحصل 2026'!F12</f>
+        <v/>
+      </c>
+      <c r="F13" s="6">
+        <f>'توقع المحصل 2026'!G12</f>
+        <v/>
+      </c>
+      <c r="G13" s="6">
+        <f>'توقع المحصل 2026'!H12</f>
+        <v/>
+      </c>
+      <c r="H13" s="15">
+        <f>IF(F13=0,"",G13/F13)</f>
+        <v/>
+      </c>
+      <c r="I13" s="6">
+        <f>J13-G13</f>
+        <v/>
+      </c>
+      <c r="J13" s="6">
+        <f>'توقع المحصل 2026'!K12</f>
+        <v/>
+      </c>
+      <c r="K13" s="6">
+        <f>IF(J13=0,0,MAX(G13,MIN(J13,F13)))</f>
+        <v/>
+      </c>
+      <c r="L13" s="6">
+        <f>K13-J13</f>
+        <v/>
+      </c>
+      <c r="M13" s="7">
+        <f>J13/J$43</f>
+        <v/>
+      </c>
+      <c r="N13" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O13" s="16" t="inlineStr">
+        <is>
+          <t>قفزة: المحصل حتى سبتمبر (134.1م) يعادل 223% من كل 2025 (60.1م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>144122</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  متنوعه</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D14" s="6">
+        <f>'توقع المحصل 2026'!E13</f>
+        <v/>
+      </c>
+      <c r="E14" s="6">
+        <f>'توقع المحصل 2026'!F13</f>
+        <v/>
+      </c>
+      <c r="F14" s="6">
+        <f>'توقع المحصل 2026'!G13</f>
+        <v/>
+      </c>
+      <c r="G14" s="6">
+        <f>'توقع المحصل 2026'!H13</f>
+        <v/>
+      </c>
+      <c r="H14" s="15">
+        <f>IF(F14=0,"",G14/F14)</f>
+        <v/>
+      </c>
+      <c r="I14" s="6">
+        <f>J14-G14</f>
+        <v/>
+      </c>
+      <c r="J14" s="6">
+        <f>'توقع المحصل 2026'!K13</f>
+        <v/>
+      </c>
+      <c r="K14" s="6">
+        <f>IF(J14=0,0,MAX(G14,MIN(J14,F14)))</f>
+        <v/>
+      </c>
+      <c r="L14" s="6">
+        <f>K14-J14</f>
+        <v/>
+      </c>
+      <c r="M14" s="7">
+        <f>J14/J$43</f>
+        <v/>
+      </c>
+      <c r="N14" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O14" s="16" t="inlineStr">
+        <is>
+          <t>قفزة: المحصل حتى سبتمبر (20.8م) يعادل 840% من كل 2025 (2.5م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>1421911</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>رسم مبيعات محلات تقديم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D15" s="6">
+        <f>'توقع المحصل 2026'!E14</f>
+        <v/>
+      </c>
+      <c r="E15" s="6">
+        <f>'توقع المحصل 2026'!F14</f>
+        <v/>
+      </c>
+      <c r="F15" s="6">
+        <f>'توقع المحصل 2026'!G14</f>
+        <v/>
+      </c>
+      <c r="G15" s="6">
+        <f>'توقع المحصل 2026'!H14</f>
+        <v/>
+      </c>
+      <c r="H15" s="15">
+        <f>IF(F15=0,"",G15/F15)</f>
+        <v/>
+      </c>
+      <c r="I15" s="6">
+        <f>J15-G15</f>
+        <v/>
+      </c>
+      <c r="J15" s="6">
+        <f>'توقع المحصل 2026'!K14</f>
+        <v/>
+      </c>
+      <c r="K15" s="6">
+        <f>IF(J15=0,0,MAX(G15,MIN(J15,F15)))</f>
+        <v/>
+      </c>
+      <c r="L15" s="6">
+        <f>K15-J15</f>
+        <v/>
+      </c>
+      <c r="M15" s="7">
+        <f>J15/J$43</f>
+        <v/>
+      </c>
+      <c r="N15" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O15" s="16" t="inlineStr">
+        <is>
+          <t>مستقر: التوقع (75.6م) قريب من محصل 2025 (67.6م).</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>1421909</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>جمع النفايات</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D16" s="6">
+        <f>'توقع المحصل 2026'!E15</f>
+        <v/>
+      </c>
+      <c r="E16" s="6">
+        <f>'توقع المحصل 2026'!F15</f>
+        <v/>
+      </c>
+      <c r="F16" s="6">
+        <f>'توقع المحصل 2026'!G15</f>
+        <v/>
+      </c>
+      <c r="G16" s="6">
+        <f>'توقع المحصل 2026'!H15</f>
+        <v/>
+      </c>
+      <c r="H16" s="15">
+        <f>IF(F16=0,"",G16/F16)</f>
+        <v/>
+      </c>
+      <c r="I16" s="6">
+        <f>J16-G16</f>
+        <v/>
+      </c>
+      <c r="J16" s="6">
+        <f>'توقع المحصل 2026'!K15</f>
+        <v/>
+      </c>
+      <c r="K16" s="6">
+        <f>IF(J16=0,0,MAX(G16,MIN(J16,F16)))</f>
+        <v/>
+      </c>
+      <c r="L16" s="6">
+        <f>K16-J16</f>
+        <v/>
+      </c>
+      <c r="M16" s="7">
+        <f>J16/J$43</f>
+        <v/>
+      </c>
+      <c r="N16" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O16" s="16" t="inlineStr">
+        <is>
+          <t>المحصل حتى سبتمبر (72.2م) بلغ 99% من كل 2025 (72.8م). إضافة الربع الأخير بنفس الوتيرة ترفع التوقع 32% فوق 2025، وإن كان التحصيل يتركز في بداية السنة فالتوقع مبالغ فيه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>11452105</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>رسوم تراخيص حفر الشوارع</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D17" s="6">
+        <f>'توقع المحصل 2026'!E16</f>
+        <v/>
+      </c>
+      <c r="E17" s="6">
+        <f>'توقع المحصل 2026'!F16</f>
+        <v/>
+      </c>
+      <c r="F17" s="6">
+        <f>'توقع المحصل 2026'!G16</f>
+        <v/>
+      </c>
+      <c r="G17" s="6">
+        <f>'توقع المحصل 2026'!H16</f>
+        <v/>
+      </c>
+      <c r="H17" s="15">
+        <f>IF(F17=0,"",G17/F17)</f>
+        <v/>
+      </c>
+      <c r="I17" s="6">
+        <f>J17-G17</f>
+        <v/>
+      </c>
+      <c r="J17" s="6">
+        <f>'توقع المحصل 2026'!K16</f>
+        <v/>
+      </c>
+      <c r="K17" s="6">
+        <f>IF(J17=0,0,MAX(G17,MIN(J17,F17)))</f>
+        <v/>
+      </c>
+      <c r="L17" s="6">
+        <f>K17-J17</f>
+        <v/>
+      </c>
+      <c r="M17" s="7">
+        <f>J17/J$43</f>
+        <v/>
+      </c>
+      <c r="N17" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O17" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (0.0م) يعادل 0% فقط من 2025 (0.6م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>11452108</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>ايراد اصدار القرارات المساحية - أمانة منطقة الرياض</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D18" s="6">
+        <f>'توقع المحصل 2026'!E17</f>
+        <v/>
+      </c>
+      <c r="E18" s="6">
+        <f>'توقع المحصل 2026'!F17</f>
+        <v/>
+      </c>
+      <c r="F18" s="6">
+        <f>'توقع المحصل 2026'!G17</f>
+        <v/>
+      </c>
+      <c r="G18" s="6">
+        <f>'توقع المحصل 2026'!H17</f>
+        <v/>
+      </c>
+      <c r="H18" s="15">
+        <f>IF(F18=0,"",G18/F18)</f>
+        <v/>
+      </c>
+      <c r="I18" s="6">
+        <f>J18-G18</f>
+        <v/>
+      </c>
+      <c r="J18" s="6">
+        <f>'توقع المحصل 2026'!K17</f>
+        <v/>
+      </c>
+      <c r="K18" s="6">
+        <f>IF(J18=0,0,MAX(G18,MIN(J18,F18)))</f>
+        <v/>
+      </c>
+      <c r="L18" s="6">
+        <f>K18-J18</f>
+        <v/>
+      </c>
+      <c r="M18" s="7">
+        <f>J18/J$43</f>
+        <v/>
+      </c>
+      <c r="N18" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O18" s="16" t="inlineStr">
+        <is>
+          <t>قفزة: المحصل حتى سبتمبر (31.2م) يعادل 127% من كل 2025 (24.5م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>1422108</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>الشهادات الصحية</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D19" s="6">
+        <f>'توقع المحصل 2026'!E18</f>
+        <v/>
+      </c>
+      <c r="E19" s="6">
+        <f>'توقع المحصل 2026'!F18</f>
+        <v/>
+      </c>
+      <c r="F19" s="6">
+        <f>'توقع المحصل 2026'!G18</f>
+        <v/>
+      </c>
+      <c r="G19" s="6">
+        <f>'توقع المحصل 2026'!H18</f>
+        <v/>
+      </c>
+      <c r="H19" s="15">
+        <f>IF(F19=0,"",G19/F19)</f>
+        <v/>
+      </c>
+      <c r="I19" s="6">
+        <f>J19-G19</f>
+        <v/>
+      </c>
+      <c r="J19" s="6">
+        <f>'توقع المحصل 2026'!K18</f>
+        <v/>
+      </c>
+      <c r="K19" s="6">
+        <f>IF(J19=0,0,MAX(G19,MIN(J19,F19)))</f>
+        <v/>
+      </c>
+      <c r="L19" s="6">
+        <f>K19-J19</f>
+        <v/>
+      </c>
+      <c r="M19" s="7">
+        <f>J19/J$43</f>
+        <v/>
+      </c>
+      <c r="N19" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O19" s="16" t="inlineStr">
+        <is>
+          <t>مستقر: التوقع (23.5م) قريب من محصل 2025 (26.1م).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>1422121</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>رسم ترخيص نشاط تقديم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D20" s="6">
+        <f>'توقع المحصل 2026'!E19</f>
+        <v/>
+      </c>
+      <c r="E20" s="6">
+        <f>'توقع المحصل 2026'!F19</f>
+        <v/>
+      </c>
+      <c r="F20" s="6">
+        <f>'توقع المحصل 2026'!G19</f>
+        <v/>
+      </c>
+      <c r="G20" s="6">
+        <f>'توقع المحصل 2026'!H19</f>
+        <v/>
+      </c>
+      <c r="H20" s="15">
+        <f>IF(F20=0,"",G20/F20)</f>
+        <v/>
+      </c>
+      <c r="I20" s="6">
+        <f>J20-G20</f>
+        <v/>
+      </c>
+      <c r="J20" s="6">
+        <f>'توقع المحصل 2026'!K19</f>
+        <v/>
+      </c>
+      <c r="K20" s="6">
+        <f>IF(J20=0,0,MAX(G20,MIN(J20,F20)))</f>
+        <v/>
+      </c>
+      <c r="L20" s="6">
+        <f>K20-J20</f>
+        <v/>
+      </c>
+      <c r="M20" s="7">
+        <f>J20/J$43</f>
+        <v/>
+      </c>
+      <c r="N20" s="5" t="inlineStr">
+        <is>
+          <t>متوسط</t>
+        </is>
+      </c>
+      <c r="O20" s="16" t="inlineStr">
+        <is>
+          <t>التوقع أعلى من 2025 بنسبة 18% لأن وتيرة التحصيل حتى سبتمبر أعلى.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>بدون رقم</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>بدون رقم (خدمات علم + جزاءات)</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>علم / جزاءات</t>
+        </is>
+      </c>
+      <c r="D21" s="6">
+        <f>'توقع المحصل 2026'!E20</f>
+        <v/>
+      </c>
+      <c r="E21" s="6">
+        <f>'توقع المحصل 2026'!F20</f>
+        <v/>
+      </c>
+      <c r="F21" s="6">
+        <f>'توقع المحصل 2026'!G20</f>
+        <v/>
+      </c>
+      <c r="G21" s="6">
+        <f>'توقع المحصل 2026'!H20</f>
+        <v/>
+      </c>
+      <c r="H21" s="15">
+        <f>IF(F21=0,"",G21/F21)</f>
+        <v/>
+      </c>
+      <c r="I21" s="6">
+        <f>J21-G21</f>
+        <v/>
+      </c>
+      <c r="J21" s="6">
+        <f>'توقع المحصل 2026'!K20</f>
+        <v/>
+      </c>
+      <c r="K21" s="6">
+        <f>IF(J21=0,0,MAX(G21,MIN(J21,F21)))</f>
+        <v/>
+      </c>
+      <c r="L21" s="6">
+        <f>K21-J21</f>
+        <v/>
+      </c>
+      <c r="M21" s="7">
+        <f>J21/J$43</f>
+        <v/>
+      </c>
+      <c r="N21" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O21" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (2.1م) يعادل 10% فقط من 2025 (21.8م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>142163</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  تأجير مباني تجارية</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D22" s="6">
+        <f>'توقع المحصل 2026'!E21</f>
+        <v/>
+      </c>
+      <c r="E22" s="6">
+        <f>'توقع المحصل 2026'!F21</f>
+        <v/>
+      </c>
+      <c r="F22" s="6">
+        <f>'توقع المحصل 2026'!G21</f>
+        <v/>
+      </c>
+      <c r="G22" s="6">
+        <f>'توقع المحصل 2026'!H21</f>
+        <v/>
+      </c>
+      <c r="H22" s="15">
+        <f>IF(F22=0,"",G22/F22)</f>
+        <v/>
+      </c>
+      <c r="I22" s="6">
+        <f>J22-G22</f>
+        <v/>
+      </c>
+      <c r="J22" s="6">
+        <f>'توقع المحصل 2026'!K21</f>
+        <v/>
+      </c>
+      <c r="K22" s="6">
+        <f>IF(J22=0,0,MAX(G22,MIN(J22,F22)))</f>
+        <v/>
+      </c>
+      <c r="L22" s="6">
+        <f>K22-J22</f>
+        <v/>
+      </c>
+      <c r="M22" s="7">
+        <f>J22/J$43</f>
+        <v/>
+      </c>
+      <c r="N22" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O22" s="16" t="inlineStr">
+        <is>
+          <t>قفزة: المحصل حتى سبتمبر (10.2م) يعادل 339% من كل 2025 (3.0م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>1422109</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  الكشفية</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D23" s="6">
+        <f>'توقع المحصل 2026'!E22</f>
+        <v/>
+      </c>
+      <c r="E23" s="6">
+        <f>'توقع المحصل 2026'!F22</f>
+        <v/>
+      </c>
+      <c r="F23" s="6">
+        <f>'توقع المحصل 2026'!G22</f>
+        <v/>
+      </c>
+      <c r="G23" s="6">
+        <f>'توقع المحصل 2026'!H22</f>
+        <v/>
+      </c>
+      <c r="H23" s="15">
+        <f>IF(F23=0,"",G23/F23)</f>
+        <v/>
+      </c>
+      <c r="I23" s="6">
+        <f>J23-G23</f>
+        <v/>
+      </c>
+      <c r="J23" s="6">
+        <f>'توقع المحصل 2026'!K22</f>
+        <v/>
+      </c>
+      <c r="K23" s="6">
+        <f>IF(J23=0,0,MAX(G23,MIN(J23,F23)))</f>
+        <v/>
+      </c>
+      <c r="L23" s="6">
+        <f>K23-J23</f>
+        <v/>
+      </c>
+      <c r="M23" s="7">
+        <f>J23/J$43</f>
+        <v/>
+      </c>
+      <c r="N23" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O23" s="16" t="inlineStr">
+        <is>
+          <t>مستقر: التوقع (7.6م) قريب من محصل 2025 (7.1م).</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>11452111</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>المقابل المالي للسماح للأنشطة التجارية بالعمل (24) ساعة</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D24" s="6">
+        <f>'توقع المحصل 2026'!E23</f>
+        <v/>
+      </c>
+      <c r="E24" s="6">
+        <f>'توقع المحصل 2026'!F23</f>
+        <v/>
+      </c>
+      <c r="F24" s="6">
+        <f>'توقع المحصل 2026'!G23</f>
+        <v/>
+      </c>
+      <c r="G24" s="6">
+        <f>'توقع المحصل 2026'!H23</f>
+        <v/>
+      </c>
+      <c r="H24" s="15">
+        <f>IF(F24=0,"",G24/F24)</f>
+        <v/>
+      </c>
+      <c r="I24" s="6">
+        <f>J24-G24</f>
+        <v/>
+      </c>
+      <c r="J24" s="6">
+        <f>'توقع المحصل 2026'!K23</f>
+        <v/>
+      </c>
+      <c r="K24" s="6">
+        <f>IF(J24=0,0,MAX(G24,MIN(J24,F24)))</f>
+        <v/>
+      </c>
+      <c r="L24" s="6">
+        <f>K24-J24</f>
+        <v/>
+      </c>
+      <c r="M24" s="7">
+        <f>J24/J$43</f>
+        <v/>
+      </c>
+      <c r="N24" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O24" s="16" t="inlineStr">
+        <is>
+          <t>قفزة: المحصل حتى سبتمبر (11.4م) يعادل 198% من كل 2025 (5.8م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>1421910</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>اصدار تراخيص اشغال الارصفة العامة و الطرق</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D25" s="6">
+        <f>'توقع المحصل 2026'!E24</f>
+        <v/>
+      </c>
+      <c r="E25" s="6">
+        <f>'توقع المحصل 2026'!F24</f>
+        <v/>
+      </c>
+      <c r="F25" s="6">
+        <f>'توقع المحصل 2026'!G24</f>
+        <v/>
+      </c>
+      <c r="G25" s="6">
+        <f>'توقع المحصل 2026'!H24</f>
+        <v/>
+      </c>
+      <c r="H25" s="15">
+        <f>IF(F25=0,"",G25/F25)</f>
+        <v/>
+      </c>
+      <c r="I25" s="6">
+        <f>J25-G25</f>
+        <v/>
+      </c>
+      <c r="J25" s="6">
+        <f>'توقع المحصل 2026'!K24</f>
+        <v/>
+      </c>
+      <c r="K25" s="6">
+        <f>IF(J25=0,0,MAX(G25,MIN(J25,F25)))</f>
+        <v/>
+      </c>
+      <c r="L25" s="6">
+        <f>K25-J25</f>
+        <v/>
+      </c>
+      <c r="M25" s="7">
+        <f>J25/J$43</f>
+        <v/>
+      </c>
+      <c r="N25" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O25" s="16" t="inlineStr">
+        <is>
+          <t>المحصل حتى سبتمبر (3.6م) بلغ 103% من كل 2025 (3.5م). إضافة الربع الأخير بنفس الوتيرة ترفع التوقع 37% فوق 2025، وإن كان التحصيل يتركز في بداية السنة فالتوقع مبالغ فيه.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>1439</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  مبيعات  ناتجه من النشاط غير مصنفة</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D26" s="6">
+        <f>'توقع المحصل 2026'!E25</f>
+        <v/>
+      </c>
+      <c r="E26" s="6">
+        <f>'توقع المحصل 2026'!F25</f>
+        <v/>
+      </c>
+      <c r="F26" s="6">
+        <f>'توقع المحصل 2026'!G25</f>
+        <v/>
+      </c>
+      <c r="G26" s="6">
+        <f>'توقع المحصل 2026'!H25</f>
+        <v/>
+      </c>
+      <c r="H26" s="15">
+        <f>IF(F26=0,"",G26/F26)</f>
+        <v/>
+      </c>
+      <c r="I26" s="6">
+        <f>J26-G26</f>
+        <v/>
+      </c>
+      <c r="J26" s="6">
+        <f>'توقع المحصل 2026'!K25</f>
+        <v/>
+      </c>
+      <c r="K26" s="6">
+        <f>IF(J26=0,0,MAX(G26,MIN(J26,F26)))</f>
+        <v/>
+      </c>
+      <c r="L26" s="6">
+        <f>K26-J26</f>
+        <v/>
+      </c>
+      <c r="M26" s="7">
+        <f>J26/J$43</f>
+        <v/>
+      </c>
+      <c r="N26" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O26" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (0.2م) يعادل 2% فقط من 2025 (8.5م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>1421901</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>بيع الوثائق والأنظمة</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D27" s="6">
+        <f>'توقع المحصل 2026'!E26</f>
+        <v/>
+      </c>
+      <c r="E27" s="6">
+        <f>'توقع المحصل 2026'!F26</f>
+        <v/>
+      </c>
+      <c r="F27" s="6">
+        <f>'توقع المحصل 2026'!G26</f>
+        <v/>
+      </c>
+      <c r="G27" s="6">
+        <f>'توقع المحصل 2026'!H26</f>
+        <v/>
+      </c>
+      <c r="H27" s="15">
+        <f>IF(F27=0,"",G27/F27)</f>
+        <v/>
+      </c>
+      <c r="I27" s="6">
+        <f>J27-G27</f>
+        <v/>
+      </c>
+      <c r="J27" s="6">
+        <f>'توقع المحصل 2026'!K26</f>
+        <v/>
+      </c>
+      <c r="K27" s="6">
+        <f>IF(J27=0,0,MAX(G27,MIN(J27,F27)))</f>
+        <v/>
+      </c>
+      <c r="L27" s="6">
+        <f>K27-J27</f>
+        <v/>
+      </c>
+      <c r="M27" s="7">
+        <f>J27/J$43</f>
+        <v/>
+      </c>
+      <c r="N27" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O27" s="16" t="inlineStr">
+        <is>
+          <t>مستقر: التوقع (2.2م) قريب من محصل 2025 (2.5م).</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>1421903</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>مبيعات التيار الكهربائي</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D28" s="6">
+        <f>'توقع المحصل 2026'!E27</f>
+        <v/>
+      </c>
+      <c r="E28" s="6">
+        <f>'توقع المحصل 2026'!F27</f>
+        <v/>
+      </c>
+      <c r="F28" s="6">
+        <f>'توقع المحصل 2026'!G27</f>
+        <v/>
+      </c>
+      <c r="G28" s="6">
+        <f>'توقع المحصل 2026'!H27</f>
+        <v/>
+      </c>
+      <c r="H28" s="15">
+        <f>IF(F28=0,"",G28/F28)</f>
+        <v/>
+      </c>
+      <c r="I28" s="6">
+        <f>J28-G28</f>
+        <v/>
+      </c>
+      <c r="J28" s="6">
+        <f>'توقع المحصل 2026'!K27</f>
+        <v/>
+      </c>
+      <c r="K28" s="6">
+        <f>IF(J28=0,0,MAX(G28,MIN(J28,F28)))</f>
+        <v/>
+      </c>
+      <c r="L28" s="6">
+        <f>K28-J28</f>
+        <v/>
+      </c>
+      <c r="M28" s="7">
+        <f>J28/J$43</f>
+        <v/>
+      </c>
+      <c r="N28" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O28" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (0.3م) يعادل 19% فقط من 2025 (1.5م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>1438</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات مفروضة بموجب أنظمة الجهة</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D29" s="6">
+        <f>'توقع المحصل 2026'!E28</f>
+        <v/>
+      </c>
+      <c r="E29" s="6">
+        <f>'توقع المحصل 2026'!F28</f>
+        <v/>
+      </c>
+      <c r="F29" s="6">
+        <f>'توقع المحصل 2026'!G28</f>
+        <v/>
+      </c>
+      <c r="G29" s="6">
+        <f>'توقع المحصل 2026'!H28</f>
+        <v/>
+      </c>
+      <c r="H29" s="15">
+        <f>IF(F29=0,"",G29/F29)</f>
+        <v/>
+      </c>
+      <c r="I29" s="6">
+        <f>J29-G29</f>
+        <v/>
+      </c>
+      <c r="J29" s="6">
+        <f>'توقع المحصل 2026'!K28</f>
+        <v/>
+      </c>
+      <c r="K29" s="6">
+        <f>IF(J29=0,0,MAX(G29,MIN(J29,F29)))</f>
+        <v/>
+      </c>
+      <c r="L29" s="6">
+        <f>K29-J29</f>
+        <v/>
+      </c>
+      <c r="M29" s="7">
+        <f>J29/J$43</f>
+        <v/>
+      </c>
+      <c r="N29" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O29" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (0.1م) يعادل 17% فقط من 2025 (0.4م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>1421912</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>تأجير العقارات لأغراض مؤقته</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D30" s="6">
+        <f>'توقع المحصل 2026'!E29</f>
+        <v/>
+      </c>
+      <c r="E30" s="6">
+        <f>'توقع المحصل 2026'!F29</f>
+        <v/>
+      </c>
+      <c r="F30" s="6">
+        <f>'توقع المحصل 2026'!G29</f>
+        <v/>
+      </c>
+      <c r="G30" s="6">
+        <f>'توقع المحصل 2026'!H29</f>
+        <v/>
+      </c>
+      <c r="H30" s="15">
+        <f>IF(F30=0,"",G30/F30)</f>
+        <v/>
+      </c>
+      <c r="I30" s="6">
+        <f>J30-G30</f>
+        <v/>
+      </c>
+      <c r="J30" s="6">
+        <f>'توقع المحصل 2026'!K29</f>
+        <v/>
+      </c>
+      <c r="K30" s="6">
+        <f>IF(J30=0,0,MAX(G30,MIN(J30,F30)))</f>
+        <v/>
+      </c>
+      <c r="L30" s="6">
+        <f>K30-J30</f>
+        <v/>
+      </c>
+      <c r="M30" s="7">
+        <f>J30/J$43</f>
+        <v/>
+      </c>
+      <c r="N30" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O30" s="16" t="inlineStr">
+        <is>
+          <t>التوقع أدنى من 2025 بنسبة 26% لأن وتيرة التحصيل حتى سبتمبر أقل.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>11452106</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>اصدار التراخيص بتأسيس أو تشغيل ابراج الاتصالات</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D31" s="6">
+        <f>'توقع المحصل 2026'!E30</f>
+        <v/>
+      </c>
+      <c r="E31" s="6">
+        <f>'توقع المحصل 2026'!F30</f>
+        <v/>
+      </c>
+      <c r="F31" s="6">
+        <f>'توقع المحصل 2026'!G30</f>
+        <v/>
+      </c>
+      <c r="G31" s="6">
+        <f>'توقع المحصل 2026'!H30</f>
+        <v/>
+      </c>
+      <c r="H31" s="15">
+        <f>IF(F31=0,"",G31/F31)</f>
+        <v/>
+      </c>
+      <c r="I31" s="6">
+        <f>J31-G31</f>
+        <v/>
+      </c>
+      <c r="J31" s="6">
+        <f>'توقع المحصل 2026'!K30</f>
+        <v/>
+      </c>
+      <c r="K31" s="6">
+        <f>IF(J31=0,0,MAX(G31,MIN(J31,F31)))</f>
+        <v/>
+      </c>
+      <c r="L31" s="6">
+        <f>K31-J31</f>
+        <v/>
+      </c>
+      <c r="M31" s="7">
+        <f>J31/J$43</f>
+        <v/>
+      </c>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O31" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (0.3م) يعادل 27% فقط من 2025 (1.3م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>11452110</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>إصدار تراخيص إستخدام أملاك خاصة لإقامة فعاليات</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D32" s="6">
+        <f>'توقع المحصل 2026'!E31</f>
+        <v/>
+      </c>
+      <c r="E32" s="6">
+        <f>'توقع المحصل 2026'!F31</f>
+        <v/>
+      </c>
+      <c r="F32" s="6">
+        <f>'توقع المحصل 2026'!G31</f>
+        <v/>
+      </c>
+      <c r="G32" s="6">
+        <f>'توقع المحصل 2026'!H31</f>
+        <v/>
+      </c>
+      <c r="H32" s="15">
+        <f>IF(F32=0,"",G32/F32)</f>
+        <v/>
+      </c>
+      <c r="I32" s="6">
+        <f>J32-G32</f>
+        <v/>
+      </c>
+      <c r="J32" s="6">
+        <f>'توقع المحصل 2026'!K31</f>
+        <v/>
+      </c>
+      <c r="K32" s="6">
+        <f>IF(J32=0,0,MAX(G32,MIN(J32,F32)))</f>
+        <v/>
+      </c>
+      <c r="L32" s="6">
+        <f>K32-J32</f>
+        <v/>
+      </c>
+      <c r="M32" s="7">
+        <f>J32/J$43</f>
+        <v/>
+      </c>
+      <c r="N32" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O32" s="16" t="inlineStr">
+        <is>
+          <t>مستقر: التوقع (0.8م) قريب من محصل 2025 (0.8م).</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>141229</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>أرباح أخرى</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D33" s="6">
+        <f>'توقع المحصل 2026'!E32</f>
+        <v/>
+      </c>
+      <c r="E33" s="6">
+        <f>'توقع المحصل 2026'!F32</f>
+        <v/>
+      </c>
+      <c r="F33" s="6">
+        <f>'توقع المحصل 2026'!G32</f>
+        <v/>
+      </c>
+      <c r="G33" s="6">
+        <f>'توقع المحصل 2026'!H32</f>
+        <v/>
+      </c>
+      <c r="H33" s="15">
+        <f>IF(F33=0,"",G33/F33)</f>
+        <v/>
+      </c>
+      <c r="I33" s="6">
+        <f>J33-G33</f>
+        <v/>
+      </c>
+      <c r="J33" s="6">
+        <f>'توقع المحصل 2026'!K32</f>
+        <v/>
+      </c>
+      <c r="K33" s="6">
+        <f>IF(J33=0,0,MAX(G33,MIN(J33,F33)))</f>
+        <v/>
+      </c>
+      <c r="L33" s="6">
+        <f>K33-J33</f>
+        <v/>
+      </c>
+      <c r="M33" s="7">
+        <f>J33/J$43</f>
+        <v/>
+      </c>
+      <c r="N33" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O33" s="16" t="inlineStr">
+        <is>
+          <t>قفزة: المحصل حتى سبتمبر (0.1م) يعادل 200% من كل 2025 (0.0م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>11452109</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>اعتماد مخططات التطوير العقاري</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D34" s="6">
+        <f>'توقع المحصل 2026'!E33</f>
+        <v/>
+      </c>
+      <c r="E34" s="6">
+        <f>'توقع المحصل 2026'!F33</f>
+        <v/>
+      </c>
+      <c r="F34" s="6">
+        <f>'توقع المحصل 2026'!G33</f>
+        <v/>
+      </c>
+      <c r="G34" s="6">
+        <f>'توقع المحصل 2026'!H33</f>
+        <v/>
+      </c>
+      <c r="H34" s="15">
+        <f>IF(F34=0,"",G34/F34)</f>
+        <v/>
+      </c>
+      <c r="I34" s="6">
+        <f>J34-G34</f>
+        <v/>
+      </c>
+      <c r="J34" s="6">
+        <f>'توقع المحصل 2026'!K33</f>
+        <v/>
+      </c>
+      <c r="K34" s="6">
+        <f>IF(J34=0,0,MAX(G34,MIN(J34,F34)))</f>
+        <v/>
+      </c>
+      <c r="L34" s="6">
+        <f>K34-J34</f>
+        <v/>
+      </c>
+      <c r="M34" s="7">
+        <f>J34/J$43</f>
+        <v/>
+      </c>
+      <c r="N34" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O34" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (0.0م) يعادل 0% فقط من 2025 (0.6م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>11452107</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>اصدار التراخيص بتأسيس أو تشغيل الصراف الآلي</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D35" s="6">
+        <f>'توقع المحصل 2026'!E34</f>
+        <v/>
+      </c>
+      <c r="E35" s="6">
+        <f>'توقع المحصل 2026'!F34</f>
+        <v/>
+      </c>
+      <c r="F35" s="6">
+        <f>'توقع المحصل 2026'!G34</f>
+        <v/>
+      </c>
+      <c r="G35" s="6">
+        <f>'توقع المحصل 2026'!H34</f>
+        <v/>
+      </c>
+      <c r="H35" s="15">
+        <f>IF(F35=0,"",G35/F35)</f>
+        <v/>
+      </c>
+      <c r="I35" s="6">
+        <f>J35-G35</f>
+        <v/>
+      </c>
+      <c r="J35" s="6">
+        <f>'توقع المحصل 2026'!K34</f>
+        <v/>
+      </c>
+      <c r="K35" s="6">
+        <f>IF(J35=0,0,MAX(G35,MIN(J35,F35)))</f>
+        <v/>
+      </c>
+      <c r="L35" s="6">
+        <f>K35-J35</f>
+        <v/>
+      </c>
+      <c r="M35" s="7">
+        <f>J35/J$43</f>
+        <v/>
+      </c>
+      <c r="N35" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O35" s="16" t="inlineStr">
+        <is>
+          <t>مستقر: التوقع (0.2م) قريب من محصل 2025 (0.2م).</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>3318212</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>مرتجع رواتب - فواتير</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D36" s="6">
+        <f>'توقع المحصل 2026'!E35</f>
+        <v/>
+      </c>
+      <c r="E36" s="6">
+        <f>'توقع المحصل 2026'!F35</f>
+        <v/>
+      </c>
+      <c r="F36" s="6">
+        <f>'توقع المحصل 2026'!G35</f>
+        <v/>
+      </c>
+      <c r="G36" s="6">
+        <f>'توقع المحصل 2026'!H35</f>
+        <v/>
+      </c>
+      <c r="H36" s="15">
+        <f>IF(F36=0,"",G36/F36)</f>
+        <v/>
+      </c>
+      <c r="I36" s="6">
+        <f>J36-G36</f>
+        <v/>
+      </c>
+      <c r="J36" s="6">
+        <f>'توقع المحصل 2026'!K35</f>
+        <v/>
+      </c>
+      <c r="K36" s="6">
+        <f>IF(J36=0,0,MAX(G36,MIN(J36,F36)))</f>
+        <v/>
+      </c>
+      <c r="L36" s="6">
+        <f>K36-J36</f>
+        <v/>
+      </c>
+      <c r="M36" s="7">
+        <f>J36/J$43</f>
+        <v/>
+      </c>
+      <c r="N36" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O36" s="16" t="inlineStr">
+        <is>
+          <t>قفزة: المحصل حتى سبتمبر (0.2م) يعادل 142% من كل 2025 (0.2م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>11422</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>رسوم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D37" s="6">
+        <f>'توقع المحصل 2026'!E36</f>
+        <v/>
+      </c>
+      <c r="E37" s="6">
+        <f>'توقع المحصل 2026'!F36</f>
+        <v/>
+      </c>
+      <c r="F37" s="6">
+        <f>'توقع المحصل 2026'!G36</f>
+        <v/>
+      </c>
+      <c r="G37" s="6">
+        <f>'توقع المحصل 2026'!H36</f>
+        <v/>
+      </c>
+      <c r="H37" s="15">
+        <f>IF(F37=0,"",G37/F37)</f>
+        <v/>
+      </c>
+      <c r="I37" s="6">
+        <f>J37-G37</f>
+        <v/>
+      </c>
+      <c r="J37" s="6">
+        <f>'توقع المحصل 2026'!K36</f>
+        <v/>
+      </c>
+      <c r="K37" s="6">
+        <f>IF(J37=0,0,MAX(G37,MIN(J37,F37)))</f>
+        <v/>
+      </c>
+      <c r="L37" s="6">
+        <f>K37-J37</f>
+        <v/>
+      </c>
+      <c r="M37" s="7">
+        <f>J37/J$43</f>
+        <v/>
+      </c>
+      <c r="N37" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O37" s="16" t="inlineStr">
+        <is>
+          <t>متوقف: لا فوترة ولا تحصيل في 2026، فتوقعه صفر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>1422103</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>تراخيص المحلات</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D38" s="6">
+        <f>'توقع المحصل 2026'!E37</f>
+        <v/>
+      </c>
+      <c r="E38" s="6">
+        <f>'توقع المحصل 2026'!F37</f>
+        <v/>
+      </c>
+      <c r="F38" s="6">
+        <f>'توقع المحصل 2026'!G37</f>
+        <v/>
+      </c>
+      <c r="G38" s="6">
+        <f>'توقع المحصل 2026'!H37</f>
+        <v/>
+      </c>
+      <c r="H38" s="15">
+        <f>IF(F38=0,"",G38/F38)</f>
+        <v/>
+      </c>
+      <c r="I38" s="6">
+        <f>J38-G38</f>
+        <v/>
+      </c>
+      <c r="J38" s="6">
+        <f>'توقع المحصل 2026'!K37</f>
+        <v/>
+      </c>
+      <c r="K38" s="6">
+        <f>IF(J38=0,0,MAX(G38,MIN(J38,F38)))</f>
+        <v/>
+      </c>
+      <c r="L38" s="6">
+        <f>K38-J38</f>
+        <v/>
+      </c>
+      <c r="M38" s="7">
+        <f>J38/J$43</f>
+        <v/>
+      </c>
+      <c r="N38" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O38" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (0.0م) يعادل 27% فقط من 2025 (0.0م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>11452513</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>لوحات إرشـادية</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D39" s="6">
+        <f>'توقع المحصل 2026'!E38</f>
+        <v/>
+      </c>
+      <c r="E39" s="6">
+        <f>'توقع المحصل 2026'!F38</f>
+        <v/>
+      </c>
+      <c r="F39" s="6">
+        <f>'توقع المحصل 2026'!G38</f>
+        <v/>
+      </c>
+      <c r="G39" s="6">
+        <f>'توقع المحصل 2026'!H38</f>
+        <v/>
+      </c>
+      <c r="H39" s="15">
+        <f>IF(F39=0,"",G39/F39)</f>
+        <v/>
+      </c>
+      <c r="I39" s="6">
+        <f>J39-G39</f>
+        <v/>
+      </c>
+      <c r="J39" s="6">
+        <f>'توقع المحصل 2026'!K38</f>
+        <v/>
+      </c>
+      <c r="K39" s="6">
+        <f>IF(J39=0,0,MAX(G39,MIN(J39,F39)))</f>
+        <v/>
+      </c>
+      <c r="L39" s="6">
+        <f>K39-J39</f>
+        <v/>
+      </c>
+      <c r="M39" s="7">
+        <f>J39/J$43</f>
+        <v/>
+      </c>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O39" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (0.0م) يعادل 7% فقط من 2025 (0.0م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>1421907</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات المخططات</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D40" s="6">
+        <f>'توقع المحصل 2026'!E39</f>
+        <v/>
+      </c>
+      <c r="E40" s="6">
+        <f>'توقع المحصل 2026'!F39</f>
+        <v/>
+      </c>
+      <c r="F40" s="6">
+        <f>'توقع المحصل 2026'!G39</f>
+        <v/>
+      </c>
+      <c r="G40" s="6">
+        <f>'توقع المحصل 2026'!H39</f>
+        <v/>
+      </c>
+      <c r="H40" s="15">
+        <f>IF(F40=0,"",G40/F40)</f>
+        <v/>
+      </c>
+      <c r="I40" s="6">
+        <f>J40-G40</f>
+        <v/>
+      </c>
+      <c r="J40" s="6">
+        <f>'توقع المحصل 2026'!K39</f>
+        <v/>
+      </c>
+      <c r="K40" s="6">
+        <f>IF(J40=0,0,MAX(G40,MIN(J40,F40)))</f>
+        <v/>
+      </c>
+      <c r="L40" s="6">
+        <f>K40-J40</f>
+        <v/>
+      </c>
+      <c r="M40" s="7">
+        <f>J40/J$43</f>
+        <v/>
+      </c>
+      <c r="N40" s="5" t="inlineStr">
+        <is>
+          <t>مرتفع</t>
+        </is>
+      </c>
+      <c r="O40" s="16" t="inlineStr">
+        <is>
+          <t>تراجع حاد: المحصل حتى سبتمبر (0.0م) يعادل 27% فقط من 2025 (0.0م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>1421908</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  رسوم خدمات  بلدية</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D41" s="6">
+        <f>'توقع المحصل 2026'!E40</f>
+        <v/>
+      </c>
+      <c r="E41" s="6">
+        <f>'توقع المحصل 2026'!F40</f>
+        <v/>
+      </c>
+      <c r="F41" s="6">
+        <f>'توقع المحصل 2026'!G40</f>
+        <v/>
+      </c>
+      <c r="G41" s="6">
+        <f>'توقع المحصل 2026'!H40</f>
+        <v/>
+      </c>
+      <c r="H41" s="15">
+        <f>IF(F41=0,"",G41/F41)</f>
+        <v/>
+      </c>
+      <c r="I41" s="6">
+        <f>J41-G41</f>
+        <v/>
+      </c>
+      <c r="J41" s="6">
+        <f>'توقع المحصل 2026'!K40</f>
+        <v/>
+      </c>
+      <c r="K41" s="6">
+        <f>IF(J41=0,0,MAX(G41,MIN(J41,F41)))</f>
+        <v/>
+      </c>
+      <c r="L41" s="6">
+        <f>K41-J41</f>
+        <v/>
+      </c>
+      <c r="M41" s="7">
+        <f>J41/J$43</f>
+        <v/>
+      </c>
+      <c r="N41" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O41" s="16" t="inlineStr">
+        <is>
+          <t>متوقف: لا فوترة ولا تحصيل في 2026، فتوقعه صفر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>142161</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>تاجير مباني سكنية</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D42" s="6">
+        <f>'توقع المحصل 2026'!E41</f>
+        <v/>
+      </c>
+      <c r="E42" s="6">
+        <f>'توقع المحصل 2026'!F41</f>
+        <v/>
+      </c>
+      <c r="F42" s="6">
+        <f>'توقع المحصل 2026'!G41</f>
+        <v/>
+      </c>
+      <c r="G42" s="6">
+        <f>'توقع المحصل 2026'!H41</f>
+        <v/>
+      </c>
+      <c r="H42" s="15">
+        <f>IF(F42=0,"",G42/F42)</f>
+        <v/>
+      </c>
+      <c r="I42" s="6">
+        <f>J42-G42</f>
+        <v/>
+      </c>
+      <c r="J42" s="6">
+        <f>'توقع المحصل 2026'!K41</f>
+        <v/>
+      </c>
+      <c r="K42" s="6">
+        <f>IF(J42=0,0,MAX(G42,MIN(J42,F42)))</f>
+        <v/>
+      </c>
+      <c r="L42" s="6">
+        <f>K42-J42</f>
+        <v/>
+      </c>
+      <c r="M42" s="7">
+        <f>J42/J$43</f>
+        <v/>
+      </c>
+      <c r="N42" s="5" t="inlineStr">
+        <is>
+          <t>منخفض</t>
+        </is>
+      </c>
+      <c r="O42" s="16" t="inlineStr">
+        <is>
+          <t>متوقف: لا فوترة ولا تحصيل في 2026، فتوقعه صفر.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="8" t="n"/>
+      <c r="B43" s="8" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="C43" s="8" t="n"/>
+      <c r="D43" s="9">
+        <f>SUM(D5:D42)</f>
+        <v/>
+      </c>
+      <c r="E43" s="9">
+        <f>SUM(E5:E42)</f>
+        <v/>
+      </c>
+      <c r="F43" s="9">
+        <f>SUM(F5:F42)</f>
+        <v/>
+      </c>
+      <c r="G43" s="9">
+        <f>SUM(G5:G42)</f>
+        <v/>
+      </c>
+      <c r="H43" s="17">
+        <f>G43/F43</f>
+        <v/>
+      </c>
+      <c r="I43" s="9">
+        <f>SUM(I5:I42)</f>
+        <v/>
+      </c>
+      <c r="J43" s="9">
+        <f>SUM(J5:J42)</f>
+        <v/>
+      </c>
+      <c r="K43" s="9">
+        <f>SUM(K5:K42)</f>
+        <v/>
+      </c>
+      <c r="L43" s="9">
+        <f>SUM(L5:L42)</f>
+        <v/>
+      </c>
+      <c r="M43" s="10">
+        <f>SUM(M5:M42)</f>
+        <v/>
+      </c>
+      <c r="N43" s="8" t="n"/>
+      <c r="O43" s="18" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:O42"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:N2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -7555,7 +10336,7 @@
           <t>معامل تحويل 2026 إلى سنة كاملة (12÷9)</t>
         </is>
       </c>
-      <c r="B4" s="12">
+      <c r="B4" s="19">
         <f>12/9</f>
         <v/>
       </c>
@@ -7571,7 +10352,7 @@
           <t>نسبة النمو – السيناريو الأول (ثابتة)</t>
         </is>
       </c>
-      <c r="B5" s="13">
+      <c r="B5" s="20">
         <f>التوقعات!C2</f>
         <v/>
       </c>
@@ -7587,7 +10368,7 @@
           <t>سقف معدل النمو التاريخي (±)</t>
         </is>
       </c>
-      <c r="B6" s="13" t="n">
+      <c r="B6" s="20" t="n">
         <v>0.25</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -7604,70 +10385,70 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="14" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>1) الإجمالي المفوتر للحساب = المفوتر + المحصل عن سنوات سابقة (حسب طلبك).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="14" t="inlineStr">
+      <c r="A11" s="21" t="inlineStr">
         <is>
           <t>2) توقع 2026 = الفعلي حتى سبتمبر × 12/9 (لا توجد بيانات شهرية، فلا موسمية في التوقع).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>3) الحسابات التي فوترتها وتحصيلها صفر في 2026 تُعتبر متوقفة وتوقعها صفر في 2026 و2027.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="14" t="inlineStr">
+      <c r="A13" s="21" t="inlineStr">
         <is>
           <t>4) 2027 – السيناريو الأول: توقع 2026 × (1 + نسبة النمو في خلية C2 بورقة التوقعات؛ الافتراضي 7%).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>5) 2027 – السيناريو الثاني: توقع 2026 × (1 + معدل النمو السنوي المركب التاريخي للحساب بين أول سنة فيها فوترة و2025، بسقف ±25%). إن توفرت سنة واحدة فقط من البيانات = نمو 0%.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="21" t="inlineStr">
         <is>
           <t>6) تم استبعاد حساب قيمة الضريبة المضافة (11411) من كل الحسابات والإجماليات.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="14" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>6b) تم دمج صفّي "بدون رقم" (خدمات علم + جزاءات، وجزاءات جزء ضئيل) في صف واحد لكل سنة.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="14" t="inlineStr">
+      <c r="A17" s="21" t="inlineStr">
         <is>
           <t>6c) أعمدة النمو لكل حساب: نمو كل سنة عن السنة السابقة (2024 عن 2023، 2025 عن 2024، 2026 توقع عن 2025، و2027 عن 2026 للسيناريوهين). تظهر فارغة عندما تكون السنة السابقة صفراً.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="14" t="inlineStr">
+      <c r="A18" s="21" t="inlineStr">
         <is>
           <t>6d) ورقة "توقع المحصل 2026": توقع إقفال 2026 كمحصّل فعلي = المحصل حتى سبتمبر × 12÷9 (مسدد عن السنة + محصل سنوات سابقة).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="14" t="inlineStr">
+      <c r="A19" s="21" t="inlineStr">
         <is>
           <t>7) تنبيه: كثير من الحسابات تتذبذب بشدة بين السنوات (لوحات دعائية، تأجير المرافق، إيرادات متنوعة)، ومضاعفة 2026 على 12/9 تضخّم أو تقلّل هذه الأرقام؛ انظر عمود "تنبيه".</t>
         </is>

</xml_diff>

<commit_message>
Add seasonal collected forecast and monthly seasonality sheets
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/توقع_الفوترة_2026_2027.xlsx
+++ b/توقع_الفوترة_2026_2027.xlsx
@@ -12,12 +12,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تفصيل المكونات" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="توقع المحصل 2026" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تحليل التوقع والأسوأ" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="توقع المحصل الموسمي" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الموسمية الشهرية" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'التوقعات'!$A$3:$R$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'توقع المحصل 2026'!$A$3:$N$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'تحليل التوقع والأسوأ'!$A$4:$O$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'توقع المحصل الموسمي'!$A$5:$Q$43</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -118,7 +121,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -150,6 +153,7 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -10298,6 +10302,3361 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:Q44"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>توقع إقفال 2026 (محصّل) بالموسمية الشهرية — بدون الضريبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="58" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>الطريقة: توقع الربع الأخير (أكتوبر–ديسمبر) = وسيط تحصيل الربع الأخير في 2023–2025 × معامل الاتجاه، ومعامل الاتجاه = المحصل يناير–سبتمبر 2026 ÷ وسيط يناير–سبتمبر للسنوات الثلاث، بين حدّين في ورقة الافتراضات. الإقفال = المحصل يناير–سبتمبر + توقع الربع الأخير. السيناريو الأسوأ: الربع الأخير = أدنى ربع أخير في السنوات الثلاث × (معامل الاتجاه بحد أقصى 1). في الحالتين لا يقل الربع الأخير عن المحصل الفعلي من أكتوبر حتى تاريخ الملف. الوسيط يخفف أثر الشهور الاستثنائية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>الملخص:</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>إقفال 2026 – أساسي</t>
+        </is>
+      </c>
+      <c r="D3" s="14">
+        <f>M44</f>
+        <v/>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>إقفال 2026 – أسوأ</t>
+        </is>
+      </c>
+      <c r="F3" s="14">
+        <f>N44</f>
+        <v/>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>الحد الأدنى (يناير–سبتمبر + أكتوبر حتى تاريخه)</t>
+        </is>
+      </c>
+      <c r="H3" s="14">
+        <f>E44+F44</f>
+        <v/>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>محصل 2025</t>
+        </is>
+      </c>
+      <c r="J3" s="14">
+        <f>D44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>رقم الحساب</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>اسم الحساب</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>التبويب</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>2025 محصّل (سنة كاملة)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>2026 محصّل يناير–سبتمبر</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>2026 محصّل أكتوبر حتى تاريخه</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>وسيط يناير–سبتمبر 2023–2025</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>وسيط الربع الأخير 2023–2025</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>أدنى ربع أخير 2023–2025</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>معامل الاتجاه</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>الربع الأخير – أساسي</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>الربع الأخير – أسوأ</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>إقفال 2026 – أساسي</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>إقفال 2026 – أسوأ</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>الطريقة البسيطة (×12÷9)</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>الفرق: أساسي − بسيط</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>نمو الأساسي عن 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>14155</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>ريع الأراضي (تأجير الأراض )</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>649331791.52</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>611923098.9299999</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>966021.95</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>469288809.82</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>228907448.88</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>204333140.13</v>
+      </c>
+      <c r="J6" s="15">
+        <f>IF(G6&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E6/G6)),IF(E6&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K6" s="6">
+        <f>IF(AND(E6=0,F6=0),0,MAX(F6,H6*J6))</f>
+        <v/>
+      </c>
+      <c r="L6" s="6">
+        <f>IF(AND(E6=0,F6=0),0,MAX(F6,I6*MIN(J6,1)))</f>
+        <v/>
+      </c>
+      <c r="M6" s="6">
+        <f>E6+K6</f>
+        <v/>
+      </c>
+      <c r="N6" s="6">
+        <f>E6+L6</f>
+        <v/>
+      </c>
+      <c r="O6" s="6">
+        <f>E6*12/9</f>
+        <v/>
+      </c>
+      <c r="P6" s="6">
+        <f>M6-O6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="7">
+        <f>IF(D6=0,"",M6/D6-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>1438001</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات و غرامات مفروضة بموجب أنظمة الجهة</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>308012204.69</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>370116478.79</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>495850</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>238450578.45</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>85816586.84999999</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>65135107.34</v>
+      </c>
+      <c r="J7" s="15">
+        <f>IF(G7&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E7/G7)),IF(E7&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K7" s="6">
+        <f>IF(AND(E7=0,F7=0),0,MAX(F7,H7*J7))</f>
+        <v/>
+      </c>
+      <c r="L7" s="6">
+        <f>IF(AND(E7=0,F7=0),0,MAX(F7,I7*MIN(J7,1)))</f>
+        <v/>
+      </c>
+      <c r="M7" s="6">
+        <f>E7+K7</f>
+        <v/>
+      </c>
+      <c r="N7" s="6">
+        <f>E7+L7</f>
+        <v/>
+      </c>
+      <c r="O7" s="6">
+        <f>E7*12/9</f>
+        <v/>
+      </c>
+      <c r="P7" s="6">
+        <f>M7-O7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="7">
+        <f>IF(D7=0,"",M7/D7-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>142162</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  تأجير المرافق</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>25602601.22</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>428454063.2</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>5982.8</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>16504314.8</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>9098286.42</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>322650</v>
+      </c>
+      <c r="J8" s="15">
+        <f>IF(G8&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E8/G8)),IF(E8&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K8" s="6">
+        <f>IF(AND(E8=0,F8=0),0,MAX(F8,H8*J8))</f>
+        <v/>
+      </c>
+      <c r="L8" s="6">
+        <f>IF(AND(E8=0,F8=0),0,MAX(F8,I8*MIN(J8,1)))</f>
+        <v/>
+      </c>
+      <c r="M8" s="6">
+        <f>E8+K8</f>
+        <v/>
+      </c>
+      <c r="N8" s="6">
+        <f>E8+L8</f>
+        <v/>
+      </c>
+      <c r="O8" s="6">
+        <f>E8*12/9</f>
+        <v/>
+      </c>
+      <c r="P8" s="6">
+        <f>M8-O8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="7">
+        <f>IF(D8=0,"",M8/D8-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>11452104</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>إصدار رخص الأنشطة التجارية</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>267496278.85</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>247515318.43</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>2860329.04</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>195619294.47</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>70733180.56999999</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>70219227.95</v>
+      </c>
+      <c r="J9" s="15">
+        <f>IF(G9&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E9/G9)),IF(E9&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K9" s="6">
+        <f>IF(AND(E9=0,F9=0),0,MAX(F9,H9*J9))</f>
+        <v/>
+      </c>
+      <c r="L9" s="6">
+        <f>IF(AND(E9=0,F9=0),0,MAX(F9,I9*MIN(J9,1)))</f>
+        <v/>
+      </c>
+      <c r="M9" s="6">
+        <f>E9+K9</f>
+        <v/>
+      </c>
+      <c r="N9" s="6">
+        <f>E9+L9</f>
+        <v/>
+      </c>
+      <c r="O9" s="6">
+        <f>E9*12/9</f>
+        <v/>
+      </c>
+      <c r="P9" s="6">
+        <f>M9-O9</f>
+        <v/>
+      </c>
+      <c r="Q9" s="7">
+        <f>IF(D9=0,"",M9/D9-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>11452103</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>ايراد اصدار تراخيص المباني والاسوار - أمانة منطقة الرياض</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>319675274.54</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>203938354.66</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>64468.55</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>171624424.4</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>72958068.90000001</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>56149701.29</v>
+      </c>
+      <c r="J10" s="15">
+        <f>IF(G10&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E10/G10)),IF(E10&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K10" s="6">
+        <f>IF(AND(E10=0,F10=0),0,MAX(F10,H10*J10))</f>
+        <v/>
+      </c>
+      <c r="L10" s="6">
+        <f>IF(AND(E10=0,F10=0),0,MAX(F10,I10*MIN(J10,1)))</f>
+        <v/>
+      </c>
+      <c r="M10" s="6">
+        <f>E10+K10</f>
+        <v/>
+      </c>
+      <c r="N10" s="6">
+        <f>E10+L10</f>
+        <v/>
+      </c>
+      <c r="O10" s="6">
+        <f>E10*12/9</f>
+        <v/>
+      </c>
+      <c r="P10" s="6">
+        <f>M10-O10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="7">
+        <f>IF(D10=0,"",M10/D10-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>11452512</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات لوحات المحلات</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>193830778.44</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>171961516.6</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>2332984.9</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>155986575</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>59354580</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>51365275.98</v>
+      </c>
+      <c r="J11" s="15">
+        <f>IF(G11&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E11/G11)),IF(E11&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K11" s="6">
+        <f>IF(AND(E11=0,F11=0),0,MAX(F11,H11*J11))</f>
+        <v/>
+      </c>
+      <c r="L11" s="6">
+        <f>IF(AND(E11=0,F11=0),0,MAX(F11,I11*MIN(J11,1)))</f>
+        <v/>
+      </c>
+      <c r="M11" s="6">
+        <f>E11+K11</f>
+        <v/>
+      </c>
+      <c r="N11" s="6">
+        <f>E11+L11</f>
+        <v/>
+      </c>
+      <c r="O11" s="6">
+        <f>E11*12/9</f>
+        <v/>
+      </c>
+      <c r="P11" s="6">
+        <f>M11-O11</f>
+        <v/>
+      </c>
+      <c r="Q11" s="7">
+        <f>IF(D11=0,"",M11/D11-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>142113</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  اللوحات الدعائية</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>1016877058.52</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>121704394.25</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>327373.48</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>402775368.76</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>159604841.42</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>35149182.39</v>
+      </c>
+      <c r="J12" s="15">
+        <f>IF(G12&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E12/G12)),IF(E12&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K12" s="6">
+        <f>IF(AND(E12=0,F12=0),0,MAX(F12,H12*J12))</f>
+        <v/>
+      </c>
+      <c r="L12" s="6">
+        <f>IF(AND(E12=0,F12=0),0,MAX(F12,I12*MIN(J12,1)))</f>
+        <v/>
+      </c>
+      <c r="M12" s="6">
+        <f>E12+K12</f>
+        <v/>
+      </c>
+      <c r="N12" s="6">
+        <f>E12+L12</f>
+        <v/>
+      </c>
+      <c r="O12" s="6">
+        <f>E12*12/9</f>
+        <v/>
+      </c>
+      <c r="P12" s="6">
+        <f>M12-O12</f>
+        <v/>
+      </c>
+      <c r="Q12" s="7">
+        <f>IF(D12=0,"",M12/D12-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>11442</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>اشغال مرافق الايواء</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>199149669.75</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>135824266.97</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>815494.87</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>152968341.46</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>66937519.73</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>57302452.03</v>
+      </c>
+      <c r="J13" s="15">
+        <f>IF(G13&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E13/G13)),IF(E13&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K13" s="6">
+        <f>IF(AND(E13=0,F13=0),0,MAX(F13,H13*J13))</f>
+        <v/>
+      </c>
+      <c r="L13" s="6">
+        <f>IF(AND(E13=0,F13=0),0,MAX(F13,I13*MIN(J13,1)))</f>
+        <v/>
+      </c>
+      <c r="M13" s="6">
+        <f>E13+K13</f>
+        <v/>
+      </c>
+      <c r="N13" s="6">
+        <f>E13+L13</f>
+        <v/>
+      </c>
+      <c r="O13" s="6">
+        <f>E13*12/9</f>
+        <v/>
+      </c>
+      <c r="P13" s="6">
+        <f>M13-O13</f>
+        <v/>
+      </c>
+      <c r="Q13" s="7">
+        <f>IF(D13=0,"",M13/D13-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>1421999</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>مبيعات أخرى</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>60096373.96</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>134076434.91</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>78879723.06</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>19648593.93</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>5322376.9</v>
+      </c>
+      <c r="J14" s="15">
+        <f>IF(G14&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E14/G14)),IF(E14&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K14" s="6">
+        <f>IF(AND(E14=0,F14=0),0,MAX(F14,H14*J14))</f>
+        <v/>
+      </c>
+      <c r="L14" s="6">
+        <f>IF(AND(E14=0,F14=0),0,MAX(F14,I14*MIN(J14,1)))</f>
+        <v/>
+      </c>
+      <c r="M14" s="6">
+        <f>E14+K14</f>
+        <v/>
+      </c>
+      <c r="N14" s="6">
+        <f>E14+L14</f>
+        <v/>
+      </c>
+      <c r="O14" s="6">
+        <f>E14*12/9</f>
+        <v/>
+      </c>
+      <c r="P14" s="6">
+        <f>M14-O14</f>
+        <v/>
+      </c>
+      <c r="Q14" s="7">
+        <f>IF(D14=0,"",M14/D14-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>1421909</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>جمع النفايات</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>72842923.63</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>71391993.31</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>831524.83</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>53175299.26</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>20735771.87</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>18851086.09</v>
+      </c>
+      <c r="J15" s="15">
+        <f>IF(G15&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E15/G15)),IF(E15&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K15" s="6">
+        <f>IF(AND(E15=0,F15=0),0,MAX(F15,H15*J15))</f>
+        <v/>
+      </c>
+      <c r="L15" s="6">
+        <f>IF(AND(E15=0,F15=0),0,MAX(F15,I15*MIN(J15,1)))</f>
+        <v/>
+      </c>
+      <c r="M15" s="6">
+        <f>E15+K15</f>
+        <v/>
+      </c>
+      <c r="N15" s="6">
+        <f>E15+L15</f>
+        <v/>
+      </c>
+      <c r="O15" s="6">
+        <f>E15*12/9</f>
+        <v/>
+      </c>
+      <c r="P15" s="6">
+        <f>M15-O15</f>
+        <v/>
+      </c>
+      <c r="Q15" s="7">
+        <f>IF(D15=0,"",M15/D15-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>1421911</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>رسم مبيعات محلات تقديم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>67630101.28</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>56321815.11</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>349894.61</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>52213518.92</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>19979808.95</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>15416582.36</v>
+      </c>
+      <c r="J16" s="15">
+        <f>IF(G16&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E16/G16)),IF(E16&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K16" s="6">
+        <f>IF(AND(E16=0,F16=0),0,MAX(F16,H16*J16))</f>
+        <v/>
+      </c>
+      <c r="L16" s="6">
+        <f>IF(AND(E16=0,F16=0),0,MAX(F16,I16*MIN(J16,1)))</f>
+        <v/>
+      </c>
+      <c r="M16" s="6">
+        <f>E16+K16</f>
+        <v/>
+      </c>
+      <c r="N16" s="6">
+        <f>E16+L16</f>
+        <v/>
+      </c>
+      <c r="O16" s="6">
+        <f>E16*12/9</f>
+        <v/>
+      </c>
+      <c r="P16" s="6">
+        <f>M16-O16</f>
+        <v/>
+      </c>
+      <c r="Q16" s="7">
+        <f>IF(D16=0,"",M16/D16-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>11452108</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>ايراد اصدار القرارات المساحية - أمانة منطقة الرياض</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>24531493.81</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>30875269.78</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>303578.42</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>13801001.77</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>5538696.05</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>1955277.89</v>
+      </c>
+      <c r="J17" s="15">
+        <f>IF(G17&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E17/G17)),IF(E17&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K17" s="6">
+        <f>IF(AND(E17=0,F17=0),0,MAX(F17,H17*J17))</f>
+        <v/>
+      </c>
+      <c r="L17" s="6">
+        <f>IF(AND(E17=0,F17=0),0,MAX(F17,I17*MIN(J17,1)))</f>
+        <v/>
+      </c>
+      <c r="M17" s="6">
+        <f>E17+K17</f>
+        <v/>
+      </c>
+      <c r="N17" s="6">
+        <f>E17+L17</f>
+        <v/>
+      </c>
+      <c r="O17" s="6">
+        <f>E17*12/9</f>
+        <v/>
+      </c>
+      <c r="P17" s="6">
+        <f>M17-O17</f>
+        <v/>
+      </c>
+      <c r="Q17" s="7">
+        <f>IF(D17=0,"",M17/D17-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>1422108</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>الشهادات الصحية</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>26098550.07</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>17590070.76</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>11040</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>14304003.57</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>6463060.62</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>3446940.2</v>
+      </c>
+      <c r="J18" s="15">
+        <f>IF(G18&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E18/G18)),IF(E18&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K18" s="6">
+        <f>IF(AND(E18=0,F18=0),0,MAX(F18,H18*J18))</f>
+        <v/>
+      </c>
+      <c r="L18" s="6">
+        <f>IF(AND(E18=0,F18=0),0,MAX(F18,I18*MIN(J18,1)))</f>
+        <v/>
+      </c>
+      <c r="M18" s="6">
+        <f>E18+K18</f>
+        <v/>
+      </c>
+      <c r="N18" s="6">
+        <f>E18+L18</f>
+        <v/>
+      </c>
+      <c r="O18" s="6">
+        <f>E18*12/9</f>
+        <v/>
+      </c>
+      <c r="P18" s="6">
+        <f>M18-O18</f>
+        <v/>
+      </c>
+      <c r="Q18" s="7">
+        <f>IF(D18=0,"",M18/D18-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>144122</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  متنوعه</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>2477531.42</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>20815252.14</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>6262033.26</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>645234.08</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>424550.96</v>
+      </c>
+      <c r="J19" s="15">
+        <f>IF(G19&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E19/G19)),IF(E19&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K19" s="6">
+        <f>IF(AND(E19=0,F19=0),0,MAX(F19,H19*J19))</f>
+        <v/>
+      </c>
+      <c r="L19" s="6">
+        <f>IF(AND(E19=0,F19=0),0,MAX(F19,I19*MIN(J19,1)))</f>
+        <v/>
+      </c>
+      <c r="M19" s="6">
+        <f>E19+K19</f>
+        <v/>
+      </c>
+      <c r="N19" s="6">
+        <f>E19+L19</f>
+        <v/>
+      </c>
+      <c r="O19" s="6">
+        <f>E19*12/9</f>
+        <v/>
+      </c>
+      <c r="P19" s="6">
+        <f>M19-O19</f>
+        <v/>
+      </c>
+      <c r="Q19" s="7">
+        <f>IF(D19=0,"",M19/D19-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>1422121</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>رسم ترخيص نشاط تقديم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>15681460.95</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>13771650.67</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>125000</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>12013210.95</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>4845000</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>3668250</v>
+      </c>
+      <c r="J20" s="15">
+        <f>IF(G20&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E20/G20)),IF(E20&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K20" s="6">
+        <f>IF(AND(E20=0,F20=0),0,MAX(F20,H20*J20))</f>
+        <v/>
+      </c>
+      <c r="L20" s="6">
+        <f>IF(AND(E20=0,F20=0),0,MAX(F20,I20*MIN(J20,1)))</f>
+        <v/>
+      </c>
+      <c r="M20" s="6">
+        <f>E20+K20</f>
+        <v/>
+      </c>
+      <c r="N20" s="6">
+        <f>E20+L20</f>
+        <v/>
+      </c>
+      <c r="O20" s="6">
+        <f>E20*12/9</f>
+        <v/>
+      </c>
+      <c r="P20" s="6">
+        <f>M20-O20</f>
+        <v/>
+      </c>
+      <c r="Q20" s="7">
+        <f>IF(D20=0,"",M20/D20-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>11452111</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>المقابل المالي للسماح للأنشطة التجارية بالعمل (24) ساعة</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>5751371.82</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>11268803.9</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>140954.87</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>3875508.86</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>1330182.55</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>1291181.74</v>
+      </c>
+      <c r="J21" s="15">
+        <f>IF(G21&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E21/G21)),IF(E21&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K21" s="6">
+        <f>IF(AND(E21=0,F21=0),0,MAX(F21,H21*J21))</f>
+        <v/>
+      </c>
+      <c r="L21" s="6">
+        <f>IF(AND(E21=0,F21=0),0,MAX(F21,I21*MIN(J21,1)))</f>
+        <v/>
+      </c>
+      <c r="M21" s="6">
+        <f>E21+K21</f>
+        <v/>
+      </c>
+      <c r="N21" s="6">
+        <f>E21+L21</f>
+        <v/>
+      </c>
+      <c r="O21" s="6">
+        <f>E21*12/9</f>
+        <v/>
+      </c>
+      <c r="P21" s="6">
+        <f>M21-O21</f>
+        <v/>
+      </c>
+      <c r="Q21" s="7">
+        <f>IF(D21=0,"",M21/D21-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>142163</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  تأجير مباني تجارية</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>3001651.75</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>10169478.26</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>3878992</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>1555970</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>1460514</v>
+      </c>
+      <c r="J22" s="15">
+        <f>IF(G22&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E22/G22)),IF(E22&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K22" s="6">
+        <f>IF(AND(E22=0,F22=0),0,MAX(F22,H22*J22))</f>
+        <v/>
+      </c>
+      <c r="L22" s="6">
+        <f>IF(AND(E22=0,F22=0),0,MAX(F22,I22*MIN(J22,1)))</f>
+        <v/>
+      </c>
+      <c r="M22" s="6">
+        <f>E22+K22</f>
+        <v/>
+      </c>
+      <c r="N22" s="6">
+        <f>E22+L22</f>
+        <v/>
+      </c>
+      <c r="O22" s="6">
+        <f>E22*12/9</f>
+        <v/>
+      </c>
+      <c r="P22" s="6">
+        <f>M22-O22</f>
+        <v/>
+      </c>
+      <c r="Q22" s="7">
+        <f>IF(D22=0,"",M22/D22-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>1422109</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  الكشفية</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>7132142.91</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>5653796.45</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>69357</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>6844995.41</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>2070998.8</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>1949868</v>
+      </c>
+      <c r="J23" s="15">
+        <f>IF(G23&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E23/G23)),IF(E23&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K23" s="6">
+        <f>IF(AND(E23=0,F23=0),0,MAX(F23,H23*J23))</f>
+        <v/>
+      </c>
+      <c r="L23" s="6">
+        <f>IF(AND(E23=0,F23=0),0,MAX(F23,I23*MIN(J23,1)))</f>
+        <v/>
+      </c>
+      <c r="M23" s="6">
+        <f>E23+K23</f>
+        <v/>
+      </c>
+      <c r="N23" s="6">
+        <f>E23+L23</f>
+        <v/>
+      </c>
+      <c r="O23" s="6">
+        <f>E23*12/9</f>
+        <v/>
+      </c>
+      <c r="P23" s="6">
+        <f>M23-O23</f>
+        <v/>
+      </c>
+      <c r="Q23" s="7">
+        <f>IF(D23=0,"",M23/D23-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>1421910</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>اصدار تراخيص اشغال الارصفة العامة و الطرق</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>3477675.2</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>3539388.27</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>25542.8</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>2228519.26</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>923715.59</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>753099.16</v>
+      </c>
+      <c r="J24" s="15">
+        <f>IF(G24&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E24/G24)),IF(E24&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K24" s="6">
+        <f>IF(AND(E24=0,F24=0),0,MAX(F24,H24*J24))</f>
+        <v/>
+      </c>
+      <c r="L24" s="6">
+        <f>IF(AND(E24=0,F24=0),0,MAX(F24,I24*MIN(J24,1)))</f>
+        <v/>
+      </c>
+      <c r="M24" s="6">
+        <f>E24+K24</f>
+        <v/>
+      </c>
+      <c r="N24" s="6">
+        <f>E24+L24</f>
+        <v/>
+      </c>
+      <c r="O24" s="6">
+        <f>E24*12/9</f>
+        <v/>
+      </c>
+      <c r="P24" s="6">
+        <f>M24-O24</f>
+        <v/>
+      </c>
+      <c r="Q24" s="7">
+        <f>IF(D24=0,"",M24/D24-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>بدون رقم</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>بدون رقم (خدمات علم + جزاءات)</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>علم</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>21814890</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>1732017.5</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>390906.25</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>9460985</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>4795561.25</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>1566843.75</v>
+      </c>
+      <c r="J25" s="15">
+        <f>IF(G25&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E25/G25)),IF(E25&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K25" s="6">
+        <f>IF(AND(E25=0,F25=0),0,MAX(F25,H25*J25))</f>
+        <v/>
+      </c>
+      <c r="L25" s="6">
+        <f>IF(AND(E25=0,F25=0),0,MAX(F25,I25*MIN(J25,1)))</f>
+        <v/>
+      </c>
+      <c r="M25" s="6">
+        <f>E25+K25</f>
+        <v/>
+      </c>
+      <c r="N25" s="6">
+        <f>E25+L25</f>
+        <v/>
+      </c>
+      <c r="O25" s="6">
+        <f>E25*12/9</f>
+        <v/>
+      </c>
+      <c r="P25" s="6">
+        <f>M25-O25</f>
+        <v/>
+      </c>
+      <c r="Q25" s="7">
+        <f>IF(D25=0,"",M25/D25-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>11452105</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>رسوم تراخيص حفر الشوارع</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>590915.4300000001</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>1350</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>48367971.36</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>6431057.76</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="15">
+        <f>IF(G26&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E26/G26)),IF(E26&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K26" s="6">
+        <f>IF(AND(E26=0,F26=0),0,MAX(F26,H26*J26))</f>
+        <v/>
+      </c>
+      <c r="L26" s="6">
+        <f>IF(AND(E26=0,F26=0),0,MAX(F26,I26*MIN(J26,1)))</f>
+        <v/>
+      </c>
+      <c r="M26" s="6">
+        <f>E26+K26</f>
+        <v/>
+      </c>
+      <c r="N26" s="6">
+        <f>E26+L26</f>
+        <v/>
+      </c>
+      <c r="O26" s="6">
+        <f>E26*12/9</f>
+        <v/>
+      </c>
+      <c r="P26" s="6">
+        <f>M26-O26</f>
+        <v/>
+      </c>
+      <c r="Q26" s="7">
+        <f>IF(D26=0,"",M26/D26-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>1421901</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>بيع الوثائق والأنظمة</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>2512377</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>1623637</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>2021695</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>714900</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>572900</v>
+      </c>
+      <c r="J27" s="15">
+        <f>IF(G27&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E27/G27)),IF(E27&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K27" s="6">
+        <f>IF(AND(E27=0,F27=0),0,MAX(F27,H27*J27))</f>
+        <v/>
+      </c>
+      <c r="L27" s="6">
+        <f>IF(AND(E27=0,F27=0),0,MAX(F27,I27*MIN(J27,1)))</f>
+        <v/>
+      </c>
+      <c r="M27" s="6">
+        <f>E27+K27</f>
+        <v/>
+      </c>
+      <c r="N27" s="6">
+        <f>E27+L27</f>
+        <v/>
+      </c>
+      <c r="O27" s="6">
+        <f>E27*12/9</f>
+        <v/>
+      </c>
+      <c r="P27" s="6">
+        <f>M27-O27</f>
+        <v/>
+      </c>
+      <c r="Q27" s="7">
+        <f>IF(D27=0,"",M27/D27-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>1421912</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>تأجير العقارات لأغراض مؤقته</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>2454143.51</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>1357611.55</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>1482330.88</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>561509.62</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>385234.73</v>
+      </c>
+      <c r="J28" s="15">
+        <f>IF(G28&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E28/G28)),IF(E28&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K28" s="6">
+        <f>IF(AND(E28=0,F28=0),0,MAX(F28,H28*J28))</f>
+        <v/>
+      </c>
+      <c r="L28" s="6">
+        <f>IF(AND(E28=0,F28=0),0,MAX(F28,I28*MIN(J28,1)))</f>
+        <v/>
+      </c>
+      <c r="M28" s="6">
+        <f>E28+K28</f>
+        <v/>
+      </c>
+      <c r="N28" s="6">
+        <f>E28+L28</f>
+        <v/>
+      </c>
+      <c r="O28" s="6">
+        <f>E28*12/9</f>
+        <v/>
+      </c>
+      <c r="P28" s="6">
+        <f>M28-O28</f>
+        <v/>
+      </c>
+      <c r="Q28" s="7">
+        <f>IF(D28=0,"",M28/D28-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>11452110</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>إصدار تراخيص إستخدام أملاك خاصة لإقامة فعاليات</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>809215.9</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>582595.83</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>11591.94</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>575291.9399999999</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>218168.33</v>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>198007.98</v>
+      </c>
+      <c r="J29" s="15">
+        <f>IF(G29&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E29/G29)),IF(E29&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K29" s="6">
+        <f>IF(AND(E29=0,F29=0),0,MAX(F29,H29*J29))</f>
+        <v/>
+      </c>
+      <c r="L29" s="6">
+        <f>IF(AND(E29=0,F29=0),0,MAX(F29,I29*MIN(J29,1)))</f>
+        <v/>
+      </c>
+      <c r="M29" s="6">
+        <f>E29+K29</f>
+        <v/>
+      </c>
+      <c r="N29" s="6">
+        <f>E29+L29</f>
+        <v/>
+      </c>
+      <c r="O29" s="6">
+        <f>E29*12/9</f>
+        <v/>
+      </c>
+      <c r="P29" s="6">
+        <f>M29-O29</f>
+        <v/>
+      </c>
+      <c r="Q29" s="7">
+        <f>IF(D29=0,"",M29/D29-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>11452106</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>اصدار التراخيص بتأسيس أو تشغيل ابراج الاتصالات</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>1275300</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>342700</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>721300</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>458800</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>423100</v>
+      </c>
+      <c r="J30" s="15">
+        <f>IF(G30&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E30/G30)),IF(E30&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K30" s="6">
+        <f>IF(AND(E30=0,F30=0),0,MAX(F30,H30*J30))</f>
+        <v/>
+      </c>
+      <c r="L30" s="6">
+        <f>IF(AND(E30=0,F30=0),0,MAX(F30,I30*MIN(J30,1)))</f>
+        <v/>
+      </c>
+      <c r="M30" s="6">
+        <f>E30+K30</f>
+        <v/>
+      </c>
+      <c r="N30" s="6">
+        <f>E30+L30</f>
+        <v/>
+      </c>
+      <c r="O30" s="6">
+        <f>E30*12/9</f>
+        <v/>
+      </c>
+      <c r="P30" s="6">
+        <f>M30-O30</f>
+        <v/>
+      </c>
+      <c r="Q30" s="7">
+        <f>IF(D30=0,"",M30/D30-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>1421903</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>مبيعات التيار الكهربائي</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>1464687.1</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>274868.65</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="15">
+        <f>IF(G31&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E31/G31)),IF(E31&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K31" s="6">
+        <f>IF(AND(E31=0,F31=0),0,MAX(F31,H31*J31))</f>
+        <v/>
+      </c>
+      <c r="L31" s="6">
+        <f>IF(AND(E31=0,F31=0),0,MAX(F31,I31*MIN(J31,1)))</f>
+        <v/>
+      </c>
+      <c r="M31" s="6">
+        <f>E31+K31</f>
+        <v/>
+      </c>
+      <c r="N31" s="6">
+        <f>E31+L31</f>
+        <v/>
+      </c>
+      <c r="O31" s="6">
+        <f>E31*12/9</f>
+        <v/>
+      </c>
+      <c r="P31" s="6">
+        <f>M31-O31</f>
+        <v/>
+      </c>
+      <c r="Q31" s="7">
+        <f>IF(D31=0,"",M31/D31-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>1439</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  مبيعات  ناتجه من النشاط غير مصنفة</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>8503508</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>183000</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>1497100</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>144348</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>14000</v>
+      </c>
+      <c r="J32" s="15">
+        <f>IF(G32&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E32/G32)),IF(E32&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K32" s="6">
+        <f>IF(AND(E32=0,F32=0),0,MAX(F32,H32*J32))</f>
+        <v/>
+      </c>
+      <c r="L32" s="6">
+        <f>IF(AND(E32=0,F32=0),0,MAX(F32,I32*MIN(J32,1)))</f>
+        <v/>
+      </c>
+      <c r="M32" s="6">
+        <f>E32+K32</f>
+        <v/>
+      </c>
+      <c r="N32" s="6">
+        <f>E32+L32</f>
+        <v/>
+      </c>
+      <c r="O32" s="6">
+        <f>E32*12/9</f>
+        <v/>
+      </c>
+      <c r="P32" s="6">
+        <f>M32-O32</f>
+        <v/>
+      </c>
+      <c r="Q32" s="7">
+        <f>IF(D32=0,"",M32/D32-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>11452109</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>اعتماد مخططات التطوير العقاري</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>591946.73</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>100</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>481600.81</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>458948.18</v>
+      </c>
+      <c r="I33" s="6" t="n">
+        <v>110345.92</v>
+      </c>
+      <c r="J33" s="15">
+        <f>IF(G33&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E33/G33)),IF(E33&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K33" s="6">
+        <f>IF(AND(E33=0,F33=0),0,MAX(F33,H33*J33))</f>
+        <v/>
+      </c>
+      <c r="L33" s="6">
+        <f>IF(AND(E33=0,F33=0),0,MAX(F33,I33*MIN(J33,1)))</f>
+        <v/>
+      </c>
+      <c r="M33" s="6">
+        <f>E33+K33</f>
+        <v/>
+      </c>
+      <c r="N33" s="6">
+        <f>E33+L33</f>
+        <v/>
+      </c>
+      <c r="O33" s="6">
+        <f>E33*12/9</f>
+        <v/>
+      </c>
+      <c r="P33" s="6">
+        <f>M33-O33</f>
+        <v/>
+      </c>
+      <c r="Q33" s="7">
+        <f>IF(D33=0,"",M33/D33-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>11452107</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>اصدار التراخيص بتأسيس أو تشغيل الصراف الآلي</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>229800</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>142784.61</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>16150</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>35000</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>49300</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>19000</v>
+      </c>
+      <c r="J34" s="15">
+        <f>IF(G34&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E34/G34)),IF(E34&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K34" s="6">
+        <f>IF(AND(E34=0,F34=0),0,MAX(F34,H34*J34))</f>
+        <v/>
+      </c>
+      <c r="L34" s="6">
+        <f>IF(AND(E34=0,F34=0),0,MAX(F34,I34*MIN(J34,1)))</f>
+        <v/>
+      </c>
+      <c r="M34" s="6">
+        <f>E34+K34</f>
+        <v/>
+      </c>
+      <c r="N34" s="6">
+        <f>E34+L34</f>
+        <v/>
+      </c>
+      <c r="O34" s="6">
+        <f>E34*12/9</f>
+        <v/>
+      </c>
+      <c r="P34" s="6">
+        <f>M34-O34</f>
+        <v/>
+      </c>
+      <c r="Q34" s="7">
+        <f>IF(D34=0,"",M34/D34-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>3318212</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>مرتجع رواتب - فواتير</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>152767.79</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>216725.66</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="15">
+        <f>IF(G35&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E35/G35)),IF(E35&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K35" s="6">
+        <f>IF(AND(E35=0,F35=0),0,MAX(F35,H35*J35))</f>
+        <v/>
+      </c>
+      <c r="L35" s="6">
+        <f>IF(AND(E35=0,F35=0),0,MAX(F35,I35*MIN(J35,1)))</f>
+        <v/>
+      </c>
+      <c r="M35" s="6">
+        <f>E35+K35</f>
+        <v/>
+      </c>
+      <c r="N35" s="6">
+        <f>E35+L35</f>
+        <v/>
+      </c>
+      <c r="O35" s="6">
+        <f>E35*12/9</f>
+        <v/>
+      </c>
+      <c r="P35" s="6">
+        <f>M35-O35</f>
+        <v/>
+      </c>
+      <c r="Q35" s="7">
+        <f>IF(D35=0,"",M35/D35-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>141229</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>أرباح أخرى</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>60000</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>80000</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>70000</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="15">
+        <f>IF(G36&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E36/G36)),IF(E36&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K36" s="6">
+        <f>IF(AND(E36=0,F36=0),0,MAX(F36,H36*J36))</f>
+        <v/>
+      </c>
+      <c r="L36" s="6">
+        <f>IF(AND(E36=0,F36=0),0,MAX(F36,I36*MIN(J36,1)))</f>
+        <v/>
+      </c>
+      <c r="M36" s="6">
+        <f>E36+K36</f>
+        <v/>
+      </c>
+      <c r="N36" s="6">
+        <f>E36+L36</f>
+        <v/>
+      </c>
+      <c r="O36" s="6">
+        <f>E36*12/9</f>
+        <v/>
+      </c>
+      <c r="P36" s="6">
+        <f>M36-O36</f>
+        <v/>
+      </c>
+      <c r="Q36" s="7">
+        <f>IF(D36=0,"",M36/D36-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>1438</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات مفروضة بموجب أنظمة الجهة</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>352900</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>59500</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>368600</v>
+      </c>
+      <c r="H37" s="6" t="n">
+        <v>81100</v>
+      </c>
+      <c r="I37" s="6" t="n">
+        <v>56700</v>
+      </c>
+      <c r="J37" s="15">
+        <f>IF(G37&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E37/G37)),IF(E37&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K37" s="6">
+        <f>IF(AND(E37=0,F37=0),0,MAX(F37,H37*J37))</f>
+        <v/>
+      </c>
+      <c r="L37" s="6">
+        <f>IF(AND(E37=0,F37=0),0,MAX(F37,I37*MIN(J37,1)))</f>
+        <v/>
+      </c>
+      <c r="M37" s="6">
+        <f>E37+K37</f>
+        <v/>
+      </c>
+      <c r="N37" s="6">
+        <f>E37+L37</f>
+        <v/>
+      </c>
+      <c r="O37" s="6">
+        <f>E37*12/9</f>
+        <v/>
+      </c>
+      <c r="P37" s="6">
+        <f>M37-O37</f>
+        <v/>
+      </c>
+      <c r="Q37" s="7">
+        <f>IF(D37=0,"",M37/D37-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>1421907</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات المخططات</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>20650</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>5550</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="15">
+        <f>IF(G38&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E38/G38)),IF(E38&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K38" s="6">
+        <f>IF(AND(E38=0,F38=0),0,MAX(F38,H38*J38))</f>
+        <v/>
+      </c>
+      <c r="L38" s="6">
+        <f>IF(AND(E38=0,F38=0),0,MAX(F38,I38*MIN(J38,1)))</f>
+        <v/>
+      </c>
+      <c r="M38" s="6">
+        <f>E38+K38</f>
+        <v/>
+      </c>
+      <c r="N38" s="6">
+        <f>E38+L38</f>
+        <v/>
+      </c>
+      <c r="O38" s="6">
+        <f>E38*12/9</f>
+        <v/>
+      </c>
+      <c r="P38" s="6">
+        <f>M38-O38</f>
+        <v/>
+      </c>
+      <c r="Q38" s="7">
+        <f>IF(D38=0,"",M38/D38-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>11452513</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>لوحات إرشـادية</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>9000</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>600</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>9475</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>3400</v>
+      </c>
+      <c r="I39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="15">
+        <f>IF(G39&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E39/G39)),IF(E39&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K39" s="6">
+        <f>IF(AND(E39=0,F39=0),0,MAX(F39,H39*J39))</f>
+        <v/>
+      </c>
+      <c r="L39" s="6">
+        <f>IF(AND(E39=0,F39=0),0,MAX(F39,I39*MIN(J39,1)))</f>
+        <v/>
+      </c>
+      <c r="M39" s="6">
+        <f>E39+K39</f>
+        <v/>
+      </c>
+      <c r="N39" s="6">
+        <f>E39+L39</f>
+        <v/>
+      </c>
+      <c r="O39" s="6">
+        <f>E39*12/9</f>
+        <v/>
+      </c>
+      <c r="P39" s="6">
+        <f>M39-O39</f>
+        <v/>
+      </c>
+      <c r="Q39" s="7">
+        <f>IF(D39=0,"",M39/D39-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>1422103</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>تراخيص المحلات</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>1603.2</v>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>432</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>10275.6</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>2091.6</v>
+      </c>
+      <c r="I40" s="6" t="n">
+        <v>528</v>
+      </c>
+      <c r="J40" s="15">
+        <f>IF(G40&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E40/G40)),IF(E40&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K40" s="6">
+        <f>IF(AND(E40=0,F40=0),0,MAX(F40,H40*J40))</f>
+        <v/>
+      </c>
+      <c r="L40" s="6">
+        <f>IF(AND(E40=0,F40=0),0,MAX(F40,I40*MIN(J40,1)))</f>
+        <v/>
+      </c>
+      <c r="M40" s="6">
+        <f>E40+K40</f>
+        <v/>
+      </c>
+      <c r="N40" s="6">
+        <f>E40+L40</f>
+        <v/>
+      </c>
+      <c r="O40" s="6">
+        <f>E40*12/9</f>
+        <v/>
+      </c>
+      <c r="P40" s="6">
+        <f>M40-O40</f>
+        <v/>
+      </c>
+      <c r="Q40" s="7">
+        <f>IF(D40=0,"",M40/D40-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>11422</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>رسوم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>27000</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v>27000</v>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="15">
+        <f>IF(G41&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E41/G41)),IF(E41&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K41" s="6">
+        <f>IF(AND(E41=0,F41=0),0,MAX(F41,H41*J41))</f>
+        <v/>
+      </c>
+      <c r="L41" s="6">
+        <f>IF(AND(E41=0,F41=0),0,MAX(F41,I41*MIN(J41,1)))</f>
+        <v/>
+      </c>
+      <c r="M41" s="6">
+        <f>E41+K41</f>
+        <v/>
+      </c>
+      <c r="N41" s="6">
+        <f>E41+L41</f>
+        <v/>
+      </c>
+      <c r="O41" s="6">
+        <f>E41*12/9</f>
+        <v/>
+      </c>
+      <c r="P41" s="6">
+        <f>M41-O41</f>
+        <v/>
+      </c>
+      <c r="Q41" s="7">
+        <f>IF(D41=0,"",M41/D41-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>142161</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>تاجير مباني سكنية</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J42" s="15">
+        <f>IF(G42&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E42/G42)),IF(E42&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K42" s="6">
+        <f>IF(AND(E42=0,F42=0),0,MAX(F42,H42*J42))</f>
+        <v/>
+      </c>
+      <c r="L42" s="6">
+        <f>IF(AND(E42=0,F42=0),0,MAX(F42,I42*MIN(J42,1)))</f>
+        <v/>
+      </c>
+      <c r="M42" s="6">
+        <f>E42+K42</f>
+        <v/>
+      </c>
+      <c r="N42" s="6">
+        <f>E42+L42</f>
+        <v/>
+      </c>
+      <c r="O42" s="6">
+        <f>E42*12/9</f>
+        <v/>
+      </c>
+      <c r="P42" s="6">
+        <f>M42-O42</f>
+        <v/>
+      </c>
+      <c r="Q42" s="7">
+        <f>IF(D42=0,"",M42/D42-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>1421908</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  رسوم خدمات  بلدية</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J43" s="15">
+        <f>IF(G43&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E43/G43)),IF(E43&gt;0,1,0))</f>
+        <v/>
+      </c>
+      <c r="K43" s="6">
+        <f>IF(AND(E43=0,F43=0),0,MAX(F43,H43*J43))</f>
+        <v/>
+      </c>
+      <c r="L43" s="6">
+        <f>IF(AND(E43=0,F43=0),0,MAX(F43,I43*MIN(J43,1)))</f>
+        <v/>
+      </c>
+      <c r="M43" s="6">
+        <f>E43+K43</f>
+        <v/>
+      </c>
+      <c r="N43" s="6">
+        <f>E43+L43</f>
+        <v/>
+      </c>
+      <c r="O43" s="6">
+        <f>E43*12/9</f>
+        <v/>
+      </c>
+      <c r="P43" s="6">
+        <f>M43-O43</f>
+        <v/>
+      </c>
+      <c r="Q43" s="7">
+        <f>IF(D43=0,"",M43/D43-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="n"/>
+      <c r="B44" s="8" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="n"/>
+      <c r="D44" s="9">
+        <f>SUM(D6:D43)</f>
+        <v/>
+      </c>
+      <c r="E44" s="9">
+        <f>SUM(E6:E43)</f>
+        <v/>
+      </c>
+      <c r="F44" s="9">
+        <f>SUM(F6:F43)</f>
+        <v/>
+      </c>
+      <c r="G44" s="9">
+        <f>SUM(G6:G43)</f>
+        <v/>
+      </c>
+      <c r="H44" s="9">
+        <f>SUM(H6:H43)</f>
+        <v/>
+      </c>
+      <c r="I44" s="9">
+        <f>SUM(I6:I43)</f>
+        <v/>
+      </c>
+      <c r="J44" s="17" t="n"/>
+      <c r="K44" s="9">
+        <f>SUM(K6:K43)</f>
+        <v/>
+      </c>
+      <c r="L44" s="9">
+        <f>SUM(L6:L43)</f>
+        <v/>
+      </c>
+      <c r="M44" s="9">
+        <f>SUM(M6:M43)</f>
+        <v/>
+      </c>
+      <c r="N44" s="9">
+        <f>SUM(N6:N43)</f>
+        <v/>
+      </c>
+      <c r="O44" s="9">
+        <f>SUM(O6:O43)</f>
+        <v/>
+      </c>
+      <c r="P44" s="9">
+        <f>SUM(P6:P43)</f>
+        <v/>
+      </c>
+      <c r="Q44" s="10">
+        <f>M44/D44-1</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:Q43"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:Q2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>المحصل الشهري الإجمالي (بدون الضريبة) وحصة كل شهر من السنة</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="11" t="inlineStr">
+        <is>
+          <t>2026: أكتوبر جزئي (حتى تاريخ الملف) ونوفمبر وديسمبر لم يحصلا بعد. شهور الذروة الاستثنائية: يوليو 2024 (اللوحات الدعائية 327م)، مايو 2025 (اللوحات الدعائية 297م)، نوفمبر 2025 (اللوحات الدعائية 598م)، يونيو 2026 (تأجير المرافق 411م).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>السنة</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>يناير</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>فبراير</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>مارس</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>أبريل</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>مايو</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>يونيو</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>يوليو</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>أغسطس</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>سبتمبر</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>أكتوبر</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>نوفمبر</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>ديسمبر</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>حتى سبتمبر %</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>الربع الأخير %</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>242718868.41</v>
+      </c>
+      <c r="C5" s="6" t="n">
+        <v>190226377.07</v>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>213693456.41</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>137496184.37</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>266781046.33</v>
+      </c>
+      <c r="G5" s="6" t="n">
+        <v>188980723.96</v>
+      </c>
+      <c r="H5" s="6" t="n">
+        <v>258110558.94</v>
+      </c>
+      <c r="I5" s="6" t="n">
+        <v>245222659.07</v>
+      </c>
+      <c r="J5" s="6" t="n">
+        <v>292626592.68</v>
+      </c>
+      <c r="K5" s="6" t="n">
+        <v>276317474.25</v>
+      </c>
+      <c r="L5" s="6" t="n">
+        <v>208973805.2</v>
+      </c>
+      <c r="M5" s="6" t="n">
+        <v>237583121.26</v>
+      </c>
+      <c r="N5" s="6">
+        <f>SUM(B5:M5)</f>
+        <v/>
+      </c>
+      <c r="O5" s="7">
+        <f>SUM(B5:J5)/N5</f>
+        <v/>
+      </c>
+      <c r="P5" s="7">
+        <f>SUM(K5:M5)/N5</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>263609897.85</v>
+      </c>
+      <c r="C6" s="6" t="n">
+        <v>225837848.51</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>167125292.76</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>140041282.92</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>224669391</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>206451120.97</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>537484963.7</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>219147762.67</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>213778511.29</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>339436921.05</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>292043473.43</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>363081833.61</v>
+      </c>
+      <c r="N6" s="6">
+        <f>SUM(B6:M6)</f>
+        <v/>
+      </c>
+      <c r="O6" s="7">
+        <f>SUM(B6:J6)/N6</f>
+        <v/>
+      </c>
+      <c r="P6" s="7">
+        <f>SUM(K6:M6)/N6</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B7" s="6" t="n">
+        <v>244629044.59</v>
+      </c>
+      <c r="C7" s="6" t="n">
+        <v>199160331.37</v>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>174627126.68</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>140777046.53</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>484593226.12</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>174638216.96</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>220552646.75</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>178058904.15</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>206613498.77</v>
+      </c>
+      <c r="K7" s="6" t="n">
+        <v>201047125.39</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>842726974.04</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>242119497.64</v>
+      </c>
+      <c r="N7" s="6">
+        <f>SUM(B7:M7)</f>
+        <v/>
+      </c>
+      <c r="O7" s="7">
+        <f>SUM(B7:J7)/N7</f>
+        <v/>
+      </c>
+      <c r="P7" s="7">
+        <f>SUM(K7:M7)/N7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="n">
+        <v>2026</v>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>229262544.24</v>
+      </c>
+      <c r="C8" s="6" t="n">
+        <v>277622602.8</v>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>166305951.68</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>263289781.16</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>251847021.46</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>712125842.35</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>271746820.91</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>256930480.94</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>244363872.65</v>
+      </c>
+      <c r="K8" s="6" t="n">
+        <v>10145046.31</v>
+      </c>
+      <c r="L8" s="6" t="n"/>
+      <c r="M8" s="6" t="n"/>
+      <c r="N8" s="6">
+        <f>SUM(B8:M8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="7" t="n"/>
+      <c r="P8" s="7" t="n"/>
+    </row>
+    <row r="9"/>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>حصة الشهر من السنة %</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="inlineStr">
+        <is>
+          <t>يناير</t>
+        </is>
+      </c>
+      <c r="C10" s="4" t="inlineStr">
+        <is>
+          <t>فبراير</t>
+        </is>
+      </c>
+      <c r="D10" s="4" t="inlineStr">
+        <is>
+          <t>مارس</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>أبريل</t>
+        </is>
+      </c>
+      <c r="F10" s="4" t="inlineStr">
+        <is>
+          <t>مايو</t>
+        </is>
+      </c>
+      <c r="G10" s="4" t="inlineStr">
+        <is>
+          <t>يونيو</t>
+        </is>
+      </c>
+      <c r="H10" s="4" t="inlineStr">
+        <is>
+          <t>يوليو</t>
+        </is>
+      </c>
+      <c r="I10" s="4" t="inlineStr">
+        <is>
+          <t>أغسطس</t>
+        </is>
+      </c>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>سبتمبر</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>أكتوبر</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>نوفمبر</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>ديسمبر</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="n">
+        <v>2023</v>
+      </c>
+      <c r="B11" s="7">
+        <f>B5/$N5</f>
+        <v/>
+      </c>
+      <c r="C11" s="7">
+        <f>C5/$N5</f>
+        <v/>
+      </c>
+      <c r="D11" s="7">
+        <f>D5/$N5</f>
+        <v/>
+      </c>
+      <c r="E11" s="7">
+        <f>E5/$N5</f>
+        <v/>
+      </c>
+      <c r="F11" s="7">
+        <f>F5/$N5</f>
+        <v/>
+      </c>
+      <c r="G11" s="7">
+        <f>G5/$N5</f>
+        <v/>
+      </c>
+      <c r="H11" s="7">
+        <f>H5/$N5</f>
+        <v/>
+      </c>
+      <c r="I11" s="7">
+        <f>I5/$N5</f>
+        <v/>
+      </c>
+      <c r="J11" s="7">
+        <f>J5/$N5</f>
+        <v/>
+      </c>
+      <c r="K11" s="7">
+        <f>K5/$N5</f>
+        <v/>
+      </c>
+      <c r="L11" s="7">
+        <f>L5/$N5</f>
+        <v/>
+      </c>
+      <c r="M11" s="7">
+        <f>M5/$N5</f>
+        <v/>
+      </c>
+      <c r="N11" s="7" t="n"/>
+      <c r="O11" s="7" t="n"/>
+      <c r="P11" s="7" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="n">
+        <v>2024</v>
+      </c>
+      <c r="B12" s="7">
+        <f>B6/$N6</f>
+        <v/>
+      </c>
+      <c r="C12" s="7">
+        <f>C6/$N6</f>
+        <v/>
+      </c>
+      <c r="D12" s="7">
+        <f>D6/$N6</f>
+        <v/>
+      </c>
+      <c r="E12" s="7">
+        <f>E6/$N6</f>
+        <v/>
+      </c>
+      <c r="F12" s="7">
+        <f>F6/$N6</f>
+        <v/>
+      </c>
+      <c r="G12" s="7">
+        <f>G6/$N6</f>
+        <v/>
+      </c>
+      <c r="H12" s="7">
+        <f>H6/$N6</f>
+        <v/>
+      </c>
+      <c r="I12" s="7">
+        <f>I6/$N6</f>
+        <v/>
+      </c>
+      <c r="J12" s="7">
+        <f>J6/$N6</f>
+        <v/>
+      </c>
+      <c r="K12" s="7">
+        <f>K6/$N6</f>
+        <v/>
+      </c>
+      <c r="L12" s="7">
+        <f>L6/$N6</f>
+        <v/>
+      </c>
+      <c r="M12" s="7">
+        <f>M6/$N6</f>
+        <v/>
+      </c>
+      <c r="N12" s="7" t="n"/>
+      <c r="O12" s="7" t="n"/>
+      <c r="P12" s="7" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="n">
+        <v>2025</v>
+      </c>
+      <c r="B13" s="7">
+        <f>B7/$N7</f>
+        <v/>
+      </c>
+      <c r="C13" s="7">
+        <f>C7/$N7</f>
+        <v/>
+      </c>
+      <c r="D13" s="7">
+        <f>D7/$N7</f>
+        <v/>
+      </c>
+      <c r="E13" s="7">
+        <f>E7/$N7</f>
+        <v/>
+      </c>
+      <c r="F13" s="7">
+        <f>F7/$N7</f>
+        <v/>
+      </c>
+      <c r="G13" s="7">
+        <f>G7/$N7</f>
+        <v/>
+      </c>
+      <c r="H13" s="7">
+        <f>H7/$N7</f>
+        <v/>
+      </c>
+      <c r="I13" s="7">
+        <f>I7/$N7</f>
+        <v/>
+      </c>
+      <c r="J13" s="7">
+        <f>J7/$N7</f>
+        <v/>
+      </c>
+      <c r="K13" s="7">
+        <f>K7/$N7</f>
+        <v/>
+      </c>
+      <c r="L13" s="7">
+        <f>L7/$N7</f>
+        <v/>
+      </c>
+      <c r="M13" s="7">
+        <f>M7/$N7</f>
+        <v/>
+      </c>
+      <c r="N13" s="7" t="n"/>
+      <c r="O13" s="7" t="n"/>
+      <c r="P13" s="7" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -10377,6 +13736,36 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>أدنى معامل اتجاه 2026 (توقع المحصل الموسمي)</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>يحدّ أثر انخفاض 2026 عن متوسط السنوات السابقة</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>أعلى معامل اتجاه 2026 (توقع المحصل الموسمي)</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>يحدّ أثر ارتفاع 2026 عن متوسط السنوات السابقة</t>
+        </is>
+      </c>
+    </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
@@ -10385,70 +13774,70 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="21" t="inlineStr">
+      <c r="A10" s="22" t="inlineStr">
         <is>
           <t>1) الإجمالي المفوتر للحساب = المفوتر + المحصل عن سنوات سابقة (حسب طلبك).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="21" t="inlineStr">
+      <c r="A11" s="22" t="inlineStr">
         <is>
           <t>2) توقع 2026 = الفعلي حتى سبتمبر × 12/9 (لا توجد بيانات شهرية، فلا موسمية في التوقع).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="21" t="inlineStr">
+      <c r="A12" s="22" t="inlineStr">
         <is>
           <t>3) الحسابات التي فوترتها وتحصيلها صفر في 2026 تُعتبر متوقفة وتوقعها صفر في 2026 و2027.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="21" t="inlineStr">
+      <c r="A13" s="22" t="inlineStr">
         <is>
           <t>4) 2027 – السيناريو الأول: توقع 2026 × (1 + نسبة النمو في خلية C2 بورقة التوقعات؛ الافتراضي 7%).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="21" t="inlineStr">
+      <c r="A14" s="22" t="inlineStr">
         <is>
           <t>5) 2027 – السيناريو الثاني: توقع 2026 × (1 + معدل النمو السنوي المركب التاريخي للحساب بين أول سنة فيها فوترة و2025، بسقف ±25%). إن توفرت سنة واحدة فقط من البيانات = نمو 0%.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="21" t="inlineStr">
+      <c r="A15" s="22" t="inlineStr">
         <is>
           <t>6) تم استبعاد حساب قيمة الضريبة المضافة (11411) من كل الحسابات والإجماليات.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="21" t="inlineStr">
+      <c r="A16" s="22" t="inlineStr">
         <is>
           <t>6b) تم دمج صفّي "بدون رقم" (خدمات علم + جزاءات، وجزاءات جزء ضئيل) في صف واحد لكل سنة.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="21" t="inlineStr">
+      <c r="A17" s="22" t="inlineStr">
         <is>
           <t>6c) أعمدة النمو لكل حساب: نمو كل سنة عن السنة السابقة (2024 عن 2023، 2025 عن 2024، 2026 توقع عن 2025، و2027 عن 2026 للسيناريوهين). تظهر فارغة عندما تكون السنة السابقة صفراً.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="21" t="inlineStr">
+      <c r="A18" s="22" t="inlineStr">
         <is>
           <t>6d) ورقة "توقع المحصل 2026": توقع إقفال 2026 كمحصّل فعلي = المحصل حتى سبتمبر × 12÷9 (مسدد عن السنة + محصل سنوات سابقة).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="21" t="inlineStr">
+      <c r="A19" s="22" t="inlineStr">
         <is>
           <t>7) تنبيه: كثير من الحسابات تتذبذب بشدة بين السنوات (لوحات دعائية، تأجير المرافق، إيرادات متنوعة)، ومضاعفة 2026 على 12/9 تضخّم أو تقلّل هذه الأرقام؛ انظر عمود "تنبيه".</t>
         </is>

</xml_diff>

<commit_message>
Reclassify 2025 facilities-rental collections out of advertising boards
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/توقع_الفوترة_2026_2027.xlsx
+++ b/توقع_الفوترة_2026_2027.xlsx
@@ -5521,7 +5521,7 @@
         <v>609523702.9299999</v>
       </c>
       <c r="G6" s="6" t="n">
-        <v>1016877058.52</v>
+        <v>103589976.04</v>
       </c>
       <c r="H6" s="6" t="n">
         <v>122031767.73</v>
@@ -5796,7 +5796,7 @@
         <v>45452213.03</v>
       </c>
       <c r="G11" s="6" t="n">
-        <v>25602601.22</v>
+        <v>938889683.7</v>
       </c>
       <c r="H11" s="6" t="n">
         <v>428460046</v>
@@ -7887,7 +7887,7 @@
       </c>
       <c r="O7" s="16" t="inlineStr">
         <is>
-          <t>تراجع حاد: المحصل حتى سبتمبر (122.0م) يعادل 12% فقط من 2025 (1,016.9م)؛ التوقع يستمر على هذا المستوى المنخفض.</t>
+          <t>قفزة: المحصل حتى سبتمبر (122.0م) يعادل 118% من كل 2025 (103.6م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
         </is>
       </c>
     </row>
@@ -8217,12 +8217,12 @@
       </c>
       <c r="N12" s="5" t="inlineStr">
         <is>
-          <t>مرتفع</t>
+          <t>منخفض</t>
         </is>
       </c>
       <c r="O12" s="16" t="inlineStr">
         <is>
-          <t>قفزة: المحصل حتى سبتمبر (428.5م) يعادل 1,674% من كل 2025 (25.6م)، والتوقع يفترض أن القفزة تستمر في الربع الأخير. احتمال المبالغة مرتفع.</t>
+          <t>التوقع أدنى من 2025 بنسبة 39% لأن وتيرة التحصيل حتى سبتمبر أقل.</t>
         </is>
       </c>
     </row>
@@ -10619,7 +10619,7 @@
         </is>
       </c>
       <c r="D8" s="6" t="n">
-        <v>25602601.22</v>
+        <v>938889683.7</v>
       </c>
       <c r="E8" s="6" t="n">
         <v>428454063.2</v>
@@ -10628,10 +10628,10 @@
         <v>5982.8</v>
       </c>
       <c r="G8" s="6" t="n">
-        <v>16504314.8</v>
+        <v>29251064.25</v>
       </c>
       <c r="H8" s="6" t="n">
-        <v>9098286.42</v>
+        <v>32592532.11</v>
       </c>
       <c r="I8" s="6" t="n">
         <v>322650</v>
@@ -10873,36 +10873,36 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>142113</t>
+          <t>11442</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t>ايرادات  اللوحات الدعائية</t>
+          <t>اشغال مرافق الايواء</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t>الرسوم والتراخيص</t>
+          <t>التبغ والإيواء</t>
         </is>
       </c>
       <c r="D12" s="6" t="n">
-        <v>1016877058.52</v>
+        <v>199149669.75</v>
       </c>
       <c r="E12" s="6" t="n">
-        <v>121704394.25</v>
+        <v>135824266.97</v>
       </c>
       <c r="F12" s="6" t="n">
-        <v>327373.48</v>
+        <v>815494.87</v>
       </c>
       <c r="G12" s="6" t="n">
-        <v>402775368.76</v>
+        <v>152968341.46</v>
       </c>
       <c r="H12" s="6" t="n">
-        <v>159604841.42</v>
+        <v>66937519.73</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>35149182.39</v>
+        <v>57302452.03</v>
       </c>
       <c r="J12" s="15">
         <f>IF(G12&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E12/G12)),IF(E12&gt;0,1,0))</f>
@@ -10940,36 +10940,36 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>11442</t>
+          <t>1421999</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>اشغال مرافق الايواء</t>
+          <t>مبيعات أخرى</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>التبغ والإيواء</t>
+          <t>أخرى</t>
         </is>
       </c>
       <c r="D13" s="6" t="n">
-        <v>199149669.75</v>
+        <v>60096373.96</v>
       </c>
       <c r="E13" s="6" t="n">
-        <v>135824266.97</v>
+        <v>134076434.91</v>
       </c>
       <c r="F13" s="6" t="n">
-        <v>815494.87</v>
+        <v>0</v>
       </c>
       <c r="G13" s="6" t="n">
-        <v>152968341.46</v>
+        <v>78879723.06</v>
       </c>
       <c r="H13" s="6" t="n">
-        <v>66937519.73</v>
+        <v>19648593.93</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>57302452.03</v>
+        <v>5322376.9</v>
       </c>
       <c r="J13" s="15">
         <f>IF(G13&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E13/G13)),IF(E13&gt;0,1,0))</f>
@@ -11007,36 +11007,36 @@
     <row r="14">
       <c r="A14" s="5" t="inlineStr">
         <is>
-          <t>1421999</t>
+          <t>142113</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t>مبيعات أخرى</t>
+          <t>ايرادات  اللوحات الدعائية</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t>أخرى</t>
+          <t>الرسوم والتراخيص</t>
         </is>
       </c>
       <c r="D14" s="6" t="n">
-        <v>60096373.96</v>
+        <v>103589976.04</v>
       </c>
       <c r="E14" s="6" t="n">
-        <v>134076434.91</v>
+        <v>121704394.25</v>
       </c>
       <c r="F14" s="6" t="n">
-        <v>0</v>
+        <v>327373.48</v>
       </c>
       <c r="G14" s="6" t="n">
-        <v>78879723.06</v>
+        <v>122797356.41</v>
       </c>
       <c r="H14" s="6" t="n">
-        <v>19648593.93</v>
+        <v>35149182.39</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>5322376.9</v>
+        <v>18399321.15</v>
       </c>
       <c r="J14" s="15">
         <f>IF(G14&gt;0,MIN(الافتراضات!$B$8,MAX(الافتراضات!$B$7,E14/G14)),IF(E14&gt;0,1,0))</f>
@@ -11754,7 +11754,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>علم</t>
+          <t>علم / جزاءات</t>
         </is>
       </c>
       <c r="D25" s="6" t="n">
@@ -13122,7 +13122,7 @@
     <row r="2">
       <c r="A2" s="11" t="inlineStr">
         <is>
-          <t>2026: أكتوبر جزئي (حتى تاريخ الملف) ونوفمبر وديسمبر لم يحصلا بعد. شهور الذروة الاستثنائية: يوليو 2024 (اللوحات الدعائية 327م)، مايو 2025 (اللوحات الدعائية 297م)، نوفمبر 2025 (اللوحات الدعائية 598م)، يونيو 2026 (تأجير المرافق 411م).</t>
+          <t>2026: أكتوبر جزئي (حتى تاريخ الملف) ونوفمبر وديسمبر لم يحصلا بعد. بعد إعادة التصنيف: نقل 913م من حساب اللوحات الدعائية (142113) إلى تأجير المرافق (142162) في 2025 (مايو 291م ونوفمبر 594م، من إدارة الدعم المالي) حسب تأكيد المستخدم. شهور الذروة المتبقية: يوليو 2024 (312م، إدارة الدعم المالي، لم تُنقل)، يونيو 2026 (تأجير المرافق 409م).</t>
         </is>
       </c>
     </row>
@@ -13657,7 +13657,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C19"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -13839,6 +13839,13 @@
     <row r="19">
       <c r="A19" s="22" t="inlineStr">
         <is>
+          <t>6e) إعادة تصنيف المحصل: حسب تأكيد المستخدم، نُقل 913م من محصل 2025 في حساب اللوحات الدعائية (142113) إلى تأجير المرافق (142162) (كلها من إدارة الدعم المالي: مايو 291م ونوفمبر 594م). ينطبق على أوراق المحصل فقط؛ أوراق الفوترة لم تُعدّل لأن مبالغ الفوترة حسب الجهة غير متوفرة. إن كانت دفعات إدارة الدعم المالي في 2024 (يوليو 312م، نوفمبر 25م، ديسمبر 102م) من نفس النوع فالتوقع الأساسي يرتفع (انظر الرد).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
           <t>7) تنبيه: كثير من الحسابات تتذبذب بشدة بين السنوات (لوحات دعائية، تأجير المرافق، إيرادات متنوعة)، ومضاعفة 2026 على 12/9 تضخّم أو تقلّل هذه الأرقام؛ انظر عمود "تنبيه".</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add collected forecast reflecting monitoring file Jan-Oct 2026 actuals
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/توقع_الفوترة_2026_2027.xlsx
+++ b/توقع_الفوترة_2026_2027.xlsx
@@ -14,13 +14,15 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="تحليل التوقع والأسوأ" sheetId="5" state="visible" r:id="rId5"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="توقع المحصل الموسمي" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الموسمية الشهرية" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="توقع المحصل (المراقبة)" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'التوقعات'!$A$3:$R$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'توقع المحصل 2026'!$A$3:$N$41</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'تحليل التوقع والأسوأ'!$A$4:$O$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'توقع المحصل الموسمي'!$A$5:$Q$43</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'توقع المحصل (المراقبة)'!$A$5:$U$48</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -13657,7 +13659,3785 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:U49"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>توقع إقفال 2026 (محصّل) بعد اعتماد إجمالي يناير–أكتوبر من ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="70" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>المحصل الفعلي يناير–أكتوبر 2026 = ورقة "الإجمالي" في ملف المراقبة (قبل الاستقطاع = بعد الاستقطاع + التوريد + المستقطع)، وأكتوبر جزئي حتى تاريخ الملف. الإقفال الأساسي = الفعلي + المتبقي من أكتوبر + نوفمبر وديسمبر؛ المتبقي من أكتوبر = المتوسط الموسمي لأكتوبر × معامل الاتجاه − المحصل حتى تاريخه (لا يقل عن صفر)؛ نوفمبر وديسمبر = وسيط 2023–2025 × معامل الاتجاه. السيناريو الأسوأ: أدنى قيمة تاريخية بدل الوسيط × (الاتجاه بحد أقصى 1). الحسابات التي في ملف المراقبة فقط ولا تاريخ لها في الملف الشهري (1431 و1422104 و1422112 و1422199 و1422202) تُبقى على الفعلي بدون إضافة. بنود التوريد (شيك/تحويل/تنفيذ) داخلة في الفعلي لكن لا تُتوقع للأشهر المتبقية لأنها غير منتظمة، فهي خطر صعودي.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>الملخص:</t>
+        </is>
+      </c>
+      <c r="C3" s="13" t="inlineStr">
+        <is>
+          <t>الفعلي يناير–أكتوبر (المراقبة)</t>
+        </is>
+      </c>
+      <c r="D3" s="14">
+        <f>D49</f>
+        <v/>
+      </c>
+      <c r="E3" s="13" t="inlineStr">
+        <is>
+          <t>إقفال 2026 – أساسي</t>
+        </is>
+      </c>
+      <c r="F3" s="14">
+        <f>M49</f>
+        <v/>
+      </c>
+      <c r="G3" s="13" t="inlineStr">
+        <is>
+          <t>إقفال 2026 – أسوأ</t>
+        </is>
+      </c>
+      <c r="H3" s="14">
+        <f>P49</f>
+        <v/>
+      </c>
+      <c r="I3" s="13" t="inlineStr">
+        <is>
+          <t>المقدر 2026 (المراقبة)</t>
+        </is>
+      </c>
+      <c r="J3" s="14">
+        <f>Q49</f>
+        <v/>
+      </c>
+      <c r="K3" s="13" t="inlineStr">
+        <is>
+          <t>المستهدف 2026</t>
+        </is>
+      </c>
+      <c r="L3" s="14">
+        <f>R49</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>رقم الحساب</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>اسم الحساب</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>التبويب</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>الفعلي يناير–أكتوبر (المراقبة)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>منه: أكتوبر حتى تاريخه</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>وسيط أكتوبر 2023–2025</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>وسيط نوفمبر+ديسمبر 2023–2025</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>أدنى أكتوبر</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>أدنى نوفمبر+ديسمبر</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>معامل الاتجاه</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>متبقي أكتوبر – أساسي</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>نوفمبر+ديسمبر – أساسي</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="inlineStr">
+        <is>
+          <t>إقفال 2026 – أساسي</t>
+        </is>
+      </c>
+      <c r="N5" s="4" t="inlineStr">
+        <is>
+          <t>متبقي أكتوبر – أسوأ</t>
+        </is>
+      </c>
+      <c r="O5" s="4" t="inlineStr">
+        <is>
+          <t>نوفمبر+ديسمبر – أسوأ</t>
+        </is>
+      </c>
+      <c r="P5" s="4" t="inlineStr">
+        <is>
+          <t>إقفال 2026 – أسوأ</t>
+        </is>
+      </c>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>المقدر 2026 (المراقبة)</t>
+        </is>
+      </c>
+      <c r="R5" s="4" t="inlineStr">
+        <is>
+          <t>المستهدف 2026 (المراقبة)</t>
+        </is>
+      </c>
+      <c r="S5" s="4" t="inlineStr">
+        <is>
+          <t>الأساسي − المقدر</t>
+        </is>
+      </c>
+      <c r="T5" s="4" t="inlineStr">
+        <is>
+          <t>الأساسي ÷ المستهدف</t>
+        </is>
+      </c>
+      <c r="U5" s="4" t="inlineStr">
+        <is>
+          <t>مصدر الفعلي</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>14155</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>ريع الأراضي (تأجير الأراض )</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>644487164.65</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>32158747.69</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>109860078.01</v>
+      </c>
+      <c r="G6" s="6" t="n">
+        <v>160048702.24</v>
+      </c>
+      <c r="H6" s="6" t="n">
+        <v>44284437.89</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>119047370.87</v>
+      </c>
+      <c r="J6" s="15">
+        <f>IFERROR(VLOOKUP(A6,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K6" s="6">
+        <f>MAX(0,F6*J6-E6)</f>
+        <v/>
+      </c>
+      <c r="L6" s="6">
+        <f>G6*J6</f>
+        <v/>
+      </c>
+      <c r="M6" s="6">
+        <f>D6+K6+L6</f>
+        <v/>
+      </c>
+      <c r="N6" s="6">
+        <f>MAX(0,H6*MIN(J6,1)-E6)</f>
+        <v/>
+      </c>
+      <c r="O6" s="6">
+        <f>I6*MIN(J6,1)</f>
+        <v/>
+      </c>
+      <c r="P6" s="6">
+        <f>D6+N6+O6</f>
+        <v/>
+      </c>
+      <c r="Q6" s="6" t="n">
+        <v>704204539.7299998</v>
+      </c>
+      <c r="R6" s="6" t="n">
+        <v>736893407.9179136</v>
+      </c>
+      <c r="S6" s="6">
+        <f>M6-Q6</f>
+        <v/>
+      </c>
+      <c r="T6" s="7">
+        <f>IF(R6=0,"",M6/R6)</f>
+        <v/>
+      </c>
+      <c r="U6" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>142162</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  تأجير المرافق</t>
+        </is>
+      </c>
+      <c r="C7" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>428714993.46</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>322955.69</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>524480.25</v>
+      </c>
+      <c r="G7" s="6" t="n">
+        <v>32068051.86</v>
+      </c>
+      <c r="H7" s="6" t="n">
+        <v>164700</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>157950</v>
+      </c>
+      <c r="J7" s="15">
+        <f>IFERROR(VLOOKUP(A7,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K7" s="6">
+        <f>MAX(0,F7*J7-E7)</f>
+        <v/>
+      </c>
+      <c r="L7" s="6">
+        <f>G7*J7</f>
+        <v/>
+      </c>
+      <c r="M7" s="6">
+        <f>D7+K7+L7</f>
+        <v/>
+      </c>
+      <c r="N7" s="6">
+        <f>MAX(0,H7*MIN(J7,1)-E7)</f>
+        <v/>
+      </c>
+      <c r="O7" s="6">
+        <f>I7*MIN(J7,1)</f>
+        <v/>
+      </c>
+      <c r="P7" s="6">
+        <f>D7+N7+O7</f>
+        <v/>
+      </c>
+      <c r="Q7" s="6" t="n">
+        <v>502882772.0000001</v>
+      </c>
+      <c r="R7" s="6" t="n">
+        <v>1003276063.144015</v>
+      </c>
+      <c r="S7" s="6">
+        <f>M7-Q7</f>
+        <v/>
+      </c>
+      <c r="T7" s="7">
+        <f>IF(R7=0,"",M7/R7)</f>
+        <v/>
+      </c>
+      <c r="U7" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>1438001</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات و غرامات مفروضة بموجب أنظمة الجهة</t>
+        </is>
+      </c>
+      <c r="C8" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>389696651.05</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>33304429</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>29549276.1</v>
+      </c>
+      <c r="G8" s="6" t="n">
+        <v>56267310.75</v>
+      </c>
+      <c r="H8" s="6" t="n">
+        <v>16531182.77</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>48603924.57</v>
+      </c>
+      <c r="J8" s="15">
+        <f>IFERROR(VLOOKUP(A8,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K8" s="6">
+        <f>MAX(0,F8*J8-E8)</f>
+        <v/>
+      </c>
+      <c r="L8" s="6">
+        <f>G8*J8</f>
+        <v/>
+      </c>
+      <c r="M8" s="6">
+        <f>D8+K8+L8</f>
+        <v/>
+      </c>
+      <c r="N8" s="6">
+        <f>MAX(0,H8*MIN(J8,1)-E8)</f>
+        <v/>
+      </c>
+      <c r="O8" s="6">
+        <f>I8*MIN(J8,1)</f>
+        <v/>
+      </c>
+      <c r="P8" s="6">
+        <f>D8+N8+O8</f>
+        <v/>
+      </c>
+      <c r="Q8" s="6" t="n">
+        <v>417587219.58</v>
+      </c>
+      <c r="R8" s="6" t="n">
+        <v>441463735.5552299</v>
+      </c>
+      <c r="S8" s="6">
+        <f>M8-Q8</f>
+        <v/>
+      </c>
+      <c r="T8" s="7">
+        <f>IF(R8=0,"",M8/R8)</f>
+        <v/>
+      </c>
+      <c r="U8" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>11452104</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>إصدار رخص الأنشطة التجارية</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>260435884.99</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>13834961.34</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>25241852.69</v>
+      </c>
+      <c r="G9" s="6" t="n">
+        <v>46330431.63</v>
+      </c>
+      <c r="H9" s="6" t="n">
+        <v>23888796.32</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>45491327.88</v>
+      </c>
+      <c r="J9" s="15">
+        <f>IFERROR(VLOOKUP(A9,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K9" s="6">
+        <f>MAX(0,F9*J9-E9)</f>
+        <v/>
+      </c>
+      <c r="L9" s="6">
+        <f>G9*J9</f>
+        <v/>
+      </c>
+      <c r="M9" s="6">
+        <f>D9+K9+L9</f>
+        <v/>
+      </c>
+      <c r="N9" s="6">
+        <f>MAX(0,H9*MIN(J9,1)-E9)</f>
+        <v/>
+      </c>
+      <c r="O9" s="6">
+        <f>I9*MIN(J9,1)</f>
+        <v/>
+      </c>
+      <c r="P9" s="6">
+        <f>D9+N9+O9</f>
+        <v/>
+      </c>
+      <c r="Q9" s="6" t="n">
+        <v>284731166.07</v>
+      </c>
+      <c r="R9" s="6" t="n">
+        <v>315914658.8484679</v>
+      </c>
+      <c r="S9" s="6">
+        <f>M9-Q9</f>
+        <v/>
+      </c>
+      <c r="T9" s="7">
+        <f>IF(R9=0,"",M9/R9)</f>
+        <v/>
+      </c>
+      <c r="U9" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>11452103</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr">
+        <is>
+          <t>ايراد اصدار تراخيص المباني والاسوار - أمانة منطقة الرياض</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>213758689.52</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>10111052.72</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>23653967.06</v>
+      </c>
+      <c r="G10" s="6" t="n">
+        <v>49304101.84</v>
+      </c>
+      <c r="H10" s="6" t="n">
+        <v>18226070.37</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>37923630.92</v>
+      </c>
+      <c r="J10" s="15">
+        <f>IFERROR(VLOOKUP(A10,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K10" s="6">
+        <f>MAX(0,F10*J10-E10)</f>
+        <v/>
+      </c>
+      <c r="L10" s="6">
+        <f>G10*J10</f>
+        <v/>
+      </c>
+      <c r="M10" s="6">
+        <f>D10+K10+L10</f>
+        <v/>
+      </c>
+      <c r="N10" s="6">
+        <f>MAX(0,H10*MIN(J10,1)-E10)</f>
+        <v/>
+      </c>
+      <c r="O10" s="6">
+        <f>I10*MIN(J10,1)</f>
+        <v/>
+      </c>
+      <c r="P10" s="6">
+        <f>D10+N10+O10</f>
+        <v/>
+      </c>
+      <c r="Q10" s="6" t="n">
+        <v>296614997.78</v>
+      </c>
+      <c r="R10" s="6" t="n">
+        <v>317404423.9819266</v>
+      </c>
+      <c r="S10" s="6">
+        <f>M10-Q10</f>
+        <v/>
+      </c>
+      <c r="T10" s="7">
+        <f>IF(R10=0,"",M10/R10)</f>
+        <v/>
+      </c>
+      <c r="U10" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>11452512</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات لوحات المحلات</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>184508812.29</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>10443752.94</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>20956485</v>
+      </c>
+      <c r="G11" s="6" t="n">
+        <v>38398095</v>
+      </c>
+      <c r="H11" s="6" t="n">
+        <v>17387315.02</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>33977960.96</v>
+      </c>
+      <c r="J11" s="15">
+        <f>IFERROR(VLOOKUP(A11,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K11" s="6">
+        <f>MAX(0,F11*J11-E11)</f>
+        <v/>
+      </c>
+      <c r="L11" s="6">
+        <f>G11*J11</f>
+        <v/>
+      </c>
+      <c r="M11" s="6">
+        <f>D11+K11+L11</f>
+        <v/>
+      </c>
+      <c r="N11" s="6">
+        <f>MAX(0,H11*MIN(J11,1)-E11)</f>
+        <v/>
+      </c>
+      <c r="O11" s="6">
+        <f>I11*MIN(J11,1)</f>
+        <v/>
+      </c>
+      <c r="P11" s="6">
+        <f>D11+N11+O11</f>
+        <v/>
+      </c>
+      <c r="Q11" s="6" t="n">
+        <v>247656264.1</v>
+      </c>
+      <c r="R11" s="6" t="n">
+        <v>248231484.51</v>
+      </c>
+      <c r="S11" s="6">
+        <f>M11-Q11</f>
+        <v/>
+      </c>
+      <c r="T11" s="7">
+        <f>IF(R11=0,"",M11/R11)</f>
+        <v/>
+      </c>
+      <c r="U11" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>1439</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  مبيعات  ناتجه من النشاط غير مصنفة</t>
+        </is>
+      </c>
+      <c r="C12" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>179433194.45</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="6" t="n">
+        <v>144348</v>
+      </c>
+      <c r="H12" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>14000</v>
+      </c>
+      <c r="J12" s="15">
+        <f>IFERROR(VLOOKUP(A12,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K12" s="6">
+        <f>MAX(0,F12*J12-E12)</f>
+        <v/>
+      </c>
+      <c r="L12" s="6">
+        <f>G12*J12</f>
+        <v/>
+      </c>
+      <c r="M12" s="6">
+        <f>D12+K12+L12</f>
+        <v/>
+      </c>
+      <c r="N12" s="6">
+        <f>MAX(0,H12*MIN(J12,1)-E12)</f>
+        <v/>
+      </c>
+      <c r="O12" s="6">
+        <f>I12*MIN(J12,1)</f>
+        <v/>
+      </c>
+      <c r="P12" s="6">
+        <f>D12+N12+O12</f>
+        <v/>
+      </c>
+      <c r="Q12" s="6" t="n">
+        <v>1036092.05</v>
+      </c>
+      <c r="R12" s="6" t="n">
+        <v>30036092.05</v>
+      </c>
+      <c r="S12" s="6">
+        <f>M12-Q12</f>
+        <v/>
+      </c>
+      <c r="T12" s="7">
+        <f>IF(R12=0,"",M12/R12)</f>
+        <v/>
+      </c>
+      <c r="U12" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>11442</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="inlineStr">
+        <is>
+          <t>اشغال مرافق الايواء</t>
+        </is>
+      </c>
+      <c r="C13" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>151739989.39</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>13283777.98</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>20391349.29</v>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>46546170.44</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>13914304.96</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>43388147.07</v>
+      </c>
+      <c r="J13" s="15">
+        <f>IFERROR(VLOOKUP(A13,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K13" s="6">
+        <f>MAX(0,F13*J13-E13)</f>
+        <v/>
+      </c>
+      <c r="L13" s="6">
+        <f>G13*J13</f>
+        <v/>
+      </c>
+      <c r="M13" s="6">
+        <f>D13+K13+L13</f>
+        <v/>
+      </c>
+      <c r="N13" s="6">
+        <f>MAX(0,H13*MIN(J13,1)-E13)</f>
+        <v/>
+      </c>
+      <c r="O13" s="6">
+        <f>I13*MIN(J13,1)</f>
+        <v/>
+      </c>
+      <c r="P13" s="6">
+        <f>D13+N13+O13</f>
+        <v/>
+      </c>
+      <c r="Q13" s="6" t="n">
+        <v>265010811.65</v>
+      </c>
+      <c r="R13" s="6" t="n">
+        <v>288111986.9440953</v>
+      </c>
+      <c r="S13" s="6">
+        <f>M13-Q13</f>
+        <v/>
+      </c>
+      <c r="T13" s="7">
+        <f>IF(R13=0,"",M13/R13)</f>
+        <v/>
+      </c>
+      <c r="U13" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>1421999</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="inlineStr">
+        <is>
+          <t>مبيعات أخرى</t>
+        </is>
+      </c>
+      <c r="C14" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>137544463.2</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>7217587.27</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>8305349.75</v>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>8433487.07</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>2826014.45</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>2496362.45</v>
+      </c>
+      <c r="J14" s="15">
+        <f>IFERROR(VLOOKUP(A14,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K14" s="6">
+        <f>MAX(0,F14*J14-E14)</f>
+        <v/>
+      </c>
+      <c r="L14" s="6">
+        <f>G14*J14</f>
+        <v/>
+      </c>
+      <c r="M14" s="6">
+        <f>D14+K14+L14</f>
+        <v/>
+      </c>
+      <c r="N14" s="6">
+        <f>MAX(0,H14*MIN(J14,1)-E14)</f>
+        <v/>
+      </c>
+      <c r="O14" s="6">
+        <f>I14*MIN(J14,1)</f>
+        <v/>
+      </c>
+      <c r="P14" s="6">
+        <f>D14+N14+O14</f>
+        <v/>
+      </c>
+      <c r="Q14" s="6" t="n">
+        <v>92115826.69999999</v>
+      </c>
+      <c r="R14" s="6" t="n">
+        <v>93151323.34705561</v>
+      </c>
+      <c r="S14" s="6">
+        <f>M14-Q14</f>
+        <v/>
+      </c>
+      <c r="T14" s="7">
+        <f>IF(R14=0,"",M14/R14)</f>
+        <v/>
+      </c>
+      <c r="U14" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>142113</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  اللوحات الدعائية</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>125120390.68</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>2451891.69</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>10807518.59</v>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>21718150.74</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>5813099.79</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>12586221.36</v>
+      </c>
+      <c r="J15" s="15">
+        <f>IFERROR(VLOOKUP(A15,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K15" s="6">
+        <f>MAX(0,F15*J15-E15)</f>
+        <v/>
+      </c>
+      <c r="L15" s="6">
+        <f>G15*J15</f>
+        <v/>
+      </c>
+      <c r="M15" s="6">
+        <f>D15+K15+L15</f>
+        <v/>
+      </c>
+      <c r="N15" s="6">
+        <f>MAX(0,H15*MIN(J15,1)-E15)</f>
+        <v/>
+      </c>
+      <c r="O15" s="6">
+        <f>I15*MIN(J15,1)</f>
+        <v/>
+      </c>
+      <c r="P15" s="6">
+        <f>D15+N15+O15</f>
+        <v/>
+      </c>
+      <c r="Q15" s="6" t="n">
+        <v>88762340.61999997</v>
+      </c>
+      <c r="R15" s="6" t="n">
+        <v>90076239.38854954</v>
+      </c>
+      <c r="S15" s="6">
+        <f>M15-Q15</f>
+        <v/>
+      </c>
+      <c r="T15" s="7">
+        <f>IF(R15=0,"",M15/R15)</f>
+        <v/>
+      </c>
+      <c r="U15" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>1431</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="inlineStr">
+        <is>
+          <t>الجزاءات والغرامات</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>103169485.22</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M16" s="6">
+        <f>D16+K16+L16</f>
+        <v/>
+      </c>
+      <c r="N16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="6">
+        <f>D16+N16+O16</f>
+        <v/>
+      </c>
+      <c r="Q16" s="6" t="n">
+        <v>36003284</v>
+      </c>
+      <c r="R16" s="6" t="n">
+        <v>90003284</v>
+      </c>
+      <c r="S16" s="6">
+        <f>M16-Q16</f>
+        <v/>
+      </c>
+      <c r="T16" s="7">
+        <f>IF(R16=0,"",M16/R16)</f>
+        <v/>
+      </c>
+      <c r="U16" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>1421909</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>جمع النفايات</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>76152734.44</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>3922507.01</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>6932993.61</v>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>13872695.64</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>6611666.54</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>11918092.48</v>
+      </c>
+      <c r="J17" s="15">
+        <f>IFERROR(VLOOKUP(A17,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K17" s="6">
+        <f>MAX(0,F17*J17-E17)</f>
+        <v/>
+      </c>
+      <c r="L17" s="6">
+        <f>G17*J17</f>
+        <v/>
+      </c>
+      <c r="M17" s="6">
+        <f>D17+K17+L17</f>
+        <v/>
+      </c>
+      <c r="N17" s="6">
+        <f>MAX(0,H17*MIN(J17,1)-E17)</f>
+        <v/>
+      </c>
+      <c r="O17" s="6">
+        <f>I17*MIN(J17,1)</f>
+        <v/>
+      </c>
+      <c r="P17" s="6">
+        <f>D17+N17+O17</f>
+        <v/>
+      </c>
+      <c r="Q17" s="6" t="n">
+        <v>86507432.33999999</v>
+      </c>
+      <c r="R17" s="6" t="n">
+        <v>97842756.86908785</v>
+      </c>
+      <c r="S17" s="6">
+        <f>M17-Q17</f>
+        <v/>
+      </c>
+      <c r="T17" s="7">
+        <f>IF(R17=0,"",M17/R17)</f>
+        <v/>
+      </c>
+      <c r="U17" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>1421911</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>رسم مبيعات محلات تقديم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>60524211.88</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>3739768.97</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>6619764.26</v>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>13360044.69</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>4881210.37</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>10535371.99</v>
+      </c>
+      <c r="J18" s="15">
+        <f>IFERROR(VLOOKUP(A18,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K18" s="6">
+        <f>MAX(0,F18*J18-E18)</f>
+        <v/>
+      </c>
+      <c r="L18" s="6">
+        <f>G18*J18</f>
+        <v/>
+      </c>
+      <c r="M18" s="6">
+        <f>D18+K18+L18</f>
+        <v/>
+      </c>
+      <c r="N18" s="6">
+        <f>MAX(0,H18*MIN(J18,1)-E18)</f>
+        <v/>
+      </c>
+      <c r="O18" s="6">
+        <f>I18*MIN(J18,1)</f>
+        <v/>
+      </c>
+      <c r="P18" s="6">
+        <f>D18+N18+O18</f>
+        <v/>
+      </c>
+      <c r="Q18" s="6" t="n">
+        <v>86279560.64999999</v>
+      </c>
+      <c r="R18" s="6" t="n">
+        <v>91313321.92602974</v>
+      </c>
+      <c r="S18" s="6">
+        <f>M18-Q18</f>
+        <v/>
+      </c>
+      <c r="T18" s="7">
+        <f>IF(R18=0,"",M18/R18)</f>
+        <v/>
+      </c>
+      <c r="U18" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>144122</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  متنوعه</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>55929677.95</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>124953</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>567745</v>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>298480.96</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>126070</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>77489.08</v>
+      </c>
+      <c r="J19" s="15">
+        <f>IFERROR(VLOOKUP(A19,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K19" s="6">
+        <f>MAX(0,F19*J19-E19)</f>
+        <v/>
+      </c>
+      <c r="L19" s="6">
+        <f>G19*J19</f>
+        <v/>
+      </c>
+      <c r="M19" s="6">
+        <f>D19+K19+L19</f>
+        <v/>
+      </c>
+      <c r="N19" s="6">
+        <f>MAX(0,H19*MIN(J19,1)-E19)</f>
+        <v/>
+      </c>
+      <c r="O19" s="6">
+        <f>I19*MIN(J19,1)</f>
+        <v/>
+      </c>
+      <c r="P19" s="6">
+        <f>D19+N19+O19</f>
+        <v/>
+      </c>
+      <c r="Q19" s="6" t="n">
+        <v>10895644.06</v>
+      </c>
+      <c r="R19" s="6" t="n">
+        <v>5397642.999999999</v>
+      </c>
+      <c r="S19" s="6">
+        <f>M19-Q19</f>
+        <v/>
+      </c>
+      <c r="T19" s="7">
+        <f>IF(R19=0,"",M19/R19)</f>
+        <v/>
+      </c>
+      <c r="U19" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>11452108</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>ايراد اصدار القرارات المساحية - أمانة منطقة الرياض</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>33095183.09</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>2067255.85</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>1896861.57</v>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>3641834.48</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>270939.62</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>1684338.27</v>
+      </c>
+      <c r="J20" s="15">
+        <f>IFERROR(VLOOKUP(A20,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K20" s="6">
+        <f>MAX(0,F20*J20-E20)</f>
+        <v/>
+      </c>
+      <c r="L20" s="6">
+        <f>G20*J20</f>
+        <v/>
+      </c>
+      <c r="M20" s="6">
+        <f>D20+K20+L20</f>
+        <v/>
+      </c>
+      <c r="N20" s="6">
+        <f>MAX(0,H20*MIN(J20,1)-E20)</f>
+        <v/>
+      </c>
+      <c r="O20" s="6">
+        <f>I20*MIN(J20,1)</f>
+        <v/>
+      </c>
+      <c r="P20" s="6">
+        <f>D20+N20+O20</f>
+        <v/>
+      </c>
+      <c r="Q20" s="6" t="n">
+        <v>17045890.37</v>
+      </c>
+      <c r="R20" s="6" t="n">
+        <v>30799388.58652012</v>
+      </c>
+      <c r="S20" s="6">
+        <f>M20-Q20</f>
+        <v/>
+      </c>
+      <c r="T20" s="7">
+        <f>IF(R20=0,"",M20/R20)</f>
+        <v/>
+      </c>
+      <c r="U20" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>1422108</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>الشهادات الصحية</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>20176446.1</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>2567043.91</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>2731752.84</v>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>3731307.78</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>1580920.2</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>1866020</v>
+      </c>
+      <c r="J21" s="15">
+        <f>IFERROR(VLOOKUP(A21,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K21" s="6">
+        <f>MAX(0,F21*J21-E21)</f>
+        <v/>
+      </c>
+      <c r="L21" s="6">
+        <f>G21*J21</f>
+        <v/>
+      </c>
+      <c r="M21" s="6">
+        <f>D21+K21+L21</f>
+        <v/>
+      </c>
+      <c r="N21" s="6">
+        <f>MAX(0,H21*MIN(J21,1)-E21)</f>
+        <v/>
+      </c>
+      <c r="O21" s="6">
+        <f>I21*MIN(J21,1)</f>
+        <v/>
+      </c>
+      <c r="P21" s="6">
+        <f>D21+N21+O21</f>
+        <v/>
+      </c>
+      <c r="Q21" s="6" t="n">
+        <v>20148582.53</v>
+      </c>
+      <c r="R21" s="6" t="n">
+        <v>21121165.60478871</v>
+      </c>
+      <c r="S21" s="6">
+        <f>M21-Q21</f>
+        <v/>
+      </c>
+      <c r="T21" s="7">
+        <f>IF(R21=0,"",M21/R21)</f>
+        <v/>
+      </c>
+      <c r="U21" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>1422121</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>رسم ترخيص نشاط تقديم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>14291699.73</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>437434.24</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>1850000</v>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>2870000</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>973250</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>2695000</v>
+      </c>
+      <c r="J22" s="15">
+        <f>IFERROR(VLOOKUP(A22,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K22" s="6">
+        <f>MAX(0,F22*J22-E22)</f>
+        <v/>
+      </c>
+      <c r="L22" s="6">
+        <f>G22*J22</f>
+        <v/>
+      </c>
+      <c r="M22" s="6">
+        <f>D22+K22+L22</f>
+        <v/>
+      </c>
+      <c r="N22" s="6">
+        <f>MAX(0,H22*MIN(J22,1)-E22)</f>
+        <v/>
+      </c>
+      <c r="O22" s="6">
+        <f>I22*MIN(J22,1)</f>
+        <v/>
+      </c>
+      <c r="P22" s="6">
+        <f>D22+N22+O22</f>
+        <v/>
+      </c>
+      <c r="Q22" s="6" t="n">
+        <v>18607310.69</v>
+      </c>
+      <c r="R22" s="6" t="n">
+        <v>19724053.61546767</v>
+      </c>
+      <c r="S22" s="6">
+        <f>M22-Q22</f>
+        <v/>
+      </c>
+      <c r="T22" s="7">
+        <f>IF(R22=0,"",M22/R22)</f>
+        <v/>
+      </c>
+      <c r="U22" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>11452111</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>المقابل المالي للسماح للأنشطة التجارية بالعمل (24) ساعة</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>12380137.91</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>990178.5</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>552605.5</v>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>816625.3</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>474556.44</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>777577.05</v>
+      </c>
+      <c r="J23" s="15">
+        <f>IFERROR(VLOOKUP(A23,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K23" s="6">
+        <f>MAX(0,F23*J23-E23)</f>
+        <v/>
+      </c>
+      <c r="L23" s="6">
+        <f>G23*J23</f>
+        <v/>
+      </c>
+      <c r="M23" s="6">
+        <f>D23+K23+L23</f>
+        <v/>
+      </c>
+      <c r="N23" s="6">
+        <f>MAX(0,H23*MIN(J23,1)-E23)</f>
+        <v/>
+      </c>
+      <c r="O23" s="6">
+        <f>I23*MIN(J23,1)</f>
+        <v/>
+      </c>
+      <c r="P23" s="6">
+        <f>D23+N23+O23</f>
+        <v/>
+      </c>
+      <c r="Q23" s="6" t="n">
+        <v>6031979.84</v>
+      </c>
+      <c r="R23" s="6" t="n">
+        <v>7104624.902319179</v>
+      </c>
+      <c r="S23" s="6">
+        <f>M23-Q23</f>
+        <v/>
+      </c>
+      <c r="T23" s="7">
+        <f>IF(R23=0,"",M23/R23)</f>
+        <v/>
+      </c>
+      <c r="U23" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>142163</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات  تأجير مباني تجارية</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>10246864.26</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>380080</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>959250</v>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>1234661</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>225853</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>596720</v>
+      </c>
+      <c r="J24" s="15">
+        <f>IFERROR(VLOOKUP(A24,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K24" s="6">
+        <f>MAX(0,F24*J24-E24)</f>
+        <v/>
+      </c>
+      <c r="L24" s="6">
+        <f>G24*J24</f>
+        <v/>
+      </c>
+      <c r="M24" s="6">
+        <f>D24+K24+L24</f>
+        <v/>
+      </c>
+      <c r="N24" s="6">
+        <f>MAX(0,H24*MIN(J24,1)-E24)</f>
+        <v/>
+      </c>
+      <c r="O24" s="6">
+        <f>I24*MIN(J24,1)</f>
+        <v/>
+      </c>
+      <c r="P24" s="6">
+        <f>D24+N24+O24</f>
+        <v/>
+      </c>
+      <c r="Q24" s="6" t="n">
+        <v>50897586.07999999</v>
+      </c>
+      <c r="R24" s="6" t="n">
+        <v>52395049.26104818</v>
+      </c>
+      <c r="S24" s="6">
+        <f>M24-Q24</f>
+        <v/>
+      </c>
+      <c r="T24" s="7">
+        <f>IF(R24=0,"",M24/R24)</f>
+        <v/>
+      </c>
+      <c r="U24" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>1422109</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  الكشفية</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>6054177.61</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>330988.56</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>702133.4</v>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>1368865.4</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>656085.2</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>1293782.8</v>
+      </c>
+      <c r="J25" s="15">
+        <f>IFERROR(VLOOKUP(A25,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K25" s="6">
+        <f>MAX(0,F25*J25-E25)</f>
+        <v/>
+      </c>
+      <c r="L25" s="6">
+        <f>G25*J25</f>
+        <v/>
+      </c>
+      <c r="M25" s="6">
+        <f>D25+K25+L25</f>
+        <v/>
+      </c>
+      <c r="N25" s="6">
+        <f>MAX(0,H25*MIN(J25,1)-E25)</f>
+        <v/>
+      </c>
+      <c r="O25" s="6">
+        <f>I25*MIN(J25,1)</f>
+        <v/>
+      </c>
+      <c r="P25" s="6">
+        <f>D25+N25+O25</f>
+        <v/>
+      </c>
+      <c r="Q25" s="6" t="n">
+        <v>9760053.120000001</v>
+      </c>
+      <c r="R25" s="6" t="n">
+        <v>10078623.04293208</v>
+      </c>
+      <c r="S25" s="6">
+        <f>M25-Q25</f>
+        <v/>
+      </c>
+      <c r="T25" s="7">
+        <f>IF(R25=0,"",M25/R25)</f>
+        <v/>
+      </c>
+      <c r="U25" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>1422202</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>نقـل الملكيـة</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>4792650</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M26" s="6">
+        <f>D26+K26+L26</f>
+        <v/>
+      </c>
+      <c r="N26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P26" s="6">
+        <f>D26+N26+O26</f>
+        <v/>
+      </c>
+      <c r="Q26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R26" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S26" s="6">
+        <f>M26-Q26</f>
+        <v/>
+      </c>
+      <c r="T26" s="7">
+        <f>IF(R26=0,"",M26/R26)</f>
+        <v/>
+      </c>
+      <c r="U26" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>1421910</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>اصدار تراخيص اشغال الارصفة العامة و الطرق</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>3716245.56</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>134647.24</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>249916</v>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>708874.1899999999</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>214841.4</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>503183.16</v>
+      </c>
+      <c r="J27" s="15">
+        <f>IFERROR(VLOOKUP(A27,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K27" s="6">
+        <f>MAX(0,F27*J27-E27)</f>
+        <v/>
+      </c>
+      <c r="L27" s="6">
+        <f>G27*J27</f>
+        <v/>
+      </c>
+      <c r="M27" s="6">
+        <f>D27+K27+L27</f>
+        <v/>
+      </c>
+      <c r="N27" s="6">
+        <f>MAX(0,H27*MIN(J27,1)-E27)</f>
+        <v/>
+      </c>
+      <c r="O27" s="6">
+        <f>I27*MIN(J27,1)</f>
+        <v/>
+      </c>
+      <c r="P27" s="6">
+        <f>D27+N27+O27</f>
+        <v/>
+      </c>
+      <c r="Q27" s="6" t="n">
+        <v>4308099.1</v>
+      </c>
+      <c r="R27" s="6" t="n">
+        <v>4541143.188332747</v>
+      </c>
+      <c r="S27" s="6">
+        <f>M27-Q27</f>
+        <v/>
+      </c>
+      <c r="T27" s="7">
+        <f>IF(R27=0,"",M27/R27)</f>
+        <v/>
+      </c>
+      <c r="U27" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>11452107</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>اصدار التراخيص بتأسيس أو تشغيل الصراف الآلي</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>2807480.73</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>57100</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>24650</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>8000</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J28" s="15">
+        <f>IFERROR(VLOOKUP(A28,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K28" s="6">
+        <f>MAX(0,F28*J28-E28)</f>
+        <v/>
+      </c>
+      <c r="L28" s="6">
+        <f>G28*J28</f>
+        <v/>
+      </c>
+      <c r="M28" s="6">
+        <f>D28+K28+L28</f>
+        <v/>
+      </c>
+      <c r="N28" s="6">
+        <f>MAX(0,H28*MIN(J28,1)-E28)</f>
+        <v/>
+      </c>
+      <c r="O28" s="6">
+        <f>I28*MIN(J28,1)</f>
+        <v/>
+      </c>
+      <c r="P28" s="6">
+        <f>D28+N28+O28</f>
+        <v/>
+      </c>
+      <c r="Q28" s="6" t="n">
+        <v>2559317.18</v>
+      </c>
+      <c r="R28" s="6" t="n">
+        <v>2621585.07964954</v>
+      </c>
+      <c r="S28" s="6">
+        <f>M28-Q28</f>
+        <v/>
+      </c>
+      <c r="T28" s="7">
+        <f>IF(R28=0,"",M28/R28)</f>
+        <v/>
+      </c>
+      <c r="U28" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>1421901</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>بيع الوثائق والأنظمة</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>2598105.71</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>179280.35</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>265200</v>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>440800</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>217400</v>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>355500</v>
+      </c>
+      <c r="J29" s="15">
+        <f>IFERROR(VLOOKUP(A29,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K29" s="6">
+        <f>MAX(0,F29*J29-E29)</f>
+        <v/>
+      </c>
+      <c r="L29" s="6">
+        <f>G29*J29</f>
+        <v/>
+      </c>
+      <c r="M29" s="6">
+        <f>D29+K29+L29</f>
+        <v/>
+      </c>
+      <c r="N29" s="6">
+        <f>MAX(0,H29*MIN(J29,1)-E29)</f>
+        <v/>
+      </c>
+      <c r="O29" s="6">
+        <f>I29*MIN(J29,1)</f>
+        <v/>
+      </c>
+      <c r="P29" s="6">
+        <f>D29+N29+O29</f>
+        <v/>
+      </c>
+      <c r="Q29" s="6" t="n">
+        <v>8797965.779999999</v>
+      </c>
+      <c r="R29" s="6" t="n">
+        <v>6675958.317713005</v>
+      </c>
+      <c r="S29" s="6">
+        <f>M29-Q29</f>
+        <v/>
+      </c>
+      <c r="T29" s="7">
+        <f>IF(R29=0,"",M29/R29)</f>
+        <v/>
+      </c>
+      <c r="U29" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>بدون رقم</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>بدون رقم (خدمات علم + جزاءات)</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>علم / جزاءات</t>
+        </is>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>2122923.75</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>390906.25</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>1662357.5</v>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>3133203.75</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>471176.25</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>1095667.5</v>
+      </c>
+      <c r="J30" s="15">
+        <f>IFERROR(VLOOKUP(A30,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K30" s="6">
+        <f>MAX(0,F30*J30-E30)</f>
+        <v/>
+      </c>
+      <c r="L30" s="6">
+        <f>G30*J30</f>
+        <v/>
+      </c>
+      <c r="M30" s="6">
+        <f>D30+K30+L30</f>
+        <v/>
+      </c>
+      <c r="N30" s="6">
+        <f>MAX(0,H30*MIN(J30,1)-E30)</f>
+        <v/>
+      </c>
+      <c r="O30" s="6">
+        <f>I30*MIN(J30,1)</f>
+        <v/>
+      </c>
+      <c r="P30" s="6">
+        <f>D30+N30+O30</f>
+        <v/>
+      </c>
+      <c r="Q30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" s="6">
+        <f>M30-Q30</f>
+        <v/>
+      </c>
+      <c r="T30" s="7">
+        <f>IF(R30=0,"",M30/R30)</f>
+        <v/>
+      </c>
+      <c r="U30" s="5" t="inlineStr">
+        <is>
+          <t>الملف الشهري</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>1421912</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>تأجير العقارات لأغراض مؤقته</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>1795620.08</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>439507.53</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>274760.4</v>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>297677.53</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>87557.2</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>286749.22</v>
+      </c>
+      <c r="J31" s="15">
+        <f>IFERROR(VLOOKUP(A31,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K31" s="6">
+        <f>MAX(0,F31*J31-E31)</f>
+        <v/>
+      </c>
+      <c r="L31" s="6">
+        <f>G31*J31</f>
+        <v/>
+      </c>
+      <c r="M31" s="6">
+        <f>D31+K31+L31</f>
+        <v/>
+      </c>
+      <c r="N31" s="6">
+        <f>MAX(0,H31*MIN(J31,1)-E31)</f>
+        <v/>
+      </c>
+      <c r="O31" s="6">
+        <f>I31*MIN(J31,1)</f>
+        <v/>
+      </c>
+      <c r="P31" s="6">
+        <f>D31+N31+O31</f>
+        <v/>
+      </c>
+      <c r="Q31" s="6" t="n">
+        <v>1715079.17</v>
+      </c>
+      <c r="R31" s="6" t="n">
+        <v>2480385.743054039</v>
+      </c>
+      <c r="S31" s="6">
+        <f>M31-Q31</f>
+        <v/>
+      </c>
+      <c r="T31" s="7">
+        <f>IF(R31=0,"",M31/R31)</f>
+        <v/>
+      </c>
+      <c r="U31" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>11452106</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>اصدار التراخيص بتأسيس أو تشغيل ابراج الاتصالات</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>1419801.03</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>56000</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>107000</v>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>326000</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>97100</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>271100</v>
+      </c>
+      <c r="J32" s="15">
+        <f>IFERROR(VLOOKUP(A32,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K32" s="6">
+        <f>MAX(0,F32*J32-E32)</f>
+        <v/>
+      </c>
+      <c r="L32" s="6">
+        <f>G32*J32</f>
+        <v/>
+      </c>
+      <c r="M32" s="6">
+        <f>D32+K32+L32</f>
+        <v/>
+      </c>
+      <c r="N32" s="6">
+        <f>MAX(0,H32*MIN(J32,1)-E32)</f>
+        <v/>
+      </c>
+      <c r="O32" s="6">
+        <f>I32*MIN(J32,1)</f>
+        <v/>
+      </c>
+      <c r="P32" s="6">
+        <f>D32+N32+O32</f>
+        <v/>
+      </c>
+      <c r="Q32" s="6" t="n">
+        <v>7078106.61</v>
+      </c>
+      <c r="R32" s="6" t="n">
+        <v>7603182.489329966</v>
+      </c>
+      <c r="S32" s="6">
+        <f>M32-Q32</f>
+        <v/>
+      </c>
+      <c r="T32" s="7">
+        <f>IF(R32=0,"",M32/R32)</f>
+        <v/>
+      </c>
+      <c r="U32" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>11452110</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>إصدار تراخيص إستخدام أملاك خاصة لإقامة فعاليات</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>615913.99</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>34158.14</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>37005.64</v>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>181162.69</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>15698.85</v>
+      </c>
+      <c r="I33" s="6" t="n">
+        <v>118880.15</v>
+      </c>
+      <c r="J33" s="15">
+        <f>IFERROR(VLOOKUP(A33,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K33" s="6">
+        <f>MAX(0,F33*J33-E33)</f>
+        <v/>
+      </c>
+      <c r="L33" s="6">
+        <f>G33*J33</f>
+        <v/>
+      </c>
+      <c r="M33" s="6">
+        <f>D33+K33+L33</f>
+        <v/>
+      </c>
+      <c r="N33" s="6">
+        <f>MAX(0,H33*MIN(J33,1)-E33)</f>
+        <v/>
+      </c>
+      <c r="O33" s="6">
+        <f>I33*MIN(J33,1)</f>
+        <v/>
+      </c>
+      <c r="P33" s="6">
+        <f>D33+N33+O33</f>
+        <v/>
+      </c>
+      <c r="Q33" s="6" t="n">
+        <v>1281240</v>
+      </c>
+      <c r="R33" s="6" t="n">
+        <v>1369461.01</v>
+      </c>
+      <c r="S33" s="6">
+        <f>M33-Q33</f>
+        <v/>
+      </c>
+      <c r="T33" s="7">
+        <f>IF(R33=0,"",M33/R33)</f>
+        <v/>
+      </c>
+      <c r="U33" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>1422104</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>رسوم وأجور ناتجة من النشاط غير مصنفة أعلاه</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>391830</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M34" s="6">
+        <f>D34+K34+L34</f>
+        <v/>
+      </c>
+      <c r="N34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P34" s="6">
+        <f>D34+N34+O34</f>
+        <v/>
+      </c>
+      <c r="Q34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S34" s="6">
+        <f>M34-Q34</f>
+        <v/>
+      </c>
+      <c r="T34" s="7">
+        <f>IF(R34=0,"",M34/R34)</f>
+        <v/>
+      </c>
+      <c r="U34" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>3318212</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>مرتجع رواتب - فواتير</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>أخرى</t>
+        </is>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>216725.66</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J35" s="15">
+        <f>IFERROR(VLOOKUP(A35,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K35" s="6">
+        <f>MAX(0,F35*J35-E35)</f>
+        <v/>
+      </c>
+      <c r="L35" s="6">
+        <f>G35*J35</f>
+        <v/>
+      </c>
+      <c r="M35" s="6">
+        <f>D35+K35+L35</f>
+        <v/>
+      </c>
+      <c r="N35" s="6">
+        <f>MAX(0,H35*MIN(J35,1)-E35)</f>
+        <v/>
+      </c>
+      <c r="O35" s="6">
+        <f>I35*MIN(J35,1)</f>
+        <v/>
+      </c>
+      <c r="P35" s="6">
+        <f>D35+N35+O35</f>
+        <v/>
+      </c>
+      <c r="Q35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S35" s="6">
+        <f>M35-Q35</f>
+        <v/>
+      </c>
+      <c r="T35" s="7">
+        <f>IF(R35=0,"",M35/R35)</f>
+        <v/>
+      </c>
+      <c r="U35" s="5" t="inlineStr">
+        <is>
+          <t>الملف الشهري</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>1421903</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>مبيعات التيار الكهربائي</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>143551.39</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J36" s="15">
+        <f>IFERROR(VLOOKUP(A36,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K36" s="6">
+        <f>MAX(0,F36*J36-E36)</f>
+        <v/>
+      </c>
+      <c r="L36" s="6">
+        <f>G36*J36</f>
+        <v/>
+      </c>
+      <c r="M36" s="6">
+        <f>D36+K36+L36</f>
+        <v/>
+      </c>
+      <c r="N36" s="6">
+        <f>MAX(0,H36*MIN(J36,1)-E36)</f>
+        <v/>
+      </c>
+      <c r="O36" s="6">
+        <f>I36*MIN(J36,1)</f>
+        <v/>
+      </c>
+      <c r="P36" s="6">
+        <f>D36+N36+O36</f>
+        <v/>
+      </c>
+      <c r="Q36" s="6" t="n">
+        <v>2391821</v>
+      </c>
+      <c r="R36" s="6" t="n">
+        <v>2391821</v>
+      </c>
+      <c r="S36" s="6">
+        <f>M36-Q36</f>
+        <v/>
+      </c>
+      <c r="T36" s="7">
+        <f>IF(R36=0,"",M36/R36)</f>
+        <v/>
+      </c>
+      <c r="U36" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>141229</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>أرباح أخرى</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>120314</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>60314</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>40000</v>
+      </c>
+      <c r="H37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J37" s="15">
+        <f>IFERROR(VLOOKUP(A37,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K37" s="6">
+        <f>MAX(0,F37*J37-E37)</f>
+        <v/>
+      </c>
+      <c r="L37" s="6">
+        <f>G37*J37</f>
+        <v/>
+      </c>
+      <c r="M37" s="6">
+        <f>D37+K37+L37</f>
+        <v/>
+      </c>
+      <c r="N37" s="6">
+        <f>MAX(0,H37*MIN(J37,1)-E37)</f>
+        <v/>
+      </c>
+      <c r="O37" s="6">
+        <f>I37*MIN(J37,1)</f>
+        <v/>
+      </c>
+      <c r="P37" s="6">
+        <f>D37+N37+O37</f>
+        <v/>
+      </c>
+      <c r="Q37" s="6" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="R37" s="6" t="n">
+        <v>30000000</v>
+      </c>
+      <c r="S37" s="6">
+        <f>M37-Q37</f>
+        <v/>
+      </c>
+      <c r="T37" s="7">
+        <f>IF(R37=0,"",M37/R37)</f>
+        <v/>
+      </c>
+      <c r="U37" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>1438</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات مفروضة بموجب أنظمة الجهة</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>جزاءات وغرامات</t>
+        </is>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>59500</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>24000</v>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>51900</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>5000</v>
+      </c>
+      <c r="I38" s="6" t="n">
+        <v>32700</v>
+      </c>
+      <c r="J38" s="15">
+        <f>IFERROR(VLOOKUP(A38,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K38" s="6">
+        <f>MAX(0,F38*J38-E38)</f>
+        <v/>
+      </c>
+      <c r="L38" s="6">
+        <f>G38*J38</f>
+        <v/>
+      </c>
+      <c r="M38" s="6">
+        <f>D38+K38+L38</f>
+        <v/>
+      </c>
+      <c r="N38" s="6">
+        <f>MAX(0,H38*MIN(J38,1)-E38)</f>
+        <v/>
+      </c>
+      <c r="O38" s="6">
+        <f>I38*MIN(J38,1)</f>
+        <v/>
+      </c>
+      <c r="P38" s="6">
+        <f>D38+N38+O38</f>
+        <v/>
+      </c>
+      <c r="Q38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S38" s="6">
+        <f>M38-Q38</f>
+        <v/>
+      </c>
+      <c r="T38" s="7">
+        <f>IF(R38=0,"",M38/R38)</f>
+        <v/>
+      </c>
+      <c r="U38" s="5" t="inlineStr">
+        <is>
+          <t>الملف الشهري</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>1421907</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات المخططات</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>5950</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I39" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J39" s="15">
+        <f>IFERROR(VLOOKUP(A39,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K39" s="6">
+        <f>MAX(0,F39*J39-E39)</f>
+        <v/>
+      </c>
+      <c r="L39" s="6">
+        <f>G39*J39</f>
+        <v/>
+      </c>
+      <c r="M39" s="6">
+        <f>D39+K39+L39</f>
+        <v/>
+      </c>
+      <c r="N39" s="6">
+        <f>MAX(0,H39*MIN(J39,1)-E39)</f>
+        <v/>
+      </c>
+      <c r="O39" s="6">
+        <f>I39*MIN(J39,1)</f>
+        <v/>
+      </c>
+      <c r="P39" s="6">
+        <f>D39+N39+O39</f>
+        <v/>
+      </c>
+      <c r="Q39" s="6" t="n">
+        <v>614036.83</v>
+      </c>
+      <c r="R39" s="6" t="n">
+        <v>614036.83</v>
+      </c>
+      <c r="S39" s="6">
+        <f>M39-Q39</f>
+        <v/>
+      </c>
+      <c r="T39" s="7">
+        <f>IF(R39=0,"",M39/R39)</f>
+        <v/>
+      </c>
+      <c r="U39" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>11452105</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>رسوم تراخيص حفر الشوارع</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>3251093.38</v>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>3179964.38</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I40" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J40" s="15">
+        <f>IFERROR(VLOOKUP(A40,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K40" s="6">
+        <f>MAX(0,F40*J40-E40)</f>
+        <v/>
+      </c>
+      <c r="L40" s="6">
+        <f>G40*J40</f>
+        <v/>
+      </c>
+      <c r="M40" s="6">
+        <f>D40+K40+L40</f>
+        <v/>
+      </c>
+      <c r="N40" s="6">
+        <f>MAX(0,H40*MIN(J40,1)-E40)</f>
+        <v/>
+      </c>
+      <c r="O40" s="6">
+        <f>I40*MIN(J40,1)</f>
+        <v/>
+      </c>
+      <c r="P40" s="6">
+        <f>D40+N40+O40</f>
+        <v/>
+      </c>
+      <c r="Q40" s="6" t="n">
+        <v>200000</v>
+      </c>
+      <c r="R40" s="6" t="n">
+        <v>442058.1764705882</v>
+      </c>
+      <c r="S40" s="6">
+        <f>M40-Q40</f>
+        <v/>
+      </c>
+      <c r="T40" s="7">
+        <f>IF(R40=0,"",M40/R40)</f>
+        <v/>
+      </c>
+      <c r="U40" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>11452513</t>
+        </is>
+      </c>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>لوحات إرشـادية</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>600</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v>2100</v>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J41" s="15">
+        <f>IFERROR(VLOOKUP(A41,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K41" s="6">
+        <f>MAX(0,F41*J41-E41)</f>
+        <v/>
+      </c>
+      <c r="L41" s="6">
+        <f>G41*J41</f>
+        <v/>
+      </c>
+      <c r="M41" s="6">
+        <f>D41+K41+L41</f>
+        <v/>
+      </c>
+      <c r="N41" s="6">
+        <f>MAX(0,H41*MIN(J41,1)-E41)</f>
+        <v/>
+      </c>
+      <c r="O41" s="6">
+        <f>I41*MIN(J41,1)</f>
+        <v/>
+      </c>
+      <c r="P41" s="6">
+        <f>D41+N41+O41</f>
+        <v/>
+      </c>
+      <c r="Q41" s="6" t="n">
+        <v>66659.70999999999</v>
+      </c>
+      <c r="R41" s="6" t="n">
+        <v>66659</v>
+      </c>
+      <c r="S41" s="6">
+        <f>M41-Q41</f>
+        <v/>
+      </c>
+      <c r="T41" s="7">
+        <f>IF(R41=0,"",M41/R41)</f>
+        <v/>
+      </c>
+      <c r="U41" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>1422103</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>تراخيص المحلات</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>432</v>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>300</v>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>1479.6</v>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="6" t="n">
+        <v>228</v>
+      </c>
+      <c r="J42" s="15">
+        <f>IFERROR(VLOOKUP(A42,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K42" s="6">
+        <f>MAX(0,F42*J42-E42)</f>
+        <v/>
+      </c>
+      <c r="L42" s="6">
+        <f>G42*J42</f>
+        <v/>
+      </c>
+      <c r="M42" s="6">
+        <f>D42+K42+L42</f>
+        <v/>
+      </c>
+      <c r="N42" s="6">
+        <f>MAX(0,H42*MIN(J42,1)-E42)</f>
+        <v/>
+      </c>
+      <c r="O42" s="6">
+        <f>I42*MIN(J42,1)</f>
+        <v/>
+      </c>
+      <c r="P42" s="6">
+        <f>D42+N42+O42</f>
+        <v/>
+      </c>
+      <c r="Q42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S42" s="6">
+        <f>M42-Q42</f>
+        <v/>
+      </c>
+      <c r="T42" s="7">
+        <f>IF(R42=0,"",M42/R42)</f>
+        <v/>
+      </c>
+      <c r="U42" s="5" t="inlineStr">
+        <is>
+          <t>الملف الشهري</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>11452109</t>
+        </is>
+      </c>
+      <c r="B43" s="5" t="inlineStr">
+        <is>
+          <t>اعتماد مخططات التطوير العقاري</t>
+        </is>
+      </c>
+      <c r="C43" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>110295.92</v>
+      </c>
+      <c r="G43" s="6" t="n">
+        <v>6100</v>
+      </c>
+      <c r="H43" s="6" t="n">
+        <v>1600</v>
+      </c>
+      <c r="I43" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="J43" s="15">
+        <f>IFERROR(VLOOKUP(A43,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K43" s="6">
+        <f>MAX(0,F43*J43-E43)</f>
+        <v/>
+      </c>
+      <c r="L43" s="6">
+        <f>G43*J43</f>
+        <v/>
+      </c>
+      <c r="M43" s="6">
+        <f>D43+K43+L43</f>
+        <v/>
+      </c>
+      <c r="N43" s="6">
+        <f>MAX(0,H43*MIN(J43,1)-E43)</f>
+        <v/>
+      </c>
+      <c r="O43" s="6">
+        <f>I43*MIN(J43,1)</f>
+        <v/>
+      </c>
+      <c r="P43" s="6">
+        <f>D43+N43+O43</f>
+        <v/>
+      </c>
+      <c r="Q43" s="6" t="n">
+        <v>854382.67</v>
+      </c>
+      <c r="R43" s="6" t="n">
+        <v>854382.67</v>
+      </c>
+      <c r="S43" s="6">
+        <f>M43-Q43</f>
+        <v/>
+      </c>
+      <c r="T43" s="7">
+        <f>IF(R43=0,"",M43/R43)</f>
+        <v/>
+      </c>
+      <c r="U43" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>11422</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>رسوم منتجات التبغ</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>التبغ والإيواء</t>
+        </is>
+      </c>
+      <c r="D44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J44" s="15">
+        <f>IFERROR(VLOOKUP(A44,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K44" s="6">
+        <f>MAX(0,F44*J44-E44)</f>
+        <v/>
+      </c>
+      <c r="L44" s="6">
+        <f>G44*J44</f>
+        <v/>
+      </c>
+      <c r="M44" s="6">
+        <f>D44+K44+L44</f>
+        <v/>
+      </c>
+      <c r="N44" s="6">
+        <f>MAX(0,H44*MIN(J44,1)-E44)</f>
+        <v/>
+      </c>
+      <c r="O44" s="6">
+        <f>I44*MIN(J44,1)</f>
+        <v/>
+      </c>
+      <c r="P44" s="6">
+        <f>D44+N44+O44</f>
+        <v/>
+      </c>
+      <c r="Q44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S44" s="6">
+        <f>M44-Q44</f>
+        <v/>
+      </c>
+      <c r="T44" s="7">
+        <f>IF(R44=0,"",M44/R44)</f>
+        <v/>
+      </c>
+      <c r="U44" s="5" t="inlineStr">
+        <is>
+          <t>الملف الشهري</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>142161</t>
+        </is>
+      </c>
+      <c r="B45" s="5" t="inlineStr">
+        <is>
+          <t>تاجير مباني سكنية</t>
+        </is>
+      </c>
+      <c r="C45" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J45" s="15">
+        <f>IFERROR(VLOOKUP(A45,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K45" s="6">
+        <f>MAX(0,F45*J45-E45)</f>
+        <v/>
+      </c>
+      <c r="L45" s="6">
+        <f>G45*J45</f>
+        <v/>
+      </c>
+      <c r="M45" s="6">
+        <f>D45+K45+L45</f>
+        <v/>
+      </c>
+      <c r="N45" s="6">
+        <f>MAX(0,H45*MIN(J45,1)-E45)</f>
+        <v/>
+      </c>
+      <c r="O45" s="6">
+        <f>I45*MIN(J45,1)</f>
+        <v/>
+      </c>
+      <c r="P45" s="6">
+        <f>D45+N45+O45</f>
+        <v/>
+      </c>
+      <c r="Q45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S45" s="6">
+        <f>M45-Q45</f>
+        <v/>
+      </c>
+      <c r="T45" s="7">
+        <f>IF(R45=0,"",M45/R45)</f>
+        <v/>
+      </c>
+      <c r="U45" s="5" t="inlineStr">
+        <is>
+          <t>الملف الشهري</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>1421908</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>ايرادات  رسوم خدمات  بلدية</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>إيرادات إستثمارية</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="15">
+        <f>IFERROR(VLOOKUP(A46,'توقع المحصل الموسمي'!$A$6:$J$43,10,FALSE),1)</f>
+        <v/>
+      </c>
+      <c r="K46" s="6">
+        <f>MAX(0,F46*J46-E46)</f>
+        <v/>
+      </c>
+      <c r="L46" s="6">
+        <f>G46*J46</f>
+        <v/>
+      </c>
+      <c r="M46" s="6">
+        <f>D46+K46+L46</f>
+        <v/>
+      </c>
+      <c r="N46" s="6">
+        <f>MAX(0,H46*MIN(J46,1)-E46)</f>
+        <v/>
+      </c>
+      <c r="O46" s="6">
+        <f>I46*MIN(J46,1)</f>
+        <v/>
+      </c>
+      <c r="P46" s="6">
+        <f>D46+N46+O46</f>
+        <v/>
+      </c>
+      <c r="Q46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S46" s="6">
+        <f>M46-Q46</f>
+        <v/>
+      </c>
+      <c r="T46" s="7">
+        <f>IF(R46=0,"",M46/R46)</f>
+        <v/>
+      </c>
+      <c r="U46" s="5" t="inlineStr">
+        <is>
+          <t>الملف الشهري</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>1422112</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>إصدار رخصة</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J47" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M47" s="6">
+        <f>D47+K47+L47</f>
+        <v/>
+      </c>
+      <c r="N47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P47" s="6">
+        <f>D47+N47+O47</f>
+        <v/>
+      </c>
+      <c r="Q47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S47" s="6">
+        <f>M47-Q47</f>
+        <v/>
+      </c>
+      <c r="T47" s="7">
+        <f>IF(R47=0,"",M47/R47)</f>
+        <v/>
+      </c>
+      <c r="U47" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>1422199</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>رسوم الخدمات العامة الأخرى</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>الرسوم والتراخيص</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M48" s="6">
+        <f>D48+K48+L48</f>
+        <v/>
+      </c>
+      <c r="N48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="O48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P48" s="6">
+        <f>D48+N48+O48</f>
+        <v/>
+      </c>
+      <c r="Q48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="R48" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="S48" s="6">
+        <f>M48-Q48</f>
+        <v/>
+      </c>
+      <c r="T48" s="7">
+        <f>IF(R48=0,"",M48/R48)</f>
+        <v/>
+      </c>
+      <c r="U48" s="5" t="inlineStr">
+        <is>
+          <t>ملف المراقبة</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="8" t="n"/>
+      <c r="B49" s="8" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="C49" s="8" t="n"/>
+      <c r="D49" s="9">
+        <f>SUM(D6:D48)</f>
+        <v/>
+      </c>
+      <c r="E49" s="9">
+        <f>SUM(E6:E48)</f>
+        <v/>
+      </c>
+      <c r="F49" s="9" t="n"/>
+      <c r="G49" s="9" t="n"/>
+      <c r="H49" s="9" t="n"/>
+      <c r="I49" s="9" t="n"/>
+      <c r="J49" s="17" t="n"/>
+      <c r="K49" s="9">
+        <f>SUM(K6:K48)</f>
+        <v/>
+      </c>
+      <c r="L49" s="9">
+        <f>SUM(L6:L48)</f>
+        <v/>
+      </c>
+      <c r="M49" s="9">
+        <f>SUM(M6:M48)</f>
+        <v/>
+      </c>
+      <c r="N49" s="9">
+        <f>SUM(N6:N48)</f>
+        <v/>
+      </c>
+      <c r="O49" s="9">
+        <f>SUM(O6:O48)</f>
+        <v/>
+      </c>
+      <c r="P49" s="9">
+        <f>SUM(P6:P48)</f>
+        <v/>
+      </c>
+      <c r="Q49" s="9">
+        <f>SUM(Q6:Q48)</f>
+        <v/>
+      </c>
+      <c r="R49" s="9">
+        <f>SUM(R6:R48)</f>
+        <v/>
+      </c>
+      <c r="S49" s="9">
+        <f>SUM(S6:S48)</f>
+        <v/>
+      </c>
+      <c r="T49" s="10">
+        <f>M49/R49</f>
+        <v/>
+      </c>
+      <c r="U49" s="8" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A5:U48"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:U2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -13846,6 +17626,13 @@
     <row r="20">
       <c r="A20" s="22" t="inlineStr">
         <is>
+          <t>6f) ورقة "توقع المحصل (المراقبة)": الفعلي يناير–أكتوبر 2026 من ملف المراقبة (ورقة الإجمالي، قبل الاستقطاع)، ثم متبقي أكتوبر ونوفمبر وديسمبر بالموسمية الشهرية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
           <t>7) تنبيه: كثير من الحسابات تتذبذب بشدة بين السنوات (لوحات دعائية، تأجير المرافق، إيرادات متنوعة)، ومضاعفة 2026 على 12/9 تضخّم أو تقلّل هذه الأرقام؛ انظر عمود "تنبيه".</t>
         </is>
       </c>

</xml_diff>

<commit_message>
Add 2023-2026 collected-by-account sheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/توقع_الفوترة_2026_2027.xlsx
+++ b/توقع_الفوترة_2026_2027.xlsx
@@ -15,7 +15,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="توقع المحصل الموسمي" sheetId="6" state="visible" r:id="rId6"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الموسمية الشهرية" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="توقع المحصل (المراقبة)" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المحصل 2023-2026" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'التوقعات'!$A$3:$R$41</definedName>
@@ -23,6 +24,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'تحليل التوقع والأسوأ'!$A$4:$O$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'توقع المحصل الموسمي'!$A$5:$Q$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'توقع المحصل (المراقبة)'!$A$5:$U$48</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'المحصل 2023-2026'!$A$4:$M$47</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -3464,6 +3466,217 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="60" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>الافتراضات (الخلايا الصفراء قابلة للتعديل)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="42" customHeight="1">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>البند</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>القيمة</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>ملاحظة</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>معامل تحويل 2026 إلى سنة كاملة (12÷9)</t>
+        </is>
+      </c>
+      <c r="B4" s="19">
+        <f>12/9</f>
+        <v/>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>المتاح فعلياً 9 أشهر (يناير–سبتمبر 2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>نسبة النمو – السيناريو الأول (ثابتة)</t>
+        </is>
+      </c>
+      <c r="B5" s="20">
+        <f>التوقعات!C2</f>
+        <v/>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>تُعدَّل من خلية C2 في ورقة التوقعات</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>سقف معدل النمو التاريخي (±)</t>
+        </is>
+      </c>
+      <c r="B6" s="20" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>لتفادي القفزات الكبيرة في الحسابات المتذبذبة؛ قابل للتعديل</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>أدنى معامل اتجاه 2026 (توقع المحصل الموسمي)</t>
+        </is>
+      </c>
+      <c r="B7" s="21" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>يحدّ أثر انخفاض 2026 عن متوسط السنوات السابقة</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>أعلى معامل اتجاه 2026 (توقع المحصل الموسمي)</t>
+        </is>
+      </c>
+      <c r="B8" s="21" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>يحدّ أثر ارتفاع 2026 عن متوسط السنوات السابقة</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>منهجية الحساب:</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="22" t="inlineStr">
+        <is>
+          <t>1) الإجمالي المفوتر للحساب = المفوتر + المحصل عن سنوات سابقة (حسب طلبك).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="22" t="inlineStr">
+        <is>
+          <t>2) توقع 2026 = الفعلي حتى سبتمبر × 12/9 (لا توجد بيانات شهرية، فلا موسمية في التوقع).</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="22" t="inlineStr">
+        <is>
+          <t>3) الحسابات التي فوترتها وتحصيلها صفر في 2026 تُعتبر متوقفة وتوقعها صفر في 2026 و2027.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="22" t="inlineStr">
+        <is>
+          <t>4) 2027 – السيناريو الأول: توقع 2026 × (1 + نسبة النمو في خلية C2 بورقة التوقعات؛ الافتراضي 7%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="22" t="inlineStr">
+        <is>
+          <t>5) 2027 – السيناريو الثاني: توقع 2026 × (1 + معدل النمو السنوي المركب التاريخي للحساب بين أول سنة فيها فوترة و2025، بسقف ±25%). إن توفرت سنة واحدة فقط من البيانات = نمو 0%.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="22" t="inlineStr">
+        <is>
+          <t>6) تم استبعاد حساب قيمة الضريبة المضافة (11411) من كل الحسابات والإجماليات.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="22" t="inlineStr">
+        <is>
+          <t>6b) تم دمج صفّي "بدون رقم" (خدمات علم + جزاءات، وجزاءات جزء ضئيل) في صف واحد لكل سنة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="22" t="inlineStr">
+        <is>
+          <t>6c) أعمدة النمو لكل حساب: نمو كل سنة عن السنة السابقة (2024 عن 2023، 2025 عن 2024، 2026 توقع عن 2025، و2027 عن 2026 للسيناريوهين). تظهر فارغة عندما تكون السنة السابقة صفراً.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="22" t="inlineStr">
+        <is>
+          <t>6d) ورقة "توقع المحصل 2026": توقع إقفال 2026 كمحصّل فعلي = المحصل حتى سبتمبر × 12÷9 (مسدد عن السنة + محصل سنوات سابقة).</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="22" t="inlineStr">
+        <is>
+          <t>6e) إعادة تصنيف المحصل: حسب تأكيد المستخدم، نُقل 913م من محصل 2025 في حساب اللوحات الدعائية (142113) إلى تأجير المرافق (142162) (كلها من إدارة الدعم المالي: مايو 291م ونوفمبر 594م). ينطبق على أوراق المحصل فقط؛ أوراق الفوترة لم تُعدّل لأن مبالغ الفوترة حسب الجهة غير متوفرة. إن كانت دفعات إدارة الدعم المالي في 2024 (يوليو 312م، نوفمبر 25م، ديسمبر 102م) من نفس النوع فالتوقع الأساسي يرتفع (انظر الرد).</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="22" t="inlineStr">
+        <is>
+          <t>6f) ورقة "توقع المحصل (المراقبة)": الفعلي يناير–أكتوبر 2026 من ملف المراقبة (ورقة الإجمالي، قبل الاستقطاع)، ثم متبقي أكتوبر ونوفمبر وديسمبر بالموسمية الشهرية.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="22" t="inlineStr">
+        <is>
+          <t>7) تنبيه: كثير من الحسابات تتذبذب بشدة بين السنوات (لوحات دعائية، تأجير المرافق، إيرادات متنوعة)، ومضاعفة 2026 على 12/9 تضخّم أو تقلّل هذه الأرقام؛ انظر عمود "تنبيه".</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -17437,207 +17650,2395 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:M48"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>الافتراضات (الخلايا الصفراء قابلة للتعديل)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="42" customHeight="1">
-      <c r="A3" s="4" t="inlineStr">
-        <is>
-          <t>البند</t>
-        </is>
-      </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>القيمة</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>ملاحظة</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>معامل تحويل 2026 إلى سنة كاملة (12÷9)</t>
-        </is>
-      </c>
-      <c r="B4" s="19">
-        <f>12/9</f>
-        <v/>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>المتاح فعلياً 9 أشهر (يناير–سبتمبر 2026)</t>
+          <t>المحصل الفعلي لكل حساب 2023–2025 وإقفال 2026 (بدون الضريبة)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>2023 و2024 و2025 = المحصل الكامل للسنة من الملف الشهري (2025 بعد نقل 913م من اللوحات الدعائية إلى تأجير المرافق؛ 2023 و2024 كما هي بدون إعادة تصنيف). 2026 = الفعلي يناير–أكتوبر من ملف المراقبة (قبل الاستقطاع) وإقفال 2026 أساسي وأسوأ من ورقة "توقع المحصل (المراقبة)". اختلاف مصدر الفعلي (المراقبة تشمل التوريد والمستقطع) يجعل مقارنة 2026 بما قبله أعلى قليلاً.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>رقم الحساب</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>اسم الحساب</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>التبويب</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>2023 محصّل</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>2024 محصّل</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>2025 محصّل</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>2026 الفعلي حتى أكتوبر</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>2026 إقفال أساسي</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>2026 إقفال أسوأ</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>نمو 2024 عن 2023</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>نمو 2025 عن 2024</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>نمو 2026 (أساسي) عن 2025</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>نمو 2026 (أسوأ) عن 2025</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>نسبة النمو – السيناريو الأول (ثابتة)</t>
-        </is>
-      </c>
-      <c r="B5" s="20">
-        <f>التوقعات!C2</f>
-        <v/>
-      </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>تُعدَّل من خلية C2 في ورقة التوقعات</t>
-        </is>
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>14155</t>
+        </is>
+      </c>
+      <c r="B5" s="5">
+        <f>'توقع المحصل (المراقبة)'!B6</f>
+        <v/>
+      </c>
+      <c r="C5" s="5">
+        <f>'توقع المحصل (المراقبة)'!C6</f>
+        <v/>
+      </c>
+      <c r="D5" s="6" t="n">
+        <v>779186906.26</v>
+      </c>
+      <c r="E5" s="6" t="n">
+        <v>803323461.12</v>
+      </c>
+      <c r="F5" s="6" t="n">
+        <v>649331791.52</v>
+      </c>
+      <c r="G5" s="6">
+        <f>'توقع المحصل (المراقبة)'!D6</f>
+        <v/>
+      </c>
+      <c r="H5" s="6">
+        <f>'توقع المحصل (المراقبة)'!M6</f>
+        <v/>
+      </c>
+      <c r="I5" s="6">
+        <f>'توقع المحصل (المراقبة)'!P6</f>
+        <v/>
+      </c>
+      <c r="J5" s="7">
+        <f>IF(D5=0,"",E5/D5-1)</f>
+        <v/>
+      </c>
+      <c r="K5" s="7">
+        <f>IF(E5=0,"",F5/E5-1)</f>
+        <v/>
+      </c>
+      <c r="L5" s="7">
+        <f>IF(F5=0,"",H5/F5-1)</f>
+        <v/>
+      </c>
+      <c r="M5" s="7">
+        <f>IF(F5=0,"",I5/F5-1)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>سقف معدل النمو التاريخي (±)</t>
-        </is>
-      </c>
-      <c r="B6" s="20" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="C6" t="inlineStr">
-        <is>
-          <t>لتفادي القفزات الكبيرة في الحسابات المتذبذبة؛ قابل للتعديل</t>
-        </is>
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>142162</t>
+        </is>
+      </c>
+      <c r="B6" s="5">
+        <f>'توقع المحصل (المراقبة)'!B7</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>'توقع المحصل (المراقبة)'!C7</f>
+        <v/>
+      </c>
+      <c r="D6" s="6" t="n">
+        <v>29573714.25</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <v>45452213.03</v>
+      </c>
+      <c r="F6" s="6" t="n">
+        <v>938889683.7</v>
+      </c>
+      <c r="G6" s="6">
+        <f>'توقع المحصل (المراقبة)'!D7</f>
+        <v/>
+      </c>
+      <c r="H6" s="6">
+        <f>'توقع المحصل (المراقبة)'!M7</f>
+        <v/>
+      </c>
+      <c r="I6" s="6">
+        <f>'توقع المحصل (المراقبة)'!P7</f>
+        <v/>
+      </c>
+      <c r="J6" s="7">
+        <f>IF(D6=0,"",E6/D6-1)</f>
+        <v/>
+      </c>
+      <c r="K6" s="7">
+        <f>IF(E6=0,"",F6/E6-1)</f>
+        <v/>
+      </c>
+      <c r="L6" s="7">
+        <f>IF(F6=0,"",H6/F6-1)</f>
+        <v/>
+      </c>
+      <c r="M6" s="7">
+        <f>IF(F6=0,"",I6/F6-1)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>أدنى معامل اتجاه 2026 (توقع المحصل الموسمي)</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>يحدّ أثر انخفاض 2026 عن متوسط السنوات السابقة</t>
-        </is>
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>1438001</t>
+        </is>
+      </c>
+      <c r="B7" s="5">
+        <f>'توقع المحصل (المراقبة)'!B8</f>
+        <v/>
+      </c>
+      <c r="C7" s="5">
+        <f>'توقع المحصل (المراقبة)'!C8</f>
+        <v/>
+      </c>
+      <c r="D7" s="6" t="n">
+        <v>459891610.83</v>
+      </c>
+      <c r="E7" s="6" t="n">
+        <v>303585685.79</v>
+      </c>
+      <c r="F7" s="6" t="n">
+        <v>308012204.69</v>
+      </c>
+      <c r="G7" s="6">
+        <f>'توقع المحصل (المراقبة)'!D8</f>
+        <v/>
+      </c>
+      <c r="H7" s="6">
+        <f>'توقع المحصل (المراقبة)'!M8</f>
+        <v/>
+      </c>
+      <c r="I7" s="6">
+        <f>'توقع المحصل (المراقبة)'!P8</f>
+        <v/>
+      </c>
+      <c r="J7" s="7">
+        <f>IF(D7=0,"",E7/D7-1)</f>
+        <v/>
+      </c>
+      <c r="K7" s="7">
+        <f>IF(E7=0,"",F7/E7-1)</f>
+        <v/>
+      </c>
+      <c r="L7" s="7">
+        <f>IF(F7=0,"",H7/F7-1)</f>
+        <v/>
+      </c>
+      <c r="M7" s="7">
+        <f>IF(F7=0,"",I7/F7-1)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>أعلى معامل اتجاه 2026 (توقع المحصل الموسمي)</t>
-        </is>
-      </c>
-      <c r="B8" s="21" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>يحدّ أثر ارتفاع 2026 عن متوسط السنوات السابقة</t>
-        </is>
+      <c r="A8" s="5" t="inlineStr">
+        <is>
+          <t>11452104</t>
+        </is>
+      </c>
+      <c r="B8" s="5">
+        <f>'توقع المحصل (المراقبة)'!B9</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>'توقع المحصل (المراقبة)'!C9</f>
+        <v/>
+      </c>
+      <c r="D8" s="6" t="n">
+        <v>260667489.98</v>
+      </c>
+      <c r="E8" s="6" t="n">
+        <v>276275913.44</v>
+      </c>
+      <c r="F8" s="6" t="n">
+        <v>267496278.85</v>
+      </c>
+      <c r="G8" s="6">
+        <f>'توقع المحصل (المراقبة)'!D9</f>
+        <v/>
+      </c>
+      <c r="H8" s="6">
+        <f>'توقع المحصل (المراقبة)'!M9</f>
+        <v/>
+      </c>
+      <c r="I8" s="6">
+        <f>'توقع المحصل (المراقبة)'!P9</f>
+        <v/>
+      </c>
+      <c r="J8" s="7">
+        <f>IF(D8=0,"",E8/D8-1)</f>
+        <v/>
+      </c>
+      <c r="K8" s="7">
+        <f>IF(E8=0,"",F8/E8-1)</f>
+        <v/>
+      </c>
+      <c r="L8" s="7">
+        <f>IF(F8=0,"",H8/F8-1)</f>
+        <v/>
+      </c>
+      <c r="M8" s="7">
+        <f>IF(F8=0,"",I8/F8-1)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>منهجية الحساب:</t>
-        </is>
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>11452103</t>
+        </is>
+      </c>
+      <c r="B9" s="5">
+        <f>'توقع المحصل (المراقبة)'!B10</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>'توقع المحصل (المراقبة)'!C10</f>
+        <v/>
+      </c>
+      <c r="D9" s="6" t="n">
+        <v>224939645.24</v>
+      </c>
+      <c r="E9" s="6" t="n">
+        <v>244582493.3</v>
+      </c>
+      <c r="F9" s="6" t="n">
+        <v>319675274.54</v>
+      </c>
+      <c r="G9" s="6">
+        <f>'توقع المحصل (المراقبة)'!D10</f>
+        <v/>
+      </c>
+      <c r="H9" s="6">
+        <f>'توقع المحصل (المراقبة)'!M10</f>
+        <v/>
+      </c>
+      <c r="I9" s="6">
+        <f>'توقع المحصل (المراقبة)'!P10</f>
+        <v/>
+      </c>
+      <c r="J9" s="7">
+        <f>IF(D9=0,"",E9/D9-1)</f>
+        <v/>
+      </c>
+      <c r="K9" s="7">
+        <f>IF(E9=0,"",F9/E9-1)</f>
+        <v/>
+      </c>
+      <c r="L9" s="7">
+        <f>IF(F9=0,"",H9/F9-1)</f>
+        <v/>
+      </c>
+      <c r="M9" s="7">
+        <f>IF(F9=0,"",I9/F9-1)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
-        <is>
-          <t>1) الإجمالي المفوتر للحساب = المفوتر + المحصل عن سنوات سابقة (حسب طلبك).</t>
-        </is>
+      <c r="A10" s="5" t="inlineStr">
+        <is>
+          <t>11452512</t>
+        </is>
+      </c>
+      <c r="B10" s="5">
+        <f>'توقع المحصل (المراقبة)'!B11</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>'توقع المحصل (المراقبة)'!C11</f>
+        <v/>
+      </c>
+      <c r="D10" s="6" t="n">
+        <v>218503365</v>
+      </c>
+      <c r="E10" s="6" t="n">
+        <v>219218740</v>
+      </c>
+      <c r="F10" s="6" t="n">
+        <v>193830778.44</v>
+      </c>
+      <c r="G10" s="6">
+        <f>'توقع المحصل (المراقبة)'!D11</f>
+        <v/>
+      </c>
+      <c r="H10" s="6">
+        <f>'توقع المحصل (المراقبة)'!M11</f>
+        <v/>
+      </c>
+      <c r="I10" s="6">
+        <f>'توقع المحصل (المراقبة)'!P11</f>
+        <v/>
+      </c>
+      <c r="J10" s="7">
+        <f>IF(D10=0,"",E10/D10-1)</f>
+        <v/>
+      </c>
+      <c r="K10" s="7">
+        <f>IF(E10=0,"",F10/E10-1)</f>
+        <v/>
+      </c>
+      <c r="L10" s="7">
+        <f>IF(F10=0,"",H10/F10-1)</f>
+        <v/>
+      </c>
+      <c r="M10" s="7">
+        <f>IF(F10=0,"",I10/F10-1)</f>
+        <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="inlineStr">
-        <is>
-          <t>2) توقع 2026 = الفعلي حتى سبتمبر × 12/9 (لا توجد بيانات شهرية، فلا موسمية في التوقع).</t>
-        </is>
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>1439</t>
+        </is>
+      </c>
+      <c r="B11" s="5">
+        <f>'توقع المحصل (المراقبة)'!B12</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>'توقع المحصل (المراقبة)'!C12</f>
+        <v/>
+      </c>
+      <c r="D11" s="6" t="n">
+        <v>3537100</v>
+      </c>
+      <c r="E11" s="6" t="n">
+        <v>227000</v>
+      </c>
+      <c r="F11" s="6" t="n">
+        <v>8503508</v>
+      </c>
+      <c r="G11" s="6">
+        <f>'توقع المحصل (المراقبة)'!D12</f>
+        <v/>
+      </c>
+      <c r="H11" s="6">
+        <f>'توقع المحصل (المراقبة)'!M12</f>
+        <v/>
+      </c>
+      <c r="I11" s="6">
+        <f>'توقع المحصل (المراقبة)'!P12</f>
+        <v/>
+      </c>
+      <c r="J11" s="7">
+        <f>IF(D11=0,"",E11/D11-1)</f>
+        <v/>
+      </c>
+      <c r="K11" s="7">
+        <f>IF(E11=0,"",F11/E11-1)</f>
+        <v/>
+      </c>
+      <c r="L11" s="7">
+        <f>IF(F11=0,"",H11/F11-1)</f>
+        <v/>
+      </c>
+      <c r="M11" s="7">
+        <f>IF(F11=0,"",I11/F11-1)</f>
+        <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
-        <is>
-          <t>3) الحسابات التي فوترتها وتحصيلها صفر في 2026 تُعتبر متوقفة وتوقعها صفر في 2026 و2027.</t>
-        </is>
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>11442</t>
+        </is>
+      </c>
+      <c r="B12" s="5">
+        <f>'توقع المحصل (المراقبة)'!B13</f>
+        <v/>
+      </c>
+      <c r="C12" s="5">
+        <f>'توقع المحصل (المراقبة)'!C13</f>
+        <v/>
+      </c>
+      <c r="D12" s="6" t="n">
+        <v>219905861.19</v>
+      </c>
+      <c r="E12" s="6" t="n">
+        <v>256726800.98</v>
+      </c>
+      <c r="F12" s="6" t="n">
+        <v>199149669.75</v>
+      </c>
+      <c r="G12" s="6">
+        <f>'توقع المحصل (المراقبة)'!D13</f>
+        <v/>
+      </c>
+      <c r="H12" s="6">
+        <f>'توقع المحصل (المراقبة)'!M13</f>
+        <v/>
+      </c>
+      <c r="I12" s="6">
+        <f>'توقع المحصل (المراقبة)'!P13</f>
+        <v/>
+      </c>
+      <c r="J12" s="7">
+        <f>IF(D12=0,"",E12/D12-1)</f>
+        <v/>
+      </c>
+      <c r="K12" s="7">
+        <f>IF(E12=0,"",F12/E12-1)</f>
+        <v/>
+      </c>
+      <c r="L12" s="7">
+        <f>IF(F12=0,"",H12/F12-1)</f>
+        <v/>
+      </c>
+      <c r="M12" s="7">
+        <f>IF(F12=0,"",I12/F12-1)</f>
+        <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
-        <is>
-          <t>4) 2027 – السيناريو الأول: توقع 2026 × (1 + نسبة النمو في خلية C2 بورقة التوقعات؛ الافتراضي 7%).</t>
-        </is>
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>1421999</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>'توقع المحصل (المراقبة)'!B14</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>'توقع المحصل (المراقبة)'!C14</f>
+        <v/>
+      </c>
+      <c r="D13" s="6" t="n">
+        <v>110542302.74</v>
+      </c>
+      <c r="E13" s="6" t="n">
+        <v>106593084.61</v>
+      </c>
+      <c r="F13" s="6" t="n">
+        <v>60096373.96</v>
+      </c>
+      <c r="G13" s="6">
+        <f>'توقع المحصل (المراقبة)'!D14</f>
+        <v/>
+      </c>
+      <c r="H13" s="6">
+        <f>'توقع المحصل (المراقبة)'!M14</f>
+        <v/>
+      </c>
+      <c r="I13" s="6">
+        <f>'توقع المحصل (المراقبة)'!P14</f>
+        <v/>
+      </c>
+      <c r="J13" s="7">
+        <f>IF(D13=0,"",E13/D13-1)</f>
+        <v/>
+      </c>
+      <c r="K13" s="7">
+        <f>IF(E13=0,"",F13/E13-1)</f>
+        <v/>
+      </c>
+      <c r="L13" s="7">
+        <f>IF(F13=0,"",H13/F13-1)</f>
+        <v/>
+      </c>
+      <c r="M13" s="7">
+        <f>IF(F13=0,"",I13/F13-1)</f>
+        <v/>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="inlineStr">
-        <is>
-          <t>5) 2027 – السيناريو الثاني: توقع 2026 × (1 + معدل النمو السنوي المركب التاريخي للحساب بين أول سنة فيها فوترة و2025، بسقف ±25%). إن توفرت سنة واحدة فقط من البيانات = نمو 0%.</t>
-        </is>
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>142113</t>
+        </is>
+      </c>
+      <c r="B14" s="5">
+        <f>'توقع المحصل (المراقبة)'!B15</f>
+        <v/>
+      </c>
+      <c r="C14" s="5">
+        <f>'توقع المحصل (المراقبة)'!C15</f>
+        <v/>
+      </c>
+      <c r="D14" s="6" t="n">
+        <v>157946538.8</v>
+      </c>
+      <c r="E14" s="6" t="n">
+        <v>609523702.9299999</v>
+      </c>
+      <c r="F14" s="6" t="n">
+        <v>103589976.04</v>
+      </c>
+      <c r="G14" s="6">
+        <f>'توقع المحصل (المراقبة)'!D15</f>
+        <v/>
+      </c>
+      <c r="H14" s="6">
+        <f>'توقع المحصل (المراقبة)'!M15</f>
+        <v/>
+      </c>
+      <c r="I14" s="6">
+        <f>'توقع المحصل (المراقبة)'!P15</f>
+        <v/>
+      </c>
+      <c r="J14" s="7">
+        <f>IF(D14=0,"",E14/D14-1)</f>
+        <v/>
+      </c>
+      <c r="K14" s="7">
+        <f>IF(E14=0,"",F14/E14-1)</f>
+        <v/>
+      </c>
+      <c r="L14" s="7">
+        <f>IF(F14=0,"",H14/F14-1)</f>
+        <v/>
+      </c>
+      <c r="M14" s="7">
+        <f>IF(F14=0,"",I14/F14-1)</f>
+        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
-        <is>
-          <t>6) تم استبعاد حساب قيمة الضريبة المضافة (11411) من كل الحسابات والإجماليات.</t>
-        </is>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>1431</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>'توقع المحصل (المراقبة)'!B16</f>
+        <v/>
+      </c>
+      <c r="C15" s="5">
+        <f>'توقع المحصل (المراقبة)'!C16</f>
+        <v/>
+      </c>
+      <c r="D15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="6">
+        <f>'توقع المحصل (المراقبة)'!D16</f>
+        <v/>
+      </c>
+      <c r="H15" s="6">
+        <f>'توقع المحصل (المراقبة)'!M16</f>
+        <v/>
+      </c>
+      <c r="I15" s="6">
+        <f>'توقع المحصل (المراقبة)'!P16</f>
+        <v/>
+      </c>
+      <c r="J15" s="7">
+        <f>IF(D15=0,"",E15/D15-1)</f>
+        <v/>
+      </c>
+      <c r="K15" s="7">
+        <f>IF(E15=0,"",F15/E15-1)</f>
+        <v/>
+      </c>
+      <c r="L15" s="7">
+        <f>IF(F15=0,"",H15/F15-1)</f>
+        <v/>
+      </c>
+      <c r="M15" s="7">
+        <f>IF(F15=0,"",I15/F15-1)</f>
+        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
-        <is>
-          <t>6b) تم دمج صفّي "بدون رقم" (خدمات علم + جزاءات، وجزاءات جزء ضئيل) في صف واحد لكل سنة.</t>
-        </is>
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>1421909</t>
+        </is>
+      </c>
+      <c r="B16" s="5">
+        <f>'توقع المحصل (المراقبة)'!B17</f>
+        <v/>
+      </c>
+      <c r="C16" s="5">
+        <f>'توقع المحصل (المراقبة)'!C17</f>
+        <v/>
+      </c>
+      <c r="D16" s="6" t="n">
+        <v>72026385.34999999</v>
+      </c>
+      <c r="E16" s="6" t="n">
+        <v>76106716.86</v>
+      </c>
+      <c r="F16" s="6" t="n">
+        <v>72842923.63</v>
+      </c>
+      <c r="G16" s="6">
+        <f>'توقع المحصل (المراقبة)'!D17</f>
+        <v/>
+      </c>
+      <c r="H16" s="6">
+        <f>'توقع المحصل (المراقبة)'!M17</f>
+        <v/>
+      </c>
+      <c r="I16" s="6">
+        <f>'توقع المحصل (المراقبة)'!P17</f>
+        <v/>
+      </c>
+      <c r="J16" s="7">
+        <f>IF(D16=0,"",E16/D16-1)</f>
+        <v/>
+      </c>
+      <c r="K16" s="7">
+        <f>IF(E16=0,"",F16/E16-1)</f>
+        <v/>
+      </c>
+      <c r="L16" s="7">
+        <f>IF(F16=0,"",H16/F16-1)</f>
+        <v/>
+      </c>
+      <c r="M16" s="7">
+        <f>IF(F16=0,"",I16/F16-1)</f>
+        <v/>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
-        <is>
-          <t>6c) أعمدة النمو لكل حساب: نمو كل سنة عن السنة السابقة (2024 عن 2023، 2025 عن 2024، 2026 توقع عن 2025، و2027 عن 2026 للسيناريوهين). تظهر فارغة عندما تكون السنة السابقة صفراً.</t>
-        </is>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>1421911</t>
+        </is>
+      </c>
+      <c r="B17" s="5">
+        <f>'توقع المحصل (المراقبة)'!B18</f>
+        <v/>
+      </c>
+      <c r="C17" s="5">
+        <f>'توقع المحصل (المراقبة)'!C18</f>
+        <v/>
+      </c>
+      <c r="D17" s="6" t="n">
+        <v>65864668.18</v>
+      </c>
+      <c r="E17" s="6" t="n">
+        <v>79278364.97</v>
+      </c>
+      <c r="F17" s="6" t="n">
+        <v>67630101.28</v>
+      </c>
+      <c r="G17" s="6">
+        <f>'توقع المحصل (المراقبة)'!D18</f>
+        <v/>
+      </c>
+      <c r="H17" s="6">
+        <f>'توقع المحصل (المراقبة)'!M18</f>
+        <v/>
+      </c>
+      <c r="I17" s="6">
+        <f>'توقع المحصل (المراقبة)'!P18</f>
+        <v/>
+      </c>
+      <c r="J17" s="7">
+        <f>IF(D17=0,"",E17/D17-1)</f>
+        <v/>
+      </c>
+      <c r="K17" s="7">
+        <f>IF(E17=0,"",F17/E17-1)</f>
+        <v/>
+      </c>
+      <c r="L17" s="7">
+        <f>IF(F17=0,"",H17/F17-1)</f>
+        <v/>
+      </c>
+      <c r="M17" s="7">
+        <f>IF(F17=0,"",I17/F17-1)</f>
+        <v/>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr">
-        <is>
-          <t>6d) ورقة "توقع المحصل 2026": توقع إقفال 2026 كمحصّل فعلي = المحصل حتى سبتمبر × 12÷9 (مسدد عن السنة + محصل سنوات سابقة).</t>
-        </is>
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>144122</t>
+        </is>
+      </c>
+      <c r="B18" s="5">
+        <f>'توقع المحصل (المراقبة)'!B19</f>
+        <v/>
+      </c>
+      <c r="C18" s="5">
+        <f>'توقع المحصل (المراقبة)'!C19</f>
+        <v/>
+      </c>
+      <c r="D18" s="6" t="n">
+        <v>8992323.98</v>
+      </c>
+      <c r="E18" s="6" t="n">
+        <v>8297789.75</v>
+      </c>
+      <c r="F18" s="6" t="n">
+        <v>2477531.42</v>
+      </c>
+      <c r="G18" s="6">
+        <f>'توقع المحصل (المراقبة)'!D19</f>
+        <v/>
+      </c>
+      <c r="H18" s="6">
+        <f>'توقع المحصل (المراقبة)'!M19</f>
+        <v/>
+      </c>
+      <c r="I18" s="6">
+        <f>'توقع المحصل (المراقبة)'!P19</f>
+        <v/>
+      </c>
+      <c r="J18" s="7">
+        <f>IF(D18=0,"",E18/D18-1)</f>
+        <v/>
+      </c>
+      <c r="K18" s="7">
+        <f>IF(E18=0,"",F18/E18-1)</f>
+        <v/>
+      </c>
+      <c r="L18" s="7">
+        <f>IF(F18=0,"",H18/F18-1)</f>
+        <v/>
+      </c>
+      <c r="M18" s="7">
+        <f>IF(F18=0,"",I18/F18-1)</f>
+        <v/>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="inlineStr">
-        <is>
-          <t>6e) إعادة تصنيف المحصل: حسب تأكيد المستخدم، نُقل 913م من محصل 2025 في حساب اللوحات الدعائية (142113) إلى تأجير المرافق (142162) (كلها من إدارة الدعم المالي: مايو 291م ونوفمبر 594م). ينطبق على أوراق المحصل فقط؛ أوراق الفوترة لم تُعدّل لأن مبالغ الفوترة حسب الجهة غير متوفرة. إن كانت دفعات إدارة الدعم المالي في 2024 (يوليو 312م، نوفمبر 25م، ديسمبر 102م) من نفس النوع فالتوقع الأساسي يرتفع (انظر الرد).</t>
-        </is>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>11452108</t>
+        </is>
+      </c>
+      <c r="B19" s="5">
+        <f>'توقع المحصل (المراقبة)'!B20</f>
+        <v/>
+      </c>
+      <c r="C19" s="5">
+        <f>'توقع المحصل (المراقبة)'!C20</f>
+        <v/>
+      </c>
+      <c r="D19" s="6" t="n">
+        <v>4316211.89</v>
+      </c>
+      <c r="E19" s="6" t="n">
+        <v>19339697.82</v>
+      </c>
+      <c r="F19" s="6" t="n">
+        <v>24531493.81</v>
+      </c>
+      <c r="G19" s="6">
+        <f>'توقع المحصل (المراقبة)'!D20</f>
+        <v/>
+      </c>
+      <c r="H19" s="6">
+        <f>'توقع المحصل (المراقبة)'!M20</f>
+        <v/>
+      </c>
+      <c r="I19" s="6">
+        <f>'توقع المحصل (المراقبة)'!P20</f>
+        <v/>
+      </c>
+      <c r="J19" s="7">
+        <f>IF(D19=0,"",E19/D19-1)</f>
+        <v/>
+      </c>
+      <c r="K19" s="7">
+        <f>IF(E19=0,"",F19/E19-1)</f>
+        <v/>
+      </c>
+      <c r="L19" s="7">
+        <f>IF(F19=0,"",H19/F19-1)</f>
+        <v/>
+      </c>
+      <c r="M19" s="7">
+        <f>IF(F19=0,"",I19/F19-1)</f>
+        <v/>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="inlineStr">
-        <is>
-          <t>6f) ورقة "توقع المحصل (المراقبة)": الفعلي يناير–أكتوبر 2026 من ملف المراقبة (ورقة الإجمالي، قبل الاستقطاع)، ثم متبقي أكتوبر ونوفمبر وديسمبر بالموسمية الشهرية.</t>
-        </is>
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>1422108</t>
+        </is>
+      </c>
+      <c r="B20" s="5">
+        <f>'توقع المحصل (المراقبة)'!B21</f>
+        <v/>
+      </c>
+      <c r="C20" s="5">
+        <f>'توقع المحصل (المراقبة)'!C21</f>
+        <v/>
+      </c>
+      <c r="D20" s="6" t="n">
+        <v>20767064.19</v>
+      </c>
+      <c r="E20" s="6" t="n">
+        <v>12367178.86</v>
+      </c>
+      <c r="F20" s="6" t="n">
+        <v>26098550.07</v>
+      </c>
+      <c r="G20" s="6">
+        <f>'توقع المحصل (المراقبة)'!D21</f>
+        <v/>
+      </c>
+      <c r="H20" s="6">
+        <f>'توقع المحصل (المراقبة)'!M21</f>
+        <v/>
+      </c>
+      <c r="I20" s="6">
+        <f>'توقع المحصل (المراقبة)'!P21</f>
+        <v/>
+      </c>
+      <c r="J20" s="7">
+        <f>IF(D20=0,"",E20/D20-1)</f>
+        <v/>
+      </c>
+      <c r="K20" s="7">
+        <f>IF(E20=0,"",F20/E20-1)</f>
+        <v/>
+      </c>
+      <c r="L20" s="7">
+        <f>IF(F20=0,"",H20/F20-1)</f>
+        <v/>
+      </c>
+      <c r="M20" s="7">
+        <f>IF(F20=0,"",I20/F20-1)</f>
+        <v/>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="22" t="inlineStr">
-        <is>
-          <t>7) تنبيه: كثير من الحسابات تتذبذب بشدة بين السنوات (لوحات دعائية، تأجير المرافق، إيرادات متنوعة)، ومضاعفة 2026 على 12/9 تضخّم أو تقلّل هذه الأرقام؛ انظر عمود "تنبيه".</t>
-        </is>
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>1422121</t>
+        </is>
+      </c>
+      <c r="B21" s="5">
+        <f>'توقع المحصل (المراقبة)'!B22</f>
+        <v/>
+      </c>
+      <c r="C21" s="5">
+        <f>'توقع المحصل (المراقبة)'!C22</f>
+        <v/>
+      </c>
+      <c r="D21" s="6" t="n">
+        <v>13322800</v>
+      </c>
+      <c r="E21" s="6" t="n">
+        <v>17925000</v>
+      </c>
+      <c r="F21" s="6" t="n">
+        <v>15681460.95</v>
+      </c>
+      <c r="G21" s="6">
+        <f>'توقع المحصل (المراقبة)'!D22</f>
+        <v/>
+      </c>
+      <c r="H21" s="6">
+        <f>'توقع المحصل (المراقبة)'!M22</f>
+        <v/>
+      </c>
+      <c r="I21" s="6">
+        <f>'توقع المحصل (المراقبة)'!P22</f>
+        <v/>
+      </c>
+      <c r="J21" s="7">
+        <f>IF(D21=0,"",E21/D21-1)</f>
+        <v/>
+      </c>
+      <c r="K21" s="7">
+        <f>IF(E21=0,"",F21/E21-1)</f>
+        <v/>
+      </c>
+      <c r="L21" s="7">
+        <f>IF(F21=0,"",H21/F21-1)</f>
+        <v/>
+      </c>
+      <c r="M21" s="7">
+        <f>IF(F21=0,"",I21/F21-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>11452111</t>
+        </is>
+      </c>
+      <c r="B22" s="5">
+        <f>'توقع المحصل (المراقبة)'!B23</f>
+        <v/>
+      </c>
+      <c r="C22" s="5">
+        <f>'توقع المحصل (المراقبة)'!C23</f>
+        <v/>
+      </c>
+      <c r="D22" s="6" t="n">
+        <v>6031956.09</v>
+      </c>
+      <c r="E22" s="6" t="n">
+        <v>5166690.6</v>
+      </c>
+      <c r="F22" s="6" t="n">
+        <v>5751371.82</v>
+      </c>
+      <c r="G22" s="6">
+        <f>'توقع المحصل (المراقبة)'!D23</f>
+        <v/>
+      </c>
+      <c r="H22" s="6">
+        <f>'توقع المحصل (المراقبة)'!M23</f>
+        <v/>
+      </c>
+      <c r="I22" s="6">
+        <f>'توقع المحصل (المراقبة)'!P23</f>
+        <v/>
+      </c>
+      <c r="J22" s="7">
+        <f>IF(D22=0,"",E22/D22-1)</f>
+        <v/>
+      </c>
+      <c r="K22" s="7">
+        <f>IF(E22=0,"",F22/E22-1)</f>
+        <v/>
+      </c>
+      <c r="L22" s="7">
+        <f>IF(F22=0,"",H22/F22-1)</f>
+        <v/>
+      </c>
+      <c r="M22" s="7">
+        <f>IF(F22=0,"",I22/F22-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>142163</t>
+        </is>
+      </c>
+      <c r="B23" s="5">
+        <f>'توقع المحصل (المراقبة)'!B24</f>
+        <v/>
+      </c>
+      <c r="C23" s="5">
+        <f>'توقع المحصل (المراقبة)'!C24</f>
+        <v/>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>6866663.43</v>
+      </c>
+      <c r="E23" s="6" t="n">
+        <v>6179302.5</v>
+      </c>
+      <c r="F23" s="6" t="n">
+        <v>3001651.75</v>
+      </c>
+      <c r="G23" s="6">
+        <f>'توقع المحصل (المراقبة)'!D24</f>
+        <v/>
+      </c>
+      <c r="H23" s="6">
+        <f>'توقع المحصل (المراقبة)'!M24</f>
+        <v/>
+      </c>
+      <c r="I23" s="6">
+        <f>'توقع المحصل (المراقبة)'!P24</f>
+        <v/>
+      </c>
+      <c r="J23" s="7">
+        <f>IF(D23=0,"",E23/D23-1)</f>
+        <v/>
+      </c>
+      <c r="K23" s="7">
+        <f>IF(E23=0,"",F23/E23-1)</f>
+        <v/>
+      </c>
+      <c r="L23" s="7">
+        <f>IF(F23=0,"",H23/F23-1)</f>
+        <v/>
+      </c>
+      <c r="M23" s="7">
+        <f>IF(F23=0,"",I23/F23-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>1422109</t>
+        </is>
+      </c>
+      <c r="B24" s="5">
+        <f>'توقع المحصل (المراقبة)'!B25</f>
+        <v/>
+      </c>
+      <c r="C24" s="5">
+        <f>'توقع المحصل (المراقبة)'!C25</f>
+        <v/>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>9211384.77</v>
+      </c>
+      <c r="E24" s="6" t="n">
+        <v>8995823.25</v>
+      </c>
+      <c r="F24" s="6" t="n">
+        <v>7132142.91</v>
+      </c>
+      <c r="G24" s="6">
+        <f>'توقع المحصل (المراقبة)'!D25</f>
+        <v/>
+      </c>
+      <c r="H24" s="6">
+        <f>'توقع المحصل (المراقبة)'!M25</f>
+        <v/>
+      </c>
+      <c r="I24" s="6">
+        <f>'توقع المحصل (المراقبة)'!P25</f>
+        <v/>
+      </c>
+      <c r="J24" s="7">
+        <f>IF(D24=0,"",E24/D24-1)</f>
+        <v/>
+      </c>
+      <c r="K24" s="7">
+        <f>IF(E24=0,"",F24/E24-1)</f>
+        <v/>
+      </c>
+      <c r="L24" s="7">
+        <f>IF(F24=0,"",H24/F24-1)</f>
+        <v/>
+      </c>
+      <c r="M24" s="7">
+        <f>IF(F24=0,"",I24/F24-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>1422202</t>
+        </is>
+      </c>
+      <c r="B25" s="5">
+        <f>'توقع المحصل (المراقبة)'!B26</f>
+        <v/>
+      </c>
+      <c r="C25" s="5">
+        <f>'توقع المحصل (المراقبة)'!C26</f>
+        <v/>
+      </c>
+      <c r="D25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="6">
+        <f>'توقع المحصل (المراقبة)'!D26</f>
+        <v/>
+      </c>
+      <c r="H25" s="6">
+        <f>'توقع المحصل (المراقبة)'!M26</f>
+        <v/>
+      </c>
+      <c r="I25" s="6">
+        <f>'توقع المحصل (المراقبة)'!P26</f>
+        <v/>
+      </c>
+      <c r="J25" s="7">
+        <f>IF(D25=0,"",E25/D25-1)</f>
+        <v/>
+      </c>
+      <c r="K25" s="7">
+        <f>IF(E25=0,"",F25/E25-1)</f>
+        <v/>
+      </c>
+      <c r="L25" s="7">
+        <f>IF(F25=0,"",H25/F25-1)</f>
+        <v/>
+      </c>
+      <c r="M25" s="7">
+        <f>IF(F25=0,"",I25/F25-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>1421910</t>
+        </is>
+      </c>
+      <c r="B26" s="5">
+        <f>'توقع المحصل (المراقبة)'!B27</f>
+        <v/>
+      </c>
+      <c r="C26" s="5">
+        <f>'توقع المحصل (المراقبة)'!C27</f>
+        <v/>
+      </c>
+      <c r="D26" s="6" t="n">
+        <v>3828676.61</v>
+      </c>
+      <c r="E26" s="6" t="n">
+        <v>2909412.61</v>
+      </c>
+      <c r="F26" s="6" t="n">
+        <v>3477675.2</v>
+      </c>
+      <c r="G26" s="6">
+        <f>'توقع المحصل (المراقبة)'!D27</f>
+        <v/>
+      </c>
+      <c r="H26" s="6">
+        <f>'توقع المحصل (المراقبة)'!M27</f>
+        <v/>
+      </c>
+      <c r="I26" s="6">
+        <f>'توقع المحصل (المراقبة)'!P27</f>
+        <v/>
+      </c>
+      <c r="J26" s="7">
+        <f>IF(D26=0,"",E26/D26-1)</f>
+        <v/>
+      </c>
+      <c r="K26" s="7">
+        <f>IF(E26=0,"",F26/E26-1)</f>
+        <v/>
+      </c>
+      <c r="L26" s="7">
+        <f>IF(F26=0,"",H26/F26-1)</f>
+        <v/>
+      </c>
+      <c r="M26" s="7">
+        <f>IF(F26=0,"",I26/F26-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>11452107</t>
+        </is>
+      </c>
+      <c r="B27" s="5">
+        <f>'توقع المحصل (المراقبة)'!B28</f>
+        <v/>
+      </c>
+      <c r="C27" s="5">
+        <f>'توقع المحصل (المراقبة)'!C28</f>
+        <v/>
+      </c>
+      <c r="D27" s="6" t="n">
+        <v>54000</v>
+      </c>
+      <c r="E27" s="6" t="n">
+        <v>90000</v>
+      </c>
+      <c r="F27" s="6" t="n">
+        <v>229800</v>
+      </c>
+      <c r="G27" s="6">
+        <f>'توقع المحصل (المراقبة)'!D28</f>
+        <v/>
+      </c>
+      <c r="H27" s="6">
+        <f>'توقع المحصل (المراقبة)'!M28</f>
+        <v/>
+      </c>
+      <c r="I27" s="6">
+        <f>'توقع المحصل (المراقبة)'!P28</f>
+        <v/>
+      </c>
+      <c r="J27" s="7">
+        <f>IF(D27=0,"",E27/D27-1)</f>
+        <v/>
+      </c>
+      <c r="K27" s="7">
+        <f>IF(E27=0,"",F27/E27-1)</f>
+        <v/>
+      </c>
+      <c r="L27" s="7">
+        <f>IF(F27=0,"",H27/F27-1)</f>
+        <v/>
+      </c>
+      <c r="M27" s="7">
+        <f>IF(F27=0,"",I27/F27-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>1421901</t>
+        </is>
+      </c>
+      <c r="B28" s="5">
+        <f>'توقع المحصل (المراقبة)'!B29</f>
+        <v/>
+      </c>
+      <c r="C28" s="5">
+        <f>'توقع المحصل (المراقبة)'!C29</f>
+        <v/>
+      </c>
+      <c r="D28" s="6" t="n">
+        <v>2928906</v>
+      </c>
+      <c r="E28" s="6" t="n">
+        <v>2736595</v>
+      </c>
+      <c r="F28" s="6" t="n">
+        <v>2512377</v>
+      </c>
+      <c r="G28" s="6">
+        <f>'توقع المحصل (المراقبة)'!D29</f>
+        <v/>
+      </c>
+      <c r="H28" s="6">
+        <f>'توقع المحصل (المراقبة)'!M29</f>
+        <v/>
+      </c>
+      <c r="I28" s="6">
+        <f>'توقع المحصل (المراقبة)'!P29</f>
+        <v/>
+      </c>
+      <c r="J28" s="7">
+        <f>IF(D28=0,"",E28/D28-1)</f>
+        <v/>
+      </c>
+      <c r="K28" s="7">
+        <f>IF(E28=0,"",F28/E28-1)</f>
+        <v/>
+      </c>
+      <c r="L28" s="7">
+        <f>IF(F28=0,"",H28/F28-1)</f>
+        <v/>
+      </c>
+      <c r="M28" s="7">
+        <f>IF(F28=0,"",I28/F28-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>بدون رقم</t>
+        </is>
+      </c>
+      <c r="B29" s="5">
+        <f>'توقع المحصل (المراقبة)'!B30</f>
+        <v/>
+      </c>
+      <c r="C29" s="5">
+        <f>'توقع المحصل (المراقبة)'!C30</f>
+        <v/>
+      </c>
+      <c r="D29" s="6" t="n">
+        <v>4815218.75</v>
+      </c>
+      <c r="E29" s="6" t="n">
+        <v>14256546.25</v>
+      </c>
+      <c r="F29" s="6" t="n">
+        <v>21814890</v>
+      </c>
+      <c r="G29" s="6">
+        <f>'توقع المحصل (المراقبة)'!D30</f>
+        <v/>
+      </c>
+      <c r="H29" s="6">
+        <f>'توقع المحصل (المراقبة)'!M30</f>
+        <v/>
+      </c>
+      <c r="I29" s="6">
+        <f>'توقع المحصل (المراقبة)'!P30</f>
+        <v/>
+      </c>
+      <c r="J29" s="7">
+        <f>IF(D29=0,"",E29/D29-1)</f>
+        <v/>
+      </c>
+      <c r="K29" s="7">
+        <f>IF(E29=0,"",F29/E29-1)</f>
+        <v/>
+      </c>
+      <c r="L29" s="7">
+        <f>IF(F29=0,"",H29/F29-1)</f>
+        <v/>
+      </c>
+      <c r="M29" s="7">
+        <f>IF(F29=0,"",I29/F29-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>1421912</t>
+        </is>
+      </c>
+      <c r="B30" s="5">
+        <f>'توقع المحصل (المراقبة)'!B31</f>
+        <v/>
+      </c>
+      <c r="C30" s="5">
+        <f>'توقع المحصل (المراقبة)'!C31</f>
+        <v/>
+      </c>
+      <c r="D30" s="6" t="n">
+        <v>838420.1899999999</v>
+      </c>
+      <c r="E30" s="6" t="n">
+        <v>2043840.5</v>
+      </c>
+      <c r="F30" s="6" t="n">
+        <v>2454143.51</v>
+      </c>
+      <c r="G30" s="6">
+        <f>'توقع المحصل (المراقبة)'!D31</f>
+        <v/>
+      </c>
+      <c r="H30" s="6">
+        <f>'توقع المحصل (المراقبة)'!M31</f>
+        <v/>
+      </c>
+      <c r="I30" s="6">
+        <f>'توقع المحصل (المراقبة)'!P31</f>
+        <v/>
+      </c>
+      <c r="J30" s="7">
+        <f>IF(D30=0,"",E30/D30-1)</f>
+        <v/>
+      </c>
+      <c r="K30" s="7">
+        <f>IF(E30=0,"",F30/E30-1)</f>
+        <v/>
+      </c>
+      <c r="L30" s="7">
+        <f>IF(F30=0,"",H30/F30-1)</f>
+        <v/>
+      </c>
+      <c r="M30" s="7">
+        <f>IF(F30=0,"",I30/F30-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>11452106</t>
+        </is>
+      </c>
+      <c r="B31" s="5">
+        <f>'توقع المحصل (المراقبة)'!B32</f>
+        <v/>
+      </c>
+      <c r="C31" s="5">
+        <f>'توقع المحصل (المراقبة)'!C32</f>
+        <v/>
+      </c>
+      <c r="D31" s="6" t="n">
+        <v>845300</v>
+      </c>
+      <c r="E31" s="6" t="n">
+        <v>1408700</v>
+      </c>
+      <c r="F31" s="6" t="n">
+        <v>1275300</v>
+      </c>
+      <c r="G31" s="6">
+        <f>'توقع المحصل (المراقبة)'!D32</f>
+        <v/>
+      </c>
+      <c r="H31" s="6">
+        <f>'توقع المحصل (المراقبة)'!M32</f>
+        <v/>
+      </c>
+      <c r="I31" s="6">
+        <f>'توقع المحصل (المراقبة)'!P32</f>
+        <v/>
+      </c>
+      <c r="J31" s="7">
+        <f>IF(D31=0,"",E31/D31-1)</f>
+        <v/>
+      </c>
+      <c r="K31" s="7">
+        <f>IF(E31=0,"",F31/E31-1)</f>
+        <v/>
+      </c>
+      <c r="L31" s="7">
+        <f>IF(F31=0,"",H31/F31-1)</f>
+        <v/>
+      </c>
+      <c r="M31" s="7">
+        <f>IF(F31=0,"",I31/F31-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>11452110</t>
+        </is>
+      </c>
+      <c r="B32" s="5">
+        <f>'توقع المحصل (المراقبة)'!B33</f>
+        <v/>
+      </c>
+      <c r="C32" s="5">
+        <f>'توقع المحصل (المراقبة)'!C33</f>
+        <v/>
+      </c>
+      <c r="D32" s="6" t="n">
+        <v>609446.45</v>
+      </c>
+      <c r="E32" s="6" t="n">
+        <v>1038687.25</v>
+      </c>
+      <c r="F32" s="6" t="n">
+        <v>809215.9</v>
+      </c>
+      <c r="G32" s="6">
+        <f>'توقع المحصل (المراقبة)'!D33</f>
+        <v/>
+      </c>
+      <c r="H32" s="6">
+        <f>'توقع المحصل (المراقبة)'!M33</f>
+        <v/>
+      </c>
+      <c r="I32" s="6">
+        <f>'توقع المحصل (المراقبة)'!P33</f>
+        <v/>
+      </c>
+      <c r="J32" s="7">
+        <f>IF(D32=0,"",E32/D32-1)</f>
+        <v/>
+      </c>
+      <c r="K32" s="7">
+        <f>IF(E32=0,"",F32/E32-1)</f>
+        <v/>
+      </c>
+      <c r="L32" s="7">
+        <f>IF(F32=0,"",H32/F32-1)</f>
+        <v/>
+      </c>
+      <c r="M32" s="7">
+        <f>IF(F32=0,"",I32/F32-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>1422104</t>
+        </is>
+      </c>
+      <c r="B33" s="5">
+        <f>'توقع المحصل (المراقبة)'!B34</f>
+        <v/>
+      </c>
+      <c r="C33" s="5">
+        <f>'توقع المحصل (المراقبة)'!C34</f>
+        <v/>
+      </c>
+      <c r="D33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="6">
+        <f>'توقع المحصل (المراقبة)'!D34</f>
+        <v/>
+      </c>
+      <c r="H33" s="6">
+        <f>'توقع المحصل (المراقبة)'!M34</f>
+        <v/>
+      </c>
+      <c r="I33" s="6">
+        <f>'توقع المحصل (المراقبة)'!P34</f>
+        <v/>
+      </c>
+      <c r="J33" s="7">
+        <f>IF(D33=0,"",E33/D33-1)</f>
+        <v/>
+      </c>
+      <c r="K33" s="7">
+        <f>IF(E33=0,"",F33/E33-1)</f>
+        <v/>
+      </c>
+      <c r="L33" s="7">
+        <f>IF(F33=0,"",H33/F33-1)</f>
+        <v/>
+      </c>
+      <c r="M33" s="7">
+        <f>IF(F33=0,"",I33/F33-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>3318212</t>
+        </is>
+      </c>
+      <c r="B34" s="5">
+        <f>'توقع المحصل (المراقبة)'!B35</f>
+        <v/>
+      </c>
+      <c r="C34" s="5">
+        <f>'توقع المحصل (المراقبة)'!C35</f>
+        <v/>
+      </c>
+      <c r="D34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" s="6" t="n">
+        <v>152767.79</v>
+      </c>
+      <c r="G34" s="6">
+        <f>'توقع المحصل (المراقبة)'!D35</f>
+        <v/>
+      </c>
+      <c r="H34" s="6">
+        <f>'توقع المحصل (المراقبة)'!M35</f>
+        <v/>
+      </c>
+      <c r="I34" s="6">
+        <f>'توقع المحصل (المراقبة)'!P35</f>
+        <v/>
+      </c>
+      <c r="J34" s="7">
+        <f>IF(D34=0,"",E34/D34-1)</f>
+        <v/>
+      </c>
+      <c r="K34" s="7">
+        <f>IF(E34=0,"",F34/E34-1)</f>
+        <v/>
+      </c>
+      <c r="L34" s="7">
+        <f>IF(F34=0,"",H34/F34-1)</f>
+        <v/>
+      </c>
+      <c r="M34" s="7">
+        <f>IF(F34=0,"",I34/F34-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>1421903</t>
+        </is>
+      </c>
+      <c r="B35" s="5">
+        <f>'توقع المحصل (المراقبة)'!B36</f>
+        <v/>
+      </c>
+      <c r="C35" s="5">
+        <f>'توقع المحصل (المراقبة)'!C36</f>
+        <v/>
+      </c>
+      <c r="D35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F35" s="6" t="n">
+        <v>1464687.1</v>
+      </c>
+      <c r="G35" s="6">
+        <f>'توقع المحصل (المراقبة)'!D36</f>
+        <v/>
+      </c>
+      <c r="H35" s="6">
+        <f>'توقع المحصل (المراقبة)'!M36</f>
+        <v/>
+      </c>
+      <c r="I35" s="6">
+        <f>'توقع المحصل (المراقبة)'!P36</f>
+        <v/>
+      </c>
+      <c r="J35" s="7">
+        <f>IF(D35=0,"",E35/D35-1)</f>
+        <v/>
+      </c>
+      <c r="K35" s="7">
+        <f>IF(E35=0,"",F35/E35-1)</f>
+        <v/>
+      </c>
+      <c r="L35" s="7">
+        <f>IF(F35=0,"",H35/F35-1)</f>
+        <v/>
+      </c>
+      <c r="M35" s="7">
+        <f>IF(F35=0,"",I35/F35-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>141229</t>
+        </is>
+      </c>
+      <c r="B36" s="5">
+        <f>'توقع المحصل (المراقبة)'!B37</f>
+        <v/>
+      </c>
+      <c r="C36" s="5">
+        <f>'توقع المحصل (المراقبة)'!C37</f>
+        <v/>
+      </c>
+      <c r="D36" s="6" t="n">
+        <v>910572</v>
+      </c>
+      <c r="E36" s="6" t="n">
+        <v>2120000</v>
+      </c>
+      <c r="F36" s="6" t="n">
+        <v>30000</v>
+      </c>
+      <c r="G36" s="6">
+        <f>'توقع المحصل (المراقبة)'!D37</f>
+        <v/>
+      </c>
+      <c r="H36" s="6">
+        <f>'توقع المحصل (المراقبة)'!M37</f>
+        <v/>
+      </c>
+      <c r="I36" s="6">
+        <f>'توقع المحصل (المراقبة)'!P37</f>
+        <v/>
+      </c>
+      <c r="J36" s="7">
+        <f>IF(D36=0,"",E36/D36-1)</f>
+        <v/>
+      </c>
+      <c r="K36" s="7">
+        <f>IF(E36=0,"",F36/E36-1)</f>
+        <v/>
+      </c>
+      <c r="L36" s="7">
+        <f>IF(F36=0,"",H36/F36-1)</f>
+        <v/>
+      </c>
+      <c r="M36" s="7">
+        <f>IF(F36=0,"",I36/F36-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>1438</t>
+        </is>
+      </c>
+      <c r="B37" s="5">
+        <f>'توقع المحصل (المراقبة)'!B38</f>
+        <v/>
+      </c>
+      <c r="C37" s="5">
+        <f>'توقع المحصل (المراقبة)'!C38</f>
+        <v/>
+      </c>
+      <c r="D37" s="6" t="n">
+        <v>4544553</v>
+      </c>
+      <c r="E37" s="6" t="n">
+        <v>486100</v>
+      </c>
+      <c r="F37" s="6" t="n">
+        <v>352900</v>
+      </c>
+      <c r="G37" s="6">
+        <f>'توقع المحصل (المراقبة)'!D38</f>
+        <v/>
+      </c>
+      <c r="H37" s="6">
+        <f>'توقع المحصل (المراقبة)'!M38</f>
+        <v/>
+      </c>
+      <c r="I37" s="6">
+        <f>'توقع المحصل (المراقبة)'!P38</f>
+        <v/>
+      </c>
+      <c r="J37" s="7">
+        <f>IF(D37=0,"",E37/D37-1)</f>
+        <v/>
+      </c>
+      <c r="K37" s="7">
+        <f>IF(E37=0,"",F37/E37-1)</f>
+        <v/>
+      </c>
+      <c r="L37" s="7">
+        <f>IF(F37=0,"",H37/F37-1)</f>
+        <v/>
+      </c>
+      <c r="M37" s="7">
+        <f>IF(F37=0,"",I37/F37-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>1421907</t>
+        </is>
+      </c>
+      <c r="B38" s="5">
+        <f>'توقع المحصل (المراقبة)'!B39</f>
+        <v/>
+      </c>
+      <c r="C38" s="5">
+        <f>'توقع المحصل (المراقبة)'!C39</f>
+        <v/>
+      </c>
+      <c r="D38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F38" s="6" t="n">
+        <v>20650</v>
+      </c>
+      <c r="G38" s="6">
+        <f>'توقع المحصل (المراقبة)'!D39</f>
+        <v/>
+      </c>
+      <c r="H38" s="6">
+        <f>'توقع المحصل (المراقبة)'!M39</f>
+        <v/>
+      </c>
+      <c r="I38" s="6">
+        <f>'توقع المحصل (المراقبة)'!P39</f>
+        <v/>
+      </c>
+      <c r="J38" s="7">
+        <f>IF(D38=0,"",E38/D38-1)</f>
+        <v/>
+      </c>
+      <c r="K38" s="7">
+        <f>IF(E38=0,"",F38/E38-1)</f>
+        <v/>
+      </c>
+      <c r="L38" s="7">
+        <f>IF(F38=0,"",H38/F38-1)</f>
+        <v/>
+      </c>
+      <c r="M38" s="7">
+        <f>IF(F38=0,"",I38/F38-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>11452105</t>
+        </is>
+      </c>
+      <c r="B39" s="5">
+        <f>'توقع المحصل (المراقبة)'!B40</f>
+        <v/>
+      </c>
+      <c r="C39" s="5">
+        <f>'توقع المحصل (المراقبة)'!C40</f>
+        <v/>
+      </c>
+      <c r="D39" s="6" t="n">
+        <v>66558861.24</v>
+      </c>
+      <c r="E39" s="6" t="n">
+        <v>65200590.52</v>
+      </c>
+      <c r="F39" s="6" t="n">
+        <v>590915.4300000001</v>
+      </c>
+      <c r="G39" s="6">
+        <f>'توقع المحصل (المراقبة)'!D40</f>
+        <v/>
+      </c>
+      <c r="H39" s="6">
+        <f>'توقع المحصل (المراقبة)'!M40</f>
+        <v/>
+      </c>
+      <c r="I39" s="6">
+        <f>'توقع المحصل (المراقبة)'!P40</f>
+        <v/>
+      </c>
+      <c r="J39" s="7">
+        <f>IF(D39=0,"",E39/D39-1)</f>
+        <v/>
+      </c>
+      <c r="K39" s="7">
+        <f>IF(E39=0,"",F39/E39-1)</f>
+        <v/>
+      </c>
+      <c r="L39" s="7">
+        <f>IF(F39=0,"",H39/F39-1)</f>
+        <v/>
+      </c>
+      <c r="M39" s="7">
+        <f>IF(F39=0,"",I39/F39-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>11452513</t>
+        </is>
+      </c>
+      <c r="B40" s="5">
+        <f>'توقع المحصل (المراقبة)'!B41</f>
+        <v/>
+      </c>
+      <c r="C40" s="5">
+        <f>'توقع المحصل (المراقبة)'!C41</f>
+        <v/>
+      </c>
+      <c r="D40" s="6" t="n">
+        <v>55525</v>
+      </c>
+      <c r="E40" s="6" t="n">
+        <v>12875</v>
+      </c>
+      <c r="F40" s="6" t="n">
+        <v>9000</v>
+      </c>
+      <c r="G40" s="6">
+        <f>'توقع المحصل (المراقبة)'!D41</f>
+        <v/>
+      </c>
+      <c r="H40" s="6">
+        <f>'توقع المحصل (المراقبة)'!M41</f>
+        <v/>
+      </c>
+      <c r="I40" s="6">
+        <f>'توقع المحصل (المراقبة)'!P41</f>
+        <v/>
+      </c>
+      <c r="J40" s="7">
+        <f>IF(D40=0,"",E40/D40-1)</f>
+        <v/>
+      </c>
+      <c r="K40" s="7">
+        <f>IF(E40=0,"",F40/E40-1)</f>
+        <v/>
+      </c>
+      <c r="L40" s="7">
+        <f>IF(F40=0,"",H40/F40-1)</f>
+        <v/>
+      </c>
+      <c r="M40" s="7">
+        <f>IF(F40=0,"",I40/F40-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>1422103</t>
+        </is>
+      </c>
+      <c r="B41" s="5">
+        <f>'توقع المحصل (المراقبة)'!B42</f>
+        <v/>
+      </c>
+      <c r="C41" s="5">
+        <f>'توقع المحصل (المراقبة)'!C42</f>
+        <v/>
+      </c>
+      <c r="D41" s="6" t="n">
+        <v>67711.60000000001</v>
+      </c>
+      <c r="E41" s="6" t="n">
+        <v>16269.6</v>
+      </c>
+      <c r="F41" s="6" t="n">
+        <v>1603.2</v>
+      </c>
+      <c r="G41" s="6">
+        <f>'توقع المحصل (المراقبة)'!D42</f>
+        <v/>
+      </c>
+      <c r="H41" s="6">
+        <f>'توقع المحصل (المراقبة)'!M42</f>
+        <v/>
+      </c>
+      <c r="I41" s="6">
+        <f>'توقع المحصل (المراقبة)'!P42</f>
+        <v/>
+      </c>
+      <c r="J41" s="7">
+        <f>IF(D41=0,"",E41/D41-1)</f>
+        <v/>
+      </c>
+      <c r="K41" s="7">
+        <f>IF(E41=0,"",F41/E41-1)</f>
+        <v/>
+      </c>
+      <c r="L41" s="7">
+        <f>IF(F41=0,"",H41/F41-1)</f>
+        <v/>
+      </c>
+      <c r="M41" s="7">
+        <f>IF(F41=0,"",I41/F41-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>11452109</t>
+        </is>
+      </c>
+      <c r="B42" s="5">
+        <f>'توقع المحصل (المراقبة)'!B43</f>
+        <v/>
+      </c>
+      <c r="C42" s="5">
+        <f>'توقع المحصل (المراقبة)'!C43</f>
+        <v/>
+      </c>
+      <c r="D42" s="6" t="n">
+        <v>536299.9399999999</v>
+      </c>
+      <c r="E42" s="6" t="n">
+        <v>1217856.22</v>
+      </c>
+      <c r="F42" s="6" t="n">
+        <v>591946.73</v>
+      </c>
+      <c r="G42" s="6">
+        <f>'توقع المحصل (المراقبة)'!D43</f>
+        <v/>
+      </c>
+      <c r="H42" s="6">
+        <f>'توقع المحصل (المراقبة)'!M43</f>
+        <v/>
+      </c>
+      <c r="I42" s="6">
+        <f>'توقع المحصل (المراقبة)'!P43</f>
+        <v/>
+      </c>
+      <c r="J42" s="7">
+        <f>IF(D42=0,"",E42/D42-1)</f>
+        <v/>
+      </c>
+      <c r="K42" s="7">
+        <f>IF(E42=0,"",F42/E42-1)</f>
+        <v/>
+      </c>
+      <c r="L42" s="7">
+        <f>IF(F42=0,"",H42/F42-1)</f>
+        <v/>
+      </c>
+      <c r="M42" s="7">
+        <f>IF(F42=0,"",I42/F42-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>11422</t>
+        </is>
+      </c>
+      <c r="B43" s="5">
+        <f>'توقع المحصل (المراقبة)'!B44</f>
+        <v/>
+      </c>
+      <c r="C43" s="5">
+        <f>'توقع المحصل (المراقبة)'!C44</f>
+        <v/>
+      </c>
+      <c r="D43" s="6" t="n">
+        <v>27000</v>
+      </c>
+      <c r="E43" s="6" t="n">
+        <v>5167</v>
+      </c>
+      <c r="F43" s="6" t="n">
+        <v>27000</v>
+      </c>
+      <c r="G43" s="6">
+        <f>'توقع المحصل (المراقبة)'!D44</f>
+        <v/>
+      </c>
+      <c r="H43" s="6">
+        <f>'توقع المحصل (المراقبة)'!M44</f>
+        <v/>
+      </c>
+      <c r="I43" s="6">
+        <f>'توقع المحصل (المراقبة)'!P44</f>
+        <v/>
+      </c>
+      <c r="J43" s="7">
+        <f>IF(D43=0,"",E43/D43-1)</f>
+        <v/>
+      </c>
+      <c r="K43" s="7">
+        <f>IF(E43=0,"",F43/E43-1)</f>
+        <v/>
+      </c>
+      <c r="L43" s="7">
+        <f>IF(F43=0,"",H43/F43-1)</f>
+        <v/>
+      </c>
+      <c r="M43" s="7">
+        <f>IF(F43=0,"",I43/F43-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>142161</t>
+        </is>
+      </c>
+      <c r="B44" s="5">
+        <f>'توقع المحصل (المراقبة)'!B45</f>
+        <v/>
+      </c>
+      <c r="C44" s="5">
+        <f>'توقع المحصل (المراقبة)'!C45</f>
+        <v/>
+      </c>
+      <c r="D44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F44" s="6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="G44" s="6">
+        <f>'توقع المحصل (المراقبة)'!D45</f>
+        <v/>
+      </c>
+      <c r="H44" s="6">
+        <f>'توقع المحصل (المراقبة)'!M45</f>
+        <v/>
+      </c>
+      <c r="I44" s="6">
+        <f>'توقع المحصل (المراقبة)'!P45</f>
+        <v/>
+      </c>
+      <c r="J44" s="7">
+        <f>IF(D44=0,"",E44/D44-1)</f>
+        <v/>
+      </c>
+      <c r="K44" s="7">
+        <f>IF(E44=0,"",F44/E44-1)</f>
+        <v/>
+      </c>
+      <c r="L44" s="7">
+        <f>IF(F44=0,"",H44/F44-1)</f>
+        <v/>
+      </c>
+      <c r="M44" s="7">
+        <f>IF(F44=0,"",I44/F44-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>1421908</t>
+        </is>
+      </c>
+      <c r="B45" s="5">
+        <f>'توقع المحصل (المراقبة)'!B46</f>
+        <v/>
+      </c>
+      <c r="C45" s="5">
+        <f>'توقع المحصل (المراقبة)'!C46</f>
+        <v/>
+      </c>
+      <c r="D45" s="6" t="n">
+        <v>16385</v>
+      </c>
+      <c r="E45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G45" s="6">
+        <f>'توقع المحصل (المراقبة)'!D46</f>
+        <v/>
+      </c>
+      <c r="H45" s="6">
+        <f>'توقع المحصل (المراقبة)'!M46</f>
+        <v/>
+      </c>
+      <c r="I45" s="6">
+        <f>'توقع المحصل (المراقبة)'!P46</f>
+        <v/>
+      </c>
+      <c r="J45" s="7">
+        <f>IF(D45=0,"",E45/D45-1)</f>
+        <v/>
+      </c>
+      <c r="K45" s="7">
+        <f>IF(E45=0,"",F45/E45-1)</f>
+        <v/>
+      </c>
+      <c r="L45" s="7">
+        <f>IF(F45=0,"",H45/F45-1)</f>
+        <v/>
+      </c>
+      <c r="M45" s="7">
+        <f>IF(F45=0,"",I45/F45-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>1422112</t>
+        </is>
+      </c>
+      <c r="B46" s="5">
+        <f>'توقع المحصل (المراقبة)'!B47</f>
+        <v/>
+      </c>
+      <c r="C46" s="5">
+        <f>'توقع المحصل (المراقبة)'!C47</f>
+        <v/>
+      </c>
+      <c r="D46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F46" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G46" s="6">
+        <f>'توقع المحصل (المراقبة)'!D47</f>
+        <v/>
+      </c>
+      <c r="H46" s="6">
+        <f>'توقع المحصل (المراقبة)'!M47</f>
+        <v/>
+      </c>
+      <c r="I46" s="6">
+        <f>'توقع المحصل (المراقبة)'!P47</f>
+        <v/>
+      </c>
+      <c r="J46" s="7">
+        <f>IF(D46=0,"",E46/D46-1)</f>
+        <v/>
+      </c>
+      <c r="K46" s="7">
+        <f>IF(E46=0,"",F46/E46-1)</f>
+        <v/>
+      </c>
+      <c r="L46" s="7">
+        <f>IF(F46=0,"",H46/F46-1)</f>
+        <v/>
+      </c>
+      <c r="M46" s="7">
+        <f>IF(F46=0,"",I46/F46-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>1422199</t>
+        </is>
+      </c>
+      <c r="B47" s="5">
+        <f>'توقع المحصل (المراقبة)'!B48</f>
+        <v/>
+      </c>
+      <c r="C47" s="5">
+        <f>'توقع المحصل (المراقبة)'!C48</f>
+        <v/>
+      </c>
+      <c r="D47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="E47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="G47" s="6">
+        <f>'توقع المحصل (المراقبة)'!D48</f>
+        <v/>
+      </c>
+      <c r="H47" s="6">
+        <f>'توقع المحصل (المراقبة)'!M48</f>
+        <v/>
+      </c>
+      <c r="I47" s="6">
+        <f>'توقع المحصل (المراقبة)'!P48</f>
+        <v/>
+      </c>
+      <c r="J47" s="7">
+        <f>IF(D47=0,"",E47/D47-1)</f>
+        <v/>
+      </c>
+      <c r="K47" s="7">
+        <f>IF(E47=0,"",F47/E47-1)</f>
+        <v/>
+      </c>
+      <c r="L47" s="7">
+        <f>IF(F47=0,"",H47/F47-1)</f>
+        <v/>
+      </c>
+      <c r="M47" s="7">
+        <f>IF(F47=0,"",I47/F47-1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="8" t="n"/>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="C48" s="8" t="n"/>
+      <c r="D48" s="9">
+        <f>SUM(D5:D47)</f>
+        <v/>
+      </c>
+      <c r="E48" s="9">
+        <f>SUM(E5:E47)</f>
+        <v/>
+      </c>
+      <c r="F48" s="9">
+        <f>SUM(F5:F47)</f>
+        <v/>
+      </c>
+      <c r="G48" s="9">
+        <f>SUM(G5:G47)</f>
+        <v/>
+      </c>
+      <c r="H48" s="9">
+        <f>SUM(H5:H47)</f>
+        <v/>
+      </c>
+      <c r="I48" s="9">
+        <f>SUM(I5:I47)</f>
+        <v/>
+      </c>
+      <c r="J48" s="10">
+        <f>E48/D48-1</f>
+        <v/>
+      </c>
+      <c r="K48" s="10">
+        <f>F48/E48-1</f>
+        <v/>
+      </c>
+      <c r="L48" s="10">
+        <f>H48/F48-1</f>
+        <v/>
+      </c>
+      <c r="M48" s="10">
+        <f>I48/F48-1</f>
+        <v/>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A4:M47"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:M2"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Add remaining-months sheet (Oct/Nov/Dec forecast vs target)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01D73U26FQnMJ6VM9LfvsWf3
</commit_message>
<xml_diff>
--- a/توقع_الفوترة_2026_2027.xlsx
+++ b/توقع_الفوترة_2026_2027.xlsx
@@ -16,7 +16,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الموسمية الشهرية" sheetId="7" state="visible" r:id="rId7"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="توقع المحصل (المراقبة)" sheetId="8" state="visible" r:id="rId8"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="المحصل 2023-2026" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الأشهر المتبقية 2026" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="الافتراضات" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'التوقعات'!$A$3:$R$41</definedName>
@@ -25,6 +26,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'توقع المحصل الموسمي'!$A$5:$Q$43</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'توقع المحصل (المراقبة)'!$A$5:$U$48</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'المحصل 2023-2026'!$A$4:$M$47</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'الأشهر المتبقية 2026'!$A$12:$Q$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -125,7 +127,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -155,6 +157,8 @@
     <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="9" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -3472,7 +3476,3147 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:Q56"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="16" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>أكتوبر ونوفمبر وديسمبر 2026: المحصل/المتوقع مقابل المستهدف والمقدر</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="48" customHeight="1">
+      <c r="A2" s="12" t="inlineStr">
+        <is>
+          <t>أكتوبر: المحصل حتى تاريخ ملف المراقبة، والمتوقع = المحصل حتى تاريخه + المتبقي (الأساسي والأسوأ). نوفمبر وديسمبر: المتوقع الأساسي والأسوأ بالموسمية الشهرية، موزّع بين الشهرين بحسب نسبتهما التاريخية لكل حساب (وسيط 2023–2025) بحيث يطابق مجموعهما ورقة "توقع المحصل (المراقبة)". المستهدف والمقدر من ورقتي "المستهدف 2026" و"المقدر 2026" في ملف المراقبة. بدون الضريبة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>الشهر</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>المحصل حتى تاريخه</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>المتوقع أساسي</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>المتوقع أسوأ</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>المستهدف</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>المقدر</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>الأساسي ÷ المستهدف</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>الأسوأ ÷ المستهدف</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>أكتوبر</t>
+        </is>
+      </c>
+      <c r="B5" s="6">
+        <f>D56</f>
+        <v/>
+      </c>
+      <c r="C5" s="6">
+        <f>E56</f>
+        <v/>
+      </c>
+      <c r="D5" s="6">
+        <f>F56</f>
+        <v/>
+      </c>
+      <c r="E5" s="6">
+        <f>G56</f>
+        <v/>
+      </c>
+      <c r="F5" s="6">
+        <f>H56</f>
+        <v/>
+      </c>
+      <c r="G5" s="7">
+        <f>IF(E5=0,"",C5/E5)</f>
+        <v/>
+      </c>
+      <c r="H5" s="7">
+        <f>IF(E5=0,"",D5/E5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>نوفمبر</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>لم يبدأ</t>
+        </is>
+      </c>
+      <c r="C6" s="6">
+        <f>I56</f>
+        <v/>
+      </c>
+      <c r="D6" s="6">
+        <f>J56</f>
+        <v/>
+      </c>
+      <c r="E6" s="6">
+        <f>K56</f>
+        <v/>
+      </c>
+      <c r="F6" s="6">
+        <f>L56</f>
+        <v/>
+      </c>
+      <c r="G6" s="7">
+        <f>IF(E6=0,"",C6/E6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="7">
+        <f>IF(E6=0,"",D6/E6)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>ديسمبر</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>لم يبدأ</t>
+        </is>
+      </c>
+      <c r="C7" s="6">
+        <f>M56</f>
+        <v/>
+      </c>
+      <c r="D7" s="6">
+        <f>N56</f>
+        <v/>
+      </c>
+      <c r="E7" s="6">
+        <f>O56</f>
+        <v/>
+      </c>
+      <c r="F7" s="6">
+        <f>P56</f>
+        <v/>
+      </c>
+      <c r="G7" s="7">
+        <f>IF(E7=0,"",C7/E7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="7">
+        <f>IF(E7=0,"",D7/E7)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>مجموع الثلاثة أشهر</t>
+        </is>
+      </c>
+      <c r="B8" s="9" t="n"/>
+      <c r="C8" s="9">
+        <f>SUM(C5:C7)</f>
+        <v/>
+      </c>
+      <c r="D8" s="9">
+        <f>SUM(D5:D7)</f>
+        <v/>
+      </c>
+      <c r="E8" s="9">
+        <f>SUM(E5:E7)</f>
+        <v/>
+      </c>
+      <c r="F8" s="9">
+        <f>SUM(F5:F7)</f>
+        <v/>
+      </c>
+      <c r="G8" s="10">
+        <f>IF(E8=0,"",C8/E8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="10">
+        <f>IF(E8=0,"",D8/E8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>ملاحظة: أكتوبر لم ينتهِ؛ المحصل حتى تاريخه جزئي. المتوقع لأكتوبر هو الشهر كاملاً.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
+        <is>
+          <t>رقم الحساب</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="inlineStr">
+        <is>
+          <t>اسم الحساب</t>
+        </is>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>التبويب</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="inlineStr">
+        <is>
+          <t>أكتوبر: المحصل حتى تاريخه</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>أكتوبر: المتوقع أساسي</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>أكتوبر: المتوقع أسوأ</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>أكتوبر: المستهدف</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>أكتوبر: المقدر</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>نوفمبر: المتوقع أساسي</t>
+        </is>
+      </c>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>نوفمبر: المتوقع أسوأ</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>نوفمبر: المستهدف</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>نوفمبر: المقدر</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>ديسمبر: المتوقع أساسي</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>ديسمبر: المتوقع أسوأ</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>ديسمبر: المستهدف</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>ديسمبر: المقدر</t>
+        </is>
+      </c>
+      <c r="Q12" s="4" t="inlineStr">
+        <is>
+          <t>حصة نوفمبر من نوفمبر+ديسمبر</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>14155</t>
+        </is>
+      </c>
+      <c r="B13" s="5">
+        <f>'توقع المحصل (المراقبة)'!B6</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>'توقع المحصل (المراقبة)'!C6</f>
+        <v/>
+      </c>
+      <c r="D13" s="6">
+        <f>'توقع المحصل (المراقبة)'!E6</f>
+        <v/>
+      </c>
+      <c r="E13" s="6">
+        <f>'توقع المحصل (المراقبة)'!E6+'توقع المحصل (المراقبة)'!K6</f>
+        <v/>
+      </c>
+      <c r="F13" s="6">
+        <f>'توقع المحصل (المراقبة)'!E6+'توقع المحصل (المراقبة)'!N6</f>
+        <v/>
+      </c>
+      <c r="G13" s="6" t="n">
+        <v>199630948.23</v>
+      </c>
+      <c r="H13" s="6" t="n">
+        <v>170742307.37</v>
+      </c>
+      <c r="I13" s="6">
+        <f>'توقع المحصل (المراقبة)'!L6*Q13</f>
+        <v/>
+      </c>
+      <c r="J13" s="6">
+        <f>'توقع المحصل (المراقبة)'!O6*Q13</f>
+        <v/>
+      </c>
+      <c r="K13" s="6" t="n">
+        <v>66228430.48</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>56657600.43</v>
+      </c>
+      <c r="M13" s="6">
+        <f>'توقع المحصل (المراقبة)'!L6*(1-Q13)</f>
+        <v/>
+      </c>
+      <c r="N13" s="6">
+        <f>'توقع المحصل (المراقبة)'!O6*(1-Q13)</f>
+        <v/>
+      </c>
+      <c r="O13" s="6" t="n">
+        <v>42439465.39</v>
+      </c>
+      <c r="P13" s="6" t="n">
+        <v>36018078.68</v>
+      </c>
+      <c r="Q13" s="19" t="n">
+        <v>0.6493</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
+        <is>
+          <t>142162</t>
+        </is>
+      </c>
+      <c r="B14" s="5">
+        <f>'توقع المحصل (المراقبة)'!B7</f>
+        <v/>
+      </c>
+      <c r="C14" s="5">
+        <f>'توقع المحصل (المراقبة)'!C7</f>
+        <v/>
+      </c>
+      <c r="D14" s="6">
+        <f>'توقع المحصل (المراقبة)'!E7</f>
+        <v/>
+      </c>
+      <c r="E14" s="6">
+        <f>'توقع المحصل (المراقبة)'!E7+'توقع المحصل (المراقبة)'!K7</f>
+        <v/>
+      </c>
+      <c r="F14" s="6">
+        <f>'توقع المحصل (المراقبة)'!E7+'توقع المحصل (المراقبة)'!N7</f>
+        <v/>
+      </c>
+      <c r="G14" s="6" t="n">
+        <v>28067945.58</v>
+      </c>
+      <c r="H14" s="6" t="n">
+        <v>14063993.05</v>
+      </c>
+      <c r="I14" s="6">
+        <f>'توقع المحصل (المراقبة)'!L7*Q14</f>
+        <v/>
+      </c>
+      <c r="J14" s="6">
+        <f>'توقع المحصل (المراقبة)'!O7*Q14</f>
+        <v/>
+      </c>
+      <c r="K14" s="6" t="n">
+        <v>418948643.78</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>6688022.26</v>
+      </c>
+      <c r="M14" s="6">
+        <f>'توقع المحصل (المراقبة)'!L7*(1-Q14)</f>
+        <v/>
+      </c>
+      <c r="N14" s="6">
+        <f>'توقع المحصل (المراقبة)'!O7*(1-Q14)</f>
+        <v/>
+      </c>
+      <c r="O14" s="6" t="n">
+        <v>16895879.24</v>
+      </c>
+      <c r="P14" s="6" t="n">
+        <v>8879088.32</v>
+      </c>
+      <c r="Q14" s="19" t="n">
+        <v>0.4582</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>1438001</t>
+        </is>
+      </c>
+      <c r="B15" s="5">
+        <f>'توقع المحصل (المراقبة)'!B8</f>
+        <v/>
+      </c>
+      <c r="C15" s="5">
+        <f>'توقع المحصل (المراقبة)'!C8</f>
+        <v/>
+      </c>
+      <c r="D15" s="6">
+        <f>'توقع المحصل (المراقبة)'!E8</f>
+        <v/>
+      </c>
+      <c r="E15" s="6">
+        <f>'توقع المحصل (المراقبة)'!E8+'توقع المحصل (المراقبة)'!K8</f>
+        <v/>
+      </c>
+      <c r="F15" s="6">
+        <f>'توقع المحصل (المراقبة)'!E8+'توقع المحصل (المراقبة)'!N8</f>
+        <v/>
+      </c>
+      <c r="G15" s="6" t="n">
+        <v>42809498.94</v>
+      </c>
+      <c r="H15" s="6" t="n">
+        <v>40632797.85</v>
+      </c>
+      <c r="I15" s="6">
+        <f>'توقع المحصل (المراقبة)'!L8*Q15</f>
+        <v/>
+      </c>
+      <c r="J15" s="6">
+        <f>'توقع المحصل (المراقبة)'!O8*Q15</f>
+        <v/>
+      </c>
+      <c r="K15" s="6" t="n">
+        <v>28537922.26</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>27001273.44</v>
+      </c>
+      <c r="M15" s="6">
+        <f>'توقع المحصل (المراقبة)'!L8*(1-Q15)</f>
+        <v/>
+      </c>
+      <c r="N15" s="6">
+        <f>'توقع المحصل (المراقبة)'!O8*(1-Q15)</f>
+        <v/>
+      </c>
+      <c r="O15" s="6" t="n">
+        <v>27405164.21</v>
+      </c>
+      <c r="P15" s="6" t="n">
+        <v>25819765.93</v>
+      </c>
+      <c r="Q15" s="19" t="n">
+        <v>0.4733</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="5" t="inlineStr">
+        <is>
+          <t>11452104</t>
+        </is>
+      </c>
+      <c r="B16" s="5">
+        <f>'توقع المحصل (المراقبة)'!B9</f>
+        <v/>
+      </c>
+      <c r="C16" s="5">
+        <f>'توقع المحصل (المراقبة)'!C9</f>
+        <v/>
+      </c>
+      <c r="D16" s="6">
+        <f>'توقع المحصل (المراقبة)'!E9</f>
+        <v/>
+      </c>
+      <c r="E16" s="6">
+        <f>'توقع المحصل (المراقبة)'!E9+'توقع المحصل (المراقبة)'!K9</f>
+        <v/>
+      </c>
+      <c r="F16" s="6">
+        <f>'توقع المحصل (المراقبة)'!E9+'توقع المحصل (المراقبة)'!N9</f>
+        <v/>
+      </c>
+      <c r="G16" s="6" t="n">
+        <v>27386694.11</v>
+      </c>
+      <c r="H16" s="6" t="n">
+        <v>24713799.54</v>
+      </c>
+      <c r="I16" s="6">
+        <f>'توقع المحصل (المراقبة)'!L9*Q16</f>
+        <v/>
+      </c>
+      <c r="J16" s="6">
+        <f>'توقع المحصل (المراقبة)'!O9*Q16</f>
+        <v/>
+      </c>
+      <c r="K16" s="6" t="n">
+        <v>18812341.93</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>14484009.75</v>
+      </c>
+      <c r="M16" s="6">
+        <f>'توقع المحصل (المراقبة)'!L9*(1-Q16)</f>
+        <v/>
+      </c>
+      <c r="N16" s="6">
+        <f>'توقع المحصل (المراقبة)'!O9*(1-Q16)</f>
+        <v/>
+      </c>
+      <c r="O16" s="6" t="n">
+        <v>27342479.23</v>
+      </c>
+      <c r="P16" s="6" t="n">
+        <v>23009908.66</v>
+      </c>
+      <c r="Q16" s="19" t="n">
+        <v>0.4334</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>11452103</t>
+        </is>
+      </c>
+      <c r="B17" s="5">
+        <f>'توقع المحصل (المراقبة)'!B10</f>
+        <v/>
+      </c>
+      <c r="C17" s="5">
+        <f>'توقع المحصل (المراقبة)'!C10</f>
+        <v/>
+      </c>
+      <c r="D17" s="6">
+        <f>'توقع المحصل (المراقبة)'!E10</f>
+        <v/>
+      </c>
+      <c r="E17" s="6">
+        <f>'توقع المحصل (المراقبة)'!E10+'توقع المحصل (المراقبة)'!K10</f>
+        <v/>
+      </c>
+      <c r="F17" s="6">
+        <f>'توقع المحصل (المراقبة)'!E10+'توقع المحصل (المراقبة)'!N10</f>
+        <v/>
+      </c>
+      <c r="G17" s="6" t="n">
+        <v>24670480.29</v>
+      </c>
+      <c r="H17" s="6" t="n">
+        <v>27405051.69</v>
+      </c>
+      <c r="I17" s="6">
+        <f>'توقع المحصل (المراقبة)'!L10*Q17</f>
+        <v/>
+      </c>
+      <c r="J17" s="6">
+        <f>'توقع المحصل (المراقبة)'!O10*Q17</f>
+        <v/>
+      </c>
+      <c r="K17" s="6" t="n">
+        <v>20693616.54</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>17088218.34</v>
+      </c>
+      <c r="M17" s="6">
+        <f>'توقع المحصل (المراقبة)'!L10*(1-Q17)</f>
+        <v/>
+      </c>
+      <c r="N17" s="6">
+        <f>'توقع المحصل (المراقبة)'!O10*(1-Q17)</f>
+        <v/>
+      </c>
+      <c r="O17" s="6" t="n">
+        <v>25538510.67</v>
+      </c>
+      <c r="P17" s="6" t="n">
+        <v>21775502.52</v>
+      </c>
+      <c r="Q17" s="19" t="n">
+        <v>0.4359</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="inlineStr">
+        <is>
+          <t>11452512</t>
+        </is>
+      </c>
+      <c r="B18" s="5">
+        <f>'توقع المحصل (المراقبة)'!B11</f>
+        <v/>
+      </c>
+      <c r="C18" s="5">
+        <f>'توقع المحصل (المراقبة)'!C11</f>
+        <v/>
+      </c>
+      <c r="D18" s="6">
+        <f>'توقع المحصل (المراقبة)'!E11</f>
+        <v/>
+      </c>
+      <c r="E18" s="6">
+        <f>'توقع المحصل (المراقبة)'!E11+'توقع المحصل (المراقبة)'!K11</f>
+        <v/>
+      </c>
+      <c r="F18" s="6">
+        <f>'توقع المحصل (المراقبة)'!E11+'توقع المحصل (المراقبة)'!N11</f>
+        <v/>
+      </c>
+      <c r="G18" s="6" t="n">
+        <v>21887337.58</v>
+      </c>
+      <c r="H18" s="6" t="n">
+        <v>21855262.79</v>
+      </c>
+      <c r="I18" s="6">
+        <f>'توقع المحصل (المراقبة)'!L11*Q18</f>
+        <v/>
+      </c>
+      <c r="J18" s="6">
+        <f>'توقع المحصل (المراقبة)'!O11*Q18</f>
+        <v/>
+      </c>
+      <c r="K18" s="6" t="n">
+        <v>13388655.95</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>13342435.15</v>
+      </c>
+      <c r="M18" s="6">
+        <f>'توقع المحصل (المراقبة)'!L11*(1-Q18)</f>
+        <v/>
+      </c>
+      <c r="N18" s="6">
+        <f>'توقع المحصل (المراقبة)'!O11*(1-Q18)</f>
+        <v/>
+      </c>
+      <c r="O18" s="6" t="n">
+        <v>18892122.62</v>
+      </c>
+      <c r="P18" s="6" t="n">
+        <v>18860322.38</v>
+      </c>
+      <c r="Q18" s="19" t="n">
+        <v>0.417</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>1439</t>
+        </is>
+      </c>
+      <c r="B19" s="5">
+        <f>'توقع المحصل (المراقبة)'!B12</f>
+        <v/>
+      </c>
+      <c r="C19" s="5">
+        <f>'توقع المحصل (المراقبة)'!C12</f>
+        <v/>
+      </c>
+      <c r="D19" s="6">
+        <f>'توقع المحصل (المراقبة)'!E12</f>
+        <v/>
+      </c>
+      <c r="E19" s="6">
+        <f>'توقع المحصل (المراقبة)'!E12+'توقع المحصل (المراقبة)'!K12</f>
+        <v/>
+      </c>
+      <c r="F19" s="6">
+        <f>'توقع المحصل (المراقبة)'!E12+'توقع المحصل (المراقبة)'!N12</f>
+        <v/>
+      </c>
+      <c r="G19" s="6" t="n">
+        <v>153424.25</v>
+      </c>
+      <c r="H19" s="6" t="n">
+        <v>36724.19</v>
+      </c>
+      <c r="I19" s="6">
+        <f>'توقع المحصل (المراقبة)'!L12*Q19</f>
+        <v/>
+      </c>
+      <c r="J19" s="6">
+        <f>'توقع المحصل (المراقبة)'!O12*Q19</f>
+        <v/>
+      </c>
+      <c r="K19" s="6" t="n">
+        <v>3380581.8</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>112976.06</v>
+      </c>
+      <c r="M19" s="6">
+        <f>'توقع المحصل (المراقبة)'!L12*(1-Q19)</f>
+        <v/>
+      </c>
+      <c r="N19" s="6">
+        <f>'توقع المحصل (المراقبة)'!O12*(1-Q19)</f>
+        <v/>
+      </c>
+      <c r="O19" s="6" t="n">
+        <v>2982608.6</v>
+      </c>
+      <c r="P19" s="6" t="n">
+        <v>99799.22</v>
+      </c>
+      <c r="Q19" s="19" t="n">
+        <v>0.9116</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="inlineStr">
+        <is>
+          <t>11442</t>
+        </is>
+      </c>
+      <c r="B20" s="5">
+        <f>'توقع المحصل (المراقبة)'!B13</f>
+        <v/>
+      </c>
+      <c r="C20" s="5">
+        <f>'توقع المحصل (المراقبة)'!C13</f>
+        <v/>
+      </c>
+      <c r="D20" s="6">
+        <f>'توقع المحصل (المراقبة)'!E13</f>
+        <v/>
+      </c>
+      <c r="E20" s="6">
+        <f>'توقع المحصل (المراقبة)'!E13+'توقع المحصل (المراقبة)'!K13</f>
+        <v/>
+      </c>
+      <c r="F20" s="6">
+        <f>'توقع المحصل (المراقبة)'!E13+'توقع المحصل (المراقبة)'!N13</f>
+        <v/>
+      </c>
+      <c r="G20" s="6" t="n">
+        <v>25698392.79</v>
+      </c>
+      <c r="H20" s="6" t="n">
+        <v>23623576.12</v>
+      </c>
+      <c r="I20" s="6">
+        <f>'توقع المحصل (المراقبة)'!L13*Q20</f>
+        <v/>
+      </c>
+      <c r="J20" s="6">
+        <f>'توقع المحصل (المراقبة)'!O13*Q20</f>
+        <v/>
+      </c>
+      <c r="K20" s="6" t="n">
+        <v>19850210.09</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>18250834.83</v>
+      </c>
+      <c r="M20" s="6">
+        <f>'توقع المحصل (المراقبة)'!L13*(1-Q20)</f>
+        <v/>
+      </c>
+      <c r="N20" s="6">
+        <f>'توقع المحصل (المراقبة)'!O13*(1-Q20)</f>
+        <v/>
+      </c>
+      <c r="O20" s="6" t="n">
+        <v>23107944.17</v>
+      </c>
+      <c r="P20" s="6" t="n">
+        <v>21244662.85</v>
+      </c>
+      <c r="Q20" s="19" t="n">
+        <v>0.5515</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
+          <t>1421999</t>
+        </is>
+      </c>
+      <c r="B21" s="5">
+        <f>'توقع المحصل (المراقبة)'!B14</f>
+        <v/>
+      </c>
+      <c r="C21" s="5">
+        <f>'توقع المحصل (المراقبة)'!C14</f>
+        <v/>
+      </c>
+      <c r="D21" s="6">
+        <f>'توقع المحصل (المراقبة)'!E14</f>
+        <v/>
+      </c>
+      <c r="E21" s="6">
+        <f>'توقع المحصل (المراقبة)'!E14+'توقع المحصل (المراقبة)'!K14</f>
+        <v/>
+      </c>
+      <c r="F21" s="6">
+        <f>'توقع المحصل (المراقبة)'!E14+'توقع المحصل (المراقبة)'!N14</f>
+        <v/>
+      </c>
+      <c r="G21" s="6" t="n">
+        <v>7531118.23</v>
+      </c>
+      <c r="H21" s="6" t="n">
+        <v>7391205.32</v>
+      </c>
+      <c r="I21" s="6">
+        <f>'توقع المحصل (المراقبة)'!L14*Q21</f>
+        <v/>
+      </c>
+      <c r="J21" s="6">
+        <f>'توقع المحصل (المراقبة)'!O14*Q21</f>
+        <v/>
+      </c>
+      <c r="K21" s="6" t="n">
+        <v>2119658.52</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>2115740.32</v>
+      </c>
+      <c r="M21" s="6">
+        <f>'توقع المحصل (المراقبة)'!L14*(1-Q21)</f>
+        <v/>
+      </c>
+      <c r="N21" s="6">
+        <f>'توقع المحصل (المراقبة)'!O14*(1-Q21)</f>
+        <v/>
+      </c>
+      <c r="O21" s="6" t="n">
+        <v>9129947.939999999</v>
+      </c>
+      <c r="P21" s="6" t="n">
+        <v>9098069.960000001</v>
+      </c>
+      <c r="Q21" s="19" t="n">
+        <v>0.4651</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>142113</t>
+        </is>
+      </c>
+      <c r="B22" s="5">
+        <f>'توقع المحصل (المراقبة)'!B15</f>
+        <v/>
+      </c>
+      <c r="C22" s="5">
+        <f>'توقع المحصل (المراقبة)'!C15</f>
+        <v/>
+      </c>
+      <c r="D22" s="6">
+        <f>'توقع المحصل (المراقبة)'!E15</f>
+        <v/>
+      </c>
+      <c r="E22" s="6">
+        <f>'توقع المحصل (المراقبة)'!E15+'توقع المحصل (المراقبة)'!K15</f>
+        <v/>
+      </c>
+      <c r="F22" s="6">
+        <f>'توقع المحصل (المراقبة)'!E15+'توقع المحصل (المراقبة)'!N15</f>
+        <v/>
+      </c>
+      <c r="G22" s="6" t="n">
+        <v>6925446.95</v>
+      </c>
+      <c r="H22" s="6" t="n">
+        <v>6820552.85</v>
+      </c>
+      <c r="I22" s="6">
+        <f>'توقع المحصل (المراقبة)'!L15*Q22</f>
+        <v/>
+      </c>
+      <c r="J22" s="6">
+        <f>'توقع المحصل (المراقبة)'!O15*Q22</f>
+        <v/>
+      </c>
+      <c r="K22" s="6" t="n">
+        <v>7021788.87</v>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>6892069.73</v>
+      </c>
+      <c r="M22" s="6">
+        <f>'توقع المحصل (المراقبة)'!L15*(1-Q22)</f>
+        <v/>
+      </c>
+      <c r="N22" s="6">
+        <f>'توقع المحصل (المراقبة)'!O15*(1-Q22)</f>
+        <v/>
+      </c>
+      <c r="O22" s="6" t="n">
+        <v>7262073.52</v>
+      </c>
+      <c r="P22" s="6" t="n">
+        <v>7813646.82</v>
+      </c>
+      <c r="Q22" s="19" t="n">
+        <v>0.4651</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>1431</t>
+        </is>
+      </c>
+      <c r="B23" s="5">
+        <f>'توقع المحصل (المراقبة)'!B16</f>
+        <v/>
+      </c>
+      <c r="C23" s="5">
+        <f>'توقع المحصل (المراقبة)'!C16</f>
+        <v/>
+      </c>
+      <c r="D23" s="6">
+        <f>'توقع المحصل (المراقبة)'!E16</f>
+        <v/>
+      </c>
+      <c r="E23" s="6">
+        <f>'توقع المحصل (المراقبة)'!E16+'توقع المحصل (المراقبة)'!K16</f>
+        <v/>
+      </c>
+      <c r="F23" s="6">
+        <f>'توقع المحصل (المراقبة)'!E16+'توقع المحصل (المراقبة)'!N16</f>
+        <v/>
+      </c>
+      <c r="G23" s="6" t="n">
+        <v>7500273</v>
+      </c>
+      <c r="H23" s="6" t="n">
+        <v>3000273</v>
+      </c>
+      <c r="I23" s="6">
+        <f>'توقع المحصل (المراقبة)'!L16*Q23</f>
+        <v/>
+      </c>
+      <c r="J23" s="6">
+        <f>'توقع المحصل (المراقبة)'!O16*Q23</f>
+        <v/>
+      </c>
+      <c r="K23" s="6" t="n">
+        <v>7500273</v>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>3000273</v>
+      </c>
+      <c r="M23" s="6">
+        <f>'توقع المحصل (المراقبة)'!L16*(1-Q23)</f>
+        <v/>
+      </c>
+      <c r="N23" s="6">
+        <f>'توقع المحصل (المراقبة)'!O16*(1-Q23)</f>
+        <v/>
+      </c>
+      <c r="O23" s="6" t="n">
+        <v>14500281</v>
+      </c>
+      <c r="P23" s="6" t="n">
+        <v>5800281</v>
+      </c>
+      <c r="Q23" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>1421909</t>
+        </is>
+      </c>
+      <c r="B24" s="5">
+        <f>'توقع المحصل (المراقبة)'!B17</f>
+        <v/>
+      </c>
+      <c r="C24" s="5">
+        <f>'توقع المحصل (المراقبة)'!C17</f>
+        <v/>
+      </c>
+      <c r="D24" s="6">
+        <f>'توقع المحصل (المراقبة)'!E17</f>
+        <v/>
+      </c>
+      <c r="E24" s="6">
+        <f>'توقع المحصل (المراقبة)'!E17+'توقع المحصل (المراقبة)'!K17</f>
+        <v/>
+      </c>
+      <c r="F24" s="6">
+        <f>'توقع المحصل (المراقبة)'!E17+'توقع المحصل (المراقبة)'!N17</f>
+        <v/>
+      </c>
+      <c r="G24" s="6" t="n">
+        <v>9414543.6</v>
+      </c>
+      <c r="H24" s="6" t="n">
+        <v>7293692.63</v>
+      </c>
+      <c r="I24" s="6">
+        <f>'توقع المحصل (المراقبة)'!L17*Q24</f>
+        <v/>
+      </c>
+      <c r="J24" s="6">
+        <f>'توقع المحصل (المراقبة)'!O17*Q24</f>
+        <v/>
+      </c>
+      <c r="K24" s="6" t="n">
+        <v>6515033.17</v>
+      </c>
+      <c r="L24" s="6" t="n">
+        <v>5118244.93</v>
+      </c>
+      <c r="M24" s="6">
+        <f>'توقع المحصل (المراقبة)'!L17*(1-Q24)</f>
+        <v/>
+      </c>
+      <c r="N24" s="6">
+        <f>'توقع المحصل (المراقبة)'!O17*(1-Q24)</f>
+        <v/>
+      </c>
+      <c r="O24" s="6" t="n">
+        <v>5125605.45</v>
+      </c>
+      <c r="P24" s="6" t="n">
+        <v>4128451.39</v>
+      </c>
+      <c r="Q24" s="19" t="n">
+        <v>0.4552</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
+          <t>1421911</t>
+        </is>
+      </c>
+      <c r="B25" s="5">
+        <f>'توقع المحصل (المراقبة)'!B18</f>
+        <v/>
+      </c>
+      <c r="C25" s="5">
+        <f>'توقع المحصل (المراقبة)'!C18</f>
+        <v/>
+      </c>
+      <c r="D25" s="6">
+        <f>'توقع المحصل (المراقبة)'!E18</f>
+        <v/>
+      </c>
+      <c r="E25" s="6">
+        <f>'توقع المحصل (المراقبة)'!E18+'توقع المحصل (المراقبة)'!K18</f>
+        <v/>
+      </c>
+      <c r="F25" s="6">
+        <f>'توقع المحصل (المراقبة)'!E18+'توقع المحصل (المراقبة)'!N18</f>
+        <v/>
+      </c>
+      <c r="G25" s="6" t="n">
+        <v>6863252.07</v>
+      </c>
+      <c r="H25" s="6" t="n">
+        <v>6483432.13</v>
+      </c>
+      <c r="I25" s="6">
+        <f>'توقع المحصل (المراقبة)'!L18*Q25</f>
+        <v/>
+      </c>
+      <c r="J25" s="6">
+        <f>'توقع المحصل (المراقبة)'!O18*Q25</f>
+        <v/>
+      </c>
+      <c r="K25" s="6" t="n">
+        <v>5768559.67</v>
+      </c>
+      <c r="L25" s="6" t="n">
+        <v>5450693.63</v>
+      </c>
+      <c r="M25" s="6">
+        <f>'توقع المحصل (المراقبة)'!L18*(1-Q25)</f>
+        <v/>
+      </c>
+      <c r="N25" s="6">
+        <f>'توقع المحصل (المراقبة)'!O18*(1-Q25)</f>
+        <v/>
+      </c>
+      <c r="O25" s="6" t="n">
+        <v>5209792.3</v>
+      </c>
+      <c r="P25" s="6" t="n">
+        <v>4925069.99</v>
+      </c>
+      <c r="Q25" s="19" t="n">
+        <v>0.4982</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>144122</t>
+        </is>
+      </c>
+      <c r="B26" s="5">
+        <f>'توقع المحصل (المراقبة)'!B19</f>
+        <v/>
+      </c>
+      <c r="C26" s="5">
+        <f>'توقع المحصل (المراقبة)'!C19</f>
+        <v/>
+      </c>
+      <c r="D26" s="6">
+        <f>'توقع المحصل (المراقبة)'!E19</f>
+        <v/>
+      </c>
+      <c r="E26" s="6">
+        <f>'توقع المحصل (المراقبة)'!E19+'توقع المحصل (المراقبة)'!K19</f>
+        <v/>
+      </c>
+      <c r="F26" s="6">
+        <f>'توقع المحصل (المراقبة)'!E19+'توقع المحصل (المراقبة)'!N19</f>
+        <v/>
+      </c>
+      <c r="G26" s="6" t="n">
+        <v>437108.39</v>
+      </c>
+      <c r="H26" s="6" t="n">
+        <v>895275.75</v>
+      </c>
+      <c r="I26" s="6">
+        <f>'توقع المحصل (المراقبة)'!L19*Q26</f>
+        <v/>
+      </c>
+      <c r="J26" s="6">
+        <f>'توقع المحصل (المراقبة)'!O19*Q26</f>
+        <v/>
+      </c>
+      <c r="K26" s="6" t="n">
+        <v>437120.39</v>
+      </c>
+      <c r="L26" s="6" t="n">
+        <v>895281.75</v>
+      </c>
+      <c r="M26" s="6">
+        <f>'توقع المحصل (المراقبة)'!L19*(1-Q26)</f>
+        <v/>
+      </c>
+      <c r="N26" s="6">
+        <f>'توقع المحصل (المراقبة)'!O19*(1-Q26)</f>
+        <v/>
+      </c>
+      <c r="O26" s="6" t="n">
+        <v>684676.76</v>
+      </c>
+      <c r="P26" s="6" t="n">
+        <v>1247604.81</v>
+      </c>
+      <c r="Q26" s="19" t="n">
+        <v>0.4959</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>11452108</t>
+        </is>
+      </c>
+      <c r="B27" s="5">
+        <f>'توقع المحصل (المراقبة)'!B20</f>
+        <v/>
+      </c>
+      <c r="C27" s="5">
+        <f>'توقع المحصل (المراقبة)'!C20</f>
+        <v/>
+      </c>
+      <c r="D27" s="6">
+        <f>'توقع المحصل (المراقبة)'!E20</f>
+        <v/>
+      </c>
+      <c r="E27" s="6">
+        <f>'توقع المحصل (المراقبة)'!E20+'توقع المحصل (المراقبة)'!K20</f>
+        <v/>
+      </c>
+      <c r="F27" s="6">
+        <f>'توقع المحصل (المراقبة)'!E20+'توقع المحصل (المراقبة)'!N20</f>
+        <v/>
+      </c>
+      <c r="G27" s="6" t="n">
+        <v>2226695.76</v>
+      </c>
+      <c r="H27" s="6" t="n">
+        <v>1882045.8</v>
+      </c>
+      <c r="I27" s="6">
+        <f>'توقع المحصل (المراقبة)'!L20*Q27</f>
+        <v/>
+      </c>
+      <c r="J27" s="6">
+        <f>'توقع المحصل (المراقبة)'!O20*Q27</f>
+        <v/>
+      </c>
+      <c r="K27" s="6" t="n">
+        <v>2909846.24</v>
+      </c>
+      <c r="L27" s="6" t="n">
+        <v>1624824.26</v>
+      </c>
+      <c r="M27" s="6">
+        <f>'توقع المحصل (المراقبة)'!L20*(1-Q27)</f>
+        <v/>
+      </c>
+      <c r="N27" s="6">
+        <f>'توقع المحصل (المراقبة)'!O20*(1-Q27)</f>
+        <v/>
+      </c>
+      <c r="O27" s="6" t="n">
+        <v>2950894.62</v>
+      </c>
+      <c r="P27" s="6" t="n">
+        <v>1562481.6</v>
+      </c>
+      <c r="Q27" s="19" t="n">
+        <v>0.4196</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>1422108</t>
+        </is>
+      </c>
+      <c r="B28" s="5">
+        <f>'توقع المحصل (المراقبة)'!B21</f>
+        <v/>
+      </c>
+      <c r="C28" s="5">
+        <f>'توقع المحصل (المراقبة)'!C21</f>
+        <v/>
+      </c>
+      <c r="D28" s="6">
+        <f>'توقع المحصل (المراقبة)'!E21</f>
+        <v/>
+      </c>
+      <c r="E28" s="6">
+        <f>'توقع المحصل (المراقبة)'!E21+'توقع المحصل (المراقبة)'!K21</f>
+        <v/>
+      </c>
+      <c r="F28" s="6">
+        <f>'توقع المحصل (المراقبة)'!E21+'توقع المحصل (المراقبة)'!N21</f>
+        <v/>
+      </c>
+      <c r="G28" s="6" t="n">
+        <v>1100942.4</v>
+      </c>
+      <c r="H28" s="6" t="n">
+        <v>736646.91</v>
+      </c>
+      <c r="I28" s="6">
+        <f>'توقع المحصل (المراقبة)'!L21*Q28</f>
+        <v/>
+      </c>
+      <c r="J28" s="6">
+        <f>'توقع المحصل (المراقبة)'!O21*Q28</f>
+        <v/>
+      </c>
+      <c r="K28" s="6" t="n">
+        <v>1662305.66</v>
+      </c>
+      <c r="L28" s="6" t="n">
+        <v>1083911.35</v>
+      </c>
+      <c r="M28" s="6">
+        <f>'توقع المحصل (المراقبة)'!L21*(1-Q28)</f>
+        <v/>
+      </c>
+      <c r="N28" s="6">
+        <f>'توقع المحصل (المراقبة)'!O21*(1-Q28)</f>
+        <v/>
+      </c>
+      <c r="O28" s="6" t="n">
+        <v>1567129.26</v>
+      </c>
+      <c r="P28" s="6" t="n">
+        <v>753291.66</v>
+      </c>
+      <c r="Q28" s="19" t="n">
+        <v>0.5244</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>1422121</t>
+        </is>
+      </c>
+      <c r="B29" s="5">
+        <f>'توقع المحصل (المراقبة)'!B22</f>
+        <v/>
+      </c>
+      <c r="C29" s="5">
+        <f>'توقع المحصل (المراقبة)'!C22</f>
+        <v/>
+      </c>
+      <c r="D29" s="6">
+        <f>'توقع المحصل (المراقبة)'!E22</f>
+        <v/>
+      </c>
+      <c r="E29" s="6">
+        <f>'توقع المحصل (المراقبة)'!E22+'توقع المحصل (المراقبة)'!K22</f>
+        <v/>
+      </c>
+      <c r="F29" s="6">
+        <f>'توقع المحصل (المراقبة)'!E22+'توقع المحصل (المراقبة)'!N22</f>
+        <v/>
+      </c>
+      <c r="G29" s="6" t="n">
+        <v>1865536.6</v>
+      </c>
+      <c r="H29" s="6" t="n">
+        <v>1717316.24</v>
+      </c>
+      <c r="I29" s="6">
+        <f>'توقع المحصل (المراقبة)'!L22*Q29</f>
+        <v/>
+      </c>
+      <c r="J29" s="6">
+        <f>'توقع المحصل (المراقبة)'!O22*Q29</f>
+        <v/>
+      </c>
+      <c r="K29" s="6" t="n">
+        <v>1246546.67</v>
+      </c>
+      <c r="L29" s="6" t="n">
+        <v>1173450.17</v>
+      </c>
+      <c r="M29" s="6">
+        <f>'توقع المحصل (المراقبة)'!L22*(1-Q29)</f>
+        <v/>
+      </c>
+      <c r="N29" s="6">
+        <f>'توقع المحصل (المراقبة)'!O22*(1-Q29)</f>
+        <v/>
+      </c>
+      <c r="O29" s="6" t="n">
+        <v>1183471.33</v>
+      </c>
+      <c r="P29" s="6" t="n">
+        <v>1102027.12</v>
+      </c>
+      <c r="Q29" s="19" t="n">
+        <v>0.4808</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>11452111</t>
+        </is>
+      </c>
+      <c r="B30" s="5">
+        <f>'توقع المحصل (المراقبة)'!B23</f>
+        <v/>
+      </c>
+      <c r="C30" s="5">
+        <f>'توقع المحصل (المراقبة)'!C23</f>
+        <v/>
+      </c>
+      <c r="D30" s="6">
+        <f>'توقع المحصل (المراقبة)'!E23</f>
+        <v/>
+      </c>
+      <c r="E30" s="6">
+        <f>'توقع المحصل (المراقبة)'!E23+'توقع المحصل (المراقبة)'!K23</f>
+        <v/>
+      </c>
+      <c r="F30" s="6">
+        <f>'توقع المحصل (المراقبة)'!E23+'توقع المحصل (المراقبة)'!N23</f>
+        <v/>
+      </c>
+      <c r="G30" s="6" t="n">
+        <v>469447.53</v>
+      </c>
+      <c r="H30" s="6" t="n">
+        <v>552264.49</v>
+      </c>
+      <c r="I30" s="6">
+        <f>'توقع المحصل (المراقبة)'!L23*Q30</f>
+        <v/>
+      </c>
+      <c r="J30" s="6">
+        <f>'توقع المحصل (المراقبة)'!O23*Q30</f>
+        <v/>
+      </c>
+      <c r="K30" s="6" t="n">
+        <v>395145.64</v>
+      </c>
+      <c r="L30" s="6" t="n">
+        <v>299239.65</v>
+      </c>
+      <c r="M30" s="6">
+        <f>'توقع المحصل (المراقبة)'!L23*(1-Q30)</f>
+        <v/>
+      </c>
+      <c r="N30" s="6">
+        <f>'توقع المحصل (المراقبة)'!O23*(1-Q30)</f>
+        <v/>
+      </c>
+      <c r="O30" s="6" t="n">
+        <v>411424.61</v>
+      </c>
+      <c r="P30" s="6" t="n">
+        <v>301711.22</v>
+      </c>
+      <c r="Q30" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="5" t="inlineStr">
+        <is>
+          <t>142163</t>
+        </is>
+      </c>
+      <c r="B31" s="5">
+        <f>'توقع المحصل (المراقبة)'!B24</f>
+        <v/>
+      </c>
+      <c r="C31" s="5">
+        <f>'توقع المحصل (المراقبة)'!C24</f>
+        <v/>
+      </c>
+      <c r="D31" s="6">
+        <f>'توقع المحصل (المراقبة)'!E24</f>
+        <v/>
+      </c>
+      <c r="E31" s="6">
+        <f>'توقع المحصل (المراقبة)'!E24+'توقع المحصل (المراقبة)'!K24</f>
+        <v/>
+      </c>
+      <c r="F31" s="6">
+        <f>'توقع المحصل (المراقبة)'!E24+'توقع المحصل (المراقبة)'!N24</f>
+        <v/>
+      </c>
+      <c r="G31" s="6" t="n">
+        <v>1589560.87</v>
+      </c>
+      <c r="H31" s="6" t="n">
+        <v>1582915.68</v>
+      </c>
+      <c r="I31" s="6">
+        <f>'توقع المحصل (المراقبة)'!L24*Q31</f>
+        <v/>
+      </c>
+      <c r="J31" s="6">
+        <f>'توقع المحصل (المراقبة)'!O24*Q31</f>
+        <v/>
+      </c>
+      <c r="K31" s="6" t="n">
+        <v>10001631.64</v>
+      </c>
+      <c r="L31" s="6" t="n">
+        <v>9902394.689999999</v>
+      </c>
+      <c r="M31" s="6">
+        <f>'توقع المحصل (المراقبة)'!L24*(1-Q31)</f>
+        <v/>
+      </c>
+      <c r="N31" s="6">
+        <f>'توقع المحصل (المراقبة)'!O24*(1-Q31)</f>
+        <v/>
+      </c>
+      <c r="O31" s="6" t="n">
+        <v>3599329.08</v>
+      </c>
+      <c r="P31" s="6" t="n">
+        <v>3596725.38</v>
+      </c>
+      <c r="Q31" s="19" t="n">
+        <v>0.7526</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>1422109</t>
+        </is>
+      </c>
+      <c r="B32" s="5">
+        <f>'توقع المحصل (المراقبة)'!B25</f>
+        <v/>
+      </c>
+      <c r="C32" s="5">
+        <f>'توقع المحصل (المراقبة)'!C25</f>
+        <v/>
+      </c>
+      <c r="D32" s="6">
+        <f>'توقع المحصل (المراقبة)'!E25</f>
+        <v/>
+      </c>
+      <c r="E32" s="6">
+        <f>'توقع المحصل (المراقبة)'!E25+'توقع المحصل (المراقبة)'!K25</f>
+        <v/>
+      </c>
+      <c r="F32" s="6">
+        <f>'توقع المحصل (المراقبة)'!E25+'توقع المحصل (المراقبة)'!N25</f>
+        <v/>
+      </c>
+      <c r="G32" s="6" t="n">
+        <v>991297.6899999999</v>
+      </c>
+      <c r="H32" s="6" t="n">
+        <v>972478.89</v>
+      </c>
+      <c r="I32" s="6">
+        <f>'توقع المحصل (المراقبة)'!L25*Q32</f>
+        <v/>
+      </c>
+      <c r="J32" s="6">
+        <f>'توقع المحصل (المراقبة)'!O25*Q32</f>
+        <v/>
+      </c>
+      <c r="K32" s="6" t="n">
+        <v>335310.58</v>
+      </c>
+      <c r="L32" s="6" t="n">
+        <v>315787.68</v>
+      </c>
+      <c r="M32" s="6">
+        <f>'توقع المحصل (المراقبة)'!L25*(1-Q32)</f>
+        <v/>
+      </c>
+      <c r="N32" s="6">
+        <f>'توقع المحصل (المراقبة)'!O25*(1-Q32)</f>
+        <v/>
+      </c>
+      <c r="O32" s="6" t="n">
+        <v>395404.39</v>
+      </c>
+      <c r="P32" s="6" t="n">
+        <v>372358.38</v>
+      </c>
+      <c r="Q32" s="19" t="n">
+        <v>0.4935</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>1422202</t>
+        </is>
+      </c>
+      <c r="B33" s="5">
+        <f>'توقع المحصل (المراقبة)'!B26</f>
+        <v/>
+      </c>
+      <c r="C33" s="5">
+        <f>'توقع المحصل (المراقبة)'!C26</f>
+        <v/>
+      </c>
+      <c r="D33" s="6">
+        <f>'توقع المحصل (المراقبة)'!E26</f>
+        <v/>
+      </c>
+      <c r="E33" s="6">
+        <f>'توقع المحصل (المراقبة)'!E26+'توقع المحصل (المراقبة)'!K26</f>
+        <v/>
+      </c>
+      <c r="F33" s="6">
+        <f>'توقع المحصل (المراقبة)'!E26+'توقع المحصل (المراقبة)'!N26</f>
+        <v/>
+      </c>
+      <c r="G33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I33" s="6">
+        <f>'توقع المحصل (المراقبة)'!L26*Q33</f>
+        <v/>
+      </c>
+      <c r="J33" s="6">
+        <f>'توقع المحصل (المراقبة)'!O26*Q33</f>
+        <v/>
+      </c>
+      <c r="K33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M33" s="6">
+        <f>'توقع المحصل (المراقبة)'!L26*(1-Q33)</f>
+        <v/>
+      </c>
+      <c r="N33" s="6">
+        <f>'توقع المحصل (المراقبة)'!O26*(1-Q33)</f>
+        <v/>
+      </c>
+      <c r="O33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P33" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>1421910</t>
+        </is>
+      </c>
+      <c r="B34" s="5">
+        <f>'توقع المحصل (المراقبة)'!B27</f>
+        <v/>
+      </c>
+      <c r="C34" s="5">
+        <f>'توقع المحصل (المراقبة)'!C27</f>
+        <v/>
+      </c>
+      <c r="D34" s="6">
+        <f>'توقع المحصل (المراقبة)'!E27</f>
+        <v/>
+      </c>
+      <c r="E34" s="6">
+        <f>'توقع المحصل (المراقبة)'!E27+'توقع المحصل (المراقبة)'!K27</f>
+        <v/>
+      </c>
+      <c r="F34" s="6">
+        <f>'توقع المحصل (المراقبة)'!E27+'توقع المحصل (المراقبة)'!N27</f>
+        <v/>
+      </c>
+      <c r="G34" s="6" t="n">
+        <v>399206.5</v>
+      </c>
+      <c r="H34" s="6" t="n">
+        <v>361900.78</v>
+      </c>
+      <c r="I34" s="6">
+        <f>'توقع المحصل (المراقبة)'!L27*Q34</f>
+        <v/>
+      </c>
+      <c r="J34" s="6">
+        <f>'توقع المحصل (المراقبة)'!O27*Q34</f>
+        <v/>
+      </c>
+      <c r="K34" s="6" t="n">
+        <v>241075.56</v>
+      </c>
+      <c r="L34" s="6" t="n">
+        <v>218809.41</v>
+      </c>
+      <c r="M34" s="6">
+        <f>'توقع المحصل (المراقبة)'!L27*(1-Q34)</f>
+        <v/>
+      </c>
+      <c r="N34" s="6">
+        <f>'توقع المحصل (المراقبة)'!O27*(1-Q34)</f>
+        <v/>
+      </c>
+      <c r="O34" s="6" t="n">
+        <v>320808.69</v>
+      </c>
+      <c r="P34" s="6" t="n">
+        <v>294493.43</v>
+      </c>
+      <c r="Q34" s="19" t="n">
+        <v>0.5476</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="5" t="inlineStr">
+        <is>
+          <t>11452107</t>
+        </is>
+      </c>
+      <c r="B35" s="5">
+        <f>'توقع المحصل (المراقبة)'!B28</f>
+        <v/>
+      </c>
+      <c r="C35" s="5">
+        <f>'توقع المحصل (المراقبة)'!C28</f>
+        <v/>
+      </c>
+      <c r="D35" s="6">
+        <f>'توقع المحصل (المراقبة)'!E28</f>
+        <v/>
+      </c>
+      <c r="E35" s="6">
+        <f>'توقع المحصل (المراقبة)'!E28+'توقع المحصل (المراقبة)'!K28</f>
+        <v/>
+      </c>
+      <c r="F35" s="6">
+        <f>'توقع المحصل (المراقبة)'!E28+'توقع المحصل (المراقبة)'!N28</f>
+        <v/>
+      </c>
+      <c r="G35" s="6" t="n">
+        <v>202820.15</v>
+      </c>
+      <c r="H35" s="6" t="n">
+        <v>202793.8</v>
+      </c>
+      <c r="I35" s="6">
+        <f>'توقع المحصل (المراقبة)'!L28*Q35</f>
+        <v/>
+      </c>
+      <c r="J35" s="6">
+        <f>'توقع المحصل (المراقبة)'!O28*Q35</f>
+        <v/>
+      </c>
+      <c r="K35" s="6" t="n">
+        <v>222880.38</v>
+      </c>
+      <c r="L35" s="6" t="n">
+        <v>221226.66</v>
+      </c>
+      <c r="M35" s="6">
+        <f>'توقع المحصل (المراقبة)'!L28*(1-Q35)</f>
+        <v/>
+      </c>
+      <c r="N35" s="6">
+        <f>'توقع المحصل (المراقبة)'!O28*(1-Q35)</f>
+        <v/>
+      </c>
+      <c r="O35" s="6" t="n">
+        <v>327327.8</v>
+      </c>
+      <c r="P35" s="6" t="n">
+        <v>321070.35</v>
+      </c>
+      <c r="Q35" s="19" t="n">
+        <v>0.2724</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>1421901</t>
+        </is>
+      </c>
+      <c r="B36" s="5">
+        <f>'توقع المحصل (المراقبة)'!B29</f>
+        <v/>
+      </c>
+      <c r="C36" s="5">
+        <f>'توقع المحصل (المراقبة)'!C29</f>
+        <v/>
+      </c>
+      <c r="D36" s="6">
+        <f>'توقع المحصل (المراقبة)'!E29</f>
+        <v/>
+      </c>
+      <c r="E36" s="6">
+        <f>'توقع المحصل (المراقبة)'!E29+'توقع المحصل (المراقبة)'!K29</f>
+        <v/>
+      </c>
+      <c r="F36" s="6">
+        <f>'توقع المحصل (المراقبة)'!E29+'توقع المحصل (المراقبة)'!N29</f>
+        <v/>
+      </c>
+      <c r="G36" s="6" t="n">
+        <v>556368.8</v>
+      </c>
+      <c r="H36" s="6" t="n">
+        <v>733161.5</v>
+      </c>
+      <c r="I36" s="6">
+        <f>'توقع المحصل (المراقبة)'!L29*Q36</f>
+        <v/>
+      </c>
+      <c r="J36" s="6">
+        <f>'توقع المحصل (المراقبة)'!O29*Q36</f>
+        <v/>
+      </c>
+      <c r="K36" s="6" t="n">
+        <v>556377.2</v>
+      </c>
+      <c r="L36" s="6" t="n">
+        <v>733164</v>
+      </c>
+      <c r="M36" s="6">
+        <f>'توقع المحصل (المراقبة)'!L29*(1-Q36)</f>
+        <v/>
+      </c>
+      <c r="N36" s="6">
+        <f>'توقع المحصل (المراقبة)'!O29*(1-Q36)</f>
+        <v/>
+      </c>
+      <c r="O36" s="6" t="n">
+        <v>555958.98</v>
+      </c>
+      <c r="P36" s="6" t="n">
+        <v>733270.28</v>
+      </c>
+      <c r="Q36" s="19" t="n">
+        <v>0.6293</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="5" t="inlineStr">
+        <is>
+          <t>بدون رقم</t>
+        </is>
+      </c>
+      <c r="B37" s="5">
+        <f>'توقع المحصل (المراقبة)'!B30</f>
+        <v/>
+      </c>
+      <c r="C37" s="5">
+        <f>'توقع المحصل (المراقبة)'!C30</f>
+        <v/>
+      </c>
+      <c r="D37" s="6">
+        <f>'توقع المحصل (المراقبة)'!E30</f>
+        <v/>
+      </c>
+      <c r="E37" s="6">
+        <f>'توقع المحصل (المراقبة)'!E30+'توقع المحصل (المراقبة)'!K30</f>
+        <v/>
+      </c>
+      <c r="F37" s="6">
+        <f>'توقع المحصل (المراقبة)'!E30+'توقع المحصل (المراقبة)'!N30</f>
+        <v/>
+      </c>
+      <c r="G37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I37" s="6">
+        <f>'توقع المحصل (المراقبة)'!L30*Q37</f>
+        <v/>
+      </c>
+      <c r="J37" s="6">
+        <f>'توقع المحصل (المراقبة)'!O30*Q37</f>
+        <v/>
+      </c>
+      <c r="K37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M37" s="6">
+        <f>'توقع المحصل (المراقبة)'!L30*(1-Q37)</f>
+        <v/>
+      </c>
+      <c r="N37" s="6">
+        <f>'توقع المحصل (المراقبة)'!O30*(1-Q37)</f>
+        <v/>
+      </c>
+      <c r="O37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P37" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="19" t="n">
+        <v>0.4822</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>1421912</t>
+        </is>
+      </c>
+      <c r="B38" s="5">
+        <f>'توقع المحصل (المراقبة)'!B31</f>
+        <v/>
+      </c>
+      <c r="C38" s="5">
+        <f>'توقع المحصل (المراقبة)'!C31</f>
+        <v/>
+      </c>
+      <c r="D38" s="6">
+        <f>'توقع المحصل (المراقبة)'!E31</f>
+        <v/>
+      </c>
+      <c r="E38" s="6">
+        <f>'توقع المحصل (المراقبة)'!E31+'توقع المحصل (المراقبة)'!K31</f>
+        <v/>
+      </c>
+      <c r="F38" s="6">
+        <f>'توقع المحصل (المراقبة)'!E31+'توقع المحصل (المراقبة)'!N31</f>
+        <v/>
+      </c>
+      <c r="G38" s="6" t="n">
+        <v>210967.17</v>
+      </c>
+      <c r="H38" s="6" t="n">
+        <v>140781.12</v>
+      </c>
+      <c r="I38" s="6">
+        <f>'توقع المحصل (المراقبة)'!L31*Q38</f>
+        <v/>
+      </c>
+      <c r="J38" s="6">
+        <f>'توقع المحصل (المراقبة)'!O31*Q38</f>
+        <v/>
+      </c>
+      <c r="K38" s="6" t="n">
+        <v>150620.18</v>
+      </c>
+      <c r="L38" s="6" t="n">
+        <v>98514.17</v>
+      </c>
+      <c r="M38" s="6">
+        <f>'توقع المحصل (المراقبة)'!L31*(1-Q38)</f>
+        <v/>
+      </c>
+      <c r="N38" s="6">
+        <f>'توقع المحصل (المراقبة)'!O31*(1-Q38)</f>
+        <v/>
+      </c>
+      <c r="O38" s="6" t="n">
+        <v>150849.35</v>
+      </c>
+      <c r="P38" s="6" t="n">
+        <v>98721.61</v>
+      </c>
+      <c r="Q38" s="19" t="n">
+        <v>0.7126</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="5" t="inlineStr">
+        <is>
+          <t>11452106</t>
+        </is>
+      </c>
+      <c r="B39" s="5">
+        <f>'توقع المحصل (المراقبة)'!B32</f>
+        <v/>
+      </c>
+      <c r="C39" s="5">
+        <f>'توقع المحصل (المراقبة)'!C32</f>
+        <v/>
+      </c>
+      <c r="D39" s="6">
+        <f>'توقع المحصل (المراقبة)'!E32</f>
+        <v/>
+      </c>
+      <c r="E39" s="6">
+        <f>'توقع المحصل (المراقبة)'!E32+'توقع المحصل (المراقبة)'!K32</f>
+        <v/>
+      </c>
+      <c r="F39" s="6">
+        <f>'توقع المحصل (المراقبة)'!E32+'توقع المحصل (المراقبة)'!N32</f>
+        <v/>
+      </c>
+      <c r="G39" s="6" t="n">
+        <v>759323.62</v>
+      </c>
+      <c r="H39" s="6" t="n">
+        <v>741972.55</v>
+      </c>
+      <c r="I39" s="6">
+        <f>'توقع المحصل (المراقبة)'!L32*Q39</f>
+        <v/>
+      </c>
+      <c r="J39" s="6">
+        <f>'توقع المحصل (المراقبة)'!O32*Q39</f>
+        <v/>
+      </c>
+      <c r="K39" s="6" t="n">
+        <v>685167.54</v>
+      </c>
+      <c r="L39" s="6" t="n">
+        <v>654274.2</v>
+      </c>
+      <c r="M39" s="6">
+        <f>'توقع المحصل (المراقبة)'!L32*(1-Q39)</f>
+        <v/>
+      </c>
+      <c r="N39" s="6">
+        <f>'توقع المحصل (المراقبة)'!O32*(1-Q39)</f>
+        <v/>
+      </c>
+      <c r="O39" s="6" t="n">
+        <v>572770.48</v>
+      </c>
+      <c r="P39" s="6" t="n">
+        <v>558666.08</v>
+      </c>
+      <c r="Q39" s="19" t="n">
+        <v>0.4988</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>11452110</t>
+        </is>
+      </c>
+      <c r="B40" s="5">
+        <f>'توقع المحصل (المراقبة)'!B33</f>
+        <v/>
+      </c>
+      <c r="C40" s="5">
+        <f>'توقع المحصل (المراقبة)'!C33</f>
+        <v/>
+      </c>
+      <c r="D40" s="6">
+        <f>'توقع المحصل (المراقبة)'!E33</f>
+        <v/>
+      </c>
+      <c r="E40" s="6">
+        <f>'توقع المحصل (المراقبة)'!E33+'توقع المحصل (المراقبة)'!K33</f>
+        <v/>
+      </c>
+      <c r="F40" s="6">
+        <f>'توقع المحصل (المراقبة)'!E33+'توقع المحصل (المراقبة)'!N33</f>
+        <v/>
+      </c>
+      <c r="G40" s="6" t="n">
+        <v>99448.75999999999</v>
+      </c>
+      <c r="H40" s="6" t="n">
+        <v>91679.33</v>
+      </c>
+      <c r="I40" s="6">
+        <f>'توقع المحصل (المراقبة)'!L33*Q40</f>
+        <v/>
+      </c>
+      <c r="J40" s="6">
+        <f>'توقع المحصل (المراقبة)'!O33*Q40</f>
+        <v/>
+      </c>
+      <c r="K40" s="6" t="n">
+        <v>88463.77</v>
+      </c>
+      <c r="L40" s="6" t="n">
+        <v>79248.89999999999</v>
+      </c>
+      <c r="M40" s="6">
+        <f>'توقع المحصل (المراقبة)'!L33*(1-Q40)</f>
+        <v/>
+      </c>
+      <c r="N40" s="6">
+        <f>'توقع المحصل (المراقبة)'!O33*(1-Q40)</f>
+        <v/>
+      </c>
+      <c r="O40" s="6" t="n">
+        <v>146186.3</v>
+      </c>
+      <c r="P40" s="6" t="n">
+        <v>141754.94</v>
+      </c>
+      <c r="Q40" s="19" t="n">
+        <v>0.6289</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="5" t="inlineStr">
+        <is>
+          <t>1422104</t>
+        </is>
+      </c>
+      <c r="B41" s="5">
+        <f>'توقع المحصل (المراقبة)'!B34</f>
+        <v/>
+      </c>
+      <c r="C41" s="5">
+        <f>'توقع المحصل (المراقبة)'!C34</f>
+        <v/>
+      </c>
+      <c r="D41" s="6">
+        <f>'توقع المحصل (المراقبة)'!E34</f>
+        <v/>
+      </c>
+      <c r="E41" s="6">
+        <f>'توقع المحصل (المراقبة)'!E34+'توقع المحصل (المراقبة)'!K34</f>
+        <v/>
+      </c>
+      <c r="F41" s="6">
+        <f>'توقع المحصل (المراقبة)'!E34+'توقع المحصل (المراقبة)'!N34</f>
+        <v/>
+      </c>
+      <c r="G41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I41" s="6">
+        <f>'توقع المحصل (المراقبة)'!L34*Q41</f>
+        <v/>
+      </c>
+      <c r="J41" s="6">
+        <f>'توقع المحصل (المراقبة)'!O34*Q41</f>
+        <v/>
+      </c>
+      <c r="K41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M41" s="6">
+        <f>'توقع المحصل (المراقبة)'!L34*(1-Q41)</f>
+        <v/>
+      </c>
+      <c r="N41" s="6">
+        <f>'توقع المحصل (المراقبة)'!O34*(1-Q41)</f>
+        <v/>
+      </c>
+      <c r="O41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P41" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>3318212</t>
+        </is>
+      </c>
+      <c r="B42" s="5">
+        <f>'توقع المحصل (المراقبة)'!B35</f>
+        <v/>
+      </c>
+      <c r="C42" s="5">
+        <f>'توقع المحصل (المراقبة)'!C35</f>
+        <v/>
+      </c>
+      <c r="D42" s="6">
+        <f>'توقع المحصل (المراقبة)'!E35</f>
+        <v/>
+      </c>
+      <c r="E42" s="6">
+        <f>'توقع المحصل (المراقبة)'!E35+'توقع المحصل (المراقبة)'!K35</f>
+        <v/>
+      </c>
+      <c r="F42" s="6">
+        <f>'توقع المحصل (المراقبة)'!E35+'توقع المحصل (المراقبة)'!N35</f>
+        <v/>
+      </c>
+      <c r="G42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I42" s="6">
+        <f>'توقع المحصل (المراقبة)'!L35*Q42</f>
+        <v/>
+      </c>
+      <c r="J42" s="6">
+        <f>'توقع المحصل (المراقبة)'!O35*Q42</f>
+        <v/>
+      </c>
+      <c r="K42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M42" s="6">
+        <f>'توقع المحصل (المراقبة)'!L35*(1-Q42)</f>
+        <v/>
+      </c>
+      <c r="N42" s="6">
+        <f>'توقع المحصل (المراقبة)'!O35*(1-Q42)</f>
+        <v/>
+      </c>
+      <c r="O42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P42" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>1421903</t>
+        </is>
+      </c>
+      <c r="B43" s="5">
+        <f>'توقع المحصل (المراقبة)'!B36</f>
+        <v/>
+      </c>
+      <c r="C43" s="5">
+        <f>'توقع المحصل (المراقبة)'!C36</f>
+        <v/>
+      </c>
+      <c r="D43" s="6">
+        <f>'توقع المحصل (المراقبة)'!E36</f>
+        <v/>
+      </c>
+      <c r="E43" s="6">
+        <f>'توقع المحصل (المراقبة)'!E36+'توقع المحصل (المراقبة)'!K36</f>
+        <v/>
+      </c>
+      <c r="F43" s="6">
+        <f>'توقع المحصل (المراقبة)'!E36+'توقع المحصل (المراقبة)'!N36</f>
+        <v/>
+      </c>
+      <c r="G43" s="6" t="n">
+        <v>187900</v>
+      </c>
+      <c r="H43" s="6" t="n">
+        <v>187900</v>
+      </c>
+      <c r="I43" s="6">
+        <f>'توقع المحصل (المراقبة)'!L36*Q43</f>
+        <v/>
+      </c>
+      <c r="J43" s="6">
+        <f>'توقع المحصل (المراقبة)'!O36*Q43</f>
+        <v/>
+      </c>
+      <c r="K43" s="6" t="n">
+        <v>219900</v>
+      </c>
+      <c r="L43" s="6" t="n">
+        <v>219900</v>
+      </c>
+      <c r="M43" s="6">
+        <f>'توقع المحصل (المراقبة)'!L36*(1-Q43)</f>
+        <v/>
+      </c>
+      <c r="N43" s="6">
+        <f>'توقع المحصل (المراقبة)'!O36*(1-Q43)</f>
+        <v/>
+      </c>
+      <c r="O43" s="6" t="n">
+        <v>298820</v>
+      </c>
+      <c r="P43" s="6" t="n">
+        <v>298820</v>
+      </c>
+      <c r="Q43" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>141229</t>
+        </is>
+      </c>
+      <c r="B44" s="5">
+        <f>'توقع المحصل (المراقبة)'!B37</f>
+        <v/>
+      </c>
+      <c r="C44" s="5">
+        <f>'توقع المحصل (المراقبة)'!C37</f>
+        <v/>
+      </c>
+      <c r="D44" s="6">
+        <f>'توقع المحصل (المراقبة)'!E37</f>
+        <v/>
+      </c>
+      <c r="E44" s="6">
+        <f>'توقع المحصل (المراقبة)'!E37+'توقع المحصل (المراقبة)'!K37</f>
+        <v/>
+      </c>
+      <c r="F44" s="6">
+        <f>'توقع المحصل (المراقبة)'!E37+'توقع المحصل (المراقبة)'!N37</f>
+        <v/>
+      </c>
+      <c r="G44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I44" s="6">
+        <f>'توقع المحصل (المراقبة)'!L37*Q44</f>
+        <v/>
+      </c>
+      <c r="J44" s="6">
+        <f>'توقع المحصل (المراقبة)'!O37*Q44</f>
+        <v/>
+      </c>
+      <c r="K44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M44" s="6">
+        <f>'توقع المحصل (المراقبة)'!L37*(1-Q44)</f>
+        <v/>
+      </c>
+      <c r="N44" s="6">
+        <f>'توقع المحصل (المراقبة)'!O37*(1-Q44)</f>
+        <v/>
+      </c>
+      <c r="O44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P44" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="19" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="5" t="inlineStr">
+        <is>
+          <t>1438</t>
+        </is>
+      </c>
+      <c r="B45" s="5">
+        <f>'توقع المحصل (المراقبة)'!B38</f>
+        <v/>
+      </c>
+      <c r="C45" s="5">
+        <f>'توقع المحصل (المراقبة)'!C38</f>
+        <v/>
+      </c>
+      <c r="D45" s="6">
+        <f>'توقع المحصل (المراقبة)'!E38</f>
+        <v/>
+      </c>
+      <c r="E45" s="6">
+        <f>'توقع المحصل (المراقبة)'!E38+'توقع المحصل (المراقبة)'!K38</f>
+        <v/>
+      </c>
+      <c r="F45" s="6">
+        <f>'توقع المحصل (المراقبة)'!E38+'توقع المحصل (المراقبة)'!N38</f>
+        <v/>
+      </c>
+      <c r="G45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I45" s="6">
+        <f>'توقع المحصل (المراقبة)'!L38*Q45</f>
+        <v/>
+      </c>
+      <c r="J45" s="6">
+        <f>'توقع المحصل (المراقبة)'!O38*Q45</f>
+        <v/>
+      </c>
+      <c r="K45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M45" s="6">
+        <f>'توقع المحصل (المراقبة)'!L38*(1-Q45)</f>
+        <v/>
+      </c>
+      <c r="N45" s="6">
+        <f>'توقع المحصل (المراقبة)'!O38*(1-Q45)</f>
+        <v/>
+      </c>
+      <c r="O45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P45" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="19" t="n">
+        <v>0.4401</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>1421907</t>
+        </is>
+      </c>
+      <c r="B46" s="5">
+        <f>'توقع المحصل (المراقبة)'!B39</f>
+        <v/>
+      </c>
+      <c r="C46" s="5">
+        <f>'توقع المحصل (المراقبة)'!C39</f>
+        <v/>
+      </c>
+      <c r="D46" s="6">
+        <f>'توقع المحصل (المراقبة)'!E39</f>
+        <v/>
+      </c>
+      <c r="E46" s="6">
+        <f>'توقع المحصل (المراقبة)'!E39+'توقع المحصل (المراقبة)'!K39</f>
+        <v/>
+      </c>
+      <c r="F46" s="6">
+        <f>'توقع المحصل (المراقبة)'!E39+'توقع المحصل (المراقبة)'!N39</f>
+        <v/>
+      </c>
+      <c r="G46" s="6" t="n">
+        <v>55366.58</v>
+      </c>
+      <c r="H46" s="6" t="n">
+        <v>55366.58</v>
+      </c>
+      <c r="I46" s="6">
+        <f>'توقع المحصل (المراقبة)'!L39*Q46</f>
+        <v/>
+      </c>
+      <c r="J46" s="6">
+        <f>'توقع المحصل (المراقبة)'!O39*Q46</f>
+        <v/>
+      </c>
+      <c r="K46" s="6" t="n">
+        <v>32730.78</v>
+      </c>
+      <c r="L46" s="6" t="n">
+        <v>32730.78</v>
+      </c>
+      <c r="M46" s="6">
+        <f>'توقع المحصل (المراقبة)'!L39*(1-Q46)</f>
+        <v/>
+      </c>
+      <c r="N46" s="6">
+        <f>'توقع المحصل (المراقبة)'!O39*(1-Q46)</f>
+        <v/>
+      </c>
+      <c r="O46" s="6" t="n">
+        <v>26407.51</v>
+      </c>
+      <c r="P46" s="6" t="n">
+        <v>26407.51</v>
+      </c>
+      <c r="Q46" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="5" t="inlineStr">
+        <is>
+          <t>11452105</t>
+        </is>
+      </c>
+      <c r="B47" s="5">
+        <f>'توقع المحصل (المراقبة)'!B40</f>
+        <v/>
+      </c>
+      <c r="C47" s="5">
+        <f>'توقع المحصل (المراقبة)'!C40</f>
+        <v/>
+      </c>
+      <c r="D47" s="6">
+        <f>'توقع المحصل (المراقبة)'!E40</f>
+        <v/>
+      </c>
+      <c r="E47" s="6">
+        <f>'توقع المحصل (المراقبة)'!E40+'توقع المحصل (المراقبة)'!K40</f>
+        <v/>
+      </c>
+      <c r="F47" s="6">
+        <f>'توقع المحصل (المراقبة)'!E40+'توقع المحصل (المراقبة)'!N40</f>
+        <v/>
+      </c>
+      <c r="G47" s="6" t="n">
+        <v>32296.3</v>
+      </c>
+      <c r="H47" s="6" t="n">
+        <v>9335.940000000001</v>
+      </c>
+      <c r="I47" s="6">
+        <f>'توقع المحصل (المراقبة)'!L40*Q47</f>
+        <v/>
+      </c>
+      <c r="J47" s="6">
+        <f>'توقع المحصل (المراقبة)'!O40*Q47</f>
+        <v/>
+      </c>
+      <c r="K47" s="6" t="n">
+        <v>27957.08</v>
+      </c>
+      <c r="L47" s="6" t="n">
+        <v>7407.4</v>
+      </c>
+      <c r="M47" s="6">
+        <f>'توقع المحصل (المراقبة)'!L40*(1-Q47)</f>
+        <v/>
+      </c>
+      <c r="N47" s="6">
+        <f>'توقع المحصل (المراقبة)'!O40*(1-Q47)</f>
+        <v/>
+      </c>
+      <c r="O47" s="6" t="n">
+        <v>25146.7</v>
+      </c>
+      <c r="P47" s="6" t="n">
+        <v>6755.12</v>
+      </c>
+      <c r="Q47" s="19" t="n">
+        <v>0.6049</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>11452513</t>
+        </is>
+      </c>
+      <c r="B48" s="5">
+        <f>'توقع المحصل (المراقبة)'!B41</f>
+        <v/>
+      </c>
+      <c r="C48" s="5">
+        <f>'توقع المحصل (المراقبة)'!C41</f>
+        <v/>
+      </c>
+      <c r="D48" s="6">
+        <f>'توقع المحصل (المراقبة)'!E41</f>
+        <v/>
+      </c>
+      <c r="E48" s="6">
+        <f>'توقع المحصل (المراقبة)'!E41+'توقع المحصل (المراقبة)'!K41</f>
+        <v/>
+      </c>
+      <c r="F48" s="6">
+        <f>'توقع المحصل (المراقبة)'!E41+'توقع المحصل (المراقبة)'!N41</f>
+        <v/>
+      </c>
+      <c r="G48" s="6" t="n">
+        <v>5715</v>
+      </c>
+      <c r="H48" s="6" t="n">
+        <v>5715</v>
+      </c>
+      <c r="I48" s="6">
+        <f>'توقع المحصل (المراقبة)'!L41*Q48</f>
+        <v/>
+      </c>
+      <c r="J48" s="6">
+        <f>'توقع المحصل (المراقبة)'!O41*Q48</f>
+        <v/>
+      </c>
+      <c r="K48" s="6" t="n">
+        <v>5723</v>
+      </c>
+      <c r="L48" s="6" t="n">
+        <v>5723</v>
+      </c>
+      <c r="M48" s="6">
+        <f>'توقع المحصل (المراقبة)'!L41*(1-Q48)</f>
+        <v/>
+      </c>
+      <c r="N48" s="6">
+        <f>'توقع المحصل (المراقبة)'!O41*(1-Q48)</f>
+        <v/>
+      </c>
+      <c r="O48" s="6" t="n">
+        <v>7794</v>
+      </c>
+      <c r="P48" s="6" t="n">
+        <v>7794.71</v>
+      </c>
+      <c r="Q48" s="19" t="n">
+        <v>0.619</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="5" t="inlineStr">
+        <is>
+          <t>1422103</t>
+        </is>
+      </c>
+      <c r="B49" s="5">
+        <f>'توقع المحصل (المراقبة)'!B42</f>
+        <v/>
+      </c>
+      <c r="C49" s="5">
+        <f>'توقع المحصل (المراقبة)'!C42</f>
+        <v/>
+      </c>
+      <c r="D49" s="6">
+        <f>'توقع المحصل (المراقبة)'!E42</f>
+        <v/>
+      </c>
+      <c r="E49" s="6">
+        <f>'توقع المحصل (المراقبة)'!E42+'توقع المحصل (المراقبة)'!K42</f>
+        <v/>
+      </c>
+      <c r="F49" s="6">
+        <f>'توقع المحصل (المراقبة)'!E42+'توقع المحصل (المراقبة)'!N42</f>
+        <v/>
+      </c>
+      <c r="G49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I49" s="6">
+        <f>'توقع المحصل (المراقبة)'!L42*Q49</f>
+        <v/>
+      </c>
+      <c r="J49" s="6">
+        <f>'توقع المحصل (المراقبة)'!O42*Q49</f>
+        <v/>
+      </c>
+      <c r="K49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M49" s="6">
+        <f>'توقع المحصل (المراقبة)'!L42*(1-Q49)</f>
+        <v/>
+      </c>
+      <c r="N49" s="6">
+        <f>'توقع المحصل (المراقبة)'!O42*(1-Q49)</f>
+        <v/>
+      </c>
+      <c r="O49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P49" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="19" t="n">
+        <v>0.8496</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>11452109</t>
+        </is>
+      </c>
+      <c r="B50" s="5">
+        <f>'توقع المحصل (المراقبة)'!B43</f>
+        <v/>
+      </c>
+      <c r="C50" s="5">
+        <f>'توقع المحصل (المراقبة)'!C43</f>
+        <v/>
+      </c>
+      <c r="D50" s="6">
+        <f>'توقع المحصل (المراقبة)'!E43</f>
+        <v/>
+      </c>
+      <c r="E50" s="6">
+        <f>'توقع المحصل (المراقبة)'!E43+'توقع المحصل (المراقبة)'!K43</f>
+        <v/>
+      </c>
+      <c r="F50" s="6">
+        <f>'توقع المحصل (المراقبة)'!E43+'توقع المحصل (المراقبة)'!N43</f>
+        <v/>
+      </c>
+      <c r="G50" s="6" t="n">
+        <v>212196.25</v>
+      </c>
+      <c r="H50" s="6" t="n">
+        <v>212196.25</v>
+      </c>
+      <c r="I50" s="6">
+        <f>'توقع المحصل (المراقبة)'!L43*Q50</f>
+        <v/>
+      </c>
+      <c r="J50" s="6">
+        <f>'توقع المحصل (المراقبة)'!O43*Q50</f>
+        <v/>
+      </c>
+      <c r="K50" s="6" t="n">
+        <v>49663.18</v>
+      </c>
+      <c r="L50" s="6" t="n">
+        <v>49663.18</v>
+      </c>
+      <c r="M50" s="6">
+        <f>'توقع المحصل (المراقبة)'!L43*(1-Q50)</f>
+        <v/>
+      </c>
+      <c r="N50" s="6">
+        <f>'توقع المحصل (المراقبة)'!O43*(1-Q50)</f>
+        <v/>
+      </c>
+      <c r="O50" s="6" t="n">
+        <v>185890.8</v>
+      </c>
+      <c r="P50" s="6" t="n">
+        <v>185890.8</v>
+      </c>
+      <c r="Q50" s="19" t="n">
+        <v>0.2869</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="5" t="inlineStr">
+        <is>
+          <t>11422</t>
+        </is>
+      </c>
+      <c r="B51" s="5">
+        <f>'توقع المحصل (المراقبة)'!B44</f>
+        <v/>
+      </c>
+      <c r="C51" s="5">
+        <f>'توقع المحصل (المراقبة)'!C44</f>
+        <v/>
+      </c>
+      <c r="D51" s="6">
+        <f>'توقع المحصل (المراقبة)'!E44</f>
+        <v/>
+      </c>
+      <c r="E51" s="6">
+        <f>'توقع المحصل (المراقبة)'!E44+'توقع المحصل (المراقبة)'!K44</f>
+        <v/>
+      </c>
+      <c r="F51" s="6">
+        <f>'توقع المحصل (المراقبة)'!E44+'توقع المحصل (المراقبة)'!N44</f>
+        <v/>
+      </c>
+      <c r="G51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I51" s="6">
+        <f>'توقع المحصل (المراقبة)'!L44*Q51</f>
+        <v/>
+      </c>
+      <c r="J51" s="6">
+        <f>'توقع المحصل (المراقبة)'!O44*Q51</f>
+        <v/>
+      </c>
+      <c r="K51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M51" s="6">
+        <f>'توقع المحصل (المراقبة)'!L44*(1-Q51)</f>
+        <v/>
+      </c>
+      <c r="N51" s="6">
+        <f>'توقع المحصل (المراقبة)'!O44*(1-Q51)</f>
+        <v/>
+      </c>
+      <c r="O51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P51" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>142161</t>
+        </is>
+      </c>
+      <c r="B52" s="5">
+        <f>'توقع المحصل (المراقبة)'!B45</f>
+        <v/>
+      </c>
+      <c r="C52" s="5">
+        <f>'توقع المحصل (المراقبة)'!C45</f>
+        <v/>
+      </c>
+      <c r="D52" s="6">
+        <f>'توقع المحصل (المراقبة)'!E45</f>
+        <v/>
+      </c>
+      <c r="E52" s="6">
+        <f>'توقع المحصل (المراقبة)'!E45+'توقع المحصل (المراقبة)'!K45</f>
+        <v/>
+      </c>
+      <c r="F52" s="6">
+        <f>'توقع المحصل (المراقبة)'!E45+'توقع المحصل (المراقبة)'!N45</f>
+        <v/>
+      </c>
+      <c r="G52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I52" s="6">
+        <f>'توقع المحصل (المراقبة)'!L45*Q52</f>
+        <v/>
+      </c>
+      <c r="J52" s="6">
+        <f>'توقع المحصل (المراقبة)'!O45*Q52</f>
+        <v/>
+      </c>
+      <c r="K52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M52" s="6">
+        <f>'توقع المحصل (المراقبة)'!L45*(1-Q52)</f>
+        <v/>
+      </c>
+      <c r="N52" s="6">
+        <f>'توقع المحصل (المراقبة)'!O45*(1-Q52)</f>
+        <v/>
+      </c>
+      <c r="O52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P52" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="5" t="inlineStr">
+        <is>
+          <t>1421908</t>
+        </is>
+      </c>
+      <c r="B53" s="5">
+        <f>'توقع المحصل (المراقبة)'!B46</f>
+        <v/>
+      </c>
+      <c r="C53" s="5">
+        <f>'توقع المحصل (المراقبة)'!C46</f>
+        <v/>
+      </c>
+      <c r="D53" s="6">
+        <f>'توقع المحصل (المراقبة)'!E46</f>
+        <v/>
+      </c>
+      <c r="E53" s="6">
+        <f>'توقع المحصل (المراقبة)'!E46+'توقع المحصل (المراقبة)'!K46</f>
+        <v/>
+      </c>
+      <c r="F53" s="6">
+        <f>'توقع المحصل (المراقبة)'!E46+'توقع المحصل (المراقبة)'!N46</f>
+        <v/>
+      </c>
+      <c r="G53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I53" s="6">
+        <f>'توقع المحصل (المراقبة)'!L46*Q53</f>
+        <v/>
+      </c>
+      <c r="J53" s="6">
+        <f>'توقع المحصل (المراقبة)'!O46*Q53</f>
+        <v/>
+      </c>
+      <c r="K53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M53" s="6">
+        <f>'توقع المحصل (المراقبة)'!L46*(1-Q53)</f>
+        <v/>
+      </c>
+      <c r="N53" s="6">
+        <f>'توقع المحصل (المراقبة)'!O46*(1-Q53)</f>
+        <v/>
+      </c>
+      <c r="O53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P53" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>1422112</t>
+        </is>
+      </c>
+      <c r="B54" s="5">
+        <f>'توقع المحصل (المراقبة)'!B47</f>
+        <v/>
+      </c>
+      <c r="C54" s="5">
+        <f>'توقع المحصل (المراقبة)'!C47</f>
+        <v/>
+      </c>
+      <c r="D54" s="6">
+        <f>'توقع المحصل (المراقبة)'!E47</f>
+        <v/>
+      </c>
+      <c r="E54" s="6">
+        <f>'توقع المحصل (المراقبة)'!E47+'توقع المحصل (المراقبة)'!K47</f>
+        <v/>
+      </c>
+      <c r="F54" s="6">
+        <f>'توقع المحصل (المراقبة)'!E47+'توقع المحصل (المراقبة)'!N47</f>
+        <v/>
+      </c>
+      <c r="G54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I54" s="6">
+        <f>'توقع المحصل (المراقبة)'!L47*Q54</f>
+        <v/>
+      </c>
+      <c r="J54" s="6">
+        <f>'توقع المحصل (المراقبة)'!O47*Q54</f>
+        <v/>
+      </c>
+      <c r="K54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M54" s="6">
+        <f>'توقع المحصل (المراقبة)'!L47*(1-Q54)</f>
+        <v/>
+      </c>
+      <c r="N54" s="6">
+        <f>'توقع المحصل (المراقبة)'!O47*(1-Q54)</f>
+        <v/>
+      </c>
+      <c r="O54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P54" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="5" t="inlineStr">
+        <is>
+          <t>1422199</t>
+        </is>
+      </c>
+      <c r="B55" s="5">
+        <f>'توقع المحصل (المراقبة)'!B48</f>
+        <v/>
+      </c>
+      <c r="C55" s="5">
+        <f>'توقع المحصل (المراقبة)'!C48</f>
+        <v/>
+      </c>
+      <c r="D55" s="6">
+        <f>'توقع المحصل (المراقبة)'!E48</f>
+        <v/>
+      </c>
+      <c r="E55" s="6">
+        <f>'توقع المحصل (المراقبة)'!E48+'توقع المحصل (المراقبة)'!K48</f>
+        <v/>
+      </c>
+      <c r="F55" s="6">
+        <f>'توقع المحصل (المراقبة)'!E48+'توقع المحصل (المراقبة)'!N48</f>
+        <v/>
+      </c>
+      <c r="G55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="I55" s="6">
+        <f>'توقع المحصل (المراقبة)'!L48*Q55</f>
+        <v/>
+      </c>
+      <c r="J55" s="6">
+        <f>'توقع المحصل (المراقبة)'!O48*Q55</f>
+        <v/>
+      </c>
+      <c r="K55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="M55" s="6">
+        <f>'توقع المحصل (المراقبة)'!L48*(1-Q55)</f>
+        <v/>
+      </c>
+      <c r="N55" s="6">
+        <f>'توقع المحصل (المراقبة)'!O48*(1-Q55)</f>
+        <v/>
+      </c>
+      <c r="O55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="P55" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="19" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="8" t="n"/>
+      <c r="B56" s="8" t="inlineStr">
+        <is>
+          <t>الإجمالي</t>
+        </is>
+      </c>
+      <c r="C56" s="8" t="n"/>
+      <c r="D56" s="9">
+        <f>SUM(D13:D55)</f>
+        <v/>
+      </c>
+      <c r="E56" s="9">
+        <f>SUM(E13:E55)</f>
+        <v/>
+      </c>
+      <c r="F56" s="9">
+        <f>SUM(F13:F55)</f>
+        <v/>
+      </c>
+      <c r="G56" s="9">
+        <f>SUM(G13:G55)</f>
+        <v/>
+      </c>
+      <c r="H56" s="9">
+        <f>SUM(H13:H55)</f>
+        <v/>
+      </c>
+      <c r="I56" s="9">
+        <f>SUM(I13:I55)</f>
+        <v/>
+      </c>
+      <c r="J56" s="9">
+        <f>SUM(J13:J55)</f>
+        <v/>
+      </c>
+      <c r="K56" s="9">
+        <f>SUM(K13:K55)</f>
+        <v/>
+      </c>
+      <c r="L56" s="9">
+        <f>SUM(L13:L55)</f>
+        <v/>
+      </c>
+      <c r="M56" s="9">
+        <f>SUM(M13:M55)</f>
+        <v/>
+      </c>
+      <c r="N56" s="9">
+        <f>SUM(N13:N55)</f>
+        <v/>
+      </c>
+      <c r="O56" s="9">
+        <f>SUM(O13:O55)</f>
+        <v/>
+      </c>
+      <c r="P56" s="9">
+        <f>SUM(P13:P55)</f>
+        <v/>
+      </c>
+      <c r="Q56" s="20" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A12:Q55"/>
+  <mergeCells count="1">
+    <mergeCell ref="A2:Q2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="60" customWidth="1" min="1" max="1"/>
@@ -3510,7 +6654,7 @@
           <t>معامل تحويل 2026 إلى سنة كاملة (12÷9)</t>
         </is>
       </c>
-      <c r="B4" s="19">
+      <c r="B4" s="21">
         <f>12/9</f>
         <v/>
       </c>
@@ -3526,7 +6670,7 @@
           <t>نسبة النمو – السيناريو الأول (ثابتة)</t>
         </is>
       </c>
-      <c r="B5" s="20">
+      <c r="B5" s="22">
         <f>التوقعات!C2</f>
         <v/>
       </c>
@@ -3542,7 +6686,7 @@
           <t>سقف معدل النمو التاريخي (±)</t>
         </is>
       </c>
-      <c r="B6" s="20" t="n">
+      <c r="B6" s="22" t="n">
         <v>0.25</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -3557,7 +6701,7 @@
           <t>أدنى معامل اتجاه 2026 (توقع المحصل الموسمي)</t>
         </is>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="23" t="n">
         <v>0.5</v>
       </c>
       <c r="C7" t="inlineStr">
@@ -3572,7 +6716,7 @@
           <t>أعلى معامل اتجاه 2026 (توقع المحصل الموسمي)</t>
         </is>
       </c>
-      <c r="B8" s="21" t="n">
+      <c r="B8" s="23" t="n">
         <v>1.5</v>
       </c>
       <c r="C8" t="inlineStr">
@@ -3589,84 +6733,91 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="22" t="inlineStr">
+      <c r="A10" s="24" t="inlineStr">
         <is>
           <t>1) الإجمالي المفوتر للحساب = المفوتر + المحصل عن سنوات سابقة (حسب طلبك).</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="22" t="inlineStr">
+      <c r="A11" s="24" t="inlineStr">
         <is>
           <t>2) توقع 2026 = الفعلي حتى سبتمبر × 12/9 (لا توجد بيانات شهرية، فلا موسمية في التوقع).</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="22" t="inlineStr">
+      <c r="A12" s="24" t="inlineStr">
         <is>
           <t>3) الحسابات التي فوترتها وتحصيلها صفر في 2026 تُعتبر متوقفة وتوقعها صفر في 2026 و2027.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="22" t="inlineStr">
+      <c r="A13" s="24" t="inlineStr">
         <is>
           <t>4) 2027 – السيناريو الأول: توقع 2026 × (1 + نسبة النمو في خلية C2 بورقة التوقعات؛ الافتراضي 7%).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="22" t="inlineStr">
+      <c r="A14" s="24" t="inlineStr">
         <is>
           <t>5) 2027 – السيناريو الثاني: توقع 2026 × (1 + معدل النمو السنوي المركب التاريخي للحساب بين أول سنة فيها فوترة و2025، بسقف ±25%). إن توفرت سنة واحدة فقط من البيانات = نمو 0%.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="22" t="inlineStr">
+      <c r="A15" s="24" t="inlineStr">
         <is>
           <t>6) تم استبعاد حساب قيمة الضريبة المضافة (11411) من كل الحسابات والإجماليات.</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="22" t="inlineStr">
+      <c r="A16" s="24" t="inlineStr">
         <is>
           <t>6b) تم دمج صفّي "بدون رقم" (خدمات علم + جزاءات، وجزاءات جزء ضئيل) في صف واحد لكل سنة.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="22" t="inlineStr">
+      <c r="A17" s="24" t="inlineStr">
         <is>
           <t>6c) أعمدة النمو لكل حساب: نمو كل سنة عن السنة السابقة (2024 عن 2023، 2025 عن 2024، 2026 توقع عن 2025، و2027 عن 2026 للسيناريوهين). تظهر فارغة عندما تكون السنة السابقة صفراً.</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="22" t="inlineStr">
+      <c r="A18" s="24" t="inlineStr">
         <is>
           <t>6d) ورقة "توقع المحصل 2026": توقع إقفال 2026 كمحصّل فعلي = المحصل حتى سبتمبر × 12÷9 (مسدد عن السنة + محصل سنوات سابقة).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="22" t="inlineStr">
+      <c r="A19" s="24" t="inlineStr">
         <is>
           <t>6e) إعادة تصنيف المحصل: حسب تأكيد المستخدم، نُقل 913م من محصل 2025 في حساب اللوحات الدعائية (142113) إلى تأجير المرافق (142162) (كلها من إدارة الدعم المالي: مايو 291م ونوفمبر 594م). ينطبق على أوراق المحصل فقط؛ أوراق الفوترة لم تُعدّل لأن مبالغ الفوترة حسب الجهة غير متوفرة. إن كانت دفعات إدارة الدعم المالي في 2024 (يوليو 312م، نوفمبر 25م، ديسمبر 102م) من نفس النوع فالتوقع الأساسي يرتفع (انظر الرد).</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="22" t="inlineStr">
+      <c r="A20" s="24" t="inlineStr">
         <is>
           <t>6f) ورقة "توقع المحصل (المراقبة)": الفعلي يناير–أكتوبر 2026 من ملف المراقبة (ورقة الإجمالي، قبل الاستقطاع)، ثم متبقي أكتوبر ونوفمبر وديسمبر بالموسمية الشهرية.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="22" t="inlineStr">
+      <c r="A21" s="24" t="inlineStr">
+        <is>
+          <t>6g) ورقة "الأشهر المتبقية 2026": أكتوبر ونوفمبر وديسمبر (المحصل حتى تاريخه والمتوقع أساسي وأسوأ) مقابل المستهدف والمقدر من ملف المراقبة.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="24" t="inlineStr">
         <is>
           <t>7) تنبيه: كثير من الحسابات تتذبذب بشدة بين السنوات (لوحات دعائية، تأجير المرافق، إيرادات متنوعة)، ومضاعفة 2026 على 12/9 تضخّم أو تقلّل هذه الأرقام؛ انظر عمود "تنبيه".</t>
         </is>

</xml_diff>